<commit_message>
index change to remove mock services and the data model file
</commit_message>
<xml_diff>
--- a/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
+++ b/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Loyalty Program\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MynikaTech\memgine\docs\domain\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{646D5A51-6C36-4BD2-8DEB-5E38F5904CBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17ED9FA7-6F98-478F-A575-B59115CC1FBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{AA28BC4D-8219-43B9-8C16-6977709D904A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{AA28BC4D-8219-43B9-8C16-6977709D904A}"/>
   </bookViews>
   <sheets>
     <sheet name="Entity Catalogue" sheetId="1" r:id="rId1"/>
@@ -8379,7 +8379,7 @@
         <v>1139</v>
       </c>
     </row>
-    <row r="22" spans="1:17" ht="45">
+    <row r="22" spans="1:17" ht="30">
       <c r="A22" s="4" t="s">
         <v>1173</v>
       </c>
@@ -14481,7 +14481,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="78" spans="1:23" ht="45">
+    <row r="78" spans="1:23" ht="30">
       <c r="A78" s="4" t="s">
         <v>10</v>
       </c>
@@ -14552,7 +14552,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="79" spans="1:23" ht="45">
+    <row r="79" spans="1:23" ht="30">
       <c r="A79" s="4" t="s">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Status Ref data changes -  generic and out of ref data services
</commit_message>
<xml_diff>
--- a/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
+++ b/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MynikaTech\memgine\docs\domain\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17ED9FA7-6F98-478F-A575-B59115CC1FBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D0E5EAC-9517-4640-A34C-6226E976EC36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{AA28BC4D-8219-43B9-8C16-6977709D904A}"/>
   </bookViews>
@@ -16,13 +16,14 @@
     <sheet name="Entity Catalogue" sheetId="1" r:id="rId1"/>
     <sheet name="Atributes" sheetId="2" r:id="rId2"/>
     <sheet name="Reference Data" sheetId="3" r:id="rId3"/>
-    <sheet name="Relationships" sheetId="4" r:id="rId4"/>
-    <sheet name="Validation Rules" sheetId="5" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="6" r:id="rId4"/>
+    <sheet name="Relationships" sheetId="4" r:id="rId5"/>
+    <sheet name="Validation Rules" sheetId="5" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Atributes!$A$1:$W$396</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Reference Data'!$A$1:$H$92</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Relationships!$A$1:$K$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Relationships!$A$1:$K$63</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10209" uniqueCount="2225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10285" uniqueCount="2258">
   <si>
     <t>Domain</t>
   </si>
@@ -6709,6 +6710,105 @@
   </si>
   <si>
     <t>Store must belong to the Offer's Organization.</t>
+  </si>
+  <si>
+    <t>Entity Type Code</t>
+  </si>
+  <si>
+    <t>ORGANIZATION</t>
+  </si>
+  <si>
+    <t>ORGANIZATION_USER</t>
+  </si>
+  <si>
+    <t>MEMBERSHIP_PRODUCT</t>
+  </si>
+  <si>
+    <t>SUBSCRIPTION_PLAN</t>
+  </si>
+  <si>
+    <t>REDEMPTION</t>
+  </si>
+  <si>
+    <t>ORGANIZATION_BRANDING</t>
+  </si>
+  <si>
+    <t>NOTIFICATION_CONFIGURATION</t>
+  </si>
+  <si>
+    <t>#</t>
+  </si>
+  <si>
+    <t>Statuses</t>
+  </si>
+  <si>
+    <t>PENDING, ACTIVE, INACTIVE, SUSPENDED, CLOSED</t>
+  </si>
+  <si>
+    <t>USER</t>
+  </si>
+  <si>
+    <t>PENDING, ACTIVE, INACTIVE, SUSPENDED, LOCKED, CLOSED</t>
+  </si>
+  <si>
+    <t>ACTIVE, INACTIVE, RETIRED</t>
+  </si>
+  <si>
+    <t>ORGANIZATION_USER_ROLE</t>
+  </si>
+  <si>
+    <t>PENDING, ACTIVE, INACTIVE, REVOKED*</t>
+  </si>
+  <si>
+    <t>PRIVILEGE</t>
+  </si>
+  <si>
+    <t>Organization User / Platform User Role</t>
+  </si>
+  <si>
+    <t>PLATFORM_USER_ROLE</t>
+  </si>
+  <si>
+    <t>DRAFT, ACTIVE, INACTIVE, EXPIRED, RETIRED</t>
+  </si>
+  <si>
+    <t>PENDING, ACTIVE, INACTIVE, EXPIRED, CANCELLED</t>
+  </si>
+  <si>
+    <t>SUCCESS, FAILED, REVERSED</t>
+  </si>
+  <si>
+    <t>PENDING, ACTIVE, INACTIVE, CLOSED</t>
+  </si>
+  <si>
+    <t>PENDING, ACTIVE, INACTIVE, RELIEVED, RETIRED</t>
+  </si>
+  <si>
+    <t>STAFF_STORE_ASSIGNMENT</t>
+  </si>
+  <si>
+    <t>DRAFT, ACTIVE, INACTIVE</t>
+  </si>
+  <si>
+    <t>PENDING, SUCCESS, FAILED, REVERSED</t>
+  </si>
+  <si>
+    <t>DRAFT, ACTIVE, INACTIVE, SUSPENDED</t>
+  </si>
+  <si>
+    <t>ACTIVE, INACTIVE</t>
+  </si>
+  <si>
+    <t>TEMPLATE</t>
+  </si>
+  <si>
+    <t>DRAFT, ACTIVE, INACTIVE, RETIRED</t>
+  </si>
+  <si>
+    <t>TEMPLATE_TYPE</t>
+  </si>
+  <si>
+    <t>DRAFT, ACTIVE, INACTIVE, EXPIRED, CANCELLED</t>
   </si>
 </sst>
 </file>
@@ -6757,12 +6857,18 @@
       <name val="Arial Unicode MS"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -6778,7 +6884,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -6828,6 +6934,9 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -8379,7 +8488,7 @@
         <v>1139</v>
       </c>
     </row>
-    <row r="22" spans="1:17" ht="30">
+    <row r="22" spans="1:17" ht="45">
       <c r="A22" s="4" t="s">
         <v>1173</v>
       </c>
@@ -9237,6 +9346,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E21F442-9136-4C15-8BA3-92E07332B93A}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:W396"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -9336,7 +9446,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="2" spans="1:23" ht="30">
+    <row r="2" spans="1:23" ht="30" hidden="1">
       <c r="A2" s="10" t="s">
         <v>5</v>
       </c>
@@ -9402,7 +9512,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:23" ht="30">
+    <row r="3" spans="1:23" ht="30" hidden="1">
       <c r="A3" s="10" t="s">
         <v>5</v>
       </c>
@@ -9470,7 +9580,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:23" ht="30">
+    <row r="4" spans="1:23" ht="30" hidden="1">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -9538,7 +9648,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:23" ht="60">
+    <row r="5" spans="1:23" ht="60" hidden="1">
       <c r="A5" s="10" t="s">
         <v>5</v>
       </c>
@@ -9607,7 +9717,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:23" ht="30">
+    <row r="6" spans="1:23" ht="30" hidden="1">
       <c r="A6" s="10" t="s">
         <v>5</v>
       </c>
@@ -9675,7 +9785,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:23">
+    <row r="7" spans="1:23" hidden="1">
       <c r="A7" s="10" t="s">
         <v>5</v>
       </c>
@@ -9811,7 +9921,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:23">
+    <row r="9" spans="1:23" hidden="1">
       <c r="A9" s="10" t="s">
         <v>5</v>
       </c>
@@ -9879,7 +9989,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="10" spans="1:23">
+    <row r="10" spans="1:23" hidden="1">
       <c r="A10" s="10" t="s">
         <v>5</v>
       </c>
@@ -9947,7 +10057,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="11" spans="1:23">
+    <row r="11" spans="1:23" hidden="1">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -10015,7 +10125,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:23" ht="30">
+    <row r="12" spans="1:23" ht="30" hidden="1">
       <c r="A12" s="10" t="s">
         <v>5</v>
       </c>
@@ -10083,7 +10193,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:23">
+    <row r="13" spans="1:23" hidden="1">
       <c r="A13" s="10" t="s">
         <v>5</v>
       </c>
@@ -10151,7 +10261,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:23" ht="30">
+    <row r="14" spans="1:23" ht="30" hidden="1">
       <c r="A14" s="10" t="s">
         <v>5</v>
       </c>
@@ -10219,7 +10329,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:23">
+    <row r="15" spans="1:23" hidden="1">
       <c r="A15" s="10" t="s">
         <v>5</v>
       </c>
@@ -10287,7 +10397,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:23" ht="30">
+    <row r="16" spans="1:23" ht="30" hidden="1">
       <c r="A16" s="10" t="s">
         <v>5</v>
       </c>
@@ -10355,7 +10465,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:23">
+    <row r="17" spans="1:23" hidden="1">
       <c r="A17" s="10" t="s">
         <v>5</v>
       </c>
@@ -10423,7 +10533,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:23" ht="30">
+    <row r="18" spans="1:23" ht="30" hidden="1">
       <c r="A18" s="3" t="s">
         <v>8</v>
       </c>
@@ -10490,7 +10600,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:23" ht="30">
+    <row r="19" spans="1:23" ht="30" hidden="1">
       <c r="A19" s="3" t="s">
         <v>8</v>
       </c>
@@ -10559,7 +10669,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="1:23">
+    <row r="20" spans="1:23" hidden="1">
       <c r="A20" s="3" t="s">
         <v>8</v>
       </c>
@@ -10626,7 +10736,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="21" spans="1:23">
+    <row r="21" spans="1:23" hidden="1">
       <c r="A21" s="3" t="s">
         <v>8</v>
       </c>
@@ -10693,7 +10803,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="22" spans="1:23">
+    <row r="22" spans="1:23" hidden="1">
       <c r="A22" s="3" t="s">
         <v>8</v>
       </c>
@@ -10760,7 +10870,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="23" spans="1:23" ht="30">
+    <row r="23" spans="1:23" ht="30" hidden="1">
       <c r="A23" s="3" t="s">
         <v>8</v>
       </c>
@@ -10829,7 +10939,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="24" spans="1:23" ht="30">
+    <row r="24" spans="1:23" ht="30" hidden="1">
       <c r="A24" s="3" t="s">
         <v>8</v>
       </c>
@@ -10896,7 +11006,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="25" spans="1:23" ht="30">
+    <row r="25" spans="1:23" ht="30" hidden="1">
       <c r="A25" s="3" t="s">
         <v>8</v>
       </c>
@@ -10963,7 +11073,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="26" spans="1:23" ht="30">
+    <row r="26" spans="1:23" ht="30" hidden="1">
       <c r="A26" s="3" t="s">
         <v>8</v>
       </c>
@@ -11101,7 +11211,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="28" spans="1:23" ht="30">
+    <row r="28" spans="1:23" ht="30" hidden="1">
       <c r="A28" s="3" t="s">
         <v>8</v>
       </c>
@@ -11168,7 +11278,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="29" spans="1:23">
+    <row r="29" spans="1:23" hidden="1">
       <c r="A29" s="3" t="s">
         <v>8</v>
       </c>
@@ -11237,7 +11347,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="30" spans="1:23" ht="30">
+    <row r="30" spans="1:23" ht="30" hidden="1">
       <c r="A30" s="3" t="s">
         <v>8</v>
       </c>
@@ -11304,7 +11414,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="31" spans="1:23">
+    <row r="31" spans="1:23" hidden="1">
       <c r="A31" s="3" t="s">
         <v>8</v>
       </c>
@@ -11373,7 +11483,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="32" spans="1:23" ht="30">
+    <row r="32" spans="1:23" ht="30" hidden="1">
       <c r="A32" s="3" t="s">
         <v>8</v>
       </c>
@@ -11440,7 +11550,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="33" spans="1:23">
+    <row r="33" spans="1:23" hidden="1">
       <c r="A33" s="3" t="s">
         <v>8</v>
       </c>
@@ -11507,7 +11617,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="34" spans="1:23" ht="30">
+    <row r="34" spans="1:23" ht="30" hidden="1">
       <c r="A34" s="3" t="s">
         <v>37</v>
       </c>
@@ -11578,7 +11688,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="35" spans="1:23" ht="30">
+    <row r="35" spans="1:23" ht="30" hidden="1">
       <c r="A35" s="3" t="s">
         <v>37</v>
       </c>
@@ -11649,7 +11759,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="36" spans="1:23">
+    <row r="36" spans="1:23" hidden="1">
       <c r="A36" s="3" t="s">
         <v>37</v>
       </c>
@@ -11720,7 +11830,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="37" spans="1:23" ht="45">
+    <row r="37" spans="1:23" ht="45" hidden="1">
       <c r="A37" s="3" t="s">
         <v>37</v>
       </c>
@@ -11862,7 +11972,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="39" spans="1:23" ht="30">
+    <row r="39" spans="1:23" ht="30" hidden="1">
       <c r="A39" s="3" t="s">
         <v>37</v>
       </c>
@@ -11933,7 +12043,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="40" spans="1:23" ht="30">
+    <row r="40" spans="1:23" ht="30" hidden="1">
       <c r="A40" s="3" t="s">
         <v>37</v>
       </c>
@@ -12004,7 +12114,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="41" spans="1:23">
+    <row r="41" spans="1:23" hidden="1">
       <c r="A41" s="3" t="s">
         <v>37</v>
       </c>
@@ -12075,7 +12185,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="42" spans="1:23" ht="30">
+    <row r="42" spans="1:23" ht="30" hidden="1">
       <c r="A42" s="3" t="s">
         <v>37</v>
       </c>
@@ -12146,7 +12256,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="43" spans="1:23">
+    <row r="43" spans="1:23" hidden="1">
       <c r="A43" s="3" t="s">
         <v>37</v>
       </c>
@@ -12217,7 +12327,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="44" spans="1:23">
+    <row r="44" spans="1:23" hidden="1">
       <c r="A44" s="3" t="s">
         <v>37</v>
       </c>
@@ -12288,7 +12398,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="45" spans="1:23">
+    <row r="45" spans="1:23" hidden="1">
       <c r="A45" s="3" t="s">
         <v>37</v>
       </c>
@@ -12359,7 +12469,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="46" spans="1:23" ht="30">
+    <row r="46" spans="1:23" ht="30" hidden="1">
       <c r="A46" s="3" t="s">
         <v>317</v>
       </c>
@@ -12406,7 +12516,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="47" spans="1:23" ht="30">
+    <row r="47" spans="1:23" ht="30" hidden="1">
       <c r="A47" s="3" t="s">
         <v>317</v>
       </c>
@@ -12453,7 +12563,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="48" spans="1:23" ht="45">
+    <row r="48" spans="1:23" ht="45" hidden="1">
       <c r="A48" s="3" t="s">
         <v>317</v>
       </c>
@@ -12500,7 +12610,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="49" spans="1:23" ht="30">
+    <row r="49" spans="1:23" ht="30" hidden="1">
       <c r="A49" s="3" t="s">
         <v>317</v>
       </c>
@@ -12594,7 +12704,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="51" spans="1:23" ht="30">
+    <row r="51" spans="1:23" ht="30" hidden="1">
       <c r="A51" s="4" t="s">
         <v>341</v>
       </c>
@@ -12662,7 +12772,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="52" spans="1:23" ht="30">
+    <row r="52" spans="1:23" ht="30" hidden="1">
       <c r="A52" s="4" t="s">
         <v>341</v>
       </c>
@@ -12730,7 +12840,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="53" spans="1:23" ht="30">
+    <row r="53" spans="1:23" ht="30" hidden="1">
       <c r="A53" s="4" t="s">
         <v>341</v>
       </c>
@@ -12866,7 +12976,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="55" spans="1:23" ht="30">
+    <row r="55" spans="1:23" ht="30" hidden="1">
       <c r="A55" s="4" t="s">
         <v>341</v>
       </c>
@@ -12934,7 +13044,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="56" spans="1:23" ht="30">
+    <row r="56" spans="1:23" ht="30" hidden="1">
       <c r="A56" s="4" t="s">
         <v>341</v>
       </c>
@@ -13002,7 +13112,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="57" spans="1:23" ht="30">
+    <row r="57" spans="1:23" ht="30" hidden="1">
       <c r="A57" s="4" t="s">
         <v>341</v>
       </c>
@@ -13070,7 +13180,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="58" spans="1:23" ht="30">
+    <row r="58" spans="1:23" ht="30" hidden="1">
       <c r="A58" s="4" t="s">
         <v>341</v>
       </c>
@@ -13138,7 +13248,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="59" spans="1:23" ht="45">
+    <row r="59" spans="1:23" ht="45" hidden="1">
       <c r="A59" s="4" t="s">
         <v>341</v>
       </c>
@@ -13206,7 +13316,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="60" spans="1:23" ht="30">
+    <row r="60" spans="1:23" ht="30" hidden="1">
       <c r="A60" s="4" t="s">
         <v>341</v>
       </c>
@@ -13274,7 +13384,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="61" spans="1:23" ht="30">
+    <row r="61" spans="1:23" ht="30" hidden="1">
       <c r="A61" s="4" t="s">
         <v>370</v>
       </c>
@@ -13345,7 +13455,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="62" spans="1:23" ht="30">
+    <row r="62" spans="1:23" ht="30" hidden="1">
       <c r="A62" s="4" t="s">
         <v>370</v>
       </c>
@@ -13416,7 +13526,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="63" spans="1:23" ht="30">
+    <row r="63" spans="1:23" ht="30" hidden="1">
       <c r="A63" s="4" t="s">
         <v>370</v>
       </c>
@@ -13487,7 +13597,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="64" spans="1:23" ht="30">
+    <row r="64" spans="1:23" ht="30" hidden="1">
       <c r="A64" s="4" t="s">
         <v>370</v>
       </c>
@@ -13629,7 +13739,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="66" spans="1:23" ht="30">
+    <row r="66" spans="1:23" ht="30" hidden="1">
       <c r="A66" s="4" t="s">
         <v>377</v>
       </c>
@@ -13700,7 +13810,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="67" spans="1:23" ht="30">
+    <row r="67" spans="1:23" ht="30" hidden="1">
       <c r="A67" s="4" t="s">
         <v>377</v>
       </c>
@@ -13771,7 +13881,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="68" spans="1:23" ht="30">
+    <row r="68" spans="1:23" ht="30" hidden="1">
       <c r="A68" s="4" t="s">
         <v>377</v>
       </c>
@@ -13842,7 +13952,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="69" spans="1:23" ht="30">
+    <row r="69" spans="1:23" ht="30" hidden="1">
       <c r="A69" s="4" t="s">
         <v>10</v>
       </c>
@@ -13913,7 +14023,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="70" spans="1:23" ht="30">
+    <row r="70" spans="1:23" ht="30" hidden="1">
       <c r="A70" s="4" t="s">
         <v>10</v>
       </c>
@@ -13984,7 +14094,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="71" spans="1:23" ht="45">
+    <row r="71" spans="1:23" ht="45" hidden="1">
       <c r="A71" s="4" t="s">
         <v>10</v>
       </c>
@@ -14055,7 +14165,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="72" spans="1:23" ht="45">
+    <row r="72" spans="1:23" ht="45" hidden="1">
       <c r="A72" s="4" t="s">
         <v>10</v>
       </c>
@@ -14126,7 +14236,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="73" spans="1:23" ht="30">
+    <row r="73" spans="1:23" ht="30" hidden="1">
       <c r="A73" s="4" t="s">
         <v>10</v>
       </c>
@@ -14197,7 +14307,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="74" spans="1:23" ht="30">
+    <row r="74" spans="1:23" ht="30" hidden="1">
       <c r="A74" s="4" t="s">
         <v>10</v>
       </c>
@@ -14268,7 +14378,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="75" spans="1:23" ht="30">
+    <row r="75" spans="1:23" ht="30" hidden="1">
       <c r="A75" s="4" t="s">
         <v>10</v>
       </c>
@@ -14339,7 +14449,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="76" spans="1:23" ht="30">
+    <row r="76" spans="1:23" ht="30" hidden="1">
       <c r="A76" s="4" t="s">
         <v>10</v>
       </c>
@@ -14481,7 +14591,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="78" spans="1:23" ht="30">
+    <row r="78" spans="1:23" ht="45" hidden="1">
       <c r="A78" s="4" t="s">
         <v>10</v>
       </c>
@@ -14552,7 +14662,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="79" spans="1:23" ht="30">
+    <row r="79" spans="1:23" ht="45" hidden="1">
       <c r="A79" s="4" t="s">
         <v>10</v>
       </c>
@@ -14623,7 +14733,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="80" spans="1:23" ht="30">
+    <row r="80" spans="1:23" ht="30" hidden="1">
       <c r="A80" s="4" t="s">
         <v>10</v>
       </c>
@@ -14694,7 +14804,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="81" spans="1:23" ht="30">
+    <row r="81" spans="1:23" ht="30" hidden="1">
       <c r="A81" s="4" t="s">
         <v>10</v>
       </c>
@@ -14765,7 +14875,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="82" spans="1:23" ht="30">
+    <row r="82" spans="1:23" ht="30" hidden="1">
       <c r="A82" s="4" t="s">
         <v>10</v>
       </c>
@@ -14836,7 +14946,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="83" spans="1:23" ht="30">
+    <row r="83" spans="1:23" ht="30" hidden="1">
       <c r="A83" s="4" t="s">
         <v>10</v>
       </c>
@@ -14907,7 +15017,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="84" spans="1:23" ht="45">
+    <row r="84" spans="1:23" ht="45" hidden="1">
       <c r="A84" s="4" t="s">
         <v>10</v>
       </c>
@@ -14978,7 +15088,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="85" spans="1:23" ht="30">
+    <row r="85" spans="1:23" ht="30" hidden="1">
       <c r="A85" s="4" t="s">
         <v>10</v>
       </c>
@@ -15049,7 +15159,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="86" spans="1:23" ht="30">
+    <row r="86" spans="1:23" ht="30" hidden="1">
       <c r="A86" s="4" t="s">
         <v>490</v>
       </c>
@@ -15120,7 +15230,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="87" spans="1:23" ht="30">
+    <row r="87" spans="1:23" ht="30" hidden="1">
       <c r="A87" s="4" t="s">
         <v>490</v>
       </c>
@@ -15191,7 +15301,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="88" spans="1:23" ht="30">
+    <row r="88" spans="1:23" ht="30" hidden="1">
       <c r="A88" s="4" t="s">
         <v>490</v>
       </c>
@@ -15262,7 +15372,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="89" spans="1:23" ht="30">
+    <row r="89" spans="1:23" ht="30" hidden="1">
       <c r="A89" s="4" t="s">
         <v>490</v>
       </c>
@@ -15333,7 +15443,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="90" spans="1:23">
+    <row r="90" spans="1:23" hidden="1">
       <c r="A90" s="4" t="s">
         <v>490</v>
       </c>
@@ -15404,7 +15514,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="91" spans="1:23">
+    <row r="91" spans="1:23" hidden="1">
       <c r="A91" s="4" t="s">
         <v>490</v>
       </c>
@@ -15475,7 +15585,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="92" spans="1:23" ht="45">
+    <row r="92" spans="1:23" ht="45" hidden="1">
       <c r="A92" s="4" t="s">
         <v>490</v>
       </c>
@@ -15617,7 +15727,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="94" spans="1:23" ht="30">
+    <row r="94" spans="1:23" ht="30" hidden="1">
       <c r="A94" s="4" t="s">
         <v>490</v>
       </c>
@@ -15688,7 +15798,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="95" spans="1:23" ht="30">
+    <row r="95" spans="1:23" ht="30" hidden="1">
       <c r="A95" s="4" t="s">
         <v>490</v>
       </c>
@@ -15759,7 +15869,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="96" spans="1:23" ht="30">
+    <row r="96" spans="1:23" ht="30" hidden="1">
       <c r="A96" s="4" t="s">
         <v>490</v>
       </c>
@@ -15830,7 +15940,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="97" spans="1:23" ht="30">
+    <row r="97" spans="1:23" ht="30" hidden="1">
       <c r="A97" s="4" t="s">
         <v>490</v>
       </c>
@@ -15901,7 +16011,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="98" spans="1:23" ht="30">
+    <row r="98" spans="1:23" ht="30" hidden="1">
       <c r="A98" s="4" t="s">
         <v>490</v>
       </c>
@@ -15972,7 +16082,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="99" spans="1:23" ht="30">
+    <row r="99" spans="1:23" ht="30" hidden="1">
       <c r="A99" s="4" t="s">
         <v>490</v>
       </c>
@@ -16043,7 +16153,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="100" spans="1:23" ht="30">
+    <row r="100" spans="1:23" ht="30" hidden="1">
       <c r="A100" s="4" t="s">
         <v>490</v>
       </c>
@@ -16114,7 +16224,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="101" spans="1:23" ht="30">
+    <row r="101" spans="1:23" ht="30" hidden="1">
       <c r="A101" s="4" t="s">
         <v>490</v>
       </c>
@@ -16185,7 +16295,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="102" spans="1:23" ht="30">
+    <row r="102" spans="1:23" ht="30" hidden="1">
       <c r="A102" s="4" t="s">
         <v>548</v>
       </c>
@@ -16256,7 +16366,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="103" spans="1:23" ht="30">
+    <row r="103" spans="1:23" ht="30" hidden="1">
       <c r="A103" s="4" t="s">
         <v>548</v>
       </c>
@@ -16327,7 +16437,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="104" spans="1:23" ht="30">
+    <row r="104" spans="1:23" ht="30" hidden="1">
       <c r="A104" s="4" t="s">
         <v>548</v>
       </c>
@@ -16398,7 +16508,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="105" spans="1:23" ht="30">
+    <row r="105" spans="1:23" ht="30" hidden="1">
       <c r="A105" s="4" t="s">
         <v>548</v>
       </c>
@@ -16469,7 +16579,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="106" spans="1:23" ht="30">
+    <row r="106" spans="1:23" ht="30" hidden="1">
       <c r="A106" s="4" t="s">
         <v>548</v>
       </c>
@@ -16540,7 +16650,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="107" spans="1:23">
+    <row r="107" spans="1:23" hidden="1">
       <c r="A107" s="4" t="s">
         <v>548</v>
       </c>
@@ -16611,7 +16721,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="108" spans="1:23">
+    <row r="108" spans="1:23" hidden="1">
       <c r="A108" s="4" t="s">
         <v>548</v>
       </c>
@@ -16682,7 +16792,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="109" spans="1:23">
+    <row r="109" spans="1:23" hidden="1">
       <c r="A109" s="4" t="s">
         <v>548</v>
       </c>
@@ -16753,7 +16863,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="110" spans="1:23" ht="30">
+    <row r="110" spans="1:23" ht="30" hidden="1">
       <c r="A110" s="4" t="s">
         <v>548</v>
       </c>
@@ -16895,7 +17005,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="112" spans="1:23" ht="30">
+    <row r="112" spans="1:23" ht="30" hidden="1">
       <c r="A112" s="4" t="s">
         <v>548</v>
       </c>
@@ -16966,7 +17076,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="113" spans="1:23">
+    <row r="113" spans="1:23" hidden="1">
       <c r="A113" s="4" t="s">
         <v>548</v>
       </c>
@@ -17037,7 +17147,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="114" spans="1:23" ht="30">
+    <row r="114" spans="1:23" ht="30" hidden="1">
       <c r="A114" s="4" t="s">
         <v>548</v>
       </c>
@@ -17108,7 +17218,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="115" spans="1:23">
+    <row r="115" spans="1:23" hidden="1">
       <c r="A115" s="4" t="s">
         <v>548</v>
       </c>
@@ -17179,7 +17289,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="116" spans="1:23" ht="30">
+    <row r="116" spans="1:23" ht="30" hidden="1">
       <c r="A116" s="4" t="s">
         <v>548</v>
       </c>
@@ -17250,7 +17360,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="117" spans="1:23">
+    <row r="117" spans="1:23" hidden="1">
       <c r="A117" s="4" t="s">
         <v>548</v>
       </c>
@@ -17321,7 +17431,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="118" spans="1:23">
+    <row r="118" spans="1:23" hidden="1">
       <c r="A118" s="4" t="s">
         <v>548</v>
       </c>
@@ -17392,7 +17502,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="119" spans="1:23">
+    <row r="119" spans="1:23" hidden="1">
       <c r="A119" s="4" t="s">
         <v>548</v>
       </c>
@@ -17463,7 +17573,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="120" spans="1:23" ht="30">
+    <row r="120" spans="1:23" ht="30" hidden="1">
       <c r="A120" s="4" t="s">
         <v>620</v>
       </c>
@@ -17534,7 +17644,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="121" spans="1:23" ht="30">
+    <row r="121" spans="1:23" ht="30" hidden="1">
       <c r="A121" s="4" t="s">
         <v>620</v>
       </c>
@@ -17605,7 +17715,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="122" spans="1:23">
+    <row r="122" spans="1:23" hidden="1">
       <c r="A122" s="4" t="s">
         <v>620</v>
       </c>
@@ -17676,7 +17786,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="123" spans="1:23" ht="30">
+    <row r="123" spans="1:23" ht="30" hidden="1">
       <c r="A123" s="4" t="s">
         <v>620</v>
       </c>
@@ -17747,7 +17857,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="124" spans="1:23">
+    <row r="124" spans="1:23" hidden="1">
       <c r="A124" s="4" t="s">
         <v>620</v>
       </c>
@@ -17818,7 +17928,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="125" spans="1:23" ht="30">
+    <row r="125" spans="1:23" ht="30" hidden="1">
       <c r="A125" s="4" t="s">
         <v>620</v>
       </c>
@@ -17889,7 +17999,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="126" spans="1:23">
+    <row r="126" spans="1:23" hidden="1">
       <c r="A126" s="4" t="s">
         <v>620</v>
       </c>
@@ -18031,7 +18141,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="128" spans="1:23" ht="30">
+    <row r="128" spans="1:23" ht="30" hidden="1">
       <c r="A128" s="4" t="s">
         <v>620</v>
       </c>
@@ -18102,7 +18212,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="129" spans="1:23" ht="30">
+    <row r="129" spans="1:23" ht="30" hidden="1">
       <c r="A129" s="4" t="s">
         <v>620</v>
       </c>
@@ -18173,7 +18283,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="130" spans="1:23">
+    <row r="130" spans="1:23" hidden="1">
       <c r="A130" s="4" t="s">
         <v>620</v>
       </c>
@@ -18244,7 +18354,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="131" spans="1:23" ht="30">
+    <row r="131" spans="1:23" ht="30" hidden="1">
       <c r="A131" s="4" t="s">
         <v>620</v>
       </c>
@@ -18315,7 +18425,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="132" spans="1:23">
+    <row r="132" spans="1:23" hidden="1">
       <c r="A132" s="4" t="s">
         <v>620</v>
       </c>
@@ -18386,7 +18496,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="133" spans="1:23">
+    <row r="133" spans="1:23" hidden="1">
       <c r="A133" s="4" t="s">
         <v>620</v>
       </c>
@@ -18457,7 +18567,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="134" spans="1:23">
+    <row r="134" spans="1:23" hidden="1">
       <c r="A134" s="4" t="s">
         <v>620</v>
       </c>
@@ -18528,7 +18638,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="135" spans="1:23" ht="30">
+    <row r="135" spans="1:23" ht="30" hidden="1">
       <c r="A135" s="4" t="s">
         <v>673</v>
       </c>
@@ -18599,7 +18709,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="136" spans="1:23" ht="30">
+    <row r="136" spans="1:23" ht="30" hidden="1">
       <c r="A136" s="4" t="s">
         <v>673</v>
       </c>
@@ -18670,7 +18780,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="137" spans="1:23" ht="30">
+    <row r="137" spans="1:23" ht="30" hidden="1">
       <c r="A137" s="4" t="s">
         <v>673</v>
       </c>
@@ -18741,7 +18851,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="138" spans="1:23" ht="30">
+    <row r="138" spans="1:23" ht="30" hidden="1">
       <c r="A138" s="4" t="s">
         <v>673</v>
       </c>
@@ -18812,7 +18922,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="139" spans="1:23" ht="30">
+    <row r="139" spans="1:23" ht="30" hidden="1">
       <c r="A139" s="4" t="s">
         <v>673</v>
       </c>
@@ -18883,7 +18993,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="140" spans="1:23" ht="30">
+    <row r="140" spans="1:23" ht="30" hidden="1">
       <c r="A140" s="4" t="s">
         <v>673</v>
       </c>
@@ -18954,7 +19064,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="141" spans="1:23" ht="30">
+    <row r="141" spans="1:23" ht="30" hidden="1">
       <c r="A141" s="4" t="s">
         <v>673</v>
       </c>
@@ -19025,7 +19135,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="142" spans="1:23">
+    <row r="142" spans="1:23" hidden="1">
       <c r="A142" s="4" t="s">
         <v>673</v>
       </c>
@@ -19167,7 +19277,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="144" spans="1:23" ht="30">
+    <row r="144" spans="1:23" ht="30" hidden="1">
       <c r="A144" s="4" t="s">
         <v>673</v>
       </c>
@@ -19238,7 +19348,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="145" spans="1:23" ht="30">
+    <row r="145" spans="1:23" ht="30" hidden="1">
       <c r="A145" s="4" t="s">
         <v>673</v>
       </c>
@@ -19309,7 +19419,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="146" spans="1:23" ht="30">
+    <row r="146" spans="1:23" ht="30" hidden="1">
       <c r="A146" s="4" t="s">
         <v>673</v>
       </c>
@@ -19380,7 +19490,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="147" spans="1:23" ht="30">
+    <row r="147" spans="1:23" ht="30" hidden="1">
       <c r="A147" s="4" t="s">
         <v>673</v>
       </c>
@@ -19451,7 +19561,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="148" spans="1:23" ht="30">
+    <row r="148" spans="1:23" ht="30" hidden="1">
       <c r="A148" s="4" t="s">
         <v>673</v>
       </c>
@@ -19522,7 +19632,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="149" spans="1:23">
+    <row r="149" spans="1:23" hidden="1">
       <c r="A149" s="4" t="s">
         <v>673</v>
       </c>
@@ -19593,7 +19703,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="150" spans="1:23" ht="30">
+    <row r="150" spans="1:23" ht="30" hidden="1">
       <c r="A150" s="4" t="s">
         <v>34</v>
       </c>
@@ -19664,7 +19774,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="151" spans="1:23" ht="30">
+    <row r="151" spans="1:23" ht="30" hidden="1">
       <c r="A151" s="4" t="s">
         <v>34</v>
       </c>
@@ -19735,7 +19845,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="152" spans="1:23" ht="30">
+    <row r="152" spans="1:23" ht="30" hidden="1">
       <c r="A152" s="4" t="s">
         <v>34</v>
       </c>
@@ -19806,7 +19916,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="153" spans="1:23" ht="30">
+    <row r="153" spans="1:23" ht="30" hidden="1">
       <c r="A153" s="4" t="s">
         <v>34</v>
       </c>
@@ -19877,7 +19987,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="154" spans="1:23">
+    <row r="154" spans="1:23" hidden="1">
       <c r="A154" s="4" t="s">
         <v>34</v>
       </c>
@@ -19948,7 +20058,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="155" spans="1:23" ht="30">
+    <row r="155" spans="1:23" ht="30" hidden="1">
       <c r="A155" s="4" t="s">
         <v>34</v>
       </c>
@@ -20019,7 +20129,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="156" spans="1:23" ht="30">
+    <row r="156" spans="1:23" ht="30" hidden="1">
       <c r="A156" s="4" t="s">
         <v>34</v>
       </c>
@@ -20161,7 +20271,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="158" spans="1:23" ht="30">
+    <row r="158" spans="1:23" ht="30" hidden="1">
       <c r="A158" s="4" t="s">
         <v>34</v>
       </c>
@@ -20232,7 +20342,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="159" spans="1:23" ht="30">
+    <row r="159" spans="1:23" ht="30" hidden="1">
       <c r="A159" s="4" t="s">
         <v>34</v>
       </c>
@@ -20303,7 +20413,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="160" spans="1:23" ht="30">
+    <row r="160" spans="1:23" ht="30" hidden="1">
       <c r="A160" s="4" t="s">
         <v>34</v>
       </c>
@@ -20374,7 +20484,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="161" spans="1:23">
+    <row r="161" spans="1:23" hidden="1">
       <c r="A161" s="4" t="s">
         <v>34</v>
       </c>
@@ -20445,7 +20555,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="162" spans="1:23" ht="30">
+    <row r="162" spans="1:23" ht="30" hidden="1">
       <c r="A162" s="4" t="s">
         <v>34</v>
       </c>
@@ -20516,7 +20626,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="163" spans="1:23" ht="30">
+    <row r="163" spans="1:23" ht="30" hidden="1">
       <c r="A163" s="4" t="s">
         <v>34</v>
       </c>
@@ -20587,7 +20697,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="164" spans="1:23" ht="30">
+    <row r="164" spans="1:23" ht="30" hidden="1">
       <c r="A164" s="4" t="s">
         <v>34</v>
       </c>
@@ -20658,7 +20768,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="165" spans="1:23" ht="30">
+    <row r="165" spans="1:23" ht="30" hidden="1">
       <c r="A165" s="4" t="s">
         <v>34</v>
       </c>
@@ -20729,7 +20839,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="166" spans="1:23" ht="30">
+    <row r="166" spans="1:23" ht="30" hidden="1">
       <c r="A166" s="4" t="s">
         <v>35</v>
       </c>
@@ -20800,7 +20910,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="167" spans="1:23" ht="30">
+    <row r="167" spans="1:23" ht="30" hidden="1">
       <c r="A167" s="4" t="s">
         <v>35</v>
       </c>
@@ -20871,7 +20981,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="168" spans="1:23" ht="30">
+    <row r="168" spans="1:23" ht="30" hidden="1">
       <c r="A168" s="4" t="s">
         <v>35</v>
       </c>
@@ -20942,7 +21052,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="169" spans="1:23" ht="30">
+    <row r="169" spans="1:23" ht="30" hidden="1">
       <c r="A169" s="4" t="s">
         <v>35</v>
       </c>
@@ -21013,7 +21123,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="170" spans="1:23" ht="30">
+    <row r="170" spans="1:23" ht="30" hidden="1">
       <c r="A170" s="4" t="s">
         <v>35</v>
       </c>
@@ -21084,7 +21194,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="171" spans="1:23" ht="30">
+    <row r="171" spans="1:23" ht="30" hidden="1">
       <c r="A171" s="4" t="s">
         <v>35</v>
       </c>
@@ -21155,7 +21265,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="172" spans="1:23" ht="30">
+    <row r="172" spans="1:23" ht="30" hidden="1">
       <c r="A172" s="4" t="s">
         <v>35</v>
       </c>
@@ -21226,7 +21336,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="173" spans="1:23" ht="30">
+    <row r="173" spans="1:23" ht="30" hidden="1">
       <c r="A173" s="4" t="s">
         <v>35</v>
       </c>
@@ -21368,7 +21478,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="175" spans="1:23" ht="30">
+    <row r="175" spans="1:23" ht="30" hidden="1">
       <c r="A175" s="4" t="s">
         <v>35</v>
       </c>
@@ -21439,7 +21549,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="176" spans="1:23" ht="30">
+    <row r="176" spans="1:23" ht="30" hidden="1">
       <c r="A176" s="4" t="s">
         <v>35</v>
       </c>
@@ -21510,7 +21620,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="177" spans="1:23" ht="30">
+    <row r="177" spans="1:23" ht="30" hidden="1">
       <c r="A177" s="4" t="s">
         <v>35</v>
       </c>
@@ -21581,7 +21691,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="178" spans="1:23" ht="30">
+    <row r="178" spans="1:23" ht="30" hidden="1">
       <c r="A178" s="4" t="s">
         <v>35</v>
       </c>
@@ -21652,7 +21762,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="179" spans="1:23" ht="30">
+    <row r="179" spans="1:23" ht="30" hidden="1">
       <c r="A179" s="4" t="s">
         <v>35</v>
       </c>
@@ -21723,7 +21833,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="180" spans="1:23" ht="30">
+    <row r="180" spans="1:23" ht="30" hidden="1">
       <c r="A180" s="4" t="s">
         <v>35</v>
       </c>
@@ -21794,7 +21904,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="181" spans="1:23" ht="30">
+    <row r="181" spans="1:23" ht="30" hidden="1">
       <c r="A181" s="3" t="s">
         <v>94</v>
       </c>
@@ -21861,7 +21971,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="182" spans="1:23" ht="30">
+    <row r="182" spans="1:23" ht="30" hidden="1">
       <c r="A182" s="3" t="s">
         <v>94</v>
       </c>
@@ -21930,7 +22040,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="183" spans="1:23" ht="30">
+    <row r="183" spans="1:23" ht="30" hidden="1">
       <c r="A183" s="3" t="s">
         <v>94</v>
       </c>
@@ -21999,7 +22109,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="184" spans="1:23" ht="30">
+    <row r="184" spans="1:23" ht="30" hidden="1">
       <c r="A184" s="3" t="s">
         <v>94</v>
       </c>
@@ -22068,7 +22178,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="185" spans="1:23" ht="30">
+    <row r="185" spans="1:23" ht="30" hidden="1">
       <c r="A185" s="3" t="s">
         <v>94</v>
       </c>
@@ -22137,7 +22247,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="186" spans="1:23" ht="30">
+    <row r="186" spans="1:23" ht="30" hidden="1">
       <c r="A186" s="3" t="s">
         <v>94</v>
       </c>
@@ -22206,7 +22316,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="187" spans="1:23">
+    <row r="187" spans="1:23" hidden="1">
       <c r="A187" s="3" t="s">
         <v>42</v>
       </c>
@@ -22273,7 +22383,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="188" spans="1:23">
+    <row r="188" spans="1:23" hidden="1">
       <c r="A188" s="3" t="s">
         <v>42</v>
       </c>
@@ -22342,7 +22452,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="189" spans="1:23">
+    <row r="189" spans="1:23" hidden="1">
       <c r="A189" s="3" t="s">
         <v>42</v>
       </c>
@@ -22411,7 +22521,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="190" spans="1:23" ht="30">
+    <row r="190" spans="1:23" ht="30" hidden="1">
       <c r="A190" s="3" t="s">
         <v>42</v>
       </c>
@@ -22480,7 +22590,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="191" spans="1:23">
+    <row r="191" spans="1:23" hidden="1">
       <c r="A191" s="3" t="s">
         <v>42</v>
       </c>
@@ -22549,7 +22659,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="192" spans="1:23" ht="30">
+    <row r="192" spans="1:23" ht="30" hidden="1">
       <c r="A192" s="3" t="s">
         <v>42</v>
       </c>
@@ -22618,7 +22728,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="193" spans="1:23">
+    <row r="193" spans="1:23" hidden="1">
       <c r="A193" s="3" t="s">
         <v>129</v>
       </c>
@@ -22685,7 +22795,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="194" spans="1:23">
+    <row r="194" spans="1:23" hidden="1">
       <c r="A194" s="3" t="s">
         <v>129</v>
       </c>
@@ -22754,7 +22864,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="195" spans="1:23">
+    <row r="195" spans="1:23" hidden="1">
       <c r="A195" s="3" t="s">
         <v>129</v>
       </c>
@@ -22823,7 +22933,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="196" spans="1:23">
+    <row r="196" spans="1:23" hidden="1">
       <c r="A196" s="3" t="s">
         <v>129</v>
       </c>
@@ -22892,7 +23002,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="197" spans="1:23">
+    <row r="197" spans="1:23" hidden="1">
       <c r="A197" s="3" t="s">
         <v>129</v>
       </c>
@@ -22961,7 +23071,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="198" spans="1:23" ht="30">
+    <row r="198" spans="1:23" ht="30" hidden="1">
       <c r="A198" s="3" t="s">
         <v>129</v>
       </c>
@@ -23030,7 +23140,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="199" spans="1:23" ht="30">
+    <row r="199" spans="1:23" ht="30" hidden="1">
       <c r="A199" s="3" t="s">
         <v>129</v>
       </c>
@@ -23099,7 +23209,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="200" spans="1:23">
+    <row r="200" spans="1:23" hidden="1">
       <c r="A200" s="3" t="s">
         <v>126</v>
       </c>
@@ -23166,7 +23276,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="201" spans="1:23">
+    <row r="201" spans="1:23" hidden="1">
       <c r="A201" s="3" t="s">
         <v>126</v>
       </c>
@@ -23235,7 +23345,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="202" spans="1:23">
+    <row r="202" spans="1:23" hidden="1">
       <c r="A202" s="3" t="s">
         <v>126</v>
       </c>
@@ -23304,7 +23414,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="203" spans="1:23" ht="30">
+    <row r="203" spans="1:23" ht="30" hidden="1">
       <c r="A203" s="3" t="s">
         <v>126</v>
       </c>
@@ -23373,7 +23483,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="204" spans="1:23" ht="30">
+    <row r="204" spans="1:23" ht="30" hidden="1">
       <c r="A204" s="3" t="s">
         <v>126</v>
       </c>
@@ -23442,7 +23552,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="205" spans="1:23">
+    <row r="205" spans="1:23" hidden="1">
       <c r="A205" s="3" t="s">
         <v>126</v>
       </c>
@@ -23511,7 +23621,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="206" spans="1:23" ht="30">
+    <row r="206" spans="1:23" ht="30" hidden="1">
       <c r="A206" s="3" t="s">
         <v>126</v>
       </c>
@@ -23580,7 +23690,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="207" spans="1:23" ht="30">
+    <row r="207" spans="1:23" ht="30" hidden="1">
       <c r="A207" s="3" t="s">
         <v>126</v>
       </c>
@@ -23649,7 +23759,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="208" spans="1:23" ht="30">
+    <row r="208" spans="1:23" ht="30" hidden="1">
       <c r="A208" s="3" t="s">
         <v>313</v>
       </c>
@@ -23716,7 +23826,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="209" spans="1:23" ht="30">
+    <row r="209" spans="1:23" ht="30" hidden="1">
       <c r="A209" s="3" t="s">
         <v>313</v>
       </c>
@@ -23785,7 +23895,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="210" spans="1:23" ht="30">
+    <row r="210" spans="1:23" ht="30" hidden="1">
       <c r="A210" s="3" t="s">
         <v>313</v>
       </c>
@@ -23854,7 +23964,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="211" spans="1:23" ht="30">
+    <row r="211" spans="1:23" ht="30" hidden="1">
       <c r="A211" s="3" t="s">
         <v>313</v>
       </c>
@@ -23923,7 +24033,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="212" spans="1:23" ht="30">
+    <row r="212" spans="1:23" ht="30" hidden="1">
       <c r="A212" s="3" t="s">
         <v>313</v>
       </c>
@@ -23992,7 +24102,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="213" spans="1:23" ht="45">
+    <row r="213" spans="1:23" ht="45" hidden="1">
       <c r="A213" s="3" t="s">
         <v>313</v>
       </c>
@@ -24061,7 +24171,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="214" spans="1:23" ht="30">
+    <row r="214" spans="1:23" ht="30" hidden="1">
       <c r="A214" s="3" t="s">
         <v>445</v>
       </c>
@@ -24128,7 +24238,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="215" spans="1:23" ht="30">
+    <row r="215" spans="1:23" ht="30" hidden="1">
       <c r="A215" s="3" t="s">
         <v>445</v>
       </c>
@@ -24197,7 +24307,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="216" spans="1:23" ht="30">
+    <row r="216" spans="1:23" ht="30" hidden="1">
       <c r="A216" s="3" t="s">
         <v>445</v>
       </c>
@@ -24266,7 +24376,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="217" spans="1:23" ht="30">
+    <row r="217" spans="1:23" ht="30" hidden="1">
       <c r="A217" s="3" t="s">
         <v>445</v>
       </c>
@@ -24335,7 +24445,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="218" spans="1:23" ht="30">
+    <row r="218" spans="1:23" ht="30" hidden="1">
       <c r="A218" s="3" t="s">
         <v>445</v>
       </c>
@@ -24404,7 +24514,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="219" spans="1:23" ht="30">
+    <row r="219" spans="1:23" ht="30" hidden="1">
       <c r="A219" s="3" t="s">
         <v>445</v>
       </c>
@@ -24473,7 +24583,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="220" spans="1:23" ht="30">
+    <row r="220" spans="1:23" ht="30" hidden="1">
       <c r="A220" s="3" t="s">
         <v>451</v>
       </c>
@@ -24540,7 +24650,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="221" spans="1:23">
+    <row r="221" spans="1:23" hidden="1">
       <c r="A221" s="3" t="s">
         <v>451</v>
       </c>
@@ -24609,7 +24719,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="222" spans="1:23">
+    <row r="222" spans="1:23" hidden="1">
       <c r="A222" s="3" t="s">
         <v>451</v>
       </c>
@@ -24678,7 +24788,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="223" spans="1:23" ht="30">
+    <row r="223" spans="1:23" ht="30" hidden="1">
       <c r="A223" s="3" t="s">
         <v>451</v>
       </c>
@@ -24747,7 +24857,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="224" spans="1:23">
+    <row r="224" spans="1:23" hidden="1">
       <c r="A224" s="3" t="s">
         <v>451</v>
       </c>
@@ -24816,7 +24926,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="225" spans="1:23" ht="30">
+    <row r="225" spans="1:23" ht="30" hidden="1">
       <c r="A225" s="3" t="s">
         <v>451</v>
       </c>
@@ -24885,7 +24995,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="226" spans="1:23" ht="30">
+    <row r="226" spans="1:23" ht="30" hidden="1">
       <c r="A226" s="3" t="s">
         <v>512</v>
       </c>
@@ -24952,7 +25062,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="227" spans="1:23" ht="30">
+    <row r="227" spans="1:23" ht="30" hidden="1">
       <c r="A227" s="3" t="s">
         <v>512</v>
       </c>
@@ -25021,7 +25131,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="228" spans="1:23" ht="30">
+    <row r="228" spans="1:23" ht="30" hidden="1">
       <c r="A228" s="3" t="s">
         <v>512</v>
       </c>
@@ -25090,7 +25200,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="229" spans="1:23" ht="30">
+    <row r="229" spans="1:23" ht="30" hidden="1">
       <c r="A229" s="3" t="s">
         <v>512</v>
       </c>
@@ -25159,7 +25269,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="230" spans="1:23" ht="30">
+    <row r="230" spans="1:23" ht="30" hidden="1">
       <c r="A230" s="3" t="s">
         <v>512</v>
       </c>
@@ -25228,7 +25338,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="231" spans="1:23" ht="30">
+    <row r="231" spans="1:23" ht="30" hidden="1">
       <c r="A231" s="3" t="s">
         <v>512</v>
       </c>
@@ -25297,7 +25407,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="232" spans="1:23" ht="30">
+    <row r="232" spans="1:23" ht="30" hidden="1">
       <c r="A232" s="3" t="s">
         <v>518</v>
       </c>
@@ -25364,7 +25474,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="233" spans="1:23">
+    <row r="233" spans="1:23" hidden="1">
       <c r="A233" s="3" t="s">
         <v>518</v>
       </c>
@@ -25433,7 +25543,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="234" spans="1:23">
+    <row r="234" spans="1:23" hidden="1">
       <c r="A234" s="3" t="s">
         <v>518</v>
       </c>
@@ -25502,7 +25612,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="235" spans="1:23" ht="30">
+    <row r="235" spans="1:23" ht="30" hidden="1">
       <c r="A235" s="3" t="s">
         <v>518</v>
       </c>
@@ -25571,7 +25681,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="236" spans="1:23">
+    <row r="236" spans="1:23" hidden="1">
       <c r="A236" s="3" t="s">
         <v>518</v>
       </c>
@@ -25640,7 +25750,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="237" spans="1:23" ht="30">
+    <row r="237" spans="1:23" ht="30" hidden="1">
       <c r="A237" s="3" t="s">
         <v>518</v>
       </c>
@@ -25709,7 +25819,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="238" spans="1:23" ht="30">
+    <row r="238" spans="1:23" ht="30" hidden="1">
       <c r="A238" s="3" t="s">
         <v>757</v>
       </c>
@@ -25776,7 +25886,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="239" spans="1:23">
+    <row r="239" spans="1:23" hidden="1">
       <c r="A239" s="3" t="s">
         <v>757</v>
       </c>
@@ -25845,7 +25955,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="240" spans="1:23">
+    <row r="240" spans="1:23" hidden="1">
       <c r="A240" s="3" t="s">
         <v>757</v>
       </c>
@@ -25914,7 +26024,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="241" spans="1:23">
+    <row r="241" spans="1:23" hidden="1">
       <c r="A241" s="3" t="s">
         <v>757</v>
       </c>
@@ -25983,7 +26093,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="242" spans="1:23">
+    <row r="242" spans="1:23" hidden="1">
       <c r="A242" s="3" t="s">
         <v>757</v>
       </c>
@@ -26052,7 +26162,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="243" spans="1:23" ht="30">
+    <row r="243" spans="1:23" ht="30" hidden="1">
       <c r="A243" s="3" t="s">
         <v>757</v>
       </c>
@@ -26121,7 +26231,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="244" spans="1:23" ht="30">
+    <row r="244" spans="1:23" ht="30" hidden="1">
       <c r="A244" s="3" t="s">
         <v>1517</v>
       </c>
@@ -26188,7 +26298,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="245" spans="1:23" ht="30">
+    <row r="245" spans="1:23" ht="30" hidden="1">
       <c r="A245" s="3" t="s">
         <v>1517</v>
       </c>
@@ -26255,7 +26365,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="246" spans="1:23" ht="30">
+    <row r="246" spans="1:23" ht="30" hidden="1">
       <c r="A246" s="3" t="s">
         <v>1517</v>
       </c>
@@ -26324,7 +26434,7 @@
         <v>1446</v>
       </c>
     </row>
-    <row r="247" spans="1:23" ht="30">
+    <row r="247" spans="1:23" ht="30" hidden="1">
       <c r="A247" s="3" t="s">
         <v>1517</v>
       </c>
@@ -26393,7 +26503,7 @@
         <v>1446</v>
       </c>
     </row>
-    <row r="248" spans="1:23">
+    <row r="248" spans="1:23" hidden="1">
       <c r="A248" s="3" t="s">
         <v>1517</v>
       </c>
@@ -26462,7 +26572,7 @@
         <v>1446</v>
       </c>
     </row>
-    <row r="249" spans="1:23" ht="30">
+    <row r="249" spans="1:23" ht="30" hidden="1">
       <c r="A249" s="3" t="s">
         <v>1517</v>
       </c>
@@ -26531,7 +26641,7 @@
         <v>1446</v>
       </c>
     </row>
-    <row r="250" spans="1:23">
+    <row r="250" spans="1:23" hidden="1">
       <c r="A250" s="3" t="s">
         <v>1517</v>
       </c>
@@ -26600,7 +26710,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="251" spans="1:23">
+    <row r="251" spans="1:23" hidden="1">
       <c r="A251" s="3" t="s">
         <v>1517</v>
       </c>
@@ -26669,7 +26779,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="252" spans="1:23">
+    <row r="252" spans="1:23" hidden="1">
       <c r="A252" s="3" t="s">
         <v>1517</v>
       </c>
@@ -26738,7 +26848,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="253" spans="1:23">
+    <row r="253" spans="1:23" hidden="1">
       <c r="A253" s="3" t="s">
         <v>1517</v>
       </c>
@@ -26807,7 +26917,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="254" spans="1:23">
+    <row r="254" spans="1:23" hidden="1">
       <c r="A254" s="3" t="s">
         <v>1517</v>
       </c>
@@ -26876,7 +26986,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="255" spans="1:23">
+    <row r="255" spans="1:23" hidden="1">
       <c r="A255" s="3" t="s">
         <v>1517</v>
       </c>
@@ -26945,7 +27055,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="256" spans="1:23" ht="30">
+    <row r="256" spans="1:23" ht="30" hidden="1">
       <c r="A256" s="3" t="s">
         <v>1517</v>
       </c>
@@ -27014,7 +27124,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="257" spans="1:23" ht="30">
+    <row r="257" spans="1:23" ht="30" hidden="1">
       <c r="A257" s="3" t="s">
         <v>1517</v>
       </c>
@@ -27083,7 +27193,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="258" spans="1:23">
+    <row r="258" spans="1:23" hidden="1">
       <c r="A258" s="3" t="s">
         <v>1517</v>
       </c>
@@ -27150,7 +27260,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="259" spans="1:23">
+    <row r="259" spans="1:23" hidden="1">
       <c r="A259" s="3" t="s">
         <v>1517</v>
       </c>
@@ -27217,7 +27327,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="260" spans="1:23">
+    <row r="260" spans="1:23" hidden="1">
       <c r="A260" s="3" t="s">
         <v>1517</v>
       </c>
@@ -27284,7 +27394,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="261" spans="1:23">
+    <row r="261" spans="1:23" hidden="1">
       <c r="A261" s="3" t="s">
         <v>1517</v>
       </c>
@@ -27353,7 +27463,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="262" spans="1:23">
+    <row r="262" spans="1:23" hidden="1">
       <c r="A262" s="3" t="s">
         <v>1517</v>
       </c>
@@ -27422,7 +27532,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="263" spans="1:23" ht="30">
+    <row r="263" spans="1:23" ht="30" hidden="1">
       <c r="A263" s="3" t="s">
         <v>1518</v>
       </c>
@@ -27489,7 +27599,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="264" spans="1:23" ht="30">
+    <row r="264" spans="1:23" ht="30" hidden="1">
       <c r="A264" s="3" t="s">
         <v>1518</v>
       </c>
@@ -27556,7 +27666,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="265" spans="1:23" ht="30">
+    <row r="265" spans="1:23" ht="30" hidden="1">
       <c r="A265" s="3" t="s">
         <v>1518</v>
       </c>
@@ -27627,7 +27737,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="266" spans="1:23">
+    <row r="266" spans="1:23" hidden="1">
       <c r="A266" s="3" t="s">
         <v>1518</v>
       </c>
@@ -27694,7 +27804,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="267" spans="1:23" ht="30">
+    <row r="267" spans="1:23" ht="30" hidden="1">
       <c r="A267" s="3" t="s">
         <v>1518</v>
       </c>
@@ -27763,7 +27873,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="268" spans="1:23">
+    <row r="268" spans="1:23" hidden="1">
       <c r="A268" s="3" t="s">
         <v>1518</v>
       </c>
@@ -27832,7 +27942,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="269" spans="1:23">
+    <row r="269" spans="1:23" hidden="1">
       <c r="A269" s="3" t="s">
         <v>1518</v>
       </c>
@@ -27968,7 +28078,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="271" spans="1:23" ht="30">
+    <row r="271" spans="1:23" ht="30" hidden="1">
       <c r="A271" s="3" t="s">
         <v>1518</v>
       </c>
@@ -28035,7 +28145,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="272" spans="1:23">
+    <row r="272" spans="1:23" hidden="1">
       <c r="A272" s="3" t="s">
         <v>1518</v>
       </c>
@@ -28100,7 +28210,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="273" spans="1:23">
+    <row r="273" spans="1:23" hidden="1">
       <c r="A273" s="3" t="s">
         <v>1518</v>
       </c>
@@ -28165,7 +28275,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="274" spans="1:23">
+    <row r="274" spans="1:23" hidden="1">
       <c r="A274" s="3" t="s">
         <v>1518</v>
       </c>
@@ -28230,7 +28340,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="275" spans="1:23">
+    <row r="275" spans="1:23" hidden="1">
       <c r="A275" s="3" t="s">
         <v>1518</v>
       </c>
@@ -28299,7 +28409,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="276" spans="1:23">
+    <row r="276" spans="1:23" hidden="1">
       <c r="A276" s="3" t="s">
         <v>1518</v>
       </c>
@@ -28368,7 +28478,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="277" spans="1:23" ht="30">
+    <row r="277" spans="1:23" ht="30" hidden="1">
       <c r="A277" s="3" t="s">
         <v>1578</v>
       </c>
@@ -28435,7 +28545,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="278" spans="1:23" ht="30">
+    <row r="278" spans="1:23" ht="30" hidden="1">
       <c r="A278" s="3" t="s">
         <v>1578</v>
       </c>
@@ -28502,7 +28612,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="279" spans="1:23" ht="45">
+    <row r="279" spans="1:23" ht="45" hidden="1">
       <c r="A279" s="3" t="s">
         <v>1578</v>
       </c>
@@ -28573,7 +28683,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="280" spans="1:23" ht="30">
+    <row r="280" spans="1:23" ht="30" hidden="1">
       <c r="A280" s="3" t="s">
         <v>1578</v>
       </c>
@@ -28642,7 +28752,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="281" spans="1:23" ht="30">
+    <row r="281" spans="1:23" ht="30" hidden="1">
       <c r="A281" s="3" t="s">
         <v>1578</v>
       </c>
@@ -28711,7 +28821,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="282" spans="1:23" ht="30">
+    <row r="282" spans="1:23" ht="30" hidden="1">
       <c r="A282" s="3" t="s">
         <v>1578</v>
       </c>
@@ -28780,7 +28890,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="283" spans="1:23" ht="30">
+    <row r="283" spans="1:23" ht="30" hidden="1">
       <c r="A283" s="3" t="s">
         <v>1578</v>
       </c>
@@ -28849,7 +28959,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="284" spans="1:23" ht="30">
+    <row r="284" spans="1:23" ht="30" hidden="1">
       <c r="A284" s="3" t="s">
         <v>1578</v>
       </c>
@@ -28985,7 +29095,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="286" spans="1:23" ht="30">
+    <row r="286" spans="1:23" ht="30" hidden="1">
       <c r="A286" s="3" t="s">
         <v>1578</v>
       </c>
@@ -29052,7 +29162,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="287" spans="1:23" ht="30">
+    <row r="287" spans="1:23" ht="30" hidden="1">
       <c r="A287" s="3" t="s">
         <v>1578</v>
       </c>
@@ -29117,7 +29227,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="288" spans="1:23" ht="30">
+    <row r="288" spans="1:23" ht="30" hidden="1">
       <c r="A288" s="3" t="s">
         <v>1578</v>
       </c>
@@ -29182,7 +29292,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="289" spans="1:23" ht="30">
+    <row r="289" spans="1:23" ht="30" hidden="1">
       <c r="A289" s="3" t="s">
         <v>1578</v>
       </c>
@@ -29247,7 +29357,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="290" spans="1:23" ht="30">
+    <row r="290" spans="1:23" ht="30" hidden="1">
       <c r="A290" s="3" t="s">
         <v>1578</v>
       </c>
@@ -29316,7 +29426,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="291" spans="1:23" ht="30">
+    <row r="291" spans="1:23" ht="30" hidden="1">
       <c r="A291" s="3" t="s">
         <v>1578</v>
       </c>
@@ -29385,7 +29495,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="292" spans="1:23" ht="30">
+    <row r="292" spans="1:23" ht="30" hidden="1">
       <c r="A292" s="3" t="s">
         <v>1635</v>
       </c>
@@ -29452,7 +29562,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="293" spans="1:23" ht="30">
+    <row r="293" spans="1:23" ht="30" hidden="1">
       <c r="A293" s="3" t="s">
         <v>1635</v>
       </c>
@@ -29519,7 +29629,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="294" spans="1:23" ht="45">
+    <row r="294" spans="1:23" ht="45" hidden="1">
       <c r="A294" s="3" t="s">
         <v>1635</v>
       </c>
@@ -29588,7 +29698,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="295" spans="1:23">
+    <row r="295" spans="1:23" hidden="1">
       <c r="A295" s="3" t="s">
         <v>1635</v>
       </c>
@@ -29655,7 +29765,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="296" spans="1:23">
+    <row r="296" spans="1:23" hidden="1">
       <c r="A296" s="3" t="s">
         <v>1635</v>
       </c>
@@ -29722,7 +29832,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="297" spans="1:23" ht="30">
+    <row r="297" spans="1:23" ht="30" hidden="1">
       <c r="A297" s="3" t="s">
         <v>1635</v>
       </c>
@@ -29856,7 +29966,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="299" spans="1:23" ht="45">
+    <row r="299" spans="1:23" ht="45" hidden="1">
       <c r="A299" s="3" t="s">
         <v>1635</v>
       </c>
@@ -29925,7 +30035,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="300" spans="1:23" ht="30">
+    <row r="300" spans="1:23" ht="30" hidden="1">
       <c r="A300" s="3" t="s">
         <v>1635</v>
       </c>
@@ -29990,7 +30100,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="301" spans="1:23" ht="30">
+    <row r="301" spans="1:23" ht="30" hidden="1">
       <c r="A301" s="3" t="s">
         <v>1635</v>
       </c>
@@ -30059,7 +30169,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="302" spans="1:23" ht="30">
+    <row r="302" spans="1:23" ht="30" hidden="1">
       <c r="A302" s="3" t="s">
         <v>1635</v>
       </c>
@@ -30126,7 +30236,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="303" spans="1:23" ht="30">
+    <row r="303" spans="1:23" ht="30" hidden="1">
       <c r="A303" s="3" t="s">
         <v>1689</v>
       </c>
@@ -30193,7 +30303,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="304" spans="1:23" ht="30">
+    <row r="304" spans="1:23" ht="30" hidden="1">
       <c r="A304" s="3" t="s">
         <v>1689</v>
       </c>
@@ -30260,7 +30370,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="305" spans="1:23" ht="30">
+    <row r="305" spans="1:23" ht="30" hidden="1">
       <c r="A305" s="3" t="s">
         <v>1689</v>
       </c>
@@ -30329,7 +30439,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="306" spans="1:23" ht="30">
+    <row r="306" spans="1:23" ht="30" hidden="1">
       <c r="A306" s="3" t="s">
         <v>1689</v>
       </c>
@@ -30396,7 +30506,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="307" spans="1:23" ht="30">
+    <row r="307" spans="1:23" ht="30" hidden="1">
       <c r="A307" s="3" t="s">
         <v>1689</v>
       </c>
@@ -30534,7 +30644,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="309" spans="1:23" ht="30">
+    <row r="309" spans="1:23" ht="30" hidden="1">
       <c r="A309" s="3" t="s">
         <v>1689</v>
       </c>
@@ -30601,7 +30711,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="310" spans="1:23" ht="30">
+    <row r="310" spans="1:23" ht="30" hidden="1">
       <c r="A310" s="3" t="s">
         <v>1689</v>
       </c>
@@ -30668,7 +30778,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="311" spans="1:23" ht="30">
+    <row r="311" spans="1:23" ht="30" hidden="1">
       <c r="A311" s="3" t="s">
         <v>1689</v>
       </c>
@@ -30733,7 +30843,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="312" spans="1:23" ht="30">
+    <row r="312" spans="1:23" ht="30" hidden="1">
       <c r="A312" s="3" t="s">
         <v>1689</v>
       </c>
@@ -30800,7 +30910,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="313" spans="1:23" ht="45">
+    <row r="313" spans="1:23" ht="45" hidden="1">
       <c r="A313" s="3" t="s">
         <v>1689</v>
       </c>
@@ -30869,7 +30979,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="314" spans="1:23" ht="30">
+    <row r="314" spans="1:23" ht="30" hidden="1">
       <c r="A314" s="3" t="s">
         <v>1689</v>
       </c>
@@ -30938,7 +31048,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="315" spans="1:23" ht="30">
+    <row r="315" spans="1:23" ht="30" hidden="1">
       <c r="A315" s="3" t="s">
         <v>1704</v>
       </c>
@@ -31005,7 +31115,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="316" spans="1:23" ht="30">
+    <row r="316" spans="1:23" ht="30" hidden="1">
       <c r="A316" s="3" t="s">
         <v>1704</v>
       </c>
@@ -31074,7 +31184,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="317" spans="1:23">
+    <row r="317" spans="1:23" hidden="1">
       <c r="A317" s="3" t="s">
         <v>1704</v>
       </c>
@@ -31143,7 +31253,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="318" spans="1:23" ht="30">
+    <row r="318" spans="1:23" ht="30" hidden="1">
       <c r="A318" s="3" t="s">
         <v>1704</v>
       </c>
@@ -31212,7 +31322,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="319" spans="1:23">
+    <row r="319" spans="1:23" hidden="1">
       <c r="A319" s="3" t="s">
         <v>1704</v>
       </c>
@@ -31350,7 +31460,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="321" spans="1:23" ht="30">
+    <row r="321" spans="1:23" ht="30" hidden="1">
       <c r="A321" s="3" t="s">
         <v>1704</v>
       </c>
@@ -31417,7 +31527,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="322" spans="1:23">
+    <row r="322" spans="1:23" hidden="1">
       <c r="A322" s="3" t="s">
         <v>1704</v>
       </c>
@@ -31482,7 +31592,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="323" spans="1:23" ht="30">
+    <row r="323" spans="1:23" ht="30" hidden="1">
       <c r="A323" s="3" t="s">
         <v>1704</v>
       </c>
@@ -31551,7 +31661,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="324" spans="1:23">
+    <row r="324" spans="1:23" hidden="1">
       <c r="A324" s="3" t="s">
         <v>1704</v>
       </c>
@@ -31620,7 +31730,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="325" spans="1:23" ht="30">
+    <row r="325" spans="1:23" ht="30" hidden="1">
       <c r="A325" s="3" t="s">
         <v>1806</v>
       </c>
@@ -31687,7 +31797,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="326" spans="1:23" ht="30">
+    <row r="326" spans="1:23" ht="30" hidden="1">
       <c r="A326" s="3" t="s">
         <v>1806</v>
       </c>
@@ -31754,7 +31864,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="327" spans="1:23" ht="30">
+    <row r="327" spans="1:23" ht="30" hidden="1">
       <c r="A327" s="3" t="s">
         <v>1806</v>
       </c>
@@ -31821,7 +31931,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="328" spans="1:23" ht="30">
+    <row r="328" spans="1:23" ht="30" hidden="1">
       <c r="A328" s="3" t="s">
         <v>1806</v>
       </c>
@@ -31890,7 +32000,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="329" spans="1:23" ht="45">
+    <row r="329" spans="1:23" ht="45" hidden="1">
       <c r="A329" s="3" t="s">
         <v>1806</v>
       </c>
@@ -31959,7 +32069,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="330" spans="1:23" ht="30">
+    <row r="330" spans="1:23" ht="30" hidden="1">
       <c r="A330" s="3" t="s">
         <v>1806</v>
       </c>
@@ -32026,7 +32136,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="331" spans="1:23" ht="30">
+    <row r="331" spans="1:23" ht="30" hidden="1">
       <c r="A331" s="3" t="s">
         <v>1806</v>
       </c>
@@ -32162,7 +32272,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="333" spans="1:23" ht="30">
+    <row r="333" spans="1:23" ht="30" hidden="1">
       <c r="A333" s="3" t="s">
         <v>1806</v>
       </c>
@@ -32229,7 +32339,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="334" spans="1:23" ht="30">
+    <row r="334" spans="1:23" ht="30" hidden="1">
       <c r="A334" s="3" t="s">
         <v>1806</v>
       </c>
@@ -32296,7 +32406,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="335" spans="1:23" ht="30">
+    <row r="335" spans="1:23" ht="30" hidden="1">
       <c r="A335" s="3" t="s">
         <v>1806</v>
       </c>
@@ -32361,7 +32471,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="336" spans="1:23" ht="30">
+    <row r="336" spans="1:23" ht="30" hidden="1">
       <c r="A336" s="3" t="s">
         <v>1806</v>
       </c>
@@ -32428,7 +32538,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="337" spans="1:23" ht="45">
+    <row r="337" spans="1:23" ht="45" hidden="1">
       <c r="A337" s="3" t="s">
         <v>1806</v>
       </c>
@@ -32497,7 +32607,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="338" spans="1:23" ht="30">
+    <row r="338" spans="1:23" ht="30" hidden="1">
       <c r="A338" s="3" t="s">
         <v>1806</v>
       </c>
@@ -32566,7 +32676,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="339" spans="1:23">
+    <row r="339" spans="1:23" hidden="1">
       <c r="A339" s="3" t="s">
         <v>1914</v>
       </c>
@@ -32635,7 +32745,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="340" spans="1:23">
+    <row r="340" spans="1:23" hidden="1">
       <c r="A340" s="3" t="s">
         <v>1914</v>
       </c>
@@ -32704,7 +32814,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="341" spans="1:23">
+    <row r="341" spans="1:23" hidden="1">
       <c r="A341" s="3" t="s">
         <v>1914</v>
       </c>
@@ -32773,7 +32883,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="342" spans="1:23" ht="30">
+    <row r="342" spans="1:23" ht="30" hidden="1">
       <c r="A342" s="3" t="s">
         <v>1914</v>
       </c>
@@ -32842,7 +32952,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="343" spans="1:23" ht="30">
+    <row r="343" spans="1:23" ht="30" hidden="1">
       <c r="A343" s="3" t="s">
         <v>1914</v>
       </c>
@@ -32913,7 +33023,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="344" spans="1:23" ht="30">
+    <row r="344" spans="1:23" ht="30" hidden="1">
       <c r="A344" s="3" t="s">
         <v>1914</v>
       </c>
@@ -32982,7 +33092,7 @@
         <v>1960</v>
       </c>
     </row>
-    <row r="345" spans="1:23">
+    <row r="345" spans="1:23" hidden="1">
       <c r="A345" s="3" t="s">
         <v>1914</v>
       </c>
@@ -33124,7 +33234,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="347" spans="1:23" ht="30">
+    <row r="347" spans="1:23" ht="30" hidden="1">
       <c r="A347" s="3" t="s">
         <v>1914</v>
       </c>
@@ -33195,7 +33305,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="348" spans="1:23">
+    <row r="348" spans="1:23" hidden="1">
       <c r="A348" s="3" t="s">
         <v>1914</v>
       </c>
@@ -33264,7 +33374,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="349" spans="1:23" ht="30">
+    <row r="349" spans="1:23" ht="30" hidden="1">
       <c r="A349" s="3" t="s">
         <v>1914</v>
       </c>
@@ -33335,7 +33445,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="350" spans="1:23" ht="30">
+    <row r="350" spans="1:23" ht="30" hidden="1">
       <c r="A350" s="3" t="s">
         <v>1914</v>
       </c>
@@ -33404,7 +33514,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="351" spans="1:23" ht="30">
+    <row r="351" spans="1:23" ht="30" hidden="1">
       <c r="A351" s="3" t="s">
         <v>1914</v>
       </c>
@@ -33475,7 +33585,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="352" spans="1:23" ht="30">
+    <row r="352" spans="1:23" ht="30" hidden="1">
       <c r="A352" s="3" t="s">
         <v>1914</v>
       </c>
@@ -33546,7 +33656,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="353" spans="1:23" ht="30">
+    <row r="353" spans="1:23" ht="30" hidden="1">
       <c r="A353" s="3" t="s">
         <v>1922</v>
       </c>
@@ -33615,7 +33725,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="354" spans="1:23" ht="30">
+    <row r="354" spans="1:23" ht="30" hidden="1">
       <c r="A354" s="3" t="s">
         <v>1922</v>
       </c>
@@ -33684,7 +33794,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="355" spans="1:23">
+    <row r="355" spans="1:23" hidden="1">
       <c r="A355" s="3" t="s">
         <v>1922</v>
       </c>
@@ -33753,7 +33863,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="356" spans="1:23" ht="45">
+    <row r="356" spans="1:23" ht="45" hidden="1">
       <c r="A356" s="3" t="s">
         <v>1922</v>
       </c>
@@ -33893,7 +34003,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="358" spans="1:23" ht="30">
+    <row r="358" spans="1:23" ht="30" hidden="1">
       <c r="A358" s="4" t="s">
         <v>2018</v>
       </c>
@@ -33964,7 +34074,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="359" spans="1:23" ht="30">
+    <row r="359" spans="1:23" ht="30" hidden="1">
       <c r="A359" s="4" t="s">
         <v>2018</v>
       </c>
@@ -34035,7 +34145,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="360" spans="1:23" ht="30">
+    <row r="360" spans="1:23" ht="30" hidden="1">
       <c r="A360" s="4" t="s">
         <v>2018</v>
       </c>
@@ -34177,7 +34287,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="362" spans="1:23" ht="30">
+    <row r="362" spans="1:23" ht="30" hidden="1">
       <c r="A362" s="4" t="s">
         <v>2018</v>
       </c>
@@ -34248,7 +34358,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="363" spans="1:23" ht="30">
+    <row r="363" spans="1:23" ht="30" hidden="1">
       <c r="A363" s="4" t="s">
         <v>2018</v>
       </c>
@@ -34319,7 +34429,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="364" spans="1:23" ht="30">
+    <row r="364" spans="1:23" ht="30" hidden="1">
       <c r="A364" s="4" t="s">
         <v>2018</v>
       </c>
@@ -34390,7 +34500,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="365" spans="1:23" ht="30">
+    <row r="365" spans="1:23" ht="30" hidden="1">
       <c r="A365" s="4" t="s">
         <v>2018</v>
       </c>
@@ -34461,7 +34571,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="366" spans="1:23" ht="30">
+    <row r="366" spans="1:23" ht="30" hidden="1">
       <c r="A366" s="4" t="s">
         <v>2018</v>
       </c>
@@ -34532,7 +34642,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="367" spans="1:23" ht="30">
+    <row r="367" spans="1:23" ht="30" hidden="1">
       <c r="A367" s="4" t="s">
         <v>2018</v>
       </c>
@@ -34603,7 +34713,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="368" spans="1:23" ht="30">
+    <row r="368" spans="1:23" ht="30" hidden="1">
       <c r="A368" s="4" t="s">
         <v>2062</v>
       </c>
@@ -34674,7 +34784,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="369" spans="1:23" ht="30">
+    <row r="369" spans="1:23" ht="30" hidden="1">
       <c r="A369" s="4" t="s">
         <v>2062</v>
       </c>
@@ -34745,7 +34855,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="370" spans="1:23" ht="30">
+    <row r="370" spans="1:23" ht="30" hidden="1">
       <c r="A370" s="4" t="s">
         <v>2062</v>
       </c>
@@ -34887,7 +34997,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="372" spans="1:23" ht="30">
+    <row r="372" spans="1:23" ht="30" hidden="1">
       <c r="A372" s="4" t="s">
         <v>2062</v>
       </c>
@@ -34958,7 +35068,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="373" spans="1:23" ht="45">
+    <row r="373" spans="1:23" ht="45" hidden="1">
       <c r="A373" s="4" t="s">
         <v>2062</v>
       </c>
@@ -35029,7 +35139,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="374" spans="1:23" ht="30">
+    <row r="374" spans="1:23" ht="30" hidden="1">
       <c r="A374" s="4" t="s">
         <v>2062</v>
       </c>
@@ -35100,7 +35210,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="375" spans="1:23" ht="30">
+    <row r="375" spans="1:23" ht="30" hidden="1">
       <c r="A375" s="4" t="s">
         <v>2062</v>
       </c>
@@ -35171,7 +35281,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="376" spans="1:23" ht="30">
+    <row r="376" spans="1:23" ht="30" hidden="1">
       <c r="A376" s="4" t="s">
         <v>2062</v>
       </c>
@@ -35242,7 +35352,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="377" spans="1:23" ht="30">
+    <row r="377" spans="1:23" ht="30" hidden="1">
       <c r="A377" s="4" t="s">
         <v>2062</v>
       </c>
@@ -35313,7 +35423,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="378" spans="1:23" ht="30">
+    <row r="378" spans="1:23" ht="30" hidden="1">
       <c r="A378" s="4" t="s">
         <v>2062</v>
       </c>
@@ -35384,7 +35494,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="379" spans="1:23" ht="30">
+    <row r="379" spans="1:23" ht="30" hidden="1">
       <c r="A379" s="4" t="s">
         <v>2062</v>
       </c>
@@ -35455,7 +35565,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="380" spans="1:23">
+    <row r="380" spans="1:23" hidden="1">
       <c r="A380" s="4" t="s">
         <v>2110</v>
       </c>
@@ -35526,7 +35636,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="381" spans="1:23" ht="30">
+    <row r="381" spans="1:23" ht="30" hidden="1">
       <c r="A381" s="4" t="s">
         <v>2110</v>
       </c>
@@ -35597,7 +35707,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="382" spans="1:23" ht="30">
+    <row r="382" spans="1:23" ht="30" hidden="1">
       <c r="A382" s="4" t="s">
         <v>2110</v>
       </c>
@@ -35668,7 +35778,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="383" spans="1:23" ht="45">
+    <row r="383" spans="1:23" ht="45" hidden="1">
       <c r="A383" s="4" t="s">
         <v>2110</v>
       </c>
@@ -35736,7 +35846,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="384" spans="1:23" ht="30">
+    <row r="384" spans="1:23" ht="30" hidden="1">
       <c r="A384" s="4" t="s">
         <v>2110</v>
       </c>
@@ -35804,7 +35914,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="385" spans="1:23" ht="45">
+    <row r="385" spans="1:23" ht="45" hidden="1">
       <c r="A385" s="4" t="s">
         <v>2110</v>
       </c>
@@ -35875,7 +35985,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="386" spans="1:23" ht="30">
+    <row r="386" spans="1:23" ht="30" hidden="1">
       <c r="A386" s="4" t="s">
         <v>2110</v>
       </c>
@@ -35946,7 +36056,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="387" spans="1:23" ht="30">
+    <row r="387" spans="1:23" ht="30" hidden="1">
       <c r="A387" s="4" t="s">
         <v>2110</v>
       </c>
@@ -36014,7 +36124,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="388" spans="1:23" ht="30">
+    <row r="388" spans="1:23" ht="30" hidden="1">
       <c r="A388" s="4" t="s">
         <v>2110</v>
       </c>
@@ -36082,7 +36192,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="389" spans="1:23" ht="30">
+    <row r="389" spans="1:23" ht="30" hidden="1">
       <c r="A389" s="4" t="s">
         <v>2110</v>
       </c>
@@ -36221,7 +36331,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="391" spans="1:23" ht="30">
+    <row r="391" spans="1:23" ht="30" hidden="1">
       <c r="A391" s="4" t="s">
         <v>2110</v>
       </c>
@@ -36292,7 +36402,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="392" spans="1:23" ht="30">
+    <row r="392" spans="1:23" ht="30" hidden="1">
       <c r="A392" s="4" t="s">
         <v>2110</v>
       </c>
@@ -36363,7 +36473,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="393" spans="1:23" ht="30">
+    <row r="393" spans="1:23" ht="30" hidden="1">
       <c r="A393" s="4" t="s">
         <v>2110</v>
       </c>
@@ -36434,7 +36544,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="394" spans="1:23" ht="30">
+    <row r="394" spans="1:23" ht="30" hidden="1">
       <c r="A394" s="4" t="s">
         <v>2110</v>
       </c>
@@ -36505,7 +36615,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="395" spans="1:23" ht="30">
+    <row r="395" spans="1:23" ht="30" hidden="1">
       <c r="A395" s="4" t="s">
         <v>2110</v>
       </c>
@@ -36576,7 +36686,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="396" spans="1:23" ht="30">
+    <row r="396" spans="1:23" ht="30" hidden="1">
       <c r="A396" s="4" t="s">
         <v>2110</v>
       </c>
@@ -36648,7 +36758,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W396" xr:uid="{7E21F442-9136-4C15-8BA3-92E07332B93A}"/>
+  <autoFilter ref="A1:W396" xr:uid="{7E21F442-9136-4C15-8BA3-92E07332B93A}">
+    <filterColumn colId="10">
+      <filters>
+        <filter val="Status"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <hyperlinks>
     <hyperlink ref="Q9" r:id="rId1" display="mailto:admin@memgine.com" xr:uid="{93170BB8-77D4-4002-829B-D89928109808}"/>
     <hyperlink ref="Q11" r:id="rId2" display="https://memgine.com/" xr:uid="{F8EB4105-6CCB-4B06-B657-948DB365F556}"/>
@@ -38981,6 +39097,373 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B7B29B1-81FD-48F8-9727-C5470F35164D}">
+  <dimension ref="A1:D25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="3" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="48.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="67.85546875" style="4" customWidth="1"/>
+    <col min="5" max="16384" width="9.140625" style="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="18" t="s">
+        <v>2233</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>2225</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>2234</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="5">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="16" t="s">
+        <v>2226</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>2235</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="5">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>2236</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>2237</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="5">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>2227</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>2235</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>315</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>2238</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="5">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>341</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>2239</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>2240</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="5">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>370</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>2241</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>2238</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="30">
+      <c r="A8" s="5">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>2242</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>2243</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>2240</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="5">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>2228</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>2244</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="5">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>490</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>489</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>2244</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="5">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>548</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>2229</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>2244</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="5">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>620</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>964</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" s="5">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>673</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>2230</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>2246</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" s="5">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" s="16" t="s">
+        <v>732</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>2247</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" s="5">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>796</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>2248</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" s="5">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>2062</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>2249</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>2240</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" s="5">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>1518</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>2231</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>2250</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" s="5">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>1578</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>2232</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>2250</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" s="5">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>1635</v>
+      </c>
+      <c r="C19" s="16" t="s">
+        <v>1633</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>2251</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" s="5">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>1689</v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>1688</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>2252</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
+      <c r="A21" s="5">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>1704</v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>1729</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>2238</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
+      <c r="A22" s="5">
+        <v>21</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>1806</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>1805</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>2253</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" s="5">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>1914</v>
+      </c>
+      <c r="C23" s="16" t="s">
+        <v>2254</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>2255</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24" s="5">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>1922</v>
+      </c>
+      <c r="C24" s="16" t="s">
+        <v>2256</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>2238</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" s="5">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>2110</v>
+      </c>
+      <c r="C25" s="16" t="s">
+        <v>2107</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>2257</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C85B9BC7-C8C8-4E3E-A0EF-02B9554CEAE5}">
   <dimension ref="A1:K63"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -41211,7 +41694,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6E5E88D-7637-4195-842B-FF426225AADB}">
   <dimension ref="A1:I36"/>
   <sheetFormatPr defaultRowHeight="15"/>

</xml_diff>

<commit_message>
ref data update for all ref data in a separate sheet
</commit_message>
<xml_diff>
--- a/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
+++ b/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MynikaTech\memgine\docs\domain\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D0E5EAC-9517-4640-A34C-6226E976EC36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2482C28D-D177-4072-94BA-F6C6E384582F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{AA28BC4D-8219-43B9-8C16-6977709D904A}"/>
   </bookViews>
@@ -16,14 +16,15 @@
     <sheet name="Entity Catalogue" sheetId="1" r:id="rId1"/>
     <sheet name="Atributes" sheetId="2" r:id="rId2"/>
     <sheet name="Reference Data" sheetId="3" r:id="rId3"/>
-    <sheet name="Sheet1" sheetId="6" r:id="rId4"/>
-    <sheet name="Relationships" sheetId="4" r:id="rId5"/>
-    <sheet name="Validation Rules" sheetId="5" r:id="rId6"/>
+    <sheet name="Status Ref Data" sheetId="6" r:id="rId4"/>
+    <sheet name="Entity Ref Data" sheetId="7" r:id="rId5"/>
+    <sheet name="Relationships" sheetId="4" r:id="rId6"/>
+    <sheet name="Validation Rules" sheetId="5" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Atributes!$A$1:$W$396</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Reference Data'!$A$1:$H$92</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Relationships!$A$1:$K$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Relationships!$A$1:$K$63</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10285" uniqueCount="2258">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10694" uniqueCount="2298">
   <si>
     <t>Domain</t>
   </si>
@@ -6809,6 +6810,126 @@
   </si>
   <si>
     <t>DRAFT, ACTIVE, INACTIVE, EXPIRED, CANCELLED</t>
+  </si>
+  <si>
+    <t>Company-owned physical branch</t>
+  </si>
+  <si>
+    <t>Canadian Dollar</t>
+  </si>
+  <si>
+    <t>Coffee chain</t>
+  </si>
+  <si>
+    <t>Fitness centre</t>
+  </si>
+  <si>
+    <t>Yoga studio</t>
+  </si>
+  <si>
+    <t>Retail store</t>
+  </si>
+  <si>
+    <t>Educational institute</t>
+  </si>
+  <si>
+    <t>Theme park</t>
+  </si>
+  <si>
+    <t>Coworking space</t>
+  </si>
+  <si>
+    <t>Automobile service centre</t>
+  </si>
+  <si>
+    <t>External payment gateway or payment service integration</t>
+  </si>
+  <si>
+    <t>Point of Sale system integration</t>
+  </si>
+  <si>
+    <t>ERP system integration</t>
+  </si>
+  <si>
+    <t>CRM platform integration</t>
+  </si>
+  <si>
+    <t>SMS gateway integration</t>
+  </si>
+  <si>
+    <t>Cloud file storage integration</t>
+  </si>
+  <si>
+    <t>Needs final catalogue</t>
+  </si>
+  <si>
+    <t>CA</t>
+  </si>
+  <si>
+    <t>Canada</t>
+  </si>
+  <si>
+    <t>ISO 3166-1 alpha-2</t>
+  </si>
+  <si>
+    <t>US</t>
+  </si>
+  <si>
+    <t>United States</t>
+  </si>
+  <si>
+    <t>IN</t>
+  </si>
+  <si>
+    <t>Region / State / Province</t>
+  </si>
+  <si>
+    <t>First-level administrative region within a country</t>
+  </si>
+  <si>
+    <t>Country-dependent; use ISO/official administrative codes where available</t>
+  </si>
+  <si>
+    <t>City/locality within a country and region</t>
+  </si>
+  <si>
+    <t>Country + Region dependent</t>
+  </si>
+  <si>
+    <t>Accounting/bookkeeping integration</t>
+  </si>
+  <si>
+    <t>Loyalty/rewards integration</t>
+  </si>
+  <si>
+    <t>Online commerce integration</t>
+  </si>
+  <si>
+    <t>Authentication/SSO integration</t>
+  </si>
+  <si>
+    <t>Email provider integration</t>
+  </si>
+  <si>
+    <t>WhatsApp messaging integration</t>
+  </si>
+  <si>
+    <t>Push notification integration</t>
+  </si>
+  <si>
+    <t>Reporting/analytics integration</t>
+  </si>
+  <si>
+    <t>Inbound/outbound webhook integration</t>
+  </si>
+  <si>
+    <t>Generic API integration</t>
+  </si>
+  <si>
+    <t>Proprietary external integration</t>
+  </si>
+  <si>
+    <t>Platform presentation template</t>
   </si>
 </sst>
 </file>
@@ -6884,7 +7005,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -6937,6 +7058,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -9785,7 +9909,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:23" hidden="1">
+    <row r="7" spans="1:23">
       <c r="A7" s="10" t="s">
         <v>5</v>
       </c>
@@ -9853,7 +9977,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:23">
+    <row r="8" spans="1:23" hidden="1">
       <c r="A8" s="10" t="s">
         <v>5</v>
       </c>
@@ -11142,7 +11266,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="27" spans="1:23" ht="30">
+    <row r="27" spans="1:23" ht="30" hidden="1">
       <c r="A27" s="3" t="s">
         <v>8</v>
       </c>
@@ -11830,7 +11954,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="37" spans="1:23" ht="45" hidden="1">
+    <row r="37" spans="1:23" ht="45">
       <c r="A37" s="3" t="s">
         <v>37</v>
       </c>
@@ -11901,7 +12025,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="38" spans="1:23" ht="30">
+    <row r="38" spans="1:23" ht="30" hidden="1">
       <c r="A38" s="3" t="s">
         <v>37</v>
       </c>
@@ -12657,7 +12781,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="50" spans="1:23" ht="30">
+    <row r="50" spans="1:23" ht="30" hidden="1">
       <c r="A50" s="3" t="s">
         <v>317</v>
       </c>
@@ -12908,7 +13032,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="54" spans="1:23" ht="30">
+    <row r="54" spans="1:23" ht="30" hidden="1">
       <c r="A54" s="4" t="s">
         <v>341</v>
       </c>
@@ -13668,7 +13792,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="65" spans="1:23" ht="30">
+    <row r="65" spans="1:23" ht="30" hidden="1">
       <c r="A65" s="4" t="s">
         <v>370</v>
       </c>
@@ -14307,7 +14431,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="74" spans="1:23" ht="30" hidden="1">
+    <row r="74" spans="1:23" ht="30">
       <c r="A74" s="4" t="s">
         <v>10</v>
       </c>
@@ -14378,7 +14502,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="75" spans="1:23" ht="30" hidden="1">
+    <row r="75" spans="1:23" ht="30">
       <c r="A75" s="4" t="s">
         <v>10</v>
       </c>
@@ -14520,7 +14644,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="77" spans="1:23" ht="30">
+    <row r="77" spans="1:23" ht="30" hidden="1">
       <c r="A77" s="4" t="s">
         <v>10</v>
       </c>
@@ -15443,7 +15567,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="90" spans="1:23" hidden="1">
+    <row r="90" spans="1:23">
       <c r="A90" s="4" t="s">
         <v>490</v>
       </c>
@@ -15514,7 +15638,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="91" spans="1:23" hidden="1">
+    <row r="91" spans="1:23">
       <c r="A91" s="4" t="s">
         <v>490</v>
       </c>
@@ -15656,7 +15780,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="93" spans="1:23" ht="30">
+    <row r="93" spans="1:23" ht="30" hidden="1">
       <c r="A93" s="4" t="s">
         <v>490</v>
       </c>
@@ -16863,7 +16987,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="110" spans="1:23" ht="30" hidden="1">
+    <row r="110" spans="1:23" ht="30">
       <c r="A110" s="4" t="s">
         <v>548</v>
       </c>
@@ -16934,7 +17058,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="111" spans="1:23">
+    <row r="111" spans="1:23" hidden="1">
       <c r="A111" s="4" t="s">
         <v>548</v>
       </c>
@@ -18070,7 +18194,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="127" spans="1:23">
+    <row r="127" spans="1:23" hidden="1">
       <c r="A127" s="4" t="s">
         <v>620</v>
       </c>
@@ -19206,7 +19330,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="143" spans="1:23" ht="30">
+    <row r="143" spans="1:23" ht="30" hidden="1">
       <c r="A143" s="4" t="s">
         <v>673</v>
       </c>
@@ -19987,7 +20111,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="154" spans="1:23" hidden="1">
+    <row r="154" spans="1:23">
       <c r="A154" s="4" t="s">
         <v>34</v>
       </c>
@@ -20200,7 +20324,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="157" spans="1:23" ht="30">
+    <row r="157" spans="1:23" ht="30" hidden="1">
       <c r="A157" s="4" t="s">
         <v>34</v>
       </c>
@@ -21407,7 +21531,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="174" spans="1:23" ht="30">
+    <row r="174" spans="1:23" ht="30" hidden="1">
       <c r="A174" s="4" t="s">
         <v>35</v>
       </c>
@@ -28011,7 +28135,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="270" spans="1:23" ht="30">
+    <row r="270" spans="1:23" ht="30" hidden="1">
       <c r="A270" s="3" t="s">
         <v>1518</v>
       </c>
@@ -29028,7 +29152,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="285" spans="1:23" ht="30">
+    <row r="285" spans="1:23" ht="30" hidden="1">
       <c r="A285" s="3" t="s">
         <v>1578</v>
       </c>
@@ -29765,7 +29889,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="296" spans="1:23" hidden="1">
+    <row r="296" spans="1:23">
       <c r="A296" s="3" t="s">
         <v>1635</v>
       </c>
@@ -29899,7 +30023,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="298" spans="1:23">
+    <row r="298" spans="1:23" hidden="1">
       <c r="A298" s="3" t="s">
         <v>1635</v>
       </c>
@@ -30439,7 +30563,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="306" spans="1:23" ht="30" hidden="1">
+    <row r="306" spans="1:23" ht="30">
       <c r="A306" s="3" t="s">
         <v>1689</v>
       </c>
@@ -30575,7 +30699,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="308" spans="1:23" ht="30">
+    <row r="308" spans="1:23" ht="30" hidden="1">
       <c r="A308" s="3" t="s">
         <v>1689</v>
       </c>
@@ -31391,7 +31515,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="320" spans="1:23" ht="30">
+    <row r="320" spans="1:23" ht="30" hidden="1">
       <c r="A320" s="3" t="s">
         <v>1704</v>
       </c>
@@ -32203,7 +32327,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="332" spans="1:23" ht="30">
+    <row r="332" spans="1:23" ht="30" hidden="1">
       <c r="A332" s="3" t="s">
         <v>1806</v>
       </c>
@@ -32745,7 +32869,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="340" spans="1:23" hidden="1">
+    <row r="340" spans="1:23">
       <c r="A340" s="3" t="s">
         <v>1914</v>
       </c>
@@ -33163,7 +33287,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="346" spans="1:23" ht="30">
+    <row r="346" spans="1:23" ht="30" hidden="1">
       <c r="A346" s="3" t="s">
         <v>1914</v>
       </c>
@@ -33932,7 +34056,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="357" spans="1:23" ht="30">
+    <row r="357" spans="1:23" ht="30" hidden="1">
       <c r="A357" s="3" t="s">
         <v>1922</v>
       </c>
@@ -34216,7 +34340,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="361" spans="1:23" ht="45">
+    <row r="361" spans="1:23" ht="45" hidden="1">
       <c r="A361" s="4" t="s">
         <v>2018</v>
       </c>
@@ -34926,7 +35050,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="371" spans="1:23" ht="30">
+    <row r="371" spans="1:23" ht="30" hidden="1">
       <c r="A371" s="4" t="s">
         <v>2062</v>
       </c>
@@ -36260,7 +36384,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="390" spans="1:23" ht="30">
+    <row r="390" spans="1:23" ht="30" hidden="1">
       <c r="A390" s="4" t="s">
         <v>2110</v>
       </c>
@@ -36761,7 +36885,16 @@
   <autoFilter ref="A1:W396" xr:uid="{7E21F442-9136-4C15-8BA3-92E07332B93A}">
     <filterColumn colId="10">
       <filters>
-        <filter val="Status"/>
+        <filter val="Benefit Category"/>
+        <filter val="Benefit Type"/>
+        <filter val="Currency"/>
+        <filter val="Integration Type"/>
+        <filter val="Organization Type"/>
+        <filter val="Organization User Type"/>
+        <filter val="Product Category"/>
+        <filter val="Product Type"/>
+        <filter val="Store Type"/>
+        <filter val="Template Type"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -39464,6 +39597,1689 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DCF67D5-27CE-4C3A-997A-96A77E128378}">
+  <dimension ref="A1:H71"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="24.85546875" style="4" customWidth="1"/>
+    <col min="2" max="2" width="26.140625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="19.5703125" style="4" customWidth="1"/>
+    <col min="4" max="4" width="21.7109375" style="4" customWidth="1"/>
+    <col min="5" max="5" width="20" style="4" customWidth="1"/>
+    <col min="6" max="6" width="21" style="4" customWidth="1"/>
+    <col min="7" max="7" width="16.28515625" style="4" customWidth="1"/>
+    <col min="8" max="8" width="27.85546875" style="4" customWidth="1"/>
+    <col min="9" max="16384" width="9.140625" style="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>851</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>852</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="19" t="s">
+        <v>853</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>854</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>2275</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>2276</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="E2" s="5">
+        <v>1</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>2277</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3" t="s">
+        <v>2278</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>2279</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="E3" s="5">
+        <v>2</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>2277</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3" t="s">
+        <v>2280</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="E4" s="5">
+        <v>3</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>2277</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="45">
+      <c r="A5" s="13" t="s">
+        <v>2281</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>2282</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>2283</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="30">
+      <c r="A6" s="13" t="s">
+        <v>1480</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>2284</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>2285</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>899</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>900</v>
+      </c>
+      <c r="E7" s="5">
+        <v>1</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>901</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" s="3"/>
+      <c r="B8" s="3" t="s">
+        <v>902</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>903</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>904</v>
+      </c>
+      <c r="E8" s="5">
+        <v>2</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>901</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="30">
+      <c r="A9" s="13" t="s">
+        <v>757</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>887</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>762</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>2258</v>
+      </c>
+      <c r="E9" s="5">
+        <v>1</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H9" s="3"/>
+    </row>
+    <row r="10" spans="1:8" ht="30">
+      <c r="A10" s="3"/>
+      <c r="B10" s="3" t="s">
+        <v>889</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>890</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>891</v>
+      </c>
+      <c r="E10" s="5">
+        <v>2</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H10" s="3"/>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="3"/>
+      <c r="B11" s="3" t="s">
+        <v>892</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>893</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>894</v>
+      </c>
+      <c r="E11" s="5">
+        <v>3</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H11" s="3"/>
+    </row>
+    <row r="12" spans="1:8" ht="30">
+      <c r="A12" s="13" t="s">
+        <v>313</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>855</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>856</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>928</v>
+      </c>
+      <c r="E12" s="5">
+        <v>1</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="30">
+      <c r="A13" s="3"/>
+      <c r="B13" s="3" t="s">
+        <v>929</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>930</v>
+      </c>
+      <c r="E13" s="5">
+        <v>2</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="3"/>
+      <c r="B14" s="3" t="s">
+        <v>931</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>932</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>933</v>
+      </c>
+      <c r="E14" s="5">
+        <v>3</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="30">
+      <c r="A15" s="3"/>
+      <c r="B15" s="3" t="s">
+        <v>866</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>934</v>
+      </c>
+      <c r="E15" s="5">
+        <v>4</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" s="13" t="s">
+        <v>445</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>959</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>960</v>
+      </c>
+      <c r="E16" s="5">
+        <v>1</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H16" s="3"/>
+    </row>
+    <row r="17" spans="1:8">
+      <c r="A17" s="3"/>
+      <c r="B17" s="3" t="s">
+        <v>961</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>962</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>963</v>
+      </c>
+      <c r="E17" s="5">
+        <v>2</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H17" s="3"/>
+    </row>
+    <row r="18" spans="1:8">
+      <c r="A18" s="3"/>
+      <c r="B18" s="3" t="s">
+        <v>964</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>620</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>965</v>
+      </c>
+      <c r="E18" s="5">
+        <v>3</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H18" s="3"/>
+    </row>
+    <row r="19" spans="1:8" ht="30">
+      <c r="A19" s="13" t="s">
+        <v>451</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>966</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>456</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>967</v>
+      </c>
+      <c r="E19" s="5">
+        <v>1</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H19" s="3"/>
+    </row>
+    <row r="20" spans="1:8">
+      <c r="A20" s="3"/>
+      <c r="B20" s="3" t="s">
+        <v>968</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>969</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>970</v>
+      </c>
+      <c r="E20" s="5">
+        <v>2</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H20" s="3"/>
+    </row>
+    <row r="21" spans="1:8" ht="30">
+      <c r="A21" s="3"/>
+      <c r="B21" s="3" t="s">
+        <v>971</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>972</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>973</v>
+      </c>
+      <c r="E21" s="5">
+        <v>3</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H21" s="3"/>
+    </row>
+    <row r="22" spans="1:8">
+      <c r="A22" s="13" t="s">
+        <v>512</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>974</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>975</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>976</v>
+      </c>
+      <c r="E22" s="5">
+        <v>1</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H22" s="3"/>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23" s="3"/>
+      <c r="B23" s="3" t="s">
+        <v>977</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>978</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>979</v>
+      </c>
+      <c r="E23" s="5">
+        <v>2</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H23" s="3"/>
+    </row>
+    <row r="24" spans="1:8">
+      <c r="A24" s="3"/>
+      <c r="B24" s="3" t="s">
+        <v>980</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>523</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>981</v>
+      </c>
+      <c r="E24" s="5">
+        <v>3</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H24" s="3"/>
+    </row>
+    <row r="25" spans="1:8">
+      <c r="A25" s="3"/>
+      <c r="B25" s="3" t="s">
+        <v>982</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>983</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>984</v>
+      </c>
+      <c r="E25" s="5">
+        <v>4</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H25" s="3"/>
+    </row>
+    <row r="26" spans="1:8" ht="30">
+      <c r="A26" s="13" t="s">
+        <v>518</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>985</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>986</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>987</v>
+      </c>
+      <c r="E26" s="5">
+        <v>1</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G26" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H26" s="3"/>
+    </row>
+    <row r="27" spans="1:8" ht="30">
+      <c r="A27" s="3"/>
+      <c r="B27" s="3" t="s">
+        <v>988</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>989</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>990</v>
+      </c>
+      <c r="E27" s="5">
+        <v>2</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H27" s="3"/>
+    </row>
+    <row r="28" spans="1:8" ht="30">
+      <c r="A28" s="3"/>
+      <c r="B28" s="3" t="s">
+        <v>991</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>992</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>993</v>
+      </c>
+      <c r="E28" s="5">
+        <v>3</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G28" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H28" s="3"/>
+    </row>
+    <row r="29" spans="1:8" ht="30">
+      <c r="A29" s="3"/>
+      <c r="B29" s="3" t="s">
+        <v>980</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>523</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>994</v>
+      </c>
+      <c r="E29" s="5">
+        <v>4</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G29" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H29" s="3"/>
+    </row>
+    <row r="30" spans="1:8">
+      <c r="A30" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>995</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>995</v>
+      </c>
+      <c r="E30" s="5">
+        <v>1</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G30" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H30" s="3" t="s">
+        <v>996</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8">
+      <c r="A31" s="3"/>
+      <c r="B31" s="3" t="s">
+        <v>997</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>998</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>999</v>
+      </c>
+      <c r="E31" s="5">
+        <v>2</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G31" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H31" s="3" t="s">
+        <v>996</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8">
+      <c r="A32" s="3"/>
+      <c r="B32" s="3" t="s">
+        <v>1000</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>1001</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>1001</v>
+      </c>
+      <c r="E32" s="5">
+        <v>3</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G32" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H32" s="3" t="s">
+        <v>996</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8">
+      <c r="A33" s="3"/>
+      <c r="B33" s="3" t="s">
+        <v>1002</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>1003</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>1004</v>
+      </c>
+      <c r="E33" s="5">
+        <v>4</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G33" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H33" s="3" t="s">
+        <v>996</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8">
+      <c r="A34" s="3"/>
+      <c r="B34" s="3" t="s">
+        <v>1005</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>2259</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>2259</v>
+      </c>
+      <c r="E34" s="5">
+        <v>5</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G34" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H34" s="3" t="s">
+        <v>996</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8">
+      <c r="A35" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>1261</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>1262</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>2260</v>
+      </c>
+      <c r="E35" s="5">
+        <v>1</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G35" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H35" s="3"/>
+    </row>
+    <row r="36" spans="1:8">
+      <c r="A36" s="3"/>
+      <c r="B36" s="3" t="s">
+        <v>1263</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>1264</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>1264</v>
+      </c>
+      <c r="E36" s="5">
+        <v>2</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G36" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H36" s="3"/>
+    </row>
+    <row r="37" spans="1:8">
+      <c r="A37" s="3"/>
+      <c r="B37" s="3" t="s">
+        <v>1265</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>1266</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>1266</v>
+      </c>
+      <c r="E37" s="5">
+        <v>3</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G37" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H37" s="3"/>
+    </row>
+    <row r="38" spans="1:8">
+      <c r="A38" s="3"/>
+      <c r="B38" s="3" t="s">
+        <v>1267</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>1268</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>1268</v>
+      </c>
+      <c r="E38" s="5">
+        <v>4</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G38" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H38" s="3"/>
+    </row>
+    <row r="39" spans="1:8">
+      <c r="A39" s="3"/>
+      <c r="B39" s="3" t="s">
+        <v>1269</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>1270</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>1270</v>
+      </c>
+      <c r="E39" s="5">
+        <v>5</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G39" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H39" s="3"/>
+    </row>
+    <row r="40" spans="1:8">
+      <c r="A40" s="3"/>
+      <c r="B40" s="3" t="s">
+        <v>1271</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="E40" s="5">
+        <v>6</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G40" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H40" s="3"/>
+    </row>
+    <row r="41" spans="1:8">
+      <c r="A41" s="3"/>
+      <c r="B41" s="3" t="s">
+        <v>1272</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>1273</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>2261</v>
+      </c>
+      <c r="E41" s="5">
+        <v>7</v>
+      </c>
+      <c r="F41" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G41" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H41" s="3"/>
+    </row>
+    <row r="42" spans="1:8">
+      <c r="A42" s="3"/>
+      <c r="B42" s="3" t="s">
+        <v>1274</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>1275</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>2262</v>
+      </c>
+      <c r="E42" s="5">
+        <v>8</v>
+      </c>
+      <c r="F42" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G42" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H42" s="3"/>
+    </row>
+    <row r="43" spans="1:8">
+      <c r="A43" s="3"/>
+      <c r="B43" s="3" t="s">
+        <v>1276</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>1277</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>1277</v>
+      </c>
+      <c r="E43" s="5">
+        <v>9</v>
+      </c>
+      <c r="F43" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G43" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H43" s="3"/>
+    </row>
+    <row r="44" spans="1:8">
+      <c r="A44" s="3"/>
+      <c r="B44" s="3" t="s">
+        <v>1278</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>1279</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>1279</v>
+      </c>
+      <c r="E44" s="5">
+        <v>10</v>
+      </c>
+      <c r="F44" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G44" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H44" s="3"/>
+    </row>
+    <row r="45" spans="1:8">
+      <c r="A45" s="3"/>
+      <c r="B45" s="3" t="s">
+        <v>1250</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>1254</v>
+      </c>
+      <c r="D45" s="3" t="s">
+        <v>2263</v>
+      </c>
+      <c r="E45" s="5">
+        <v>11</v>
+      </c>
+      <c r="F45" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G45" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H45" s="3"/>
+    </row>
+    <row r="46" spans="1:8">
+      <c r="A46" s="3"/>
+      <c r="B46" s="3" t="s">
+        <v>1280</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>1281</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>1281</v>
+      </c>
+      <c r="E46" s="5">
+        <v>12</v>
+      </c>
+      <c r="F46" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G46" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H46" s="3"/>
+    </row>
+    <row r="47" spans="1:8">
+      <c r="A47" s="3"/>
+      <c r="B47" s="3" t="s">
+        <v>1282</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>1283</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>1283</v>
+      </c>
+      <c r="E47" s="5">
+        <v>13</v>
+      </c>
+      <c r="F47" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G47" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H47" s="3"/>
+    </row>
+    <row r="48" spans="1:8">
+      <c r="A48" s="3"/>
+      <c r="B48" s="3" t="s">
+        <v>1284</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>1285</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>1285</v>
+      </c>
+      <c r="E48" s="5">
+        <v>14</v>
+      </c>
+      <c r="F48" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G48" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H48" s="3"/>
+    </row>
+    <row r="49" spans="1:8">
+      <c r="A49" s="3"/>
+      <c r="B49" s="3" t="s">
+        <v>1286</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>1287</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>1287</v>
+      </c>
+      <c r="E49" s="5">
+        <v>15</v>
+      </c>
+      <c r="F49" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G49" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H49" s="3"/>
+    </row>
+    <row r="50" spans="1:8">
+      <c r="A50" s="3"/>
+      <c r="B50" s="3" t="s">
+        <v>898</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>1288</v>
+      </c>
+      <c r="D50" s="3" t="s">
+        <v>2264</v>
+      </c>
+      <c r="E50" s="5">
+        <v>16</v>
+      </c>
+      <c r="F50" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G50" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H50" s="3"/>
+    </row>
+    <row r="51" spans="1:8">
+      <c r="A51" s="3"/>
+      <c r="B51" s="3" t="s">
+        <v>1289</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>1290</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>2265</v>
+      </c>
+      <c r="E51" s="5">
+        <v>17</v>
+      </c>
+      <c r="F51" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G51" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H51" s="3"/>
+    </row>
+    <row r="52" spans="1:8">
+      <c r="A52" s="3"/>
+      <c r="B52" s="3" t="s">
+        <v>1291</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>1292</v>
+      </c>
+      <c r="D52" s="3" t="s">
+        <v>2266</v>
+      </c>
+      <c r="E52" s="5">
+        <v>18</v>
+      </c>
+      <c r="F52" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G52" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H52" s="3"/>
+    </row>
+    <row r="53" spans="1:8" ht="30">
+      <c r="A53" s="3"/>
+      <c r="B53" s="3" t="s">
+        <v>980</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>1293</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>2267</v>
+      </c>
+      <c r="E53" s="5">
+        <v>19</v>
+      </c>
+      <c r="F53" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G53" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H53" s="3"/>
+    </row>
+    <row r="54" spans="1:8" ht="45">
+      <c r="A54" s="13" t="s">
+        <v>1704</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>1759</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>1632</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>2268</v>
+      </c>
+      <c r="E54" s="5">
+        <v>1</v>
+      </c>
+      <c r="F54" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G54" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H54" s="3" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" ht="30">
+      <c r="A55" s="3"/>
+      <c r="B55" s="3" t="s">
+        <v>1709</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>1747</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>2269</v>
+      </c>
+      <c r="E55" s="5">
+        <v>2</v>
+      </c>
+      <c r="F55" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G55" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H55" s="3" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" ht="30">
+      <c r="A56" s="3"/>
+      <c r="B56" s="3" t="s">
+        <v>1762</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>1763</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>2270</v>
+      </c>
+      <c r="E56" s="5">
+        <v>3</v>
+      </c>
+      <c r="F56" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G56" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H56" s="3" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" ht="45">
+      <c r="A57" s="3"/>
+      <c r="B57" s="3" t="s">
+        <v>1765</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>1766</v>
+      </c>
+      <c r="D57" s="3" t="s">
+        <v>2271</v>
+      </c>
+      <c r="E57" s="5">
+        <v>4</v>
+      </c>
+      <c r="F57" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G57" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H57" s="3" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" ht="30">
+      <c r="A58" s="3"/>
+      <c r="B58" s="3" t="s">
+        <v>1768</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>1769</v>
+      </c>
+      <c r="D58" s="3" t="s">
+        <v>2286</v>
+      </c>
+      <c r="E58" s="5">
+        <v>5</v>
+      </c>
+      <c r="F58" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G58" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H58" s="3" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" ht="30">
+      <c r="A59" s="3"/>
+      <c r="B59" s="3" t="s">
+        <v>961</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>962</v>
+      </c>
+      <c r="D59" s="3" t="s">
+        <v>2287</v>
+      </c>
+      <c r="E59" s="5">
+        <v>6</v>
+      </c>
+      <c r="F59" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G59" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H59" s="3" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" ht="30">
+      <c r="A60" s="3"/>
+      <c r="B60" s="3" t="s">
+        <v>1772</v>
+      </c>
+      <c r="C60" s="3" t="s">
+        <v>1773</v>
+      </c>
+      <c r="D60" s="3" t="s">
+        <v>2288</v>
+      </c>
+      <c r="E60" s="5">
+        <v>7</v>
+      </c>
+      <c r="F60" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G60" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H60" s="3" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" ht="30">
+      <c r="A61" s="3"/>
+      <c r="B61" s="3" t="s">
+        <v>1775</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>1776</v>
+      </c>
+      <c r="D61" s="3" t="s">
+        <v>2289</v>
+      </c>
+      <c r="E61" s="5">
+        <v>8</v>
+      </c>
+      <c r="F61" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G61" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H61" s="3" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" ht="30">
+      <c r="A62" s="3"/>
+      <c r="B62" s="3" t="s">
+        <v>1778</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>1779</v>
+      </c>
+      <c r="D62" s="3" t="s">
+        <v>2290</v>
+      </c>
+      <c r="E62" s="5">
+        <v>9</v>
+      </c>
+      <c r="F62" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G62" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H62" s="3" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" ht="30">
+      <c r="A63" s="3"/>
+      <c r="B63" s="3" t="s">
+        <v>1781</v>
+      </c>
+      <c r="C63" s="3" t="s">
+        <v>1782</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>2272</v>
+      </c>
+      <c r="E63" s="5">
+        <v>10</v>
+      </c>
+      <c r="F63" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G63" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H63" s="3" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" ht="30">
+      <c r="A64" s="3"/>
+      <c r="B64" s="3" t="s">
+        <v>1784</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>1785</v>
+      </c>
+      <c r="D64" s="3" t="s">
+        <v>2291</v>
+      </c>
+      <c r="E64" s="5">
+        <v>11</v>
+      </c>
+      <c r="F64" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G64" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H64" s="3" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" ht="30">
+      <c r="A65" s="3"/>
+      <c r="B65" s="3" t="s">
+        <v>1787</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>1788</v>
+      </c>
+      <c r="D65" s="3" t="s">
+        <v>2292</v>
+      </c>
+      <c r="E65" s="5">
+        <v>12</v>
+      </c>
+      <c r="F65" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G65" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H65" s="3" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" ht="30">
+      <c r="A66" s="3"/>
+      <c r="B66" s="3" t="s">
+        <v>1790</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>1791</v>
+      </c>
+      <c r="D66" s="3" t="s">
+        <v>2273</v>
+      </c>
+      <c r="E66" s="5">
+        <v>13</v>
+      </c>
+      <c r="F66" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G66" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H66" s="3" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" ht="30">
+      <c r="A67" s="3"/>
+      <c r="B67" s="3" t="s">
+        <v>1793</v>
+      </c>
+      <c r="C67" s="3" t="s">
+        <v>1794</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>2293</v>
+      </c>
+      <c r="E67" s="5">
+        <v>14</v>
+      </c>
+      <c r="F67" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G67" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H67" s="3" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" ht="30">
+      <c r="A68" s="3"/>
+      <c r="B68" s="3" t="s">
+        <v>1796</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>1797</v>
+      </c>
+      <c r="D68" s="3" t="s">
+        <v>2294</v>
+      </c>
+      <c r="E68" s="5">
+        <v>15</v>
+      </c>
+      <c r="F68" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G68" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H68" s="3" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" ht="30">
+      <c r="A69" s="3"/>
+      <c r="B69" s="3" t="s">
+        <v>1799</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>1800</v>
+      </c>
+      <c r="D69" s="3" t="s">
+        <v>2295</v>
+      </c>
+      <c r="E69" s="5">
+        <v>16</v>
+      </c>
+      <c r="F69" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G69" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H69" s="3" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" ht="30">
+      <c r="A70" s="3"/>
+      <c r="B70" s="3" t="s">
+        <v>1802</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>1803</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>2296</v>
+      </c>
+      <c r="E70" s="5">
+        <v>17</v>
+      </c>
+      <c r="F70" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G70" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H70" s="3" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" ht="30">
+      <c r="A71" s="13" t="s">
+        <v>1546</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="C71" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="D71" s="3" t="s">
+        <v>2297</v>
+      </c>
+      <c r="E71" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="F71" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G71" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H71" s="3" t="s">
+        <v>2274</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C85B9BC7-C8C8-4E3E-A0EF-02B9554CEAE5}">
   <dimension ref="A1:K63"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -41694,7 +43510,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6E5E88D-7637-4195-842B-FF426225AADB}">
   <dimension ref="A1:I36"/>
   <sheetFormatPr defaultRowHeight="15"/>

</xml_diff>

<commit_message>
org admin preview of overall custoemr experience implementation
</commit_message>
<xml_diff>
--- a/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
+++ b/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MynikaTech\memgine\docs\domain\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0646BDD4-2FDE-4846-A818-98AC9DF4AD61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4F57A97-FD42-4D5F-B918-433EC83B7732}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{AA28BC4D-8219-43B9-8C16-6977709D904A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{AA28BC4D-8219-43B9-8C16-6977709D904A}"/>
   </bookViews>
   <sheets>
     <sheet name="Entity Catalogue" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10892" uniqueCount="2399">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11202" uniqueCount="2463">
   <si>
     <t>Domain</t>
   </si>
@@ -7237,6 +7237,198 @@
   </si>
   <si>
     <t>Ordering</t>
+  </si>
+  <si>
+    <t>Customer Experience</t>
+  </si>
+  <si>
+    <t>customer_experience</t>
+  </si>
+  <si>
+    <t>Represents the organization-specific customer-facing experience configuration derived from a Memgine platform template. Controls the presentation, branding, sections and configurable customer-facing content while the underlying business data remains in its respective domain entities.</t>
+  </si>
+  <si>
+    <t>customer_experience_id</t>
+  </si>
+  <si>
+    <t>Experience Name</t>
+  </si>
+  <si>
+    <t>One customer experience configuration belongs to an organization. The selected Template controls the supported experience structure and capabilities. Actual transactional/domain content such as Offers remains in its respective entity and is not duplicated here.</t>
+  </si>
+  <si>
+    <t>Customer Experience ID</t>
+  </si>
+  <si>
+    <t>Uniquely identify a customer experience</t>
+  </si>
+  <si>
+    <t>System-generated identifier for the organization customer experience configuration</t>
+  </si>
+  <si>
+    <t>Primary identifier for the customer experience configuration</t>
+  </si>
+  <si>
+    <t>ce-1001</t>
+  </si>
+  <si>
+    <t>Identify the owning organization</t>
+  </si>
+  <si>
+    <t>Identifies the organization that owns this customer experience</t>
+  </si>
+  <si>
+    <t>Tenant ownership and isolation key</t>
+  </si>
+  <si>
+    <t>org-1001</t>
+  </si>
+  <si>
+    <t>Identify the governing platform template</t>
+  </si>
+  <si>
+    <t>References the Memgine platform template that defines the structure and capabilities of the experience</t>
+  </si>
+  <si>
+    <t>Determines which sections and presentation capabilities are supported</t>
+  </si>
+  <si>
+    <t>tpl-f-and-b-bakery-v1</t>
+  </si>
+  <si>
+    <t>experience_name</t>
+  </si>
+  <si>
+    <t>Identify the customer experience configuration</t>
+  </si>
+  <si>
+    <t>Human-readable name for the organization's customer experience configuration</t>
+  </si>
+  <si>
+    <t>Administrative name used to identify the configuration</t>
+  </si>
+  <si>
+    <t>Sunrise Bakery Customer Experience</t>
+  </si>
+  <si>
+    <t>Experience Definition</t>
+  </si>
+  <si>
+    <t>experience_definition</t>
+  </si>
+  <si>
+    <t>Store configurable customer experience content and presentation</t>
+  </si>
+  <si>
+    <t>Stores flexible section configuration and customer-facing content governed by the selected template</t>
+  </si>
+  <si>
+    <t>{"hero":{"enabled":true}}</t>
+  </si>
+  <si>
+    <t>Template default</t>
+  </si>
+  <si>
+    <t>Experience Status ID</t>
+  </si>
+  <si>
+    <t>experience_status_id</t>
+  </si>
+  <si>
+    <t>Control the lifecycle of the customer experience</t>
+  </si>
+  <si>
+    <t>References the canonical Status entity controlling the lifecycle of the experience</t>
+  </si>
+  <si>
+    <t>Determines whether the experience is draft, active, inactive, etc.</t>
+  </si>
+  <si>
+    <t>status-active</t>
+  </si>
+  <si>
+    <t>Published At</t>
+  </si>
+  <si>
+    <t>published_at</t>
+  </si>
+  <si>
+    <t>Record when the current customer experience was published</t>
+  </si>
+  <si>
+    <t>Timestamp of the most recent successful publication</t>
+  </si>
+  <si>
+    <t>Publication audit timestamp</t>
+  </si>
+  <si>
+    <t>2026-08-25T10:30:00Z</t>
+  </si>
+  <si>
+    <t>Published By</t>
+  </si>
+  <si>
+    <t>published_by</t>
+  </si>
+  <si>
+    <t>Identify who published the experience</t>
+  </si>
+  <si>
+    <t>User responsible for the most recent publication</t>
+  </si>
+  <si>
+    <t>Publication audit user</t>
+  </si>
+  <si>
+    <t>user-1001</t>
+  </si>
+  <si>
+    <t>Timestamp when the customer experience record was created</t>
+  </si>
+  <si>
+    <t>Creation timestamp</t>
+  </si>
+  <si>
+    <t>2026-08-25T09:00:00Z</t>
+  </si>
+  <si>
+    <t>User that created the customer experience record</t>
+  </si>
+  <si>
+    <t>Creation audit user</t>
+  </si>
+  <si>
+    <t>Timestamp when the customer experience record was last modified</t>
+  </si>
+  <si>
+    <t>Last modification timestamp</t>
+  </si>
+  <si>
+    <t>2026-08-25T10:15:00Z</t>
+  </si>
+  <si>
+    <t>User that last modified the customer experience record</t>
+  </si>
+  <si>
+    <t>Last modification audit user</t>
+  </si>
+  <si>
+    <t>Indicates whether the customer experience record has been logically deleted</t>
+  </si>
+  <si>
+    <t>Prevents physical deletion while removing the record from normal application use</t>
+  </si>
+  <si>
+    <t>Version number used to prevent conflicting updates</t>
+  </si>
+  <si>
+    <t>Incremented whenever the record is modified</t>
+  </si>
+  <si>
+    <t>JSON/XML representation of configurable experience sections and content</t>
+  </si>
+  <si>
+    <t>customer-experience-status-draft</t>
   </si>
 </sst>
 </file>
@@ -7462,7 +7654,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3841114F-D1EC-49B1-850B-590431E39412}" name="Table2" displayName="Table2" ref="A1:Q37" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3841114F-D1EC-49B1-850B-590431E39412}" name="Table2" displayName="Table2" ref="A1:Q38" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{FEF6275C-74E6-4563-BFF3-6461E4A3D8DA}" name="Entity Code" dataDxfId="16"/>
     <tableColumn id="2" xr3:uid="{67FE23FD-539D-4023-BA73-D2A0B84718BF}" name="Domain" dataDxfId="15"/>
@@ -7783,20 +7975,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4659496D-1A4F-4BC3-BD65-377E70E6B8BE}">
-  <dimension ref="A1:Q37"/>
+  <dimension ref="A1:Q38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="31.85546875" style="4" customWidth="1"/>
     <col min="2" max="2" width="16.28515625" style="4" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.42578125" style="4" customWidth="1"/>
     <col min="5" max="5" width="30" style="4" customWidth="1"/>
     <col min="6" max="6" width="48.5703125" style="4" customWidth="1"/>
     <col min="7" max="7" width="14.140625" style="4" customWidth="1"/>
     <col min="8" max="8" width="15.28515625" style="4" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.42578125" style="4" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="9.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11" style="4" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.85546875" style="4" customWidth="1"/>
     <col min="12" max="12" width="9.7109375" style="4" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="12.42578125" style="4" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="27.42578125" style="4" customWidth="1"/>
@@ -9765,6 +9957,50 @@
       </c>
       <c r="Q37" s="4" t="s">
         <v>2116</v>
+      </c>
+    </row>
+    <row r="38" spans="1:17" ht="105">
+      <c r="A38" s="4" t="s">
+        <v>2399</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>2400</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>2401</v>
+      </c>
+      <c r="G38" s="4" t="s">
+        <v>1520</v>
+      </c>
+      <c r="H38" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="I38" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="J38" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K38" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="L38" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="M38" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="N38" s="4" t="s">
+        <v>2402</v>
+      </c>
+      <c r="O38" s="4" t="s">
+        <v>2403</v>
+      </c>
+      <c r="P38" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q38" s="4" t="s">
+        <v>2404</v>
       </c>
     </row>
   </sheetData>
@@ -12964,8 +13200,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E21F442-9136-4C15-8BA3-92E07332B93A}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:W396"/>
+  <dimension ref="A1:W410"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.140625" style="4" customWidth="1"/>
@@ -13064,7 +13299,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="2" spans="1:23" ht="30" hidden="1">
+    <row r="2" spans="1:23" ht="30">
       <c r="A2" s="10" t="s">
         <v>5</v>
       </c>
@@ -13130,7 +13365,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:23" ht="30" hidden="1">
+    <row r="3" spans="1:23" ht="30">
       <c r="A3" s="10" t="s">
         <v>5</v>
       </c>
@@ -13198,7 +13433,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:23" ht="30" hidden="1">
+    <row r="4" spans="1:23" ht="30">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -13266,7 +13501,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:23" ht="60" hidden="1">
+    <row r="5" spans="1:23" ht="60">
       <c r="A5" s="10" t="s">
         <v>5</v>
       </c>
@@ -13335,7 +13570,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:23" ht="30" hidden="1">
+    <row r="6" spans="1:23" ht="30">
       <c r="A6" s="10" t="s">
         <v>5</v>
       </c>
@@ -13403,7 +13638,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:23" hidden="1">
+    <row r="7" spans="1:23">
       <c r="A7" s="10" t="s">
         <v>5</v>
       </c>
@@ -13471,7 +13706,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:23" hidden="1">
+    <row r="8" spans="1:23">
       <c r="A8" s="10" t="s">
         <v>5</v>
       </c>
@@ -13539,7 +13774,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:23" hidden="1">
+    <row r="9" spans="1:23">
       <c r="A9" s="10" t="s">
         <v>5</v>
       </c>
@@ -13607,7 +13842,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="10" spans="1:23" hidden="1">
+    <row r="10" spans="1:23">
       <c r="A10" s="10" t="s">
         <v>5</v>
       </c>
@@ -13675,7 +13910,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="11" spans="1:23" hidden="1">
+    <row r="11" spans="1:23">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -13743,7 +13978,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:23" ht="30" hidden="1">
+    <row r="12" spans="1:23" ht="30">
       <c r="A12" s="10" t="s">
         <v>5</v>
       </c>
@@ -13811,7 +14046,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:23" hidden="1">
+    <row r="13" spans="1:23">
       <c r="A13" s="10" t="s">
         <v>5</v>
       </c>
@@ -13879,7 +14114,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:23" ht="30" hidden="1">
+    <row r="14" spans="1:23" ht="30">
       <c r="A14" s="10" t="s">
         <v>5</v>
       </c>
@@ -13947,7 +14182,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:23" hidden="1">
+    <row r="15" spans="1:23">
       <c r="A15" s="10" t="s">
         <v>5</v>
       </c>
@@ -14015,7 +14250,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:23" ht="30" hidden="1">
+    <row r="16" spans="1:23" ht="30">
       <c r="A16" s="10" t="s">
         <v>5</v>
       </c>
@@ -14083,7 +14318,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:23" hidden="1">
+    <row r="17" spans="1:23">
       <c r="A17" s="10" t="s">
         <v>5</v>
       </c>
@@ -14151,7 +14386,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:23" ht="30" hidden="1">
+    <row r="18" spans="1:23" ht="30">
       <c r="A18" s="3" t="s">
         <v>8</v>
       </c>
@@ -14218,7 +14453,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:23" ht="30" hidden="1">
+    <row r="19" spans="1:23" ht="30">
       <c r="A19" s="3" t="s">
         <v>8</v>
       </c>
@@ -14287,7 +14522,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="1:23" hidden="1">
+    <row r="20" spans="1:23">
       <c r="A20" s="3" t="s">
         <v>8</v>
       </c>
@@ -14354,7 +14589,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="21" spans="1:23" hidden="1">
+    <row r="21" spans="1:23">
       <c r="A21" s="3" t="s">
         <v>8</v>
       </c>
@@ -14421,7 +14656,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="22" spans="1:23" hidden="1">
+    <row r="22" spans="1:23">
       <c r="A22" s="3" t="s">
         <v>8</v>
       </c>
@@ -14488,7 +14723,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="23" spans="1:23" ht="30" hidden="1">
+    <row r="23" spans="1:23" ht="30">
       <c r="A23" s="3" t="s">
         <v>8</v>
       </c>
@@ -14557,7 +14792,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="24" spans="1:23" ht="30" hidden="1">
+    <row r="24" spans="1:23" ht="30">
       <c r="A24" s="3" t="s">
         <v>8</v>
       </c>
@@ -14624,7 +14859,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="25" spans="1:23" ht="30" hidden="1">
+    <row r="25" spans="1:23" ht="30">
       <c r="A25" s="3" t="s">
         <v>8</v>
       </c>
@@ -14691,7 +14926,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="26" spans="1:23" ht="30" hidden="1">
+    <row r="26" spans="1:23" ht="30">
       <c r="A26" s="3" t="s">
         <v>8</v>
       </c>
@@ -14760,7 +14995,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="27" spans="1:23" ht="30" hidden="1">
+    <row r="27" spans="1:23" ht="30">
       <c r="A27" s="3" t="s">
         <v>8</v>
       </c>
@@ -14829,7 +15064,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="28" spans="1:23" ht="30" hidden="1">
+    <row r="28" spans="1:23" ht="30">
       <c r="A28" s="3" t="s">
         <v>8</v>
       </c>
@@ -14896,7 +15131,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="29" spans="1:23" hidden="1">
+    <row r="29" spans="1:23">
       <c r="A29" s="3" t="s">
         <v>8</v>
       </c>
@@ -14965,7 +15200,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="30" spans="1:23" ht="30" hidden="1">
+    <row r="30" spans="1:23" ht="30">
       <c r="A30" s="3" t="s">
         <v>8</v>
       </c>
@@ -15032,7 +15267,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="31" spans="1:23" hidden="1">
+    <row r="31" spans="1:23">
       <c r="A31" s="3" t="s">
         <v>8</v>
       </c>
@@ -15101,7 +15336,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="32" spans="1:23" ht="30" hidden="1">
+    <row r="32" spans="1:23" ht="30">
       <c r="A32" s="3" t="s">
         <v>8</v>
       </c>
@@ -15168,7 +15403,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="33" spans="1:23" hidden="1">
+    <row r="33" spans="1:23">
       <c r="A33" s="3" t="s">
         <v>8</v>
       </c>
@@ -15235,7 +15470,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="34" spans="1:23" ht="30" hidden="1">
+    <row r="34" spans="1:23" ht="30">
       <c r="A34" s="3" t="s">
         <v>37</v>
       </c>
@@ -15306,7 +15541,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="35" spans="1:23" ht="30" hidden="1">
+    <row r="35" spans="1:23" ht="30">
       <c r="A35" s="3" t="s">
         <v>37</v>
       </c>
@@ -15377,7 +15612,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="36" spans="1:23" hidden="1">
+    <row r="36" spans="1:23">
       <c r="A36" s="3" t="s">
         <v>37</v>
       </c>
@@ -15448,7 +15683,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="37" spans="1:23" ht="45" hidden="1">
+    <row r="37" spans="1:23" ht="45">
       <c r="A37" s="3" t="s">
         <v>37</v>
       </c>
@@ -15519,7 +15754,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="38" spans="1:23" ht="30" hidden="1">
+    <row r="38" spans="1:23" ht="30">
       <c r="A38" s="3" t="s">
         <v>37</v>
       </c>
@@ -15590,7 +15825,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="39" spans="1:23" ht="30" hidden="1">
+    <row r="39" spans="1:23" ht="30">
       <c r="A39" s="3" t="s">
         <v>37</v>
       </c>
@@ -15661,7 +15896,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="40" spans="1:23" ht="30" hidden="1">
+    <row r="40" spans="1:23" ht="30">
       <c r="A40" s="3" t="s">
         <v>37</v>
       </c>
@@ -15732,7 +15967,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="41" spans="1:23" hidden="1">
+    <row r="41" spans="1:23">
       <c r="A41" s="3" t="s">
         <v>37</v>
       </c>
@@ -15803,7 +16038,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="42" spans="1:23" ht="30" hidden="1">
+    <row r="42" spans="1:23" ht="30">
       <c r="A42" s="3" t="s">
         <v>37</v>
       </c>
@@ -15874,7 +16109,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="43" spans="1:23" hidden="1">
+    <row r="43" spans="1:23">
       <c r="A43" s="3" t="s">
         <v>37</v>
       </c>
@@ -15945,7 +16180,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="44" spans="1:23" hidden="1">
+    <row r="44" spans="1:23">
       <c r="A44" s="3" t="s">
         <v>37</v>
       </c>
@@ -16016,7 +16251,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="45" spans="1:23" hidden="1">
+    <row r="45" spans="1:23">
       <c r="A45" s="3" t="s">
         <v>37</v>
       </c>
@@ -16087,7 +16322,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="46" spans="1:23" ht="30" hidden="1">
+    <row r="46" spans="1:23" ht="30">
       <c r="A46" s="3" t="s">
         <v>317</v>
       </c>
@@ -16134,7 +16369,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="47" spans="1:23" ht="30" hidden="1">
+    <row r="47" spans="1:23" ht="30">
       <c r="A47" s="3" t="s">
         <v>317</v>
       </c>
@@ -16181,7 +16416,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="48" spans="1:23" ht="45" hidden="1">
+    <row r="48" spans="1:23" ht="45">
       <c r="A48" s="3" t="s">
         <v>317</v>
       </c>
@@ -16228,7 +16463,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="49" spans="1:23" ht="30" hidden="1">
+    <row r="49" spans="1:23" ht="30">
       <c r="A49" s="3" t="s">
         <v>317</v>
       </c>
@@ -16275,7 +16510,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="50" spans="1:23" ht="30" hidden="1">
+    <row r="50" spans="1:23" ht="30">
       <c r="A50" s="3" t="s">
         <v>317</v>
       </c>
@@ -16322,7 +16557,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="51" spans="1:23" ht="30" hidden="1">
+    <row r="51" spans="1:23" ht="30">
       <c r="A51" s="4" t="s">
         <v>341</v>
       </c>
@@ -16390,7 +16625,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="52" spans="1:23" ht="30" hidden="1">
+    <row r="52" spans="1:23" ht="30">
       <c r="A52" s="4" t="s">
         <v>341</v>
       </c>
@@ -16458,7 +16693,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="53" spans="1:23" ht="30" hidden="1">
+    <row r="53" spans="1:23" ht="30">
       <c r="A53" s="4" t="s">
         <v>341</v>
       </c>
@@ -16526,7 +16761,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="54" spans="1:23" ht="30" hidden="1">
+    <row r="54" spans="1:23" ht="30">
       <c r="A54" s="4" t="s">
         <v>341</v>
       </c>
@@ -16594,7 +16829,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="55" spans="1:23" ht="30" hidden="1">
+    <row r="55" spans="1:23" ht="30">
       <c r="A55" s="4" t="s">
         <v>341</v>
       </c>
@@ -16662,7 +16897,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="56" spans="1:23" ht="30" hidden="1">
+    <row r="56" spans="1:23" ht="30">
       <c r="A56" s="4" t="s">
         <v>341</v>
       </c>
@@ -16730,7 +16965,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="57" spans="1:23" ht="30" hidden="1">
+    <row r="57" spans="1:23" ht="30">
       <c r="A57" s="4" t="s">
         <v>341</v>
       </c>
@@ -16798,7 +17033,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="58" spans="1:23" ht="30" hidden="1">
+    <row r="58" spans="1:23" ht="30">
       <c r="A58" s="4" t="s">
         <v>341</v>
       </c>
@@ -16866,7 +17101,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="59" spans="1:23" ht="45" hidden="1">
+    <row r="59" spans="1:23" ht="45">
       <c r="A59" s="4" t="s">
         <v>341</v>
       </c>
@@ -16934,7 +17169,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="60" spans="1:23" ht="30" hidden="1">
+    <row r="60" spans="1:23" ht="30">
       <c r="A60" s="4" t="s">
         <v>341</v>
       </c>
@@ -17002,7 +17237,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="61" spans="1:23" ht="30" hidden="1">
+    <row r="61" spans="1:23" ht="30">
       <c r="A61" s="4" t="s">
         <v>370</v>
       </c>
@@ -17073,7 +17308,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="62" spans="1:23" ht="30" hidden="1">
+    <row r="62" spans="1:23" ht="30">
       <c r="A62" s="4" t="s">
         <v>370</v>
       </c>
@@ -17144,7 +17379,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="63" spans="1:23" ht="30" hidden="1">
+    <row r="63" spans="1:23" ht="30">
       <c r="A63" s="4" t="s">
         <v>370</v>
       </c>
@@ -17215,7 +17450,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="64" spans="1:23" ht="30" hidden="1">
+    <row r="64" spans="1:23" ht="30">
       <c r="A64" s="4" t="s">
         <v>370</v>
       </c>
@@ -17286,7 +17521,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="65" spans="1:23" ht="30" hidden="1">
+    <row r="65" spans="1:23" ht="30">
       <c r="A65" s="4" t="s">
         <v>370</v>
       </c>
@@ -17357,7 +17592,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="66" spans="1:23" ht="30" hidden="1">
+    <row r="66" spans="1:23" ht="30">
       <c r="A66" s="4" t="s">
         <v>377</v>
       </c>
@@ -17428,7 +17663,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="67" spans="1:23" ht="30" hidden="1">
+    <row r="67" spans="1:23" ht="30">
       <c r="A67" s="4" t="s">
         <v>377</v>
       </c>
@@ -17499,7 +17734,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="68" spans="1:23" ht="30" hidden="1">
+    <row r="68" spans="1:23" ht="30">
       <c r="A68" s="4" t="s">
         <v>377</v>
       </c>
@@ -17570,7 +17805,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="69" spans="1:23" ht="30" hidden="1">
+    <row r="69" spans="1:23" ht="30">
       <c r="A69" s="4" t="s">
         <v>10</v>
       </c>
@@ -17641,7 +17876,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="70" spans="1:23" ht="30" hidden="1">
+    <row r="70" spans="1:23" ht="30">
       <c r="A70" s="4" t="s">
         <v>10</v>
       </c>
@@ -17712,7 +17947,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="71" spans="1:23" ht="45" hidden="1">
+    <row r="71" spans="1:23" ht="45">
       <c r="A71" s="4" t="s">
         <v>10</v>
       </c>
@@ -17783,7 +18018,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="72" spans="1:23" ht="45" hidden="1">
+    <row r="72" spans="1:23" ht="45">
       <c r="A72" s="4" t="s">
         <v>10</v>
       </c>
@@ -17854,7 +18089,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="73" spans="1:23" ht="30" hidden="1">
+    <row r="73" spans="1:23" ht="30">
       <c r="A73" s="4" t="s">
         <v>10</v>
       </c>
@@ -17925,7 +18160,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="74" spans="1:23" ht="30" hidden="1">
+    <row r="74" spans="1:23" ht="30">
       <c r="A74" s="4" t="s">
         <v>10</v>
       </c>
@@ -17996,7 +18231,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="75" spans="1:23" ht="30" hidden="1">
+    <row r="75" spans="1:23" ht="30">
       <c r="A75" s="4" t="s">
         <v>10</v>
       </c>
@@ -18067,7 +18302,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="76" spans="1:23" ht="30" hidden="1">
+    <row r="76" spans="1:23" ht="30">
       <c r="A76" s="4" t="s">
         <v>10</v>
       </c>
@@ -18138,7 +18373,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="77" spans="1:23" ht="30" hidden="1">
+    <row r="77" spans="1:23" ht="30">
       <c r="A77" s="4" t="s">
         <v>10</v>
       </c>
@@ -18209,7 +18444,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="78" spans="1:23" ht="45" hidden="1">
+    <row r="78" spans="1:23" ht="45">
       <c r="A78" s="4" t="s">
         <v>10</v>
       </c>
@@ -18280,7 +18515,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="79" spans="1:23" ht="45" hidden="1">
+    <row r="79" spans="1:23" ht="45">
       <c r="A79" s="4" t="s">
         <v>10</v>
       </c>
@@ -18351,7 +18586,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="80" spans="1:23" ht="30" hidden="1">
+    <row r="80" spans="1:23" ht="30">
       <c r="A80" s="4" t="s">
         <v>10</v>
       </c>
@@ -18422,7 +18657,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="81" spans="1:23" ht="30" hidden="1">
+    <row r="81" spans="1:23" ht="30">
       <c r="A81" s="4" t="s">
         <v>10</v>
       </c>
@@ -18493,7 +18728,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="82" spans="1:23" ht="30" hidden="1">
+    <row r="82" spans="1:23" ht="30">
       <c r="A82" s="4" t="s">
         <v>10</v>
       </c>
@@ -18564,7 +18799,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="83" spans="1:23" ht="30" hidden="1">
+    <row r="83" spans="1:23" ht="30">
       <c r="A83" s="4" t="s">
         <v>10</v>
       </c>
@@ -18635,7 +18870,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="84" spans="1:23" ht="45" hidden="1">
+    <row r="84" spans="1:23" ht="45">
       <c r="A84" s="4" t="s">
         <v>10</v>
       </c>
@@ -18706,7 +18941,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="85" spans="1:23" ht="30" hidden="1">
+    <row r="85" spans="1:23" ht="30">
       <c r="A85" s="4" t="s">
         <v>10</v>
       </c>
@@ -18777,7 +19012,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="86" spans="1:23" ht="30" hidden="1">
+    <row r="86" spans="1:23" ht="30">
       <c r="A86" s="4" t="s">
         <v>490</v>
       </c>
@@ -18848,7 +19083,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="87" spans="1:23" ht="30" hidden="1">
+    <row r="87" spans="1:23" ht="30">
       <c r="A87" s="4" t="s">
         <v>490</v>
       </c>
@@ -18919,7 +19154,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="88" spans="1:23" ht="30" hidden="1">
+    <row r="88" spans="1:23" ht="30">
       <c r="A88" s="4" t="s">
         <v>490</v>
       </c>
@@ -18990,7 +19225,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="89" spans="1:23" ht="30" hidden="1">
+    <row r="89" spans="1:23" ht="30">
       <c r="A89" s="4" t="s">
         <v>490</v>
       </c>
@@ -19061,7 +19296,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="90" spans="1:23" hidden="1">
+    <row r="90" spans="1:23">
       <c r="A90" s="4" t="s">
         <v>490</v>
       </c>
@@ -19132,7 +19367,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="91" spans="1:23" hidden="1">
+    <row r="91" spans="1:23">
       <c r="A91" s="4" t="s">
         <v>490</v>
       </c>
@@ -19203,7 +19438,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="92" spans="1:23" ht="45" hidden="1">
+    <row r="92" spans="1:23" ht="45">
       <c r="A92" s="4" t="s">
         <v>490</v>
       </c>
@@ -19274,7 +19509,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="93" spans="1:23" ht="30" hidden="1">
+    <row r="93" spans="1:23" ht="30">
       <c r="A93" s="4" t="s">
         <v>490</v>
       </c>
@@ -19345,7 +19580,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="94" spans="1:23" ht="30" hidden="1">
+    <row r="94" spans="1:23" ht="30">
       <c r="A94" s="4" t="s">
         <v>490</v>
       </c>
@@ -19416,7 +19651,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="95" spans="1:23" ht="30" hidden="1">
+    <row r="95" spans="1:23" ht="30">
       <c r="A95" s="4" t="s">
         <v>490</v>
       </c>
@@ -19487,7 +19722,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="96" spans="1:23" ht="30" hidden="1">
+    <row r="96" spans="1:23" ht="30">
       <c r="A96" s="4" t="s">
         <v>490</v>
       </c>
@@ -19558,7 +19793,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="97" spans="1:23" ht="30" hidden="1">
+    <row r="97" spans="1:23" ht="30">
       <c r="A97" s="4" t="s">
         <v>490</v>
       </c>
@@ -19629,7 +19864,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="98" spans="1:23" ht="30" hidden="1">
+    <row r="98" spans="1:23" ht="30">
       <c r="A98" s="4" t="s">
         <v>490</v>
       </c>
@@ -19700,7 +19935,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="99" spans="1:23" ht="30" hidden="1">
+    <row r="99" spans="1:23" ht="30">
       <c r="A99" s="4" t="s">
         <v>490</v>
       </c>
@@ -19771,7 +20006,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="100" spans="1:23" ht="30" hidden="1">
+    <row r="100" spans="1:23" ht="30">
       <c r="A100" s="4" t="s">
         <v>490</v>
       </c>
@@ -19842,7 +20077,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="101" spans="1:23" ht="30" hidden="1">
+    <row r="101" spans="1:23" ht="30">
       <c r="A101" s="4" t="s">
         <v>490</v>
       </c>
@@ -19913,7 +20148,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="102" spans="1:23" ht="30" hidden="1">
+    <row r="102" spans="1:23" ht="30">
       <c r="A102" s="4" t="s">
         <v>548</v>
       </c>
@@ -19984,7 +20219,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="103" spans="1:23" ht="30" hidden="1">
+    <row r="103" spans="1:23" ht="30">
       <c r="A103" s="4" t="s">
         <v>548</v>
       </c>
@@ -20055,7 +20290,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="104" spans="1:23" ht="30" hidden="1">
+    <row r="104" spans="1:23" ht="30">
       <c r="A104" s="4" t="s">
         <v>548</v>
       </c>
@@ -20126,7 +20361,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="105" spans="1:23" ht="30" hidden="1">
+    <row r="105" spans="1:23" ht="30">
       <c r="A105" s="4" t="s">
         <v>548</v>
       </c>
@@ -20197,7 +20432,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="106" spans="1:23" ht="30" hidden="1">
+    <row r="106" spans="1:23" ht="30">
       <c r="A106" s="4" t="s">
         <v>548</v>
       </c>
@@ -20268,7 +20503,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="107" spans="1:23" hidden="1">
+    <row r="107" spans="1:23">
       <c r="A107" s="4" t="s">
         <v>548</v>
       </c>
@@ -20339,7 +20574,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="108" spans="1:23" hidden="1">
+    <row r="108" spans="1:23">
       <c r="A108" s="4" t="s">
         <v>548</v>
       </c>
@@ -20410,7 +20645,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="109" spans="1:23" hidden="1">
+    <row r="109" spans="1:23">
       <c r="A109" s="4" t="s">
         <v>548</v>
       </c>
@@ -20481,7 +20716,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="110" spans="1:23" ht="30" hidden="1">
+    <row r="110" spans="1:23" ht="30">
       <c r="A110" s="4" t="s">
         <v>548</v>
       </c>
@@ -20552,7 +20787,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="111" spans="1:23" hidden="1">
+    <row r="111" spans="1:23">
       <c r="A111" s="4" t="s">
         <v>548</v>
       </c>
@@ -20623,7 +20858,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="112" spans="1:23" ht="30" hidden="1">
+    <row r="112" spans="1:23" ht="30">
       <c r="A112" s="4" t="s">
         <v>548</v>
       </c>
@@ -20694,7 +20929,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="113" spans="1:23" hidden="1">
+    <row r="113" spans="1:23">
       <c r="A113" s="4" t="s">
         <v>548</v>
       </c>
@@ -20765,7 +21000,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="114" spans="1:23" ht="30" hidden="1">
+    <row r="114" spans="1:23" ht="30">
       <c r="A114" s="4" t="s">
         <v>548</v>
       </c>
@@ -20836,7 +21071,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="115" spans="1:23" hidden="1">
+    <row r="115" spans="1:23">
       <c r="A115" s="4" t="s">
         <v>548</v>
       </c>
@@ -20907,7 +21142,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="116" spans="1:23" ht="30" hidden="1">
+    <row r="116" spans="1:23" ht="30">
       <c r="A116" s="4" t="s">
         <v>548</v>
       </c>
@@ -20978,7 +21213,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="117" spans="1:23" hidden="1">
+    <row r="117" spans="1:23">
       <c r="A117" s="4" t="s">
         <v>548</v>
       </c>
@@ -21049,7 +21284,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="118" spans="1:23" hidden="1">
+    <row r="118" spans="1:23">
       <c r="A118" s="4" t="s">
         <v>548</v>
       </c>
@@ -21120,7 +21355,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="119" spans="1:23" hidden="1">
+    <row r="119" spans="1:23">
       <c r="A119" s="4" t="s">
         <v>548</v>
       </c>
@@ -21191,7 +21426,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="120" spans="1:23" ht="30" hidden="1">
+    <row r="120" spans="1:23" ht="30">
       <c r="A120" s="4" t="s">
         <v>620</v>
       </c>
@@ -21262,7 +21497,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="121" spans="1:23" ht="30" hidden="1">
+    <row r="121" spans="1:23" ht="30">
       <c r="A121" s="4" t="s">
         <v>620</v>
       </c>
@@ -21333,7 +21568,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="122" spans="1:23" hidden="1">
+    <row r="122" spans="1:23">
       <c r="A122" s="4" t="s">
         <v>620</v>
       </c>
@@ -21404,7 +21639,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="123" spans="1:23" ht="30" hidden="1">
+    <row r="123" spans="1:23" ht="30">
       <c r="A123" s="4" t="s">
         <v>620</v>
       </c>
@@ -21475,7 +21710,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="124" spans="1:23" hidden="1">
+    <row r="124" spans="1:23">
       <c r="A124" s="4" t="s">
         <v>620</v>
       </c>
@@ -21546,7 +21781,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="125" spans="1:23" ht="30" hidden="1">
+    <row r="125" spans="1:23" ht="30">
       <c r="A125" s="4" t="s">
         <v>620</v>
       </c>
@@ -21617,7 +21852,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="126" spans="1:23" hidden="1">
+    <row r="126" spans="1:23">
       <c r="A126" s="4" t="s">
         <v>620</v>
       </c>
@@ -21688,7 +21923,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="127" spans="1:23" hidden="1">
+    <row r="127" spans="1:23">
       <c r="A127" s="4" t="s">
         <v>620</v>
       </c>
@@ -21759,7 +21994,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="128" spans="1:23" ht="30" hidden="1">
+    <row r="128" spans="1:23" ht="30">
       <c r="A128" s="4" t="s">
         <v>620</v>
       </c>
@@ -21830,7 +22065,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="129" spans="1:23" ht="30" hidden="1">
+    <row r="129" spans="1:23" ht="30">
       <c r="A129" s="4" t="s">
         <v>620</v>
       </c>
@@ -21901,7 +22136,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="130" spans="1:23" hidden="1">
+    <row r="130" spans="1:23">
       <c r="A130" s="4" t="s">
         <v>620</v>
       </c>
@@ -21972,7 +22207,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="131" spans="1:23" ht="30" hidden="1">
+    <row r="131" spans="1:23" ht="30">
       <c r="A131" s="4" t="s">
         <v>620</v>
       </c>
@@ -22043,7 +22278,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="132" spans="1:23" hidden="1">
+    <row r="132" spans="1:23">
       <c r="A132" s="4" t="s">
         <v>620</v>
       </c>
@@ -22114,7 +22349,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="133" spans="1:23" hidden="1">
+    <row r="133" spans="1:23">
       <c r="A133" s="4" t="s">
         <v>620</v>
       </c>
@@ -22185,7 +22420,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="134" spans="1:23" hidden="1">
+    <row r="134" spans="1:23">
       <c r="A134" s="4" t="s">
         <v>620</v>
       </c>
@@ -22256,7 +22491,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="135" spans="1:23" ht="30" hidden="1">
+    <row r="135" spans="1:23" ht="30">
       <c r="A135" s="4" t="s">
         <v>673</v>
       </c>
@@ -22327,7 +22562,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="136" spans="1:23" ht="30" hidden="1">
+    <row r="136" spans="1:23" ht="30">
       <c r="A136" s="4" t="s">
         <v>673</v>
       </c>
@@ -22398,7 +22633,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="137" spans="1:23" ht="30" hidden="1">
+    <row r="137" spans="1:23" ht="30">
       <c r="A137" s="4" t="s">
         <v>673</v>
       </c>
@@ -22469,7 +22704,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="138" spans="1:23" ht="30" hidden="1">
+    <row r="138" spans="1:23" ht="30">
       <c r="A138" s="4" t="s">
         <v>673</v>
       </c>
@@ -22540,7 +22775,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="139" spans="1:23" ht="30" hidden="1">
+    <row r="139" spans="1:23" ht="30">
       <c r="A139" s="4" t="s">
         <v>673</v>
       </c>
@@ -22611,7 +22846,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="140" spans="1:23" ht="30" hidden="1">
+    <row r="140" spans="1:23" ht="30">
       <c r="A140" s="4" t="s">
         <v>673</v>
       </c>
@@ -22682,7 +22917,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="141" spans="1:23" ht="30" hidden="1">
+    <row r="141" spans="1:23" ht="30">
       <c r="A141" s="4" t="s">
         <v>673</v>
       </c>
@@ -22753,7 +22988,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="142" spans="1:23" hidden="1">
+    <row r="142" spans="1:23">
       <c r="A142" s="4" t="s">
         <v>673</v>
       </c>
@@ -22824,7 +23059,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="143" spans="1:23" ht="30" hidden="1">
+    <row r="143" spans="1:23" ht="30">
       <c r="A143" s="4" t="s">
         <v>673</v>
       </c>
@@ -22895,7 +23130,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="144" spans="1:23" ht="30" hidden="1">
+    <row r="144" spans="1:23" ht="30">
       <c r="A144" s="4" t="s">
         <v>673</v>
       </c>
@@ -22966,7 +23201,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="145" spans="1:23" ht="30" hidden="1">
+    <row r="145" spans="1:23" ht="30">
       <c r="A145" s="4" t="s">
         <v>673</v>
       </c>
@@ -23037,7 +23272,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="146" spans="1:23" ht="30" hidden="1">
+    <row r="146" spans="1:23" ht="30">
       <c r="A146" s="4" t="s">
         <v>673</v>
       </c>
@@ -23108,7 +23343,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="147" spans="1:23" ht="30" hidden="1">
+    <row r="147" spans="1:23" ht="30">
       <c r="A147" s="4" t="s">
         <v>673</v>
       </c>
@@ -23179,7 +23414,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="148" spans="1:23" ht="30" hidden="1">
+    <row r="148" spans="1:23" ht="30">
       <c r="A148" s="4" t="s">
         <v>673</v>
       </c>
@@ -23250,7 +23485,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="149" spans="1:23" hidden="1">
+    <row r="149" spans="1:23">
       <c r="A149" s="4" t="s">
         <v>673</v>
       </c>
@@ -23321,7 +23556,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="150" spans="1:23" ht="30" hidden="1">
+    <row r="150" spans="1:23" ht="30">
       <c r="A150" s="4" t="s">
         <v>34</v>
       </c>
@@ -23392,7 +23627,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="151" spans="1:23" ht="30" hidden="1">
+    <row r="151" spans="1:23" ht="30">
       <c r="A151" s="4" t="s">
         <v>34</v>
       </c>
@@ -23463,7 +23698,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="152" spans="1:23" ht="30" hidden="1">
+    <row r="152" spans="1:23" ht="30">
       <c r="A152" s="4" t="s">
         <v>34</v>
       </c>
@@ -23534,7 +23769,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="153" spans="1:23" ht="30" hidden="1">
+    <row r="153" spans="1:23" ht="30">
       <c r="A153" s="4" t="s">
         <v>34</v>
       </c>
@@ -23605,7 +23840,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="154" spans="1:23" hidden="1">
+    <row r="154" spans="1:23">
       <c r="A154" s="4" t="s">
         <v>34</v>
       </c>
@@ -23676,7 +23911,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="155" spans="1:23" ht="30" hidden="1">
+    <row r="155" spans="1:23" ht="30">
       <c r="A155" s="4" t="s">
         <v>34</v>
       </c>
@@ -23747,7 +23982,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="156" spans="1:23" ht="30" hidden="1">
+    <row r="156" spans="1:23" ht="30">
       <c r="A156" s="4" t="s">
         <v>34</v>
       </c>
@@ -23818,7 +24053,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="157" spans="1:23" ht="30" hidden="1">
+    <row r="157" spans="1:23" ht="30">
       <c r="A157" s="4" t="s">
         <v>34</v>
       </c>
@@ -23889,7 +24124,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="158" spans="1:23" ht="30" hidden="1">
+    <row r="158" spans="1:23" ht="30">
       <c r="A158" s="4" t="s">
         <v>34</v>
       </c>
@@ -23960,7 +24195,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="159" spans="1:23" ht="30" hidden="1">
+    <row r="159" spans="1:23" ht="30">
       <c r="A159" s="4" t="s">
         <v>34</v>
       </c>
@@ -24031,7 +24266,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="160" spans="1:23" ht="30" hidden="1">
+    <row r="160" spans="1:23" ht="30">
       <c r="A160" s="4" t="s">
         <v>34</v>
       </c>
@@ -24102,7 +24337,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="161" spans="1:23" hidden="1">
+    <row r="161" spans="1:23">
       <c r="A161" s="4" t="s">
         <v>34</v>
       </c>
@@ -24173,7 +24408,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="162" spans="1:23" ht="30" hidden="1">
+    <row r="162" spans="1:23" ht="30">
       <c r="A162" s="4" t="s">
         <v>34</v>
       </c>
@@ -24244,7 +24479,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="163" spans="1:23" ht="30" hidden="1">
+    <row r="163" spans="1:23" ht="30">
       <c r="A163" s="4" t="s">
         <v>34</v>
       </c>
@@ -24315,7 +24550,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="164" spans="1:23" ht="30" hidden="1">
+    <row r="164" spans="1:23" ht="30">
       <c r="A164" s="4" t="s">
         <v>34</v>
       </c>
@@ -24386,7 +24621,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="165" spans="1:23" ht="30" hidden="1">
+    <row r="165" spans="1:23" ht="30">
       <c r="A165" s="4" t="s">
         <v>34</v>
       </c>
@@ -24457,7 +24692,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="166" spans="1:23" ht="30" hidden="1">
+    <row r="166" spans="1:23" ht="30">
       <c r="A166" s="4" t="s">
         <v>35</v>
       </c>
@@ -24528,7 +24763,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="167" spans="1:23" ht="30" hidden="1">
+    <row r="167" spans="1:23" ht="30">
       <c r="A167" s="4" t="s">
         <v>35</v>
       </c>
@@ -24599,7 +24834,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="168" spans="1:23" ht="30" hidden="1">
+    <row r="168" spans="1:23" ht="30">
       <c r="A168" s="4" t="s">
         <v>35</v>
       </c>
@@ -24670,7 +24905,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="169" spans="1:23" ht="30" hidden="1">
+    <row r="169" spans="1:23" ht="30">
       <c r="A169" s="4" t="s">
         <v>35</v>
       </c>
@@ -24741,7 +24976,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="170" spans="1:23" ht="30" hidden="1">
+    <row r="170" spans="1:23" ht="30">
       <c r="A170" s="4" t="s">
         <v>35</v>
       </c>
@@ -24812,7 +25047,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="171" spans="1:23" ht="30" hidden="1">
+    <row r="171" spans="1:23" ht="30">
       <c r="A171" s="4" t="s">
         <v>35</v>
       </c>
@@ -24883,7 +25118,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="172" spans="1:23" ht="30" hidden="1">
+    <row r="172" spans="1:23" ht="30">
       <c r="A172" s="4" t="s">
         <v>35</v>
       </c>
@@ -24954,7 +25189,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="173" spans="1:23" ht="30" hidden="1">
+    <row r="173" spans="1:23" ht="30">
       <c r="A173" s="4" t="s">
         <v>35</v>
       </c>
@@ -25025,7 +25260,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="174" spans="1:23" ht="30" hidden="1">
+    <row r="174" spans="1:23" ht="30">
       <c r="A174" s="4" t="s">
         <v>35</v>
       </c>
@@ -25096,7 +25331,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="175" spans="1:23" ht="30" hidden="1">
+    <row r="175" spans="1:23" ht="30">
       <c r="A175" s="4" t="s">
         <v>35</v>
       </c>
@@ -25167,7 +25402,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="176" spans="1:23" ht="30" hidden="1">
+    <row r="176" spans="1:23" ht="30">
       <c r="A176" s="4" t="s">
         <v>35</v>
       </c>
@@ -25238,7 +25473,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="177" spans="1:23" ht="30" hidden="1">
+    <row r="177" spans="1:23" ht="30">
       <c r="A177" s="4" t="s">
         <v>35</v>
       </c>
@@ -25309,7 +25544,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="178" spans="1:23" ht="30" hidden="1">
+    <row r="178" spans="1:23" ht="30">
       <c r="A178" s="4" t="s">
         <v>35</v>
       </c>
@@ -25380,7 +25615,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="179" spans="1:23" ht="30" hidden="1">
+    <row r="179" spans="1:23" ht="30">
       <c r="A179" s="4" t="s">
         <v>35</v>
       </c>
@@ -25451,7 +25686,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="180" spans="1:23" ht="30" hidden="1">
+    <row r="180" spans="1:23" ht="30">
       <c r="A180" s="4" t="s">
         <v>35</v>
       </c>
@@ -25522,7 +25757,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="181" spans="1:23" ht="30" hidden="1">
+    <row r="181" spans="1:23" ht="30">
       <c r="A181" s="3" t="s">
         <v>94</v>
       </c>
@@ -25589,7 +25824,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="182" spans="1:23" ht="30" hidden="1">
+    <row r="182" spans="1:23" ht="30">
       <c r="A182" s="3" t="s">
         <v>94</v>
       </c>
@@ -25658,7 +25893,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="183" spans="1:23" ht="30" hidden="1">
+    <row r="183" spans="1:23" ht="30">
       <c r="A183" s="3" t="s">
         <v>94</v>
       </c>
@@ -25727,7 +25962,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="184" spans="1:23" ht="30" hidden="1">
+    <row r="184" spans="1:23" ht="30">
       <c r="A184" s="3" t="s">
         <v>94</v>
       </c>
@@ -25796,7 +26031,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="185" spans="1:23" ht="30" hidden="1">
+    <row r="185" spans="1:23" ht="30">
       <c r="A185" s="3" t="s">
         <v>94</v>
       </c>
@@ -25865,7 +26100,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="186" spans="1:23" ht="30" hidden="1">
+    <row r="186" spans="1:23" ht="30">
       <c r="A186" s="3" t="s">
         <v>94</v>
       </c>
@@ -25934,7 +26169,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="187" spans="1:23" hidden="1">
+    <row r="187" spans="1:23">
       <c r="A187" s="3" t="s">
         <v>42</v>
       </c>
@@ -26001,7 +26236,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="188" spans="1:23" hidden="1">
+    <row r="188" spans="1:23">
       <c r="A188" s="3" t="s">
         <v>42</v>
       </c>
@@ -26070,7 +26305,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="189" spans="1:23" hidden="1">
+    <row r="189" spans="1:23">
       <c r="A189" s="3" t="s">
         <v>42</v>
       </c>
@@ -26139,7 +26374,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="190" spans="1:23" ht="30" hidden="1">
+    <row r="190" spans="1:23" ht="30">
       <c r="A190" s="3" t="s">
         <v>42</v>
       </c>
@@ -26208,7 +26443,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="191" spans="1:23" hidden="1">
+    <row r="191" spans="1:23">
       <c r="A191" s="3" t="s">
         <v>42</v>
       </c>
@@ -26277,7 +26512,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="192" spans="1:23" ht="30" hidden="1">
+    <row r="192" spans="1:23" ht="30">
       <c r="A192" s="3" t="s">
         <v>42</v>
       </c>
@@ -26346,7 +26581,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="193" spans="1:23" hidden="1">
+    <row r="193" spans="1:23">
       <c r="A193" s="3" t="s">
         <v>129</v>
       </c>
@@ -26413,7 +26648,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="194" spans="1:23" hidden="1">
+    <row r="194" spans="1:23">
       <c r="A194" s="3" t="s">
         <v>129</v>
       </c>
@@ -26482,7 +26717,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="195" spans="1:23" hidden="1">
+    <row r="195" spans="1:23">
       <c r="A195" s="3" t="s">
         <v>129</v>
       </c>
@@ -26551,7 +26786,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="196" spans="1:23" hidden="1">
+    <row r="196" spans="1:23">
       <c r="A196" s="3" t="s">
         <v>129</v>
       </c>
@@ -26620,7 +26855,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="197" spans="1:23" hidden="1">
+    <row r="197" spans="1:23">
       <c r="A197" s="3" t="s">
         <v>129</v>
       </c>
@@ -26689,7 +26924,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="198" spans="1:23" ht="30" hidden="1">
+    <row r="198" spans="1:23" ht="30">
       <c r="A198" s="3" t="s">
         <v>129</v>
       </c>
@@ -26758,7 +26993,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="199" spans="1:23" ht="30" hidden="1">
+    <row r="199" spans="1:23" ht="30">
       <c r="A199" s="3" t="s">
         <v>129</v>
       </c>
@@ -26827,7 +27062,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="200" spans="1:23" hidden="1">
+    <row r="200" spans="1:23">
       <c r="A200" s="3" t="s">
         <v>126</v>
       </c>
@@ -26894,7 +27129,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="201" spans="1:23" hidden="1">
+    <row r="201" spans="1:23">
       <c r="A201" s="3" t="s">
         <v>126</v>
       </c>
@@ -26963,7 +27198,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="202" spans="1:23" hidden="1">
+    <row r="202" spans="1:23">
       <c r="A202" s="3" t="s">
         <v>126</v>
       </c>
@@ -27032,7 +27267,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="203" spans="1:23" ht="30" hidden="1">
+    <row r="203" spans="1:23" ht="30">
       <c r="A203" s="3" t="s">
         <v>126</v>
       </c>
@@ -27101,7 +27336,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="204" spans="1:23" ht="30" hidden="1">
+    <row r="204" spans="1:23" ht="30">
       <c r="A204" s="3" t="s">
         <v>126</v>
       </c>
@@ -27170,7 +27405,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="205" spans="1:23" hidden="1">
+    <row r="205" spans="1:23">
       <c r="A205" s="3" t="s">
         <v>126</v>
       </c>
@@ -27239,7 +27474,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="206" spans="1:23" ht="30" hidden="1">
+    <row r="206" spans="1:23" ht="30">
       <c r="A206" s="3" t="s">
         <v>126</v>
       </c>
@@ -27308,7 +27543,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="207" spans="1:23" ht="30" hidden="1">
+    <row r="207" spans="1:23" ht="30">
       <c r="A207" s="3" t="s">
         <v>126</v>
       </c>
@@ -27377,7 +27612,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="208" spans="1:23" ht="30" hidden="1">
+    <row r="208" spans="1:23" ht="30">
       <c r="A208" s="3" t="s">
         <v>313</v>
       </c>
@@ -27444,7 +27679,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="209" spans="1:23" ht="30" hidden="1">
+    <row r="209" spans="1:23" ht="30">
       <c r="A209" s="3" t="s">
         <v>313</v>
       </c>
@@ -27513,7 +27748,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="210" spans="1:23" ht="30" hidden="1">
+    <row r="210" spans="1:23" ht="30">
       <c r="A210" s="3" t="s">
         <v>313</v>
       </c>
@@ -27582,7 +27817,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="211" spans="1:23" ht="30" hidden="1">
+    <row r="211" spans="1:23" ht="30">
       <c r="A211" s="3" t="s">
         <v>313</v>
       </c>
@@ -27651,7 +27886,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="212" spans="1:23" ht="30" hidden="1">
+    <row r="212" spans="1:23" ht="30">
       <c r="A212" s="3" t="s">
         <v>313</v>
       </c>
@@ -27720,7 +27955,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="213" spans="1:23" ht="45" hidden="1">
+    <row r="213" spans="1:23" ht="45">
       <c r="A213" s="3" t="s">
         <v>313</v>
       </c>
@@ -27789,7 +28024,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="214" spans="1:23" ht="30" hidden="1">
+    <row r="214" spans="1:23" ht="30">
       <c r="A214" s="3" t="s">
         <v>445</v>
       </c>
@@ -27856,7 +28091,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="215" spans="1:23" ht="30" hidden="1">
+    <row r="215" spans="1:23" ht="30">
       <c r="A215" s="3" t="s">
         <v>445</v>
       </c>
@@ -27925,7 +28160,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="216" spans="1:23" ht="30" hidden="1">
+    <row r="216" spans="1:23" ht="30">
       <c r="A216" s="3" t="s">
         <v>445</v>
       </c>
@@ -27994,7 +28229,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="217" spans="1:23" ht="30" hidden="1">
+    <row r="217" spans="1:23" ht="30">
       <c r="A217" s="3" t="s">
         <v>445</v>
       </c>
@@ -28063,7 +28298,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="218" spans="1:23" ht="30" hidden="1">
+    <row r="218" spans="1:23" ht="30">
       <c r="A218" s="3" t="s">
         <v>445</v>
       </c>
@@ -28132,7 +28367,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="219" spans="1:23" ht="30" hidden="1">
+    <row r="219" spans="1:23" ht="30">
       <c r="A219" s="3" t="s">
         <v>445</v>
       </c>
@@ -28201,7 +28436,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="220" spans="1:23" ht="30" hidden="1">
+    <row r="220" spans="1:23" ht="30">
       <c r="A220" s="3" t="s">
         <v>451</v>
       </c>
@@ -28268,7 +28503,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="221" spans="1:23" hidden="1">
+    <row r="221" spans="1:23">
       <c r="A221" s="3" t="s">
         <v>451</v>
       </c>
@@ -28337,7 +28572,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="222" spans="1:23" hidden="1">
+    <row r="222" spans="1:23">
       <c r="A222" s="3" t="s">
         <v>451</v>
       </c>
@@ -28406,7 +28641,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="223" spans="1:23" ht="30" hidden="1">
+    <row r="223" spans="1:23" ht="30">
       <c r="A223" s="3" t="s">
         <v>451</v>
       </c>
@@ -28475,7 +28710,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="224" spans="1:23" hidden="1">
+    <row r="224" spans="1:23">
       <c r="A224" s="3" t="s">
         <v>451</v>
       </c>
@@ -28544,7 +28779,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="225" spans="1:23" ht="30" hidden="1">
+    <row r="225" spans="1:23" ht="30">
       <c r="A225" s="3" t="s">
         <v>451</v>
       </c>
@@ -28613,7 +28848,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="226" spans="1:23" ht="30" hidden="1">
+    <row r="226" spans="1:23" ht="30">
       <c r="A226" s="3" t="s">
         <v>512</v>
       </c>
@@ -28680,7 +28915,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="227" spans="1:23" ht="30" hidden="1">
+    <row r="227" spans="1:23" ht="30">
       <c r="A227" s="3" t="s">
         <v>512</v>
       </c>
@@ -28749,7 +28984,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="228" spans="1:23" ht="30" hidden="1">
+    <row r="228" spans="1:23" ht="30">
       <c r="A228" s="3" t="s">
         <v>512</v>
       </c>
@@ -28818,7 +29053,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="229" spans="1:23" ht="30" hidden="1">
+    <row r="229" spans="1:23" ht="30">
       <c r="A229" s="3" t="s">
         <v>512</v>
       </c>
@@ -28887,7 +29122,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="230" spans="1:23" ht="30" hidden="1">
+    <row r="230" spans="1:23" ht="30">
       <c r="A230" s="3" t="s">
         <v>512</v>
       </c>
@@ -28956,7 +29191,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="231" spans="1:23" ht="30" hidden="1">
+    <row r="231" spans="1:23" ht="30">
       <c r="A231" s="3" t="s">
         <v>512</v>
       </c>
@@ -29025,7 +29260,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="232" spans="1:23" ht="30" hidden="1">
+    <row r="232" spans="1:23" ht="30">
       <c r="A232" s="3" t="s">
         <v>518</v>
       </c>
@@ -29092,7 +29327,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="233" spans="1:23" hidden="1">
+    <row r="233" spans="1:23">
       <c r="A233" s="3" t="s">
         <v>518</v>
       </c>
@@ -29161,7 +29396,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="234" spans="1:23" hidden="1">
+    <row r="234" spans="1:23">
       <c r="A234" s="3" t="s">
         <v>518</v>
       </c>
@@ -29230,7 +29465,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="235" spans="1:23" ht="30" hidden="1">
+    <row r="235" spans="1:23" ht="30">
       <c r="A235" s="3" t="s">
         <v>518</v>
       </c>
@@ -29299,7 +29534,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="236" spans="1:23" hidden="1">
+    <row r="236" spans="1:23">
       <c r="A236" s="3" t="s">
         <v>518</v>
       </c>
@@ -29368,7 +29603,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="237" spans="1:23" ht="30" hidden="1">
+    <row r="237" spans="1:23" ht="30">
       <c r="A237" s="3" t="s">
         <v>518</v>
       </c>
@@ -29437,7 +29672,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="238" spans="1:23" ht="30" hidden="1">
+    <row r="238" spans="1:23" ht="30">
       <c r="A238" s="3" t="s">
         <v>757</v>
       </c>
@@ -29504,7 +29739,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="239" spans="1:23" hidden="1">
+    <row r="239" spans="1:23">
       <c r="A239" s="3" t="s">
         <v>757</v>
       </c>
@@ -29573,7 +29808,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="240" spans="1:23" hidden="1">
+    <row r="240" spans="1:23">
       <c r="A240" s="3" t="s">
         <v>757</v>
       </c>
@@ -29642,7 +29877,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="241" spans="1:23" hidden="1">
+    <row r="241" spans="1:23">
       <c r="A241" s="3" t="s">
         <v>757</v>
       </c>
@@ -29711,7 +29946,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="242" spans="1:23" hidden="1">
+    <row r="242" spans="1:23">
       <c r="A242" s="3" t="s">
         <v>757</v>
       </c>
@@ -29780,7 +30015,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="243" spans="1:23" ht="30" hidden="1">
+    <row r="243" spans="1:23" ht="30">
       <c r="A243" s="3" t="s">
         <v>757</v>
       </c>
@@ -29849,7 +30084,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="244" spans="1:23" ht="30" hidden="1">
+    <row r="244" spans="1:23" ht="30">
       <c r="A244" s="3" t="s">
         <v>1517</v>
       </c>
@@ -29916,7 +30151,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="245" spans="1:23" ht="30" hidden="1">
+    <row r="245" spans="1:23" ht="30">
       <c r="A245" s="3" t="s">
         <v>1517</v>
       </c>
@@ -29983,7 +30218,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="246" spans="1:23" ht="30" hidden="1">
+    <row r="246" spans="1:23" ht="30">
       <c r="A246" s="3" t="s">
         <v>1517</v>
       </c>
@@ -30052,7 +30287,7 @@
         <v>1446</v>
       </c>
     </row>
-    <row r="247" spans="1:23" ht="30" hidden="1">
+    <row r="247" spans="1:23" ht="30">
       <c r="A247" s="3" t="s">
         <v>1517</v>
       </c>
@@ -30121,7 +30356,7 @@
         <v>1446</v>
       </c>
     </row>
-    <row r="248" spans="1:23" hidden="1">
+    <row r="248" spans="1:23">
       <c r="A248" s="3" t="s">
         <v>1517</v>
       </c>
@@ -30190,7 +30425,7 @@
         <v>1446</v>
       </c>
     </row>
-    <row r="249" spans="1:23" ht="30" hidden="1">
+    <row r="249" spans="1:23" ht="30">
       <c r="A249" s="3" t="s">
         <v>1517</v>
       </c>
@@ -30259,7 +30494,7 @@
         <v>1446</v>
       </c>
     </row>
-    <row r="250" spans="1:23" hidden="1">
+    <row r="250" spans="1:23">
       <c r="A250" s="3" t="s">
         <v>1517</v>
       </c>
@@ -30328,7 +30563,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="251" spans="1:23" hidden="1">
+    <row r="251" spans="1:23">
       <c r="A251" s="3" t="s">
         <v>1517</v>
       </c>
@@ -30397,7 +30632,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="252" spans="1:23" hidden="1">
+    <row r="252" spans="1:23">
       <c r="A252" s="3" t="s">
         <v>1517</v>
       </c>
@@ -30466,7 +30701,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="253" spans="1:23" hidden="1">
+    <row r="253" spans="1:23">
       <c r="A253" s="3" t="s">
         <v>1517</v>
       </c>
@@ -30535,7 +30770,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="254" spans="1:23" hidden="1">
+    <row r="254" spans="1:23">
       <c r="A254" s="3" t="s">
         <v>1517</v>
       </c>
@@ -30604,7 +30839,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="255" spans="1:23" hidden="1">
+    <row r="255" spans="1:23">
       <c r="A255" s="3" t="s">
         <v>1517</v>
       </c>
@@ -30673,7 +30908,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="256" spans="1:23" ht="30" hidden="1">
+    <row r="256" spans="1:23" ht="30">
       <c r="A256" s="3" t="s">
         <v>1517</v>
       </c>
@@ -30742,7 +30977,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="257" spans="1:23" ht="30" hidden="1">
+    <row r="257" spans="1:23" ht="30">
       <c r="A257" s="3" t="s">
         <v>1517</v>
       </c>
@@ -30811,7 +31046,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="258" spans="1:23" hidden="1">
+    <row r="258" spans="1:23">
       <c r="A258" s="3" t="s">
         <v>1517</v>
       </c>
@@ -30878,7 +31113,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="259" spans="1:23" hidden="1">
+    <row r="259" spans="1:23">
       <c r="A259" s="3" t="s">
         <v>1517</v>
       </c>
@@ -30945,7 +31180,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="260" spans="1:23" hidden="1">
+    <row r="260" spans="1:23">
       <c r="A260" s="3" t="s">
         <v>1517</v>
       </c>
@@ -31012,7 +31247,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="261" spans="1:23" hidden="1">
+    <row r="261" spans="1:23">
       <c r="A261" s="3" t="s">
         <v>1517</v>
       </c>
@@ -31081,7 +31316,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="262" spans="1:23" hidden="1">
+    <row r="262" spans="1:23">
       <c r="A262" s="3" t="s">
         <v>1517</v>
       </c>
@@ -31150,7 +31385,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="263" spans="1:23" ht="30" hidden="1">
+    <row r="263" spans="1:23" ht="30">
       <c r="A263" s="3" t="s">
         <v>1518</v>
       </c>
@@ -31217,7 +31452,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="264" spans="1:23" ht="30" hidden="1">
+    <row r="264" spans="1:23" ht="30">
       <c r="A264" s="3" t="s">
         <v>1518</v>
       </c>
@@ -31284,7 +31519,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="265" spans="1:23" ht="30" hidden="1">
+    <row r="265" spans="1:23" ht="30">
       <c r="A265" s="3" t="s">
         <v>1518</v>
       </c>
@@ -31355,7 +31590,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="266" spans="1:23" hidden="1">
+    <row r="266" spans="1:23">
       <c r="A266" s="3" t="s">
         <v>1518</v>
       </c>
@@ -31422,7 +31657,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="267" spans="1:23" ht="30" hidden="1">
+    <row r="267" spans="1:23" ht="30">
       <c r="A267" s="3" t="s">
         <v>1518</v>
       </c>
@@ -31491,7 +31726,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="268" spans="1:23" hidden="1">
+    <row r="268" spans="1:23">
       <c r="A268" s="3" t="s">
         <v>1518</v>
       </c>
@@ -31560,7 +31795,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="269" spans="1:23" hidden="1">
+    <row r="269" spans="1:23">
       <c r="A269" s="3" t="s">
         <v>1518</v>
       </c>
@@ -31629,7 +31864,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="270" spans="1:23" ht="30" hidden="1">
+    <row r="270" spans="1:23" ht="30">
       <c r="A270" s="3" t="s">
         <v>1518</v>
       </c>
@@ -31696,7 +31931,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="271" spans="1:23" ht="30" hidden="1">
+    <row r="271" spans="1:23" ht="30">
       <c r="A271" s="3" t="s">
         <v>1518</v>
       </c>
@@ -31763,7 +31998,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="272" spans="1:23" hidden="1">
+    <row r="272" spans="1:23">
       <c r="A272" s="3" t="s">
         <v>1518</v>
       </c>
@@ -31828,7 +32063,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="273" spans="1:23" hidden="1">
+    <row r="273" spans="1:23">
       <c r="A273" s="3" t="s">
         <v>1518</v>
       </c>
@@ -31893,7 +32128,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="274" spans="1:23" hidden="1">
+    <row r="274" spans="1:23">
       <c r="A274" s="3" t="s">
         <v>1518</v>
       </c>
@@ -31958,7 +32193,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="275" spans="1:23" hidden="1">
+    <row r="275" spans="1:23">
       <c r="A275" s="3" t="s">
         <v>1518</v>
       </c>
@@ -32027,7 +32262,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="276" spans="1:23" hidden="1">
+    <row r="276" spans="1:23">
       <c r="A276" s="3" t="s">
         <v>1518</v>
       </c>
@@ -32096,7 +32331,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="277" spans="1:23" ht="30" hidden="1">
+    <row r="277" spans="1:23" ht="30">
       <c r="A277" s="3" t="s">
         <v>1578</v>
       </c>
@@ -32163,7 +32398,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="278" spans="1:23" ht="30" hidden="1">
+    <row r="278" spans="1:23" ht="30">
       <c r="A278" s="3" t="s">
         <v>1578</v>
       </c>
@@ -32230,7 +32465,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="279" spans="1:23" ht="45" hidden="1">
+    <row r="279" spans="1:23" ht="45">
       <c r="A279" s="3" t="s">
         <v>1578</v>
       </c>
@@ -32301,7 +32536,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="280" spans="1:23" ht="30" hidden="1">
+    <row r="280" spans="1:23" ht="30">
       <c r="A280" s="3" t="s">
         <v>1578</v>
       </c>
@@ -32370,7 +32605,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="281" spans="1:23" ht="30" hidden="1">
+    <row r="281" spans="1:23" ht="30">
       <c r="A281" s="3" t="s">
         <v>1578</v>
       </c>
@@ -32439,7 +32674,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="282" spans="1:23" ht="30" hidden="1">
+    <row r="282" spans="1:23" ht="30">
       <c r="A282" s="3" t="s">
         <v>1578</v>
       </c>
@@ -32508,7 +32743,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="283" spans="1:23" ht="30" hidden="1">
+    <row r="283" spans="1:23" ht="30">
       <c r="A283" s="3" t="s">
         <v>1578</v>
       </c>
@@ -32577,7 +32812,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="284" spans="1:23" ht="30" hidden="1">
+    <row r="284" spans="1:23" ht="30">
       <c r="A284" s="3" t="s">
         <v>1578</v>
       </c>
@@ -32646,7 +32881,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="285" spans="1:23" ht="30" hidden="1">
+    <row r="285" spans="1:23" ht="30">
       <c r="A285" s="3" t="s">
         <v>1578</v>
       </c>
@@ -32713,7 +32948,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="286" spans="1:23" ht="30" hidden="1">
+    <row r="286" spans="1:23" ht="30">
       <c r="A286" s="3" t="s">
         <v>1578</v>
       </c>
@@ -32780,7 +33015,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="287" spans="1:23" ht="30" hidden="1">
+    <row r="287" spans="1:23" ht="30">
       <c r="A287" s="3" t="s">
         <v>1578</v>
       </c>
@@ -32845,7 +33080,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="288" spans="1:23" ht="30" hidden="1">
+    <row r="288" spans="1:23" ht="30">
       <c r="A288" s="3" t="s">
         <v>1578</v>
       </c>
@@ -32910,7 +33145,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="289" spans="1:23" ht="30" hidden="1">
+    <row r="289" spans="1:23" ht="30">
       <c r="A289" s="3" t="s">
         <v>1578</v>
       </c>
@@ -32975,7 +33210,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="290" spans="1:23" ht="30" hidden="1">
+    <row r="290" spans="1:23" ht="30">
       <c r="A290" s="3" t="s">
         <v>1578</v>
       </c>
@@ -33044,7 +33279,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="291" spans="1:23" ht="30" hidden="1">
+    <row r="291" spans="1:23" ht="30">
       <c r="A291" s="3" t="s">
         <v>1578</v>
       </c>
@@ -33113,7 +33348,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="292" spans="1:23" ht="30" hidden="1">
+    <row r="292" spans="1:23" ht="30">
       <c r="A292" s="3" t="s">
         <v>1635</v>
       </c>
@@ -33180,7 +33415,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="293" spans="1:23" ht="30" hidden="1">
+    <row r="293" spans="1:23" ht="30">
       <c r="A293" s="3" t="s">
         <v>1635</v>
       </c>
@@ -33247,7 +33482,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="294" spans="1:23" ht="45" hidden="1">
+    <row r="294" spans="1:23" ht="45">
       <c r="A294" s="3" t="s">
         <v>1635</v>
       </c>
@@ -33316,7 +33551,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="295" spans="1:23" hidden="1">
+    <row r="295" spans="1:23">
       <c r="A295" s="3" t="s">
         <v>1635</v>
       </c>
@@ -33383,7 +33618,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="296" spans="1:23" hidden="1">
+    <row r="296" spans="1:23">
       <c r="A296" s="3" t="s">
         <v>1635</v>
       </c>
@@ -33450,7 +33685,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="297" spans="1:23" ht="30" hidden="1">
+    <row r="297" spans="1:23" ht="30">
       <c r="A297" s="3" t="s">
         <v>1635</v>
       </c>
@@ -33517,7 +33752,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="298" spans="1:23" hidden="1">
+    <row r="298" spans="1:23">
       <c r="A298" s="3" t="s">
         <v>1635</v>
       </c>
@@ -33584,7 +33819,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="299" spans="1:23" ht="45" hidden="1">
+    <row r="299" spans="1:23" ht="45">
       <c r="A299" s="3" t="s">
         <v>1635</v>
       </c>
@@ -33653,7 +33888,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="300" spans="1:23" ht="30" hidden="1">
+    <row r="300" spans="1:23" ht="30">
       <c r="A300" s="3" t="s">
         <v>1635</v>
       </c>
@@ -33718,7 +33953,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="301" spans="1:23" ht="30" hidden="1">
+    <row r="301" spans="1:23" ht="30">
       <c r="A301" s="3" t="s">
         <v>1635</v>
       </c>
@@ -33787,7 +34022,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="302" spans="1:23" ht="30" hidden="1">
+    <row r="302" spans="1:23" ht="30">
       <c r="A302" s="3" t="s">
         <v>1635</v>
       </c>
@@ -33854,7 +34089,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="303" spans="1:23" ht="30" hidden="1">
+    <row r="303" spans="1:23" ht="30">
       <c r="A303" s="3" t="s">
         <v>1689</v>
       </c>
@@ -33921,7 +34156,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="304" spans="1:23" ht="30" hidden="1">
+    <row r="304" spans="1:23" ht="30">
       <c r="A304" s="3" t="s">
         <v>1689</v>
       </c>
@@ -33988,7 +34223,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="305" spans="1:23" ht="30" hidden="1">
+    <row r="305" spans="1:23" ht="30">
       <c r="A305" s="3" t="s">
         <v>1689</v>
       </c>
@@ -34057,7 +34292,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="306" spans="1:23" ht="30" hidden="1">
+    <row r="306" spans="1:23" ht="30">
       <c r="A306" s="3" t="s">
         <v>1689</v>
       </c>
@@ -34124,7 +34359,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="307" spans="1:23" ht="30" hidden="1">
+    <row r="307" spans="1:23" ht="30">
       <c r="A307" s="3" t="s">
         <v>1689</v>
       </c>
@@ -34193,7 +34428,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="308" spans="1:23" ht="30" hidden="1">
+    <row r="308" spans="1:23" ht="30">
       <c r="A308" s="3" t="s">
         <v>1689</v>
       </c>
@@ -34262,7 +34497,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="309" spans="1:23" ht="30" hidden="1">
+    <row r="309" spans="1:23" ht="30">
       <c r="A309" s="3" t="s">
         <v>1689</v>
       </c>
@@ -34329,7 +34564,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="310" spans="1:23" ht="30" hidden="1">
+    <row r="310" spans="1:23" ht="30">
       <c r="A310" s="3" t="s">
         <v>1689</v>
       </c>
@@ -34396,7 +34631,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="311" spans="1:23" ht="30" hidden="1">
+    <row r="311" spans="1:23" ht="30">
       <c r="A311" s="3" t="s">
         <v>1689</v>
       </c>
@@ -34461,7 +34696,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="312" spans="1:23" ht="30" hidden="1">
+    <row r="312" spans="1:23" ht="30">
       <c r="A312" s="3" t="s">
         <v>1689</v>
       </c>
@@ -34528,7 +34763,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="313" spans="1:23" ht="45" hidden="1">
+    <row r="313" spans="1:23" ht="45">
       <c r="A313" s="3" t="s">
         <v>1689</v>
       </c>
@@ -34597,7 +34832,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="314" spans="1:23" ht="30" hidden="1">
+    <row r="314" spans="1:23" ht="30">
       <c r="A314" s="3" t="s">
         <v>1689</v>
       </c>
@@ -34666,7 +34901,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="315" spans="1:23" ht="30" hidden="1">
+    <row r="315" spans="1:23" ht="30">
       <c r="A315" s="3" t="s">
         <v>1704</v>
       </c>
@@ -34733,7 +34968,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="316" spans="1:23" ht="30" hidden="1">
+    <row r="316" spans="1:23" ht="30">
       <c r="A316" s="3" t="s">
         <v>1704</v>
       </c>
@@ -34802,7 +35037,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="317" spans="1:23" hidden="1">
+    <row r="317" spans="1:23">
       <c r="A317" s="3" t="s">
         <v>1704</v>
       </c>
@@ -34871,7 +35106,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="318" spans="1:23" ht="30" hidden="1">
+    <row r="318" spans="1:23" ht="30">
       <c r="A318" s="3" t="s">
         <v>1704</v>
       </c>
@@ -34940,7 +35175,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="319" spans="1:23" hidden="1">
+    <row r="319" spans="1:23">
       <c r="A319" s="3" t="s">
         <v>1704</v>
       </c>
@@ -35009,7 +35244,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="320" spans="1:23" ht="30" hidden="1">
+    <row r="320" spans="1:23" ht="30">
       <c r="A320" s="3" t="s">
         <v>1704</v>
       </c>
@@ -35078,7 +35313,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="321" spans="1:23" ht="30" hidden="1">
+    <row r="321" spans="1:23" ht="30">
       <c r="A321" s="3" t="s">
         <v>1704</v>
       </c>
@@ -35145,7 +35380,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="322" spans="1:23" hidden="1">
+    <row r="322" spans="1:23">
       <c r="A322" s="3" t="s">
         <v>1704</v>
       </c>
@@ -35210,7 +35445,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="323" spans="1:23" ht="30" hidden="1">
+    <row r="323" spans="1:23" ht="30">
       <c r="A323" s="3" t="s">
         <v>1704</v>
       </c>
@@ -35279,7 +35514,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="324" spans="1:23" hidden="1">
+    <row r="324" spans="1:23">
       <c r="A324" s="3" t="s">
         <v>1704</v>
       </c>
@@ -35348,7 +35583,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="325" spans="1:23" ht="30" hidden="1">
+    <row r="325" spans="1:23" ht="30">
       <c r="A325" s="3" t="s">
         <v>1806</v>
       </c>
@@ -35415,7 +35650,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="326" spans="1:23" ht="30" hidden="1">
+    <row r="326" spans="1:23" ht="30">
       <c r="A326" s="3" t="s">
         <v>1806</v>
       </c>
@@ -35482,7 +35717,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="327" spans="1:23" ht="30" hidden="1">
+    <row r="327" spans="1:23" ht="30">
       <c r="A327" s="3" t="s">
         <v>1806</v>
       </c>
@@ -35549,7 +35784,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="328" spans="1:23" ht="30" hidden="1">
+    <row r="328" spans="1:23" ht="30">
       <c r="A328" s="3" t="s">
         <v>1806</v>
       </c>
@@ -35618,7 +35853,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="329" spans="1:23" ht="45" hidden="1">
+    <row r="329" spans="1:23" ht="45">
       <c r="A329" s="3" t="s">
         <v>1806</v>
       </c>
@@ -35687,7 +35922,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="330" spans="1:23" ht="30" hidden="1">
+    <row r="330" spans="1:23" ht="30">
       <c r="A330" s="3" t="s">
         <v>1806</v>
       </c>
@@ -35754,7 +35989,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="331" spans="1:23" ht="30" hidden="1">
+    <row r="331" spans="1:23" ht="30">
       <c r="A331" s="3" t="s">
         <v>1806</v>
       </c>
@@ -35821,7 +36056,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="332" spans="1:23" ht="30" hidden="1">
+    <row r="332" spans="1:23" ht="30">
       <c r="A332" s="3" t="s">
         <v>1806</v>
       </c>
@@ -35890,7 +36125,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="333" spans="1:23" ht="30" hidden="1">
+    <row r="333" spans="1:23" ht="30">
       <c r="A333" s="3" t="s">
         <v>1806</v>
       </c>
@@ -35957,7 +36192,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="334" spans="1:23" ht="30" hidden="1">
+    <row r="334" spans="1:23" ht="30">
       <c r="A334" s="3" t="s">
         <v>1806</v>
       </c>
@@ -36024,7 +36259,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="335" spans="1:23" ht="30" hidden="1">
+    <row r="335" spans="1:23" ht="30">
       <c r="A335" s="3" t="s">
         <v>1806</v>
       </c>
@@ -36089,7 +36324,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="336" spans="1:23" ht="30" hidden="1">
+    <row r="336" spans="1:23" ht="30">
       <c r="A336" s="3" t="s">
         <v>1806</v>
       </c>
@@ -36156,7 +36391,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="337" spans="1:23" ht="45" hidden="1">
+    <row r="337" spans="1:23" ht="45">
       <c r="A337" s="3" t="s">
         <v>1806</v>
       </c>
@@ -36225,7 +36460,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="338" spans="1:23" ht="30" hidden="1">
+    <row r="338" spans="1:23" ht="30">
       <c r="A338" s="3" t="s">
         <v>1806</v>
       </c>
@@ -37274,7 +37509,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="353" spans="1:23" ht="30" hidden="1">
+    <row r="353" spans="1:23" ht="30">
       <c r="A353" s="3" t="s">
         <v>1922</v>
       </c>
@@ -37343,7 +37578,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="354" spans="1:23" ht="30" hidden="1">
+    <row r="354" spans="1:23" ht="30">
       <c r="A354" s="3" t="s">
         <v>1922</v>
       </c>
@@ -37412,7 +37647,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="355" spans="1:23" hidden="1">
+    <row r="355" spans="1:23">
       <c r="A355" s="3" t="s">
         <v>1922</v>
       </c>
@@ -37481,7 +37716,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="356" spans="1:23" ht="45" hidden="1">
+    <row r="356" spans="1:23" ht="45">
       <c r="A356" s="3" t="s">
         <v>1922</v>
       </c>
@@ -37550,7 +37785,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="357" spans="1:23" ht="30" hidden="1">
+    <row r="357" spans="1:23" ht="30">
       <c r="A357" s="3" t="s">
         <v>1922</v>
       </c>
@@ -37621,7 +37856,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="358" spans="1:23" ht="30" hidden="1">
+    <row r="358" spans="1:23" ht="30">
       <c r="A358" s="4" t="s">
         <v>2018</v>
       </c>
@@ -37692,7 +37927,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="359" spans="1:23" ht="30" hidden="1">
+    <row r="359" spans="1:23" ht="30">
       <c r="A359" s="4" t="s">
         <v>2018</v>
       </c>
@@ -37763,7 +37998,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="360" spans="1:23" ht="30" hidden="1">
+    <row r="360" spans="1:23" ht="30">
       <c r="A360" s="4" t="s">
         <v>2018</v>
       </c>
@@ -37834,7 +38069,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="361" spans="1:23" ht="45" hidden="1">
+    <row r="361" spans="1:23" ht="45">
       <c r="A361" s="4" t="s">
         <v>2018</v>
       </c>
@@ -37905,7 +38140,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="362" spans="1:23" ht="30" hidden="1">
+    <row r="362" spans="1:23" ht="30">
       <c r="A362" s="4" t="s">
         <v>2018</v>
       </c>
@@ -37976,7 +38211,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="363" spans="1:23" ht="30" hidden="1">
+    <row r="363" spans="1:23" ht="30">
       <c r="A363" s="4" t="s">
         <v>2018</v>
       </c>
@@ -38047,7 +38282,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="364" spans="1:23" ht="30" hidden="1">
+    <row r="364" spans="1:23" ht="30">
       <c r="A364" s="4" t="s">
         <v>2018</v>
       </c>
@@ -38118,7 +38353,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="365" spans="1:23" ht="30" hidden="1">
+    <row r="365" spans="1:23" ht="30">
       <c r="A365" s="4" t="s">
         <v>2018</v>
       </c>
@@ -38189,7 +38424,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="366" spans="1:23" ht="30" hidden="1">
+    <row r="366" spans="1:23" ht="30">
       <c r="A366" s="4" t="s">
         <v>2018</v>
       </c>
@@ -38260,7 +38495,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="367" spans="1:23" ht="30" hidden="1">
+    <row r="367" spans="1:23" ht="30">
       <c r="A367" s="4" t="s">
         <v>2018</v>
       </c>
@@ -38331,7 +38566,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="368" spans="1:23" ht="30" hidden="1">
+    <row r="368" spans="1:23" ht="30">
       <c r="A368" s="4" t="s">
         <v>2062</v>
       </c>
@@ -38402,7 +38637,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="369" spans="1:23" ht="30" hidden="1">
+    <row r="369" spans="1:23" ht="30">
       <c r="A369" s="4" t="s">
         <v>2062</v>
       </c>
@@ -38473,7 +38708,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="370" spans="1:23" ht="30" hidden="1">
+    <row r="370" spans="1:23" ht="30">
       <c r="A370" s="4" t="s">
         <v>2062</v>
       </c>
@@ -38544,7 +38779,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="371" spans="1:23" ht="30" hidden="1">
+    <row r="371" spans="1:23" ht="30">
       <c r="A371" s="4" t="s">
         <v>2062</v>
       </c>
@@ -38615,7 +38850,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="372" spans="1:23" ht="30" hidden="1">
+    <row r="372" spans="1:23" ht="30">
       <c r="A372" s="4" t="s">
         <v>2062</v>
       </c>
@@ -38686,7 +38921,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="373" spans="1:23" ht="45" hidden="1">
+    <row r="373" spans="1:23" ht="45">
       <c r="A373" s="4" t="s">
         <v>2062</v>
       </c>
@@ -38757,7 +38992,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="374" spans="1:23" ht="30" hidden="1">
+    <row r="374" spans="1:23" ht="30">
       <c r="A374" s="4" t="s">
         <v>2062</v>
       </c>
@@ -38828,7 +39063,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="375" spans="1:23" ht="30" hidden="1">
+    <row r="375" spans="1:23" ht="30">
       <c r="A375" s="4" t="s">
         <v>2062</v>
       </c>
@@ -38899,7 +39134,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="376" spans="1:23" ht="30" hidden="1">
+    <row r="376" spans="1:23" ht="30">
       <c r="A376" s="4" t="s">
         <v>2062</v>
       </c>
@@ -38970,7 +39205,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="377" spans="1:23" ht="30" hidden="1">
+    <row r="377" spans="1:23" ht="30">
       <c r="A377" s="4" t="s">
         <v>2062</v>
       </c>
@@ -39041,7 +39276,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="378" spans="1:23" ht="30" hidden="1">
+    <row r="378" spans="1:23" ht="30">
       <c r="A378" s="4" t="s">
         <v>2062</v>
       </c>
@@ -39112,7 +39347,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="379" spans="1:23" ht="30" hidden="1">
+    <row r="379" spans="1:23" ht="30">
       <c r="A379" s="4" t="s">
         <v>2062</v>
       </c>
@@ -39183,7 +39418,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="380" spans="1:23" hidden="1">
+    <row r="380" spans="1:23">
       <c r="A380" s="4" t="s">
         <v>2110</v>
       </c>
@@ -39254,7 +39489,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="381" spans="1:23" ht="30" hidden="1">
+    <row r="381" spans="1:23" ht="30">
       <c r="A381" s="4" t="s">
         <v>2110</v>
       </c>
@@ -39325,7 +39560,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="382" spans="1:23" ht="30" hidden="1">
+    <row r="382" spans="1:23" ht="30">
       <c r="A382" s="4" t="s">
         <v>2110</v>
       </c>
@@ -39396,7 +39631,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="383" spans="1:23" ht="45" hidden="1">
+    <row r="383" spans="1:23" ht="45">
       <c r="A383" s="4" t="s">
         <v>2110</v>
       </c>
@@ -39464,7 +39699,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="384" spans="1:23" ht="30" hidden="1">
+    <row r="384" spans="1:23" ht="30">
       <c r="A384" s="4" t="s">
         <v>2110</v>
       </c>
@@ -39532,7 +39767,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="385" spans="1:23" ht="45" hidden="1">
+    <row r="385" spans="1:23" ht="45">
       <c r="A385" s="4" t="s">
         <v>2110</v>
       </c>
@@ -39603,7 +39838,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="386" spans="1:23" ht="30" hidden="1">
+    <row r="386" spans="1:23" ht="30">
       <c r="A386" s="4" t="s">
         <v>2110</v>
       </c>
@@ -39674,7 +39909,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="387" spans="1:23" ht="30" hidden="1">
+    <row r="387" spans="1:23" ht="30">
       <c r="A387" s="4" t="s">
         <v>2110</v>
       </c>
@@ -39742,7 +39977,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="388" spans="1:23" ht="30" hidden="1">
+    <row r="388" spans="1:23" ht="30">
       <c r="A388" s="4" t="s">
         <v>2110</v>
       </c>
@@ -39810,7 +40045,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="389" spans="1:23" ht="30" hidden="1">
+    <row r="389" spans="1:23" ht="30">
       <c r="A389" s="4" t="s">
         <v>2110</v>
       </c>
@@ -39878,7 +40113,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="390" spans="1:23" ht="30" hidden="1">
+    <row r="390" spans="1:23" ht="30">
       <c r="A390" s="4" t="s">
         <v>2110</v>
       </c>
@@ -39949,7 +40184,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="391" spans="1:23" ht="30" hidden="1">
+    <row r="391" spans="1:23" ht="30">
       <c r="A391" s="4" t="s">
         <v>2110</v>
       </c>
@@ -40020,7 +40255,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="392" spans="1:23" ht="30" hidden="1">
+    <row r="392" spans="1:23" ht="30">
       <c r="A392" s="4" t="s">
         <v>2110</v>
       </c>
@@ -40091,7 +40326,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="393" spans="1:23" ht="30" hidden="1">
+    <row r="393" spans="1:23" ht="30">
       <c r="A393" s="4" t="s">
         <v>2110</v>
       </c>
@@ -40162,7 +40397,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="394" spans="1:23" ht="30" hidden="1">
+    <row r="394" spans="1:23" ht="30">
       <c r="A394" s="4" t="s">
         <v>2110</v>
       </c>
@@ -40233,7 +40468,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="395" spans="1:23" ht="30" hidden="1">
+    <row r="395" spans="1:23" ht="30">
       <c r="A395" s="4" t="s">
         <v>2110</v>
       </c>
@@ -40304,7 +40539,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="396" spans="1:23" ht="30" hidden="1">
+    <row r="396" spans="1:23" ht="30">
       <c r="A396" s="4" t="s">
         <v>2110</v>
       </c>
@@ -40375,14 +40610,1002 @@
         <v>21</v>
       </c>
     </row>
+    <row r="397" spans="1:23" ht="45">
+      <c r="A397" s="3" t="s">
+        <v>2399</v>
+      </c>
+      <c r="B397" s="5">
+        <v>1</v>
+      </c>
+      <c r="C397" s="3" t="s">
+        <v>2405</v>
+      </c>
+      <c r="D397" s="3" t="s">
+        <v>2402</v>
+      </c>
+      <c r="E397" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="F397" s="5">
+        <v>36</v>
+      </c>
+      <c r="G397" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H397" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I397" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="J397" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="K397" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="L397" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="M397" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="N397" s="3" t="s">
+        <v>2406</v>
+      </c>
+      <c r="O397" s="3" t="s">
+        <v>2407</v>
+      </c>
+      <c r="P397" s="3" t="s">
+        <v>2408</v>
+      </c>
+      <c r="Q397" s="3" t="s">
+        <v>2409</v>
+      </c>
+      <c r="R397" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="S397" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="T397" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="U397" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="V397" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="W397" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="398" spans="1:23" ht="30">
+      <c r="A398" s="3" t="s">
+        <v>2399</v>
+      </c>
+      <c r="B398" s="5">
+        <v>2</v>
+      </c>
+      <c r="C398" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D398" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E398" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="F398" s="5">
+        <v>36</v>
+      </c>
+      <c r="G398" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H398" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I398" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J398" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="K398" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="L398" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="M398" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="N398" s="3" t="s">
+        <v>2410</v>
+      </c>
+      <c r="O398" s="3" t="s">
+        <v>2411</v>
+      </c>
+      <c r="P398" s="3" t="s">
+        <v>2412</v>
+      </c>
+      <c r="Q398" s="3" t="s">
+        <v>2413</v>
+      </c>
+      <c r="R398" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="S398" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="T398" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="U398" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="V398" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="W398" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="399" spans="1:23" ht="45">
+      <c r="A399" s="3" t="s">
+        <v>2399</v>
+      </c>
+      <c r="B399" s="5">
+        <v>3</v>
+      </c>
+      <c r="C399" s="3" t="s">
+        <v>1928</v>
+      </c>
+      <c r="D399" s="3" t="s">
+        <v>1918</v>
+      </c>
+      <c r="E399" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="F399" s="5">
+        <v>36</v>
+      </c>
+      <c r="G399" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H399" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I399" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J399" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="K399" s="3" t="s">
+        <v>1914</v>
+      </c>
+      <c r="L399" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="M399" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="N399" s="3" t="s">
+        <v>2414</v>
+      </c>
+      <c r="O399" s="3" t="s">
+        <v>2415</v>
+      </c>
+      <c r="P399" s="3" t="s">
+        <v>2416</v>
+      </c>
+      <c r="Q399" s="3" t="s">
+        <v>2417</v>
+      </c>
+      <c r="R399" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="S399" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="T399" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="U399" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="V399" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="W399" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="400" spans="1:23" ht="30">
+      <c r="A400" s="3" t="s">
+        <v>2399</v>
+      </c>
+      <c r="B400" s="5">
+        <v>4</v>
+      </c>
+      <c r="C400" s="3" t="s">
+        <v>2403</v>
+      </c>
+      <c r="D400" s="3" t="s">
+        <v>2418</v>
+      </c>
+      <c r="E400" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="F400" s="5">
+        <v>150</v>
+      </c>
+      <c r="G400" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H400" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I400" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J400" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="K400" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="L400" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="M400" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="N400" s="3" t="s">
+        <v>2419</v>
+      </c>
+      <c r="O400" s="3" t="s">
+        <v>2420</v>
+      </c>
+      <c r="P400" s="3" t="s">
+        <v>2421</v>
+      </c>
+      <c r="Q400" s="3" t="s">
+        <v>2422</v>
+      </c>
+      <c r="R400" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="S400" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="T400" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="U400" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="V400" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="W400" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="401" spans="1:23" ht="45">
+      <c r="A401" s="3" t="s">
+        <v>2399</v>
+      </c>
+      <c r="B401" s="5">
+        <v>5</v>
+      </c>
+      <c r="C401" s="3" t="s">
+        <v>2423</v>
+      </c>
+      <c r="D401" s="3" t="s">
+        <v>2424</v>
+      </c>
+      <c r="E401" s="3" t="s">
+        <v>1955</v>
+      </c>
+      <c r="F401" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="G401" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H401" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I401" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J401" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="K401" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="L401" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="M401" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="N401" s="3" t="s">
+        <v>2425</v>
+      </c>
+      <c r="O401" s="3" t="s">
+        <v>2426</v>
+      </c>
+      <c r="P401" s="3" t="s">
+        <v>2461</v>
+      </c>
+      <c r="Q401" s="3" t="s">
+        <v>2427</v>
+      </c>
+      <c r="R401" s="3" t="s">
+        <v>2428</v>
+      </c>
+      <c r="S401" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="T401" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="U401" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="V401" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="W401" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="402" spans="1:23" ht="45">
+      <c r="A402" s="3" t="s">
+        <v>2399</v>
+      </c>
+      <c r="B402" s="5">
+        <v>6</v>
+      </c>
+      <c r="C402" s="3" t="s">
+        <v>2429</v>
+      </c>
+      <c r="D402" s="3" t="s">
+        <v>2430</v>
+      </c>
+      <c r="E402" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="F402" s="5">
+        <v>36</v>
+      </c>
+      <c r="G402" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H402" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I402" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J402" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="K402" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="L402" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="M402" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="N402" s="3" t="s">
+        <v>2431</v>
+      </c>
+      <c r="O402" s="3" t="s">
+        <v>2432</v>
+      </c>
+      <c r="P402" s="3" t="s">
+        <v>2433</v>
+      </c>
+      <c r="Q402" s="3" t="s">
+        <v>2434</v>
+      </c>
+      <c r="R402" s="3" t="s">
+        <v>2462</v>
+      </c>
+      <c r="S402" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="T402" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="U402" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="V402" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="W402" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="403" spans="1:23" ht="45">
+      <c r="A403" s="3" t="s">
+        <v>2399</v>
+      </c>
+      <c r="B403" s="5">
+        <v>7</v>
+      </c>
+      <c r="C403" s="3" t="s">
+        <v>2435</v>
+      </c>
+      <c r="D403" s="3" t="s">
+        <v>2436</v>
+      </c>
+      <c r="E403" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="F403" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="G403" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H403" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I403" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J403" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="K403" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="L403" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="M403" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="N403" s="3" t="s">
+        <v>2437</v>
+      </c>
+      <c r="O403" s="3" t="s">
+        <v>2438</v>
+      </c>
+      <c r="P403" s="3" t="s">
+        <v>2439</v>
+      </c>
+      <c r="Q403" s="3" t="s">
+        <v>2440</v>
+      </c>
+      <c r="R403" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="S403" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="T403" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="U403" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="V403" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="W403" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="404" spans="1:23" ht="30">
+      <c r="A404" s="3" t="s">
+        <v>2399</v>
+      </c>
+      <c r="B404" s="5">
+        <v>8</v>
+      </c>
+      <c r="C404" s="3" t="s">
+        <v>2441</v>
+      </c>
+      <c r="D404" s="3" t="s">
+        <v>2442</v>
+      </c>
+      <c r="E404" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="F404" s="5">
+        <v>36</v>
+      </c>
+      <c r="G404" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H404" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I404" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J404" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="K404" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="L404" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="M404" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="N404" s="3" t="s">
+        <v>2443</v>
+      </c>
+      <c r="O404" s="3" t="s">
+        <v>2444</v>
+      </c>
+      <c r="P404" s="3" t="s">
+        <v>2445</v>
+      </c>
+      <c r="Q404" s="3" t="s">
+        <v>2446</v>
+      </c>
+      <c r="R404" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="S404" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="T404" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="U404" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="V404" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="W404" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="405" spans="1:23" ht="30">
+      <c r="A405" s="3" t="s">
+        <v>2399</v>
+      </c>
+      <c r="B405" s="5">
+        <v>9</v>
+      </c>
+      <c r="C405" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="D405" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="E405" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="F405" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="G405" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H405" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I405" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J405" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="K405" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="L405" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="M405" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="N405" s="3" t="s">
+        <v>1971</v>
+      </c>
+      <c r="O405" s="3" t="s">
+        <v>2447</v>
+      </c>
+      <c r="P405" s="3" t="s">
+        <v>2448</v>
+      </c>
+      <c r="Q405" s="3" t="s">
+        <v>2449</v>
+      </c>
+      <c r="R405" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="S405" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="T405" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="U405" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="V405" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="W405" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="406" spans="1:23" ht="30">
+      <c r="A406" s="3" t="s">
+        <v>2399</v>
+      </c>
+      <c r="B406" s="5">
+        <v>10</v>
+      </c>
+      <c r="C406" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="D406" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="E406" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="F406" s="5">
+        <v>36</v>
+      </c>
+      <c r="G406" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H406" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I406" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J406" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="K406" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="L406" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="M406" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="N406" s="3" t="s">
+        <v>1974</v>
+      </c>
+      <c r="O406" s="3" t="s">
+        <v>2450</v>
+      </c>
+      <c r="P406" s="3" t="s">
+        <v>2451</v>
+      </c>
+      <c r="Q406" s="3" t="s">
+        <v>2446</v>
+      </c>
+      <c r="R406" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="S406" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="T406" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="U406" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="V406" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="W406" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="407" spans="1:23" ht="30">
+      <c r="A407" s="3" t="s">
+        <v>2399</v>
+      </c>
+      <c r="B407" s="5">
+        <v>11</v>
+      </c>
+      <c r="C407" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="D407" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="E407" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="F407" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="G407" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H407" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I407" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J407" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="K407" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="L407" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="M407" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="N407" s="3" t="s">
+        <v>1977</v>
+      </c>
+      <c r="O407" s="3" t="s">
+        <v>2452</v>
+      </c>
+      <c r="P407" s="3" t="s">
+        <v>2453</v>
+      </c>
+      <c r="Q407" s="3" t="s">
+        <v>2454</v>
+      </c>
+      <c r="R407" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="S407" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="T407" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="U407" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="V407" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="W407" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="408" spans="1:23" ht="30">
+      <c r="A408" s="3" t="s">
+        <v>2399</v>
+      </c>
+      <c r="B408" s="5">
+        <v>12</v>
+      </c>
+      <c r="C408" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="D408" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="E408" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="F408" s="5">
+        <v>36</v>
+      </c>
+      <c r="G408" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H408" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I408" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J408" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="K408" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="L408" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="M408" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="N408" s="3" t="s">
+        <v>1979</v>
+      </c>
+      <c r="O408" s="3" t="s">
+        <v>2455</v>
+      </c>
+      <c r="P408" s="3" t="s">
+        <v>2456</v>
+      </c>
+      <c r="Q408" s="3" t="s">
+        <v>2446</v>
+      </c>
+      <c r="R408" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="S408" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="T408" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="U408" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="V408" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="W408" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="409" spans="1:23" ht="30">
+      <c r="A409" s="3" t="s">
+        <v>2399</v>
+      </c>
+      <c r="B409" s="5">
+        <v>13</v>
+      </c>
+      <c r="C409" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="D409" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="E409" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="F409" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="G409" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H409" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I409" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J409" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="K409" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="L409" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="M409" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="N409" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="O409" s="3" t="s">
+        <v>2457</v>
+      </c>
+      <c r="P409" s="3" t="s">
+        <v>2458</v>
+      </c>
+      <c r="Q409" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="R409" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="S409" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="T409" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="U409" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="V409" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="W409" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="410" spans="1:23" ht="30">
+      <c r="A410" s="3" t="s">
+        <v>2399</v>
+      </c>
+      <c r="B410" s="5">
+        <v>14</v>
+      </c>
+      <c r="C410" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="D410" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="E410" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="F410" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="G410" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H410" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I410" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="J410" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="K410" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="L410" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="M410" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="N410" s="3" t="s">
+        <v>1985</v>
+      </c>
+      <c r="O410" s="3" t="s">
+        <v>2459</v>
+      </c>
+      <c r="P410" s="3" t="s">
+        <v>2460</v>
+      </c>
+      <c r="Q410" s="3">
+        <v>1</v>
+      </c>
+      <c r="R410" s="3">
+        <v>1</v>
+      </c>
+      <c r="S410" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="T410" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="U410" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="V410" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="W410" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:W396" xr:uid="{7E21F442-9136-4C15-8BA3-92E07332B93A}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="Template"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:W396" xr:uid="{7E21F442-9136-4C15-8BA3-92E07332B93A}"/>
   <hyperlinks>
     <hyperlink ref="Q9" r:id="rId1" display="mailto:admin@memgine.com" xr:uid="{93170BB8-77D4-4002-829B-D89928109808}"/>
     <hyperlink ref="Q11" r:id="rId2" display="https://memgine.com/" xr:uid="{F8EB4105-6CCB-4B06-B657-948DB365F556}"/>

</xml_diff>

<commit_message>
Platform-admin create new org with basic foundation built including logging, error handling, and draft
</commit_message>
<xml_diff>
--- a/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
+++ b/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MynikaTech\memgine\docs\domain\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4F57A97-FD42-4D5F-B918-433EC83B7732}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{331967AC-A866-4C7C-8443-77689366D5DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{AA28BC4D-8219-43B9-8C16-6977709D904A}"/>
   </bookViews>
@@ -9376,7 +9376,7 @@
         <v>1539</v>
       </c>
     </row>
-    <row r="27" spans="1:17" ht="45">
+    <row r="27" spans="1:17" ht="30">
       <c r="A27" s="4" t="s">
         <v>1576</v>
       </c>

</xml_diff>

<commit_message>
add product to domain model
</commit_message>
<xml_diff>
--- a/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
+++ b/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MynikaTech\memgine\docs\domain\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D40B066-C1C8-41D3-8BB0-AC1B2BFCB954}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC82217B-53E9-40B5-B787-178C7AA3B44B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{AA28BC4D-8219-43B9-8C16-6977709D904A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="5" activeTab="11" xr2:uid="{AA28BC4D-8219-43B9-8C16-6977709D904A}"/>
   </bookViews>
   <sheets>
     <sheet name="Entity Catalogue" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11467" uniqueCount="2552">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11807" uniqueCount="2624">
   <si>
     <t>Domain</t>
   </si>
@@ -7510,18 +7510,6 @@
     <t>product</t>
   </si>
   <si>
-    <t>Identify the product or service associated with the benefit.</t>
-  </si>
-  <si>
-    <t>Product or service that the benefit provides, discounts or otherwise relates to.</t>
-  </si>
-  <si>
-    <t>Represents the business product or service associated with the benefit.</t>
-  </si>
-  <si>
-    <t>Cappuccino</t>
-  </si>
-  <si>
     <t>Retail Price</t>
   </si>
   <si>
@@ -7697,6 +7685,234 @@
   </si>
   <si>
     <t>Unable to calculate upgraded subscription period.</t>
+  </si>
+  <si>
+    <t>PRODUCT</t>
+  </si>
+  <si>
+    <t>Commerce</t>
+  </si>
+  <si>
+    <t>Product Management</t>
+  </si>
+  <si>
+    <t>Represents an organization-owned catalogue item or service that can be associated with Memgine Benefits.</t>
+  </si>
+  <si>
+    <t>product_id</t>
+  </si>
+  <si>
+    <t>Lightweight product catalogue used by Memgine for benefit association. Product does not represent inventory or stock management. Products may be maintained manually or populated from an external POS, menu, inventory or other business system in the future.</t>
+  </si>
+  <si>
+    <t>Product ID</t>
+  </si>
+  <si>
+    <t>Uniquely identify a Product.</t>
+  </si>
+  <si>
+    <t>System-generated identifier for the Product.</t>
+  </si>
+  <si>
+    <t>Primary identifier for an organization-owned Product record.</t>
+  </si>
+  <si>
+    <t>PROD-1001</t>
+  </si>
+  <si>
+    <t>Identify the Organization that owns the Product.</t>
+  </si>
+  <si>
+    <t>References the Organization that owns and manages the Product.</t>
+  </si>
+  <si>
+    <t>Establishes tenant ownership and isolation of the Product.</t>
+  </si>
+  <si>
+    <t>Product Code</t>
+  </si>
+  <si>
+    <t>product_code</t>
+  </si>
+  <si>
+    <t>Provide a unique business identifier for the Product.</t>
+  </si>
+  <si>
+    <t>Business-defined code used to identify the Product.</t>
+  </si>
+  <si>
+    <t>Represents the organization's internal or external product/SKU code.</t>
+  </si>
+  <si>
+    <t>FC001</t>
+  </si>
+  <si>
+    <t>product_name</t>
+  </si>
+  <si>
+    <t>Identify the Product for business and customer-facing use.</t>
+  </si>
+  <si>
+    <t>Human-readable name of the Product or service.</t>
+  </si>
+  <si>
+    <t>Primary display name of the Product.</t>
+  </si>
+  <si>
+    <t>Filter Coffee</t>
+  </si>
+  <si>
+    <t>Describe the Product or service.</t>
+  </si>
+  <si>
+    <t>Additional business description of the Product.</t>
+  </si>
+  <si>
+    <t>Provides optional contextual information about the Product.</t>
+  </si>
+  <si>
+    <t>Hot brewed filter coffee</t>
+  </si>
+  <si>
+    <t>Control whether the Product is available for association with Benefits.</t>
+  </si>
+  <si>
+    <t>References the lifecycle status of the Product.</t>
+  </si>
+  <si>
+    <t>Determines whether the Product is active and available for business use.</t>
+  </si>
+  <si>
+    <t>Record Product creation time.</t>
+  </si>
+  <si>
+    <t>System-generated creation timestamp.</t>
+  </si>
+  <si>
+    <t>Audit timestamp recording when the Product was created.</t>
+  </si>
+  <si>
+    <t>2026-08-31T10:00:00</t>
+  </si>
+  <si>
+    <t>Identify who created the Product.</t>
+  </si>
+  <si>
+    <t>References the User who created the Product.</t>
+  </si>
+  <si>
+    <t>Audit reference identifying the creator of the Product.</t>
+  </si>
+  <si>
+    <t>Record the last Product modification time.</t>
+  </si>
+  <si>
+    <t>System-generated update timestamp.</t>
+  </si>
+  <si>
+    <t>Audit timestamp recording the latest Product modification.</t>
+  </si>
+  <si>
+    <t>Identify who last modified the Product.</t>
+  </si>
+  <si>
+    <t>References the User who last modified the Product.</t>
+  </si>
+  <si>
+    <t>Audit reference identifying the latest modifier.</t>
+  </si>
+  <si>
+    <t>Support logical deletion of Products.</t>
+  </si>
+  <si>
+    <t>Indicates whether the Product has been logically deleted.</t>
+  </si>
+  <si>
+    <t>Soft-delete flag; deleted Products are not available for new Benefit associations.</t>
+  </si>
+  <si>
+    <t>Support optimistic concurrency for Product updates.</t>
+  </si>
+  <si>
+    <t>System-managed version number.</t>
+  </si>
+  <si>
+    <t>Used to detect conflicting updates to the same Product.</t>
+  </si>
+  <si>
+    <t>Associate the Benefit with an organization Product.</t>
+  </si>
+  <si>
+    <t>References the Product or service associated with the Benefit.</t>
+  </si>
+  <si>
+    <t>Identifies the Product to which the Benefit applies.</t>
+  </si>
+  <si>
+    <t>Organization owns Product</t>
+  </si>
+  <si>
+    <t>Each Product belongs to exactly one Organization.</t>
+  </si>
+  <si>
+    <t>Product associated with Benefit</t>
+  </si>
+  <si>
+    <t>A Product may be associated with zero or more Benefits, while a Benefit may optionally reference one Product.</t>
+  </si>
+  <si>
+    <t>REL063</t>
+  </si>
+  <si>
+    <t>REL064</t>
+  </si>
+  <si>
+    <t>Must be unique within the Organization.</t>
+  </si>
+  <si>
+    <t>Duplicate Product Code within the Organization.</t>
+  </si>
+  <si>
+    <t>Product Code may correspond to an organization's internal SKU or an external product code.</t>
+  </si>
+  <si>
+    <t>VAL049</t>
+  </si>
+  <si>
+    <t>Organization must exist.</t>
+  </si>
+  <si>
+    <t>VAL050</t>
+  </si>
+  <si>
+    <t>Status must exist in Status reference data.</t>
+  </si>
+  <si>
+    <t>Invalid Product Status.</t>
+  </si>
+  <si>
+    <t>VAL051</t>
+  </si>
+  <si>
+    <t>If Product is specified, it must exist.</t>
+  </si>
+  <si>
+    <t>Invalid Product.</t>
+  </si>
+  <si>
+    <t>VAL052</t>
+  </si>
+  <si>
+    <t>If Product is specified, it must belong to the same Organization as the Benefit.</t>
+  </si>
+  <si>
+    <t>Product must belong to the Benefit's Organization.</t>
+  </si>
+  <si>
+    <t>VAL053</t>
+  </si>
+  <si>
+    <t>VAL054</t>
   </si>
 </sst>
 </file>
@@ -7925,7 +8141,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3841114F-D1EC-49B1-850B-590431E39412}" name="Table2" displayName="Table2" ref="A1:Q38" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3841114F-D1EC-49B1-850B-590431E39412}" name="Table2" displayName="Table2" ref="A1:Q39" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{FEF6275C-74E6-4563-BFF3-6461E4A3D8DA}" name="Entity Code" dataDxfId="16"/>
     <tableColumn id="2" xr3:uid="{67FE23FD-539D-4023-BA73-D2A0B84718BF}" name="Domain" dataDxfId="15"/>
@@ -8246,7 +8462,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4659496D-1A4F-4BC3-BD65-377E70E6B8BE}">
-  <dimension ref="A1:Q38"/>
+  <dimension ref="A1:Q39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="31.85546875" style="4" customWidth="1"/>
@@ -10272,6 +10488,59 @@
       </c>
       <c r="Q38" s="4" t="s">
         <v>2404</v>
+      </c>
+    </row>
+    <row r="39" spans="1:17" ht="105">
+      <c r="A39" s="4" t="s">
+        <v>2548</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>2549</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>2550</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>2476</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>2488</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>2551</v>
+      </c>
+      <c r="G39" s="4" t="s">
+        <v>2476</v>
+      </c>
+      <c r="H39" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="I39" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="J39" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K39" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="L39" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="M39" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="N39" s="4" t="s">
+        <v>2552</v>
+      </c>
+      <c r="O39" s="4" t="s">
+        <v>1398</v>
+      </c>
+      <c r="P39" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q39" s="4" t="s">
+        <v>2553</v>
       </c>
     </row>
   </sheetData>
@@ -11967,7 +12236,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C85B9BC7-C8C8-4E3E-A0EF-02B9554CEAE5}">
-  <dimension ref="A1:K63"/>
+  <dimension ref="A1:K65"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.5703125" style="4" bestFit="1" customWidth="1"/>
@@ -14189,6 +14458,76 @@
         <v>2185</v>
       </c>
     </row>
+    <row r="64" spans="1:11">
+      <c r="A64" s="4" t="s">
+        <v>2606</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>2476</v>
+      </c>
+      <c r="D64" s="4" t="s">
+        <v>2602</v>
+      </c>
+      <c r="E64" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F64" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="G64" s="4" t="s">
+        <v>1301</v>
+      </c>
+      <c r="H64" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I64" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="J64" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K64" s="4" t="s">
+        <v>2603</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" ht="30">
+      <c r="A65" s="4" t="s">
+        <v>2607</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>2476</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>490</v>
+      </c>
+      <c r="D65" s="4" t="s">
+        <v>2604</v>
+      </c>
+      <c r="E65" s="4" t="s">
+        <v>2552</v>
+      </c>
+      <c r="F65" s="4" t="s">
+        <v>2552</v>
+      </c>
+      <c r="G65" s="4" t="s">
+        <v>1301</v>
+      </c>
+      <c r="H65" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I65" s="4" t="s">
+        <v>1310</v>
+      </c>
+      <c r="J65" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K65" s="4" t="s">
+        <v>2605</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K63" xr:uid="{C85B9BC7-C8C8-4E3E-A0EF-02B9554CEAE5}"/>
   <phoneticPr fontId="4" type="noConversion"/>
@@ -14199,7 +14538,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6E5E88D-7637-4195-842B-FF426225AADB}">
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
@@ -15149,22 +15488,22 @@
     </row>
     <row r="37" spans="1:9">
       <c r="A37" s="3" t="s">
-        <v>2503</v>
+        <v>2499</v>
       </c>
       <c r="B37" t="s">
         <v>10</v>
       </c>
       <c r="C37" t="s">
-        <v>2504</v>
+        <v>2500</v>
       </c>
       <c r="D37" t="s">
         <v>2188</v>
       </c>
       <c r="E37" t="s">
-        <v>2505</v>
+        <v>2501</v>
       </c>
       <c r="F37" t="s">
-        <v>2506</v>
+        <v>2502</v>
       </c>
       <c r="G37" t="s">
         <v>1392</v>
@@ -15173,27 +15512,27 @@
         <v>1393</v>
       </c>
       <c r="I37" t="s">
-        <v>2507</v>
+        <v>2503</v>
       </c>
     </row>
     <row r="38" spans="1:9">
       <c r="A38" s="3" t="s">
-        <v>2508</v>
+        <v>2504</v>
       </c>
       <c r="B38" t="s">
         <v>10</v>
       </c>
       <c r="C38" t="s">
-        <v>2509</v>
+        <v>2505</v>
       </c>
       <c r="D38" t="s">
         <v>1405</v>
       </c>
       <c r="E38" t="s">
-        <v>2510</v>
+        <v>2506</v>
       </c>
       <c r="F38" t="s">
-        <v>2511</v>
+        <v>2507</v>
       </c>
       <c r="G38" t="s">
         <v>1392</v>
@@ -15202,27 +15541,27 @@
         <v>1393</v>
       </c>
       <c r="I38" t="s">
-        <v>2512</v>
+        <v>2508</v>
       </c>
     </row>
     <row r="39" spans="1:9">
       <c r="A39" s="3" t="s">
-        <v>2513</v>
+        <v>2509</v>
       </c>
       <c r="B39" t="s">
         <v>10</v>
       </c>
       <c r="C39" t="s">
-        <v>2509</v>
+        <v>2505</v>
       </c>
       <c r="D39" t="s">
         <v>61</v>
       </c>
       <c r="E39" t="s">
-        <v>2514</v>
+        <v>2510</v>
       </c>
       <c r="F39" t="s">
-        <v>2515</v>
+        <v>2511</v>
       </c>
       <c r="G39" t="s">
         <v>1392</v>
@@ -15231,27 +15570,27 @@
         <v>1393</v>
       </c>
       <c r="I39" t="s">
-        <v>2516</v>
+        <v>2512</v>
       </c>
     </row>
     <row r="40" spans="1:9">
       <c r="A40" s="3" t="s">
-        <v>2517</v>
+        <v>2513</v>
       </c>
       <c r="B40" t="s">
         <v>10</v>
       </c>
       <c r="C40" t="s">
-        <v>2518</v>
+        <v>2514</v>
       </c>
       <c r="D40" t="s">
         <v>2188</v>
       </c>
       <c r="E40" t="s">
-        <v>2519</v>
+        <v>2515</v>
       </c>
       <c r="F40" t="s">
-        <v>2520</v>
+        <v>2516</v>
       </c>
       <c r="G40" t="s">
         <v>1392</v>
@@ -15260,27 +15599,27 @@
         <v>1393</v>
       </c>
       <c r="I40" t="s">
-        <v>2521</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="41" spans="1:9">
       <c r="A41" s="3" t="s">
-        <v>2522</v>
+        <v>2518</v>
       </c>
       <c r="B41" t="s">
         <v>490</v>
       </c>
       <c r="C41" t="s">
-        <v>2493</v>
+        <v>2489</v>
       </c>
       <c r="D41" t="s">
         <v>1405</v>
       </c>
       <c r="E41" t="s">
-        <v>2523</v>
+        <v>2519</v>
       </c>
       <c r="F41" t="s">
-        <v>2524</v>
+        <v>2520</v>
       </c>
       <c r="G41" t="s">
         <v>1392</v>
@@ -15291,22 +15630,22 @@
     </row>
     <row r="42" spans="1:9">
       <c r="A42" s="3" t="s">
-        <v>2525</v>
+        <v>2521</v>
       </c>
       <c r="B42" t="s">
         <v>490</v>
       </c>
       <c r="C42" t="s">
-        <v>2498</v>
+        <v>2494</v>
       </c>
       <c r="D42" t="s">
         <v>1405</v>
       </c>
       <c r="E42" t="s">
-        <v>2526</v>
+        <v>2522</v>
       </c>
       <c r="F42" t="s">
-        <v>2527</v>
+        <v>2523</v>
       </c>
       <c r="G42" t="s">
         <v>1392</v>
@@ -15317,140 +15656,140 @@
     </row>
     <row r="43" spans="1:9">
       <c r="A43" s="3" t="s">
-        <v>2528</v>
+        <v>2524</v>
       </c>
       <c r="B43" t="s">
-        <v>2534</v>
+        <v>2530</v>
       </c>
       <c r="C43" t="s">
-        <v>2535</v>
+        <v>2531</v>
       </c>
       <c r="D43" t="s">
         <v>2188</v>
       </c>
       <c r="E43" t="s">
-        <v>2536</v>
+        <v>2532</v>
       </c>
       <c r="F43" t="s">
-        <v>2537</v>
+        <v>2533</v>
       </c>
       <c r="G43" t="s">
         <v>1392</v>
       </c>
       <c r="H43" t="s">
-        <v>2538</v>
+        <v>2534</v>
       </c>
     </row>
     <row r="44" spans="1:9">
       <c r="A44" s="3" t="s">
-        <v>2529</v>
+        <v>2525</v>
       </c>
       <c r="B44" t="s">
-        <v>2534</v>
+        <v>2530</v>
       </c>
       <c r="C44" t="s">
-        <v>2509</v>
+        <v>2505</v>
       </c>
       <c r="D44" t="s">
         <v>2188</v>
       </c>
       <c r="E44" t="s">
-        <v>2539</v>
+        <v>2535</v>
       </c>
       <c r="F44" t="s">
-        <v>2540</v>
+        <v>2536</v>
       </c>
       <c r="G44" t="s">
         <v>1392</v>
       </c>
       <c r="H44" t="s">
-        <v>2538</v>
+        <v>2534</v>
       </c>
     </row>
     <row r="45" spans="1:9">
       <c r="A45" s="3" t="s">
+        <v>2526</v>
+      </c>
+      <c r="B45" t="s">
         <v>2530</v>
       </c>
-      <c r="B45" t="s">
-        <v>2534</v>
-      </c>
       <c r="C45" t="s">
-        <v>2541</v>
+        <v>2537</v>
       </c>
       <c r="D45" t="s">
         <v>175</v>
       </c>
       <c r="E45" t="s">
-        <v>2542</v>
+        <v>2538</v>
       </c>
       <c r="F45" t="s">
-        <v>2543</v>
+        <v>2539</v>
       </c>
       <c r="G45" t="s">
         <v>1392</v>
       </c>
       <c r="H45" t="s">
-        <v>2538</v>
+        <v>2534</v>
       </c>
     </row>
     <row r="46" spans="1:9">
       <c r="A46" s="3" t="s">
-        <v>2531</v>
+        <v>2527</v>
       </c>
       <c r="B46" t="s">
-        <v>2534</v>
+        <v>2530</v>
       </c>
       <c r="C46" t="s">
-        <v>2544</v>
+        <v>2540</v>
       </c>
       <c r="D46" t="s">
         <v>175</v>
       </c>
       <c r="E46" t="s">
-        <v>2545</v>
+        <v>2541</v>
       </c>
       <c r="F46" t="s">
-        <v>2546</v>
+        <v>2542</v>
       </c>
       <c r="G46" t="s">
         <v>1392</v>
       </c>
       <c r="H46" t="s">
-        <v>2538</v>
+        <v>2534</v>
       </c>
     </row>
     <row r="47" spans="1:9">
       <c r="A47" s="3" t="s">
-        <v>2532</v>
+        <v>2528</v>
       </c>
       <c r="B47" t="s">
-        <v>2534</v>
+        <v>2530</v>
       </c>
       <c r="C47" t="s">
-        <v>2547</v>
+        <v>2543</v>
       </c>
       <c r="D47" t="s">
         <v>2188</v>
       </c>
       <c r="E47" t="s">
-        <v>2548</v>
+        <v>2544</v>
       </c>
       <c r="F47" t="s">
-        <v>2549</v>
+        <v>2545</v>
       </c>
       <c r="G47" t="s">
         <v>1392</v>
       </c>
       <c r="H47" t="s">
-        <v>2538</v>
+        <v>2534</v>
       </c>
     </row>
     <row r="48" spans="1:9">
       <c r="A48" s="3" t="s">
-        <v>2533</v>
+        <v>2529</v>
       </c>
       <c r="B48" t="s">
-        <v>2534</v>
+        <v>2530</v>
       </c>
       <c r="C48" t="s">
         <v>576</v>
@@ -15459,16 +15798,175 @@
         <v>2188</v>
       </c>
       <c r="E48" t="s">
-        <v>2550</v>
+        <v>2546</v>
       </c>
       <c r="F48" t="s">
-        <v>2551</v>
+        <v>2547</v>
       </c>
       <c r="G48" t="s">
         <v>1392</v>
       </c>
       <c r="H48" t="s">
-        <v>2538</v>
+        <v>2534</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9">
+      <c r="A49" s="3" t="s">
+        <v>2611</v>
+      </c>
+      <c r="B49" t="s">
+        <v>2476</v>
+      </c>
+      <c r="C49" t="s">
+        <v>2562</v>
+      </c>
+      <c r="D49" t="s">
+        <v>61</v>
+      </c>
+      <c r="E49" t="s">
+        <v>2608</v>
+      </c>
+      <c r="F49" t="s">
+        <v>2609</v>
+      </c>
+      <c r="G49" t="s">
+        <v>1392</v>
+      </c>
+      <c r="H49" t="s">
+        <v>1393</v>
+      </c>
+      <c r="I49" t="s">
+        <v>2610</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9">
+      <c r="A50" s="3" t="s">
+        <v>2613</v>
+      </c>
+      <c r="B50" t="s">
+        <v>2476</v>
+      </c>
+      <c r="C50" t="s">
+        <v>1398</v>
+      </c>
+      <c r="D50" t="s">
+        <v>32</v>
+      </c>
+      <c r="E50" t="s">
+        <v>1390</v>
+      </c>
+      <c r="F50" t="s">
+        <v>1399</v>
+      </c>
+      <c r="G50" t="s">
+        <v>1392</v>
+      </c>
+      <c r="H50" t="s">
+        <v>1393</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9">
+      <c r="A51" s="3" t="s">
+        <v>2616</v>
+      </c>
+      <c r="B51" t="s">
+        <v>2476</v>
+      </c>
+      <c r="C51" t="s">
+        <v>5</v>
+      </c>
+      <c r="D51" t="s">
+        <v>175</v>
+      </c>
+      <c r="E51" t="s">
+        <v>2612</v>
+      </c>
+      <c r="F51" t="s">
+        <v>1415</v>
+      </c>
+      <c r="G51" t="s">
+        <v>1392</v>
+      </c>
+      <c r="H51" t="s">
+        <v>939</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9">
+      <c r="A52" s="3" t="s">
+        <v>2619</v>
+      </c>
+      <c r="B52" t="s">
+        <v>2476</v>
+      </c>
+      <c r="C52" t="s">
+        <v>42</v>
+      </c>
+      <c r="D52" t="s">
+        <v>175</v>
+      </c>
+      <c r="E52" t="s">
+        <v>2614</v>
+      </c>
+      <c r="F52" t="s">
+        <v>2615</v>
+      </c>
+      <c r="G52" t="s">
+        <v>1392</v>
+      </c>
+      <c r="H52" t="s">
+        <v>1393</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9">
+      <c r="A53" s="3" t="s">
+        <v>2622</v>
+      </c>
+      <c r="B53" t="s">
+        <v>490</v>
+      </c>
+      <c r="C53" t="s">
+        <v>2476</v>
+      </c>
+      <c r="D53" t="s">
+        <v>175</v>
+      </c>
+      <c r="E53" t="s">
+        <v>2617</v>
+      </c>
+      <c r="F53" t="s">
+        <v>2618</v>
+      </c>
+      <c r="G53" t="s">
+        <v>1392</v>
+      </c>
+      <c r="H53" t="s">
+        <v>1393</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9">
+      <c r="A54" s="3" t="s">
+        <v>2623</v>
+      </c>
+      <c r="B54" t="s">
+        <v>490</v>
+      </c>
+      <c r="C54" t="s">
+        <v>2476</v>
+      </c>
+      <c r="D54" t="s">
+        <v>2188</v>
+      </c>
+      <c r="E54" t="s">
+        <v>2620</v>
+      </c>
+      <c r="F54" t="s">
+        <v>2621</v>
+      </c>
+      <c r="G54" t="s">
+        <v>1392</v>
+      </c>
+      <c r="H54" t="s">
+        <v>1393</v>
       </c>
     </row>
   </sheetData>
@@ -15480,7 +15978,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E21F442-9136-4C15-8BA3-92E07332B93A}">
-  <dimension ref="A1:W415"/>
+  <dimension ref="A1:W427"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.140625" style="4" customWidth="1"/>
@@ -22002,7 +22500,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="96" spans="1:23" ht="30">
+    <row r="96" spans="1:23">
       <c r="A96" s="4" t="s">
         <v>490</v>
       </c>
@@ -22013,13 +22511,13 @@
         <v>2476</v>
       </c>
       <c r="D96" s="3" t="s">
-        <v>2488</v>
+        <v>2552</v>
       </c>
       <c r="E96" s="3" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="F96" s="5">
-        <v>150</v>
+        <v>36</v>
       </c>
       <c r="G96" s="1" t="s">
         <v>6</v>
@@ -22031,10 +22529,10 @@
         <v>6</v>
       </c>
       <c r="J96" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K96" s="3" t="s">
-        <v>269</v>
+        <v>2476</v>
       </c>
       <c r="L96" s="1" t="s">
         <v>6</v>
@@ -22043,19 +22541,19 @@
         <v>6</v>
       </c>
       <c r="N96" s="3" t="s">
-        <v>2489</v>
+        <v>2599</v>
       </c>
       <c r="O96" s="3" t="s">
-        <v>2490</v>
+        <v>2600</v>
       </c>
       <c r="P96" s="3" t="s">
-        <v>2491</v>
+        <v>2601</v>
       </c>
       <c r="Q96" s="3" t="s">
-        <v>2492</v>
+        <v>2558</v>
       </c>
       <c r="R96" s="3" t="s">
-        <v>269</v>
+        <v>72</v>
       </c>
       <c r="S96" s="1" t="s">
         <v>7</v>
@@ -22070,7 +22568,7 @@
         <v>7</v>
       </c>
       <c r="W96" s="1" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
     </row>
     <row r="97" spans="1:23" ht="45">
@@ -22081,10 +22579,10 @@
         <v>10</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>2493</v>
+        <v>2489</v>
       </c>
       <c r="D97" s="3" t="s">
-        <v>2494</v>
+        <v>2490</v>
       </c>
       <c r="E97" s="3" t="s">
         <v>173</v>
@@ -22114,13 +22612,13 @@
         <v>6</v>
       </c>
       <c r="N97" s="3" t="s">
-        <v>2495</v>
+        <v>2491</v>
       </c>
       <c r="O97" s="3" t="s">
-        <v>2496</v>
+        <v>2492</v>
       </c>
       <c r="P97" s="3" t="s">
-        <v>2497</v>
+        <v>2493</v>
       </c>
       <c r="Q97" s="3">
         <v>5.5</v>
@@ -22152,10 +22650,10 @@
         <v>11</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>2498</v>
+        <v>2494</v>
       </c>
       <c r="D98" s="3" t="s">
-        <v>2499</v>
+        <v>2495</v>
       </c>
       <c r="E98" s="3" t="s">
         <v>173</v>
@@ -22185,13 +22683,13 @@
         <v>6</v>
       </c>
       <c r="N98" s="3" t="s">
-        <v>2500</v>
+        <v>2496</v>
       </c>
       <c r="O98" s="3" t="s">
-        <v>2501</v>
+        <v>2497</v>
       </c>
       <c r="P98" s="3" t="s">
-        <v>2502</v>
+        <v>2498</v>
       </c>
       <c r="Q98" s="3">
         <v>1.8</v>
@@ -44237,6 +44735,858 @@
       </c>
       <c r="W415" s="3" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="416" spans="1:23">
+      <c r="A416" s="4" t="s">
+        <v>2476</v>
+      </c>
+      <c r="B416" s="4">
+        <v>1</v>
+      </c>
+      <c r="C416" s="4" t="s">
+        <v>2554</v>
+      </c>
+      <c r="D416" s="4" t="s">
+        <v>2552</v>
+      </c>
+      <c r="E416" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F416" s="4">
+        <v>36</v>
+      </c>
+      <c r="G416" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H416" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I416" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="J416" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K416" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="L416" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="M416" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="N416" s="4" t="s">
+        <v>2555</v>
+      </c>
+      <c r="O416" s="4" t="s">
+        <v>2556</v>
+      </c>
+      <c r="P416" s="4" t="s">
+        <v>2557</v>
+      </c>
+      <c r="Q416" s="4" t="s">
+        <v>2558</v>
+      </c>
+      <c r="R416" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="S416" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T416" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="U416" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V416" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W416" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="417" spans="1:23">
+      <c r="A417" s="4" t="s">
+        <v>2476</v>
+      </c>
+      <c r="B417" s="4">
+        <v>2</v>
+      </c>
+      <c r="C417" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D417" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E417" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F417" s="4">
+        <v>36</v>
+      </c>
+      <c r="G417" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H417" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I417" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J417" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K417" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="L417" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M417" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N417" s="4" t="s">
+        <v>2559</v>
+      </c>
+      <c r="O417" s="4" t="s">
+        <v>2560</v>
+      </c>
+      <c r="P417" s="4" t="s">
+        <v>2561</v>
+      </c>
+      <c r="Q417" s="4" t="s">
+        <v>2125</v>
+      </c>
+      <c r="R417" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="S417" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T417" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U417" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="V417" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W417" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="418" spans="1:23">
+      <c r="A418" s="4" t="s">
+        <v>2476</v>
+      </c>
+      <c r="B418" s="4">
+        <v>3</v>
+      </c>
+      <c r="C418" s="4" t="s">
+        <v>2562</v>
+      </c>
+      <c r="D418" s="4" t="s">
+        <v>2563</v>
+      </c>
+      <c r="E418" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="F418" s="4">
+        <v>50</v>
+      </c>
+      <c r="G418" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H418" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I418" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J418" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K418" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="L418" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="M418" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N418" s="4" t="s">
+        <v>2564</v>
+      </c>
+      <c r="O418" s="4" t="s">
+        <v>2565</v>
+      </c>
+      <c r="P418" s="4" t="s">
+        <v>2566</v>
+      </c>
+      <c r="Q418" s="4" t="s">
+        <v>2567</v>
+      </c>
+      <c r="R418" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="S418" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T418" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U418" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V418" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="W418" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="419" spans="1:23">
+      <c r="A419" s="4" t="s">
+        <v>2476</v>
+      </c>
+      <c r="B419" s="4">
+        <v>4</v>
+      </c>
+      <c r="C419" s="4" t="s">
+        <v>1398</v>
+      </c>
+      <c r="D419" s="4" t="s">
+        <v>2568</v>
+      </c>
+      <c r="E419" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="F419" s="4">
+        <v>150</v>
+      </c>
+      <c r="G419" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H419" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I419" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J419" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K419" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="L419" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M419" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N419" s="4" t="s">
+        <v>2569</v>
+      </c>
+      <c r="O419" s="4" t="s">
+        <v>2570</v>
+      </c>
+      <c r="P419" s="4" t="s">
+        <v>2571</v>
+      </c>
+      <c r="Q419" s="4" t="s">
+        <v>2572</v>
+      </c>
+      <c r="R419" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="S419" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T419" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U419" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V419" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="W419" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="420" spans="1:23">
+      <c r="A420" s="4" t="s">
+        <v>2476</v>
+      </c>
+      <c r="B420" s="4">
+        <v>5</v>
+      </c>
+      <c r="C420" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D420" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="E420" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="F420" s="4">
+        <v>1000</v>
+      </c>
+      <c r="G420" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H420" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I420" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J420" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K420" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="L420" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M420" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N420" s="4" t="s">
+        <v>2573</v>
+      </c>
+      <c r="O420" s="4" t="s">
+        <v>2574</v>
+      </c>
+      <c r="P420" s="4" t="s">
+        <v>2575</v>
+      </c>
+      <c r="Q420" s="4" t="s">
+        <v>2576</v>
+      </c>
+      <c r="R420" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="S420" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T420" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="U420" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="V420" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="W420" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="421" spans="1:23">
+      <c r="A421" s="4" t="s">
+        <v>2476</v>
+      </c>
+      <c r="B421" s="4">
+        <v>6</v>
+      </c>
+      <c r="C421" s="4" t="s">
+        <v>461</v>
+      </c>
+      <c r="D421" s="4" t="s">
+        <v>1016</v>
+      </c>
+      <c r="E421" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F421" s="4">
+        <v>36</v>
+      </c>
+      <c r="G421" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H421" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I421" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J421" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K421" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="L421" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M421" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N421" s="4" t="s">
+        <v>2577</v>
+      </c>
+      <c r="O421" s="4" t="s">
+        <v>2578</v>
+      </c>
+      <c r="P421" s="4" t="s">
+        <v>2579</v>
+      </c>
+      <c r="Q421" s="4" t="s">
+        <v>868</v>
+      </c>
+      <c r="R421" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="S421" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T421" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U421" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V421" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="W421" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="422" spans="1:23">
+      <c r="A422" s="4" t="s">
+        <v>2476</v>
+      </c>
+      <c r="B422" s="4">
+        <v>7</v>
+      </c>
+      <c r="C422" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="D422" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="E422" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="F422" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="G422" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H422" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I422" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J422" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K422" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="L422" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M422" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="N422" s="4" t="s">
+        <v>2580</v>
+      </c>
+      <c r="O422" s="4" t="s">
+        <v>2581</v>
+      </c>
+      <c r="P422" s="4" t="s">
+        <v>2582</v>
+      </c>
+      <c r="Q422" s="4" t="s">
+        <v>2583</v>
+      </c>
+      <c r="R422" s="4" t="s">
+        <v>1570</v>
+      </c>
+      <c r="S422" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="T422" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="U422" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V422" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W422" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="423" spans="1:23">
+      <c r="A423" s="4" t="s">
+        <v>2476</v>
+      </c>
+      <c r="B423" s="4">
+        <v>8</v>
+      </c>
+      <c r="C423" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="D423" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="E423" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F423" s="4">
+        <v>36</v>
+      </c>
+      <c r="G423" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H423" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I423" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J423" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K423" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="L423" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M423" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="N423" s="4" t="s">
+        <v>2584</v>
+      </c>
+      <c r="O423" s="4" t="s">
+        <v>2585</v>
+      </c>
+      <c r="P423" s="4" t="s">
+        <v>2586</v>
+      </c>
+      <c r="Q423" s="4" t="s">
+        <v>2031</v>
+      </c>
+      <c r="R423" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="S423" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="T423" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U423" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="V423" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W423" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="424" spans="1:23">
+      <c r="A424" s="4" t="s">
+        <v>2476</v>
+      </c>
+      <c r="B424" s="4">
+        <v>9</v>
+      </c>
+      <c r="C424" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="D424" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="E424" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="F424" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="G424" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H424" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I424" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J424" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K424" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="L424" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M424" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="N424" s="4" t="s">
+        <v>2587</v>
+      </c>
+      <c r="O424" s="4" t="s">
+        <v>2588</v>
+      </c>
+      <c r="P424" s="4" t="s">
+        <v>2589</v>
+      </c>
+      <c r="Q424" s="4" t="s">
+        <v>2583</v>
+      </c>
+      <c r="R424" s="4" t="s">
+        <v>1570</v>
+      </c>
+      <c r="S424" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="T424" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="U424" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V424" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W424" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="425" spans="1:23">
+      <c r="A425" s="4" t="s">
+        <v>2476</v>
+      </c>
+      <c r="B425" s="4">
+        <v>10</v>
+      </c>
+      <c r="C425" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="D425" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="E425" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F425" s="4">
+        <v>36</v>
+      </c>
+      <c r="G425" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H425" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I425" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J425" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K425" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="L425" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M425" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="N425" s="4" t="s">
+        <v>2590</v>
+      </c>
+      <c r="O425" s="4" t="s">
+        <v>2591</v>
+      </c>
+      <c r="P425" s="4" t="s">
+        <v>2592</v>
+      </c>
+      <c r="Q425" s="4" t="s">
+        <v>2031</v>
+      </c>
+      <c r="R425" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="S425" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="T425" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U425" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="V425" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W425" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="426" spans="1:23">
+      <c r="A426" s="4" t="s">
+        <v>2476</v>
+      </c>
+      <c r="B426" s="4">
+        <v>11</v>
+      </c>
+      <c r="C426" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="D426" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="E426" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="F426" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="G426" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H426" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I426" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J426" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K426" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="L426" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M426" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="N426" s="4" t="s">
+        <v>2593</v>
+      </c>
+      <c r="O426" s="4" t="s">
+        <v>2594</v>
+      </c>
+      <c r="P426" s="4" t="s">
+        <v>2595</v>
+      </c>
+      <c r="Q426" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="R426" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="S426" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="T426" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U426" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="V426" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W426" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="427" spans="1:23">
+      <c r="A427" s="4" t="s">
+        <v>2476</v>
+      </c>
+      <c r="B427" s="4">
+        <v>12</v>
+      </c>
+      <c r="C427" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="D427" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="E427" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="F427" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="G427" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H427" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I427" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J427" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K427" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="L427" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M427" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="N427" s="4" t="s">
+        <v>2596</v>
+      </c>
+      <c r="O427" s="4" t="s">
+        <v>2597</v>
+      </c>
+      <c r="P427" s="4" t="s">
+        <v>2598</v>
+      </c>
+      <c r="Q427" s="4">
+        <v>1</v>
+      </c>
+      <c r="R427" s="4">
+        <v>1</v>
+      </c>
+      <c r="S427" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="T427" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="U427" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V427" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W427" s="4" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Benefits upgrade to save local, add new fields and save
</commit_message>
<xml_diff>
--- a/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
+++ b/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MynikaTech\memgine\docs\domain\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9C5276E-8617-4EB0-8674-509D980D0BF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5918DCBF-6558-4BBE-9C7F-EE824680324A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{AA28BC4D-8219-43B9-8C16-6977709D904A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AA28BC4D-8219-43B9-8C16-6977709D904A}"/>
   </bookViews>
   <sheets>
     <sheet name="Entity Catalogue" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Benfits form screen changes
</commit_message>
<xml_diff>
--- a/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
+++ b/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MynikaTech\memgine\docs\domain\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF80174B-274F-463E-BD86-95924B7AC6E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C1DC0D6-60E0-458B-8148-9DBF91DAF8A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="3" xr2:uid="{AA28BC4D-8219-43B9-8C16-6977709D904A}"/>
   </bookViews>
@@ -24722,7 +24722,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="2" spans="1:23" ht="30">
+    <row r="2" spans="1:23" ht="30" hidden="1">
       <c r="A2" s="10" t="s">
         <v>5</v>
       </c>
@@ -24788,7 +24788,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:23" ht="30">
+    <row r="3" spans="1:23" ht="30" hidden="1">
       <c r="A3" s="10" t="s">
         <v>5</v>
       </c>
@@ -24856,7 +24856,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:23" ht="30">
+    <row r="4" spans="1:23" ht="30" hidden="1">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -24924,7 +24924,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:23" ht="60">
+    <row r="5" spans="1:23" ht="60" hidden="1">
       <c r="A5" s="10" t="s">
         <v>5</v>
       </c>
@@ -24993,7 +24993,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:23" ht="30">
+    <row r="6" spans="1:23" ht="30" hidden="1">
       <c r="A6" s="10" t="s">
         <v>5</v>
       </c>
@@ -25061,7 +25061,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:23">
+    <row r="7" spans="1:23" hidden="1">
       <c r="A7" s="10" t="s">
         <v>5</v>
       </c>
@@ -25129,7 +25129,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:23">
+    <row r="8" spans="1:23" hidden="1">
       <c r="A8" s="10" t="s">
         <v>5</v>
       </c>
@@ -25197,7 +25197,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:23">
+    <row r="9" spans="1:23" hidden="1">
       <c r="A9" s="10" t="s">
         <v>5</v>
       </c>
@@ -25265,7 +25265,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="10" spans="1:23">
+    <row r="10" spans="1:23" hidden="1">
       <c r="A10" s="10" t="s">
         <v>5</v>
       </c>
@@ -25333,7 +25333,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="11" spans="1:23">
+    <row r="11" spans="1:23" hidden="1">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -25401,7 +25401,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:23" ht="30">
+    <row r="12" spans="1:23" ht="30" hidden="1">
       <c r="A12" s="10" t="s">
         <v>5</v>
       </c>
@@ -25469,7 +25469,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:23">
+    <row r="13" spans="1:23" hidden="1">
       <c r="A13" s="10" t="s">
         <v>5</v>
       </c>
@@ -25537,7 +25537,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:23" ht="30">
+    <row r="14" spans="1:23" ht="30" hidden="1">
       <c r="A14" s="10" t="s">
         <v>5</v>
       </c>
@@ -25605,7 +25605,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:23">
+    <row r="15" spans="1:23" hidden="1">
       <c r="A15" s="10" t="s">
         <v>5</v>
       </c>
@@ -25673,7 +25673,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:23" ht="30">
+    <row r="16" spans="1:23" ht="30" hidden="1">
       <c r="A16" s="10" t="s">
         <v>5</v>
       </c>
@@ -25741,7 +25741,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:23">
+    <row r="17" spans="1:23" hidden="1">
       <c r="A17" s="10" t="s">
         <v>5</v>
       </c>
@@ -30577,7 +30577,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="88" spans="1:23" ht="30" hidden="1">
+    <row r="88" spans="1:23" ht="30">
       <c r="A88" s="4" t="s">
         <v>490</v>
       </c>
@@ -30648,7 +30648,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="89" spans="1:23" ht="30" hidden="1">
+    <row r="89" spans="1:23" ht="30">
       <c r="A89" s="4" t="s">
         <v>490</v>
       </c>
@@ -30719,7 +30719,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="90" spans="1:23" ht="30" hidden="1">
+    <row r="90" spans="1:23" ht="30">
       <c r="A90" s="4" t="s">
         <v>490</v>
       </c>
@@ -30790,7 +30790,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="91" spans="1:23" ht="30" hidden="1">
+    <row r="91" spans="1:23" ht="30">
       <c r="A91" s="4" t="s">
         <v>490</v>
       </c>
@@ -30861,7 +30861,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="92" spans="1:23" hidden="1">
+    <row r="92" spans="1:23">
       <c r="A92" s="4" t="s">
         <v>490</v>
       </c>
@@ -30932,7 +30932,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="93" spans="1:23" hidden="1">
+    <row r="93" spans="1:23">
       <c r="A93" s="4" t="s">
         <v>490</v>
       </c>
@@ -31003,7 +31003,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="94" spans="1:23" ht="45" hidden="1">
+    <row r="94" spans="1:23" ht="45">
       <c r="A94" s="4" t="s">
         <v>490</v>
       </c>
@@ -31074,7 +31074,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="95" spans="1:23" ht="30" hidden="1">
+    <row r="95" spans="1:23" ht="30">
       <c r="A95" s="4" t="s">
         <v>490</v>
       </c>
@@ -31145,7 +31145,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="96" spans="1:23" ht="30" hidden="1">
+    <row r="96" spans="1:23" ht="30">
       <c r="A96" s="4" t="s">
         <v>490</v>
       </c>
@@ -31216,7 +31216,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="97" spans="1:23" ht="45" hidden="1">
+    <row r="97" spans="1:23" ht="45">
       <c r="A97" s="4" t="s">
         <v>490</v>
       </c>
@@ -31287,7 +31287,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="98" spans="1:23" ht="30" hidden="1">
+    <row r="98" spans="1:23" ht="30">
       <c r="A98" s="4" t="s">
         <v>490</v>
       </c>
@@ -31358,7 +31358,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="99" spans="1:23" ht="30" hidden="1">
+    <row r="99" spans="1:23" ht="30">
       <c r="A99" s="4" t="s">
         <v>490</v>
       </c>
@@ -31429,7 +31429,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="100" spans="1:23" ht="30" hidden="1">
+    <row r="100" spans="1:23" ht="30">
       <c r="A100" s="4" t="s">
         <v>490</v>
       </c>
@@ -31500,7 +31500,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="101" spans="1:23" ht="30" hidden="1">
+    <row r="101" spans="1:23" ht="30">
       <c r="A101" s="4" t="s">
         <v>490</v>
       </c>
@@ -31571,7 +31571,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="102" spans="1:23" ht="30" hidden="1">
+    <row r="102" spans="1:23" ht="30">
       <c r="A102" s="4" t="s">
         <v>490</v>
       </c>
@@ -31642,7 +31642,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="103" spans="1:23" ht="30" hidden="1">
+    <row r="103" spans="1:23" ht="30">
       <c r="A103" s="4" t="s">
         <v>490</v>
       </c>
@@ -31713,7 +31713,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="104" spans="1:23" ht="30" hidden="1">
+    <row r="104" spans="1:23" ht="30">
       <c r="A104" s="4" t="s">
         <v>490</v>
       </c>
@@ -31784,7 +31784,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="105" spans="1:23" ht="30" hidden="1">
+    <row r="105" spans="1:23" ht="30">
       <c r="A105" s="4" t="s">
         <v>490</v>
       </c>
@@ -31855,7 +31855,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="106" spans="1:23" ht="30" hidden="1">
+    <row r="106" spans="1:23" ht="30">
       <c r="A106" s="4" t="s">
         <v>490</v>
       </c>
@@ -42601,7 +42601,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="260" spans="1:23" ht="30">
+    <row r="260" spans="1:23" ht="30" hidden="1">
       <c r="A260" s="3" t="s">
         <v>1514</v>
       </c>
@@ -42668,7 +42668,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="261" spans="1:23" ht="30">
+    <row r="261" spans="1:23" ht="30" hidden="1">
       <c r="A261" s="3" t="s">
         <v>1514</v>
       </c>
@@ -42735,7 +42735,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="262" spans="1:23" ht="30">
+    <row r="262" spans="1:23" ht="30" hidden="1">
       <c r="A262" s="3" t="s">
         <v>1514</v>
       </c>
@@ -42804,7 +42804,7 @@
         <v>1443</v>
       </c>
     </row>
-    <row r="263" spans="1:23" ht="30">
+    <row r="263" spans="1:23" ht="30" hidden="1">
       <c r="A263" s="3" t="s">
         <v>1514</v>
       </c>
@@ -42873,7 +42873,7 @@
         <v>1443</v>
       </c>
     </row>
-    <row r="264" spans="1:23">
+    <row r="264" spans="1:23" hidden="1">
       <c r="A264" s="3" t="s">
         <v>1514</v>
       </c>
@@ -42942,7 +42942,7 @@
         <v>1443</v>
       </c>
     </row>
-    <row r="265" spans="1:23" ht="30">
+    <row r="265" spans="1:23" ht="30" hidden="1">
       <c r="A265" s="3" t="s">
         <v>1514</v>
       </c>
@@ -43011,7 +43011,7 @@
         <v>1443</v>
       </c>
     </row>
-    <row r="266" spans="1:23">
+    <row r="266" spans="1:23" hidden="1">
       <c r="A266" s="3" t="s">
         <v>1514</v>
       </c>
@@ -43080,7 +43080,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="267" spans="1:23">
+    <row r="267" spans="1:23" hidden="1">
       <c r="A267" s="3" t="s">
         <v>1514</v>
       </c>
@@ -43149,7 +43149,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="268" spans="1:23">
+    <row r="268" spans="1:23" hidden="1">
       <c r="A268" s="3" t="s">
         <v>1514</v>
       </c>
@@ -43218,7 +43218,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="269" spans="1:23">
+    <row r="269" spans="1:23" hidden="1">
       <c r="A269" s="3" t="s">
         <v>1514</v>
       </c>
@@ -43287,7 +43287,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="270" spans="1:23">
+    <row r="270" spans="1:23" hidden="1">
       <c r="A270" s="3" t="s">
         <v>1514</v>
       </c>
@@ -43356,7 +43356,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="271" spans="1:23">
+    <row r="271" spans="1:23" hidden="1">
       <c r="A271" s="3" t="s">
         <v>1514</v>
       </c>
@@ -43425,7 +43425,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="272" spans="1:23" ht="30">
+    <row r="272" spans="1:23" ht="30" hidden="1">
       <c r="A272" s="3" t="s">
         <v>1514</v>
       </c>
@@ -43494,7 +43494,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="273" spans="1:23" ht="30">
+    <row r="273" spans="1:23" ht="30" hidden="1">
       <c r="A273" s="3" t="s">
         <v>1514</v>
       </c>
@@ -43563,7 +43563,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="274" spans="1:23">
+    <row r="274" spans="1:23" hidden="1">
       <c r="A274" s="3" t="s">
         <v>1514</v>
       </c>
@@ -43630,7 +43630,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="275" spans="1:23">
+    <row r="275" spans="1:23" hidden="1">
       <c r="A275" s="3" t="s">
         <v>1514</v>
       </c>
@@ -43697,7 +43697,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="276" spans="1:23">
+    <row r="276" spans="1:23" hidden="1">
       <c r="A276" s="3" t="s">
         <v>1514</v>
       </c>
@@ -43764,7 +43764,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="277" spans="1:23">
+    <row r="277" spans="1:23" hidden="1">
       <c r="A277" s="3" t="s">
         <v>1514</v>
       </c>
@@ -43833,7 +43833,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="278" spans="1:23">
+    <row r="278" spans="1:23" hidden="1">
       <c r="A278" s="3" t="s">
         <v>1514</v>
       </c>
@@ -56209,8 +56209,7 @@
   <autoFilter ref="A1:W456" xr:uid="{7E21F442-9136-4C15-8BA3-92E07332B93A}">
     <filterColumn colId="0">
       <filters>
-        <filter val="Organization"/>
-        <filter val="Organization Details"/>
+        <filter val="Benefit"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
membership product save edit and view changes
</commit_message>
<xml_diff>
--- a/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
+++ b/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MynikaTech\memgine\docs\domain\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C1DC0D6-60E0-458B-8148-9DBF91DAF8A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E89E67E2-721B-4B8A-9324-DEC75EC7BB45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="3" xr2:uid="{AA28BC4D-8219-43B9-8C16-6977709D904A}"/>
   </bookViews>
@@ -29408,7 +29408,7 @@
         <v>7</v>
       </c>
       <c r="M71" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N71" s="3" t="s">
         <v>432</v>
@@ -29435,7 +29435,7 @@
         <v>7</v>
       </c>
       <c r="V71" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W71" s="1" t="s">
         <v>6</v>
@@ -30577,7 +30577,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="88" spans="1:23" ht="30">
+    <row r="88" spans="1:23" ht="30" hidden="1">
       <c r="A88" s="4" t="s">
         <v>490</v>
       </c>
@@ -30648,7 +30648,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="89" spans="1:23" ht="30">
+    <row r="89" spans="1:23" ht="30" hidden="1">
       <c r="A89" s="4" t="s">
         <v>490</v>
       </c>
@@ -30719,7 +30719,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="90" spans="1:23" ht="30">
+    <row r="90" spans="1:23" ht="30" hidden="1">
       <c r="A90" s="4" t="s">
         <v>490</v>
       </c>
@@ -30790,7 +30790,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="91" spans="1:23" ht="30">
+    <row r="91" spans="1:23" ht="30" hidden="1">
       <c r="A91" s="4" t="s">
         <v>490</v>
       </c>
@@ -30861,7 +30861,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="92" spans="1:23">
+    <row r="92" spans="1:23" hidden="1">
       <c r="A92" s="4" t="s">
         <v>490</v>
       </c>
@@ -30932,7 +30932,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="93" spans="1:23">
+    <row r="93" spans="1:23" hidden="1">
       <c r="A93" s="4" t="s">
         <v>490</v>
       </c>
@@ -31003,7 +31003,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="94" spans="1:23" ht="45">
+    <row r="94" spans="1:23" ht="45" hidden="1">
       <c r="A94" s="4" t="s">
         <v>490</v>
       </c>
@@ -31074,7 +31074,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="95" spans="1:23" ht="30">
+    <row r="95" spans="1:23" ht="30" hidden="1">
       <c r="A95" s="4" t="s">
         <v>490</v>
       </c>
@@ -31145,7 +31145,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="96" spans="1:23" ht="30">
+    <row r="96" spans="1:23" ht="30" hidden="1">
       <c r="A96" s="4" t="s">
         <v>490</v>
       </c>
@@ -31216,7 +31216,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="97" spans="1:23" ht="45">
+    <row r="97" spans="1:23" ht="45" hidden="1">
       <c r="A97" s="4" t="s">
         <v>490</v>
       </c>
@@ -31287,7 +31287,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="98" spans="1:23" ht="30">
+    <row r="98" spans="1:23" ht="30" hidden="1">
       <c r="A98" s="4" t="s">
         <v>490</v>
       </c>
@@ -31358,7 +31358,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="99" spans="1:23" ht="30">
+    <row r="99" spans="1:23" ht="30" hidden="1">
       <c r="A99" s="4" t="s">
         <v>490</v>
       </c>
@@ -31429,7 +31429,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="100" spans="1:23" ht="30">
+    <row r="100" spans="1:23" ht="30" hidden="1">
       <c r="A100" s="4" t="s">
         <v>490</v>
       </c>
@@ -31500,7 +31500,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="101" spans="1:23" ht="30">
+    <row r="101" spans="1:23" ht="30" hidden="1">
       <c r="A101" s="4" t="s">
         <v>490</v>
       </c>
@@ -31571,7 +31571,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="102" spans="1:23" ht="30">
+    <row r="102" spans="1:23" ht="30" hidden="1">
       <c r="A102" s="4" t="s">
         <v>490</v>
       </c>
@@ -31642,7 +31642,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="103" spans="1:23" ht="30">
+    <row r="103" spans="1:23" ht="30" hidden="1">
       <c r="A103" s="4" t="s">
         <v>490</v>
       </c>
@@ -31713,7 +31713,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="104" spans="1:23" ht="30">
+    <row r="104" spans="1:23" ht="30" hidden="1">
       <c r="A104" s="4" t="s">
         <v>490</v>
       </c>
@@ -31784,7 +31784,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="105" spans="1:23" ht="30">
+    <row r="105" spans="1:23" ht="30" hidden="1">
       <c r="A105" s="4" t="s">
         <v>490</v>
       </c>
@@ -31855,7 +31855,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="106" spans="1:23" ht="30">
+    <row r="106" spans="1:23" ht="30" hidden="1">
       <c r="A106" s="4" t="s">
         <v>490</v>
       </c>
@@ -31926,7 +31926,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="107" spans="1:23" ht="30" hidden="1">
+    <row r="107" spans="1:23" ht="30">
       <c r="A107" s="4" t="s">
         <v>548</v>
       </c>
@@ -31997,7 +31997,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="108" spans="1:23" ht="30" hidden="1">
+    <row r="108" spans="1:23" ht="30">
       <c r="A108" s="4" t="s">
         <v>548</v>
       </c>
@@ -32068,7 +32068,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="109" spans="1:23" ht="30" hidden="1">
+    <row r="109" spans="1:23" ht="30">
       <c r="A109" s="4" t="s">
         <v>548</v>
       </c>
@@ -32106,7 +32106,7 @@
         <v>7</v>
       </c>
       <c r="M109" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N109" s="3" t="s">
         <v>563</v>
@@ -32133,13 +32133,13 @@
         <v>7</v>
       </c>
       <c r="V109" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="W109" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="110" spans="1:23" ht="30" hidden="1">
+    <row r="110" spans="1:23" ht="30">
       <c r="A110" s="4" t="s">
         <v>548</v>
       </c>
@@ -32210,7 +32210,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="111" spans="1:23" ht="30" hidden="1">
+    <row r="111" spans="1:23" ht="30">
       <c r="A111" s="4" t="s">
         <v>548</v>
       </c>
@@ -32281,7 +32281,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="112" spans="1:23" hidden="1">
+    <row r="112" spans="1:23">
       <c r="A112" s="4" t="s">
         <v>548</v>
       </c>
@@ -32352,7 +32352,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="113" spans="1:23" hidden="1">
+    <row r="113" spans="1:23">
       <c r="A113" s="4" t="s">
         <v>548</v>
       </c>
@@ -32423,7 +32423,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="114" spans="1:23" hidden="1">
+    <row r="114" spans="1:23">
       <c r="A114" s="4" t="s">
         <v>548</v>
       </c>
@@ -32494,7 +32494,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="115" spans="1:23" ht="30" hidden="1">
+    <row r="115" spans="1:23" ht="30">
       <c r="A115" s="4" t="s">
         <v>548</v>
       </c>
@@ -32565,7 +32565,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="116" spans="1:23" hidden="1">
+    <row r="116" spans="1:23">
       <c r="A116" s="4" t="s">
         <v>548</v>
       </c>
@@ -32636,7 +32636,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="117" spans="1:23" ht="30" hidden="1">
+    <row r="117" spans="1:23" ht="30">
       <c r="A117" s="4" t="s">
         <v>548</v>
       </c>
@@ -32707,7 +32707,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="118" spans="1:23" hidden="1">
+    <row r="118" spans="1:23">
       <c r="A118" s="4" t="s">
         <v>548</v>
       </c>
@@ -32778,7 +32778,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="119" spans="1:23" ht="30" hidden="1">
+    <row r="119" spans="1:23" ht="30">
       <c r="A119" s="4" t="s">
         <v>548</v>
       </c>
@@ -32849,7 +32849,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="120" spans="1:23" hidden="1">
+    <row r="120" spans="1:23">
       <c r="A120" s="4" t="s">
         <v>548</v>
       </c>
@@ -32920,7 +32920,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="121" spans="1:23" ht="30" hidden="1">
+    <row r="121" spans="1:23" ht="30">
       <c r="A121" s="4" t="s">
         <v>548</v>
       </c>
@@ -32991,7 +32991,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="122" spans="1:23" hidden="1">
+    <row r="122" spans="1:23">
       <c r="A122" s="4" t="s">
         <v>548</v>
       </c>
@@ -33062,7 +33062,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="123" spans="1:23" hidden="1">
+    <row r="123" spans="1:23">
       <c r="A123" s="4" t="s">
         <v>548</v>
       </c>
@@ -33133,7 +33133,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="124" spans="1:23" hidden="1">
+    <row r="124" spans="1:23">
       <c r="A124" s="4" t="s">
         <v>548</v>
       </c>
@@ -56209,7 +56209,7 @@
   <autoFilter ref="A1:W456" xr:uid="{7E21F442-9136-4C15-8BA3-92E07332B93A}">
     <filterColumn colId="0">
       <filters>
-        <filter val="Benefit"/>
+        <filter val="Subscription Plan"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
Customer scree n in org admin
</commit_message>
<xml_diff>
--- a/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
+++ b/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MynikaTech\memgine\docs\domain\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0694C604-9124-46E7-B720-E703D626DD16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAB49E44-DBF9-4D80-B910-E461BF0DEE63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="3" xr2:uid="{AA28BC4D-8219-43B9-8C16-6977709D904A}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15086" uniqueCount="4031">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15068" uniqueCount="4031">
   <si>
     <t>Domain</t>
   </si>
@@ -24886,6 +24886,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E21F442-9136-4C15-8BA3-92E07332B93A}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:W462"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -24985,7 +24986,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="2" spans="1:23" ht="30">
+    <row r="2" spans="1:23" ht="30" hidden="1">
       <c r="A2" s="10" t="s">
         <v>5</v>
       </c>
@@ -25051,7 +25052,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:23" ht="30">
+    <row r="3" spans="1:23" ht="30" hidden="1">
       <c r="A3" s="10" t="s">
         <v>5</v>
       </c>
@@ -25119,7 +25120,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:23" ht="30">
+    <row r="4" spans="1:23" ht="30" hidden="1">
       <c r="A4" s="10" t="s">
         <v>5</v>
       </c>
@@ -25187,7 +25188,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:23" ht="60">
+    <row r="5" spans="1:23" ht="60" hidden="1">
       <c r="A5" s="10" t="s">
         <v>5</v>
       </c>
@@ -25256,7 +25257,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:23" ht="30">
+    <row r="6" spans="1:23" ht="30" hidden="1">
       <c r="A6" s="10" t="s">
         <v>5</v>
       </c>
@@ -25324,7 +25325,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:23">
+    <row r="7" spans="1:23" hidden="1">
       <c r="A7" s="10" t="s">
         <v>5</v>
       </c>
@@ -25392,7 +25393,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:23">
+    <row r="8" spans="1:23" hidden="1">
       <c r="A8" s="10" t="s">
         <v>5</v>
       </c>
@@ -25460,7 +25461,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:23">
+    <row r="9" spans="1:23" hidden="1">
       <c r="A9" s="10" t="s">
         <v>5</v>
       </c>
@@ -25528,7 +25529,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="10" spans="1:23">
+    <row r="10" spans="1:23" hidden="1">
       <c r="A10" s="10" t="s">
         <v>5</v>
       </c>
@@ -25596,7 +25597,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="11" spans="1:23">
+    <row r="11" spans="1:23" hidden="1">
       <c r="A11" s="10" t="s">
         <v>5</v>
       </c>
@@ -25664,7 +25665,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:23" ht="30">
+    <row r="12" spans="1:23" ht="30" hidden="1">
       <c r="A12" s="10" t="s">
         <v>5</v>
       </c>
@@ -25732,7 +25733,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:23">
+    <row r="13" spans="1:23" hidden="1">
       <c r="A13" s="10" t="s">
         <v>5</v>
       </c>
@@ -25800,7 +25801,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:23" ht="30">
+    <row r="14" spans="1:23" ht="30" hidden="1">
       <c r="A14" s="10" t="s">
         <v>5</v>
       </c>
@@ -25868,7 +25869,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:23">
+    <row r="15" spans="1:23" hidden="1">
       <c r="A15" s="10" t="s">
         <v>5</v>
       </c>
@@ -25936,7 +25937,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:23" ht="30">
+    <row r="16" spans="1:23" ht="30" hidden="1">
       <c r="A16" s="10" t="s">
         <v>5</v>
       </c>
@@ -26004,7 +26005,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:23">
+    <row r="17" spans="1:23" hidden="1">
       <c r="A17" s="10" t="s">
         <v>5</v>
       </c>
@@ -27156,7 +27157,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="34" spans="1:23" ht="30">
+    <row r="34" spans="1:23" ht="30" hidden="1">
       <c r="A34" s="3" t="s">
         <v>37</v>
       </c>
@@ -27227,7 +27228,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="35" spans="1:23" ht="30">
+    <row r="35" spans="1:23" ht="30" hidden="1">
       <c r="A35" s="3" t="s">
         <v>37</v>
       </c>
@@ -27298,7 +27299,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="36" spans="1:23">
+    <row r="36" spans="1:23" hidden="1">
       <c r="A36" s="3" t="s">
         <v>37</v>
       </c>
@@ -27369,7 +27370,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="37" spans="1:23" ht="45">
+    <row r="37" spans="1:23" ht="45" hidden="1">
       <c r="A37" s="3" t="s">
         <v>37</v>
       </c>
@@ -27440,7 +27441,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="38" spans="1:23" ht="30">
+    <row r="38" spans="1:23" ht="30" hidden="1">
       <c r="A38" s="3" t="s">
         <v>37</v>
       </c>
@@ -27511,7 +27512,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="39" spans="1:23" ht="30">
+    <row r="39" spans="1:23" ht="30" hidden="1">
       <c r="A39" s="3" t="s">
         <v>37</v>
       </c>
@@ -27582,7 +27583,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="40" spans="1:23" ht="30">
+    <row r="40" spans="1:23" ht="30" hidden="1">
       <c r="A40" s="3" t="s">
         <v>37</v>
       </c>
@@ -27653,7 +27654,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="41" spans="1:23">
+    <row r="41" spans="1:23" hidden="1">
       <c r="A41" s="3" t="s">
         <v>37</v>
       </c>
@@ -27724,7 +27725,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="42" spans="1:23" ht="30">
+    <row r="42" spans="1:23" ht="30" hidden="1">
       <c r="A42" s="3" t="s">
         <v>37</v>
       </c>
@@ -27795,7 +27796,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="43" spans="1:23">
+    <row r="43" spans="1:23" hidden="1">
       <c r="A43" s="3" t="s">
         <v>37</v>
       </c>
@@ -27866,7 +27867,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="44" spans="1:23">
+    <row r="44" spans="1:23" hidden="1">
       <c r="A44" s="3" t="s">
         <v>37</v>
       </c>
@@ -27937,7 +27938,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="45" spans="1:23">
+    <row r="45" spans="1:23" hidden="1">
       <c r="A45" s="3" t="s">
         <v>37</v>
       </c>
@@ -28008,7 +28009,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="46" spans="1:23" ht="30">
+    <row r="46" spans="1:23" ht="30" hidden="1">
       <c r="A46" s="3" t="s">
         <v>317</v>
       </c>
@@ -28055,7 +28056,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="47" spans="1:23" ht="30">
+    <row r="47" spans="1:23" ht="30" hidden="1">
       <c r="A47" s="3" t="s">
         <v>317</v>
       </c>
@@ -28102,7 +28103,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="48" spans="1:23" ht="45">
+    <row r="48" spans="1:23" ht="45" hidden="1">
       <c r="A48" s="3" t="s">
         <v>317</v>
       </c>
@@ -28149,7 +28150,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="49" spans="1:23" ht="30">
+    <row r="49" spans="1:23" ht="30" hidden="1">
       <c r="A49" s="3" t="s">
         <v>317</v>
       </c>
@@ -28196,7 +28197,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="50" spans="1:23" ht="30">
+    <row r="50" spans="1:23" ht="30" hidden="1">
       <c r="A50" s="3" t="s">
         <v>317</v>
       </c>
@@ -28243,7 +28244,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="51" spans="1:23" ht="30">
+    <row r="51" spans="1:23" ht="30" hidden="1">
       <c r="A51" s="4" t="s">
         <v>341</v>
       </c>
@@ -28311,7 +28312,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="52" spans="1:23" ht="30">
+    <row r="52" spans="1:23" ht="30" hidden="1">
       <c r="A52" s="4" t="s">
         <v>341</v>
       </c>
@@ -28379,7 +28380,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="53" spans="1:23" ht="30">
+    <row r="53" spans="1:23" ht="30" hidden="1">
       <c r="A53" s="4" t="s">
         <v>341</v>
       </c>
@@ -28447,7 +28448,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="54" spans="1:23" ht="30">
+    <row r="54" spans="1:23" ht="30" hidden="1">
       <c r="A54" s="4" t="s">
         <v>341</v>
       </c>
@@ -28515,7 +28516,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="55" spans="1:23" ht="30">
+    <row r="55" spans="1:23" ht="30" hidden="1">
       <c r="A55" s="4" t="s">
         <v>341</v>
       </c>
@@ -28583,7 +28584,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="56" spans="1:23" ht="30">
+    <row r="56" spans="1:23" ht="30" hidden="1">
       <c r="A56" s="4" t="s">
         <v>341</v>
       </c>
@@ -28651,7 +28652,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="57" spans="1:23" ht="30">
+    <row r="57" spans="1:23" ht="30" hidden="1">
       <c r="A57" s="4" t="s">
         <v>341</v>
       </c>
@@ -28719,7 +28720,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="58" spans="1:23" ht="30">
+    <row r="58" spans="1:23" ht="30" hidden="1">
       <c r="A58" s="4" t="s">
         <v>341</v>
       </c>
@@ -28787,7 +28788,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="59" spans="1:23" ht="45">
+    <row r="59" spans="1:23" ht="45" hidden="1">
       <c r="A59" s="4" t="s">
         <v>341</v>
       </c>
@@ -28855,7 +28856,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="60" spans="1:23" ht="30">
+    <row r="60" spans="1:23" ht="30" hidden="1">
       <c r="A60" s="4" t="s">
         <v>341</v>
       </c>
@@ -28923,7 +28924,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="61" spans="1:23" ht="30">
+    <row r="61" spans="1:23" ht="30" hidden="1">
       <c r="A61" s="4" t="s">
         <v>370</v>
       </c>
@@ -28994,7 +28995,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="62" spans="1:23" ht="30">
+    <row r="62" spans="1:23" ht="30" hidden="1">
       <c r="A62" s="4" t="s">
         <v>370</v>
       </c>
@@ -29065,7 +29066,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="63" spans="1:23" ht="30">
+    <row r="63" spans="1:23" ht="30" hidden="1">
       <c r="A63" s="4" t="s">
         <v>370</v>
       </c>
@@ -29136,7 +29137,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="64" spans="1:23" ht="30">
+    <row r="64" spans="1:23" ht="30" hidden="1">
       <c r="A64" s="4" t="s">
         <v>370</v>
       </c>
@@ -29207,7 +29208,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="65" spans="1:23" ht="30">
+    <row r="65" spans="1:23" ht="30" hidden="1">
       <c r="A65" s="4" t="s">
         <v>370</v>
       </c>
@@ -29278,7 +29279,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="66" spans="1:23" ht="30">
+    <row r="66" spans="1:23" ht="30" hidden="1">
       <c r="A66" s="4" t="s">
         <v>377</v>
       </c>
@@ -29349,7 +29350,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="67" spans="1:23" ht="30">
+    <row r="67" spans="1:23" ht="30" hidden="1">
       <c r="A67" s="4" t="s">
         <v>377</v>
       </c>
@@ -29420,7 +29421,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="68" spans="1:23" ht="30">
+    <row r="68" spans="1:23" ht="30" hidden="1">
       <c r="A68" s="4" t="s">
         <v>377</v>
       </c>
@@ -29491,7 +29492,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="69" spans="1:23" ht="30">
+    <row r="69" spans="1:23" ht="30" hidden="1">
       <c r="A69" s="4" t="s">
         <v>10</v>
       </c>
@@ -29562,7 +29563,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="70" spans="1:23" ht="30">
+    <row r="70" spans="1:23" ht="30" hidden="1">
       <c r="A70" s="4" t="s">
         <v>10</v>
       </c>
@@ -29633,7 +29634,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="71" spans="1:23" ht="45">
+    <row r="71" spans="1:23" ht="45" hidden="1">
       <c r="A71" s="4" t="s">
         <v>10</v>
       </c>
@@ -29704,7 +29705,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="72" spans="1:23" ht="45">
+    <row r="72" spans="1:23" ht="45" hidden="1">
       <c r="A72" s="4" t="s">
         <v>10</v>
       </c>
@@ -29775,7 +29776,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="73" spans="1:23" ht="30">
+    <row r="73" spans="1:23" ht="30" hidden="1">
       <c r="A73" s="4" t="s">
         <v>10</v>
       </c>
@@ -29846,7 +29847,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="74" spans="1:23" ht="30">
+    <row r="74" spans="1:23" ht="30" hidden="1">
       <c r="A74" s="4" t="s">
         <v>10</v>
       </c>
@@ -29917,7 +29918,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="75" spans="1:23" ht="30">
+    <row r="75" spans="1:23" ht="30" hidden="1">
       <c r="A75" s="4" t="s">
         <v>10</v>
       </c>
@@ -29988,7 +29989,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="76" spans="1:23" ht="30">
+    <row r="76" spans="1:23" ht="30" hidden="1">
       <c r="A76" s="4" t="s">
         <v>10</v>
       </c>
@@ -30059,7 +30060,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="77" spans="1:23" ht="30">
+    <row r="77" spans="1:23" ht="30" hidden="1">
       <c r="A77" s="4" t="s">
         <v>10</v>
       </c>
@@ -30130,7 +30131,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="78" spans="1:23" ht="30">
+    <row r="78" spans="1:23" ht="30" hidden="1">
       <c r="A78" s="4" t="s">
         <v>10</v>
       </c>
@@ -30201,7 +30202,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="79" spans="1:23" ht="30">
+    <row r="79" spans="1:23" ht="30" hidden="1">
       <c r="A79" s="4" t="s">
         <v>10</v>
       </c>
@@ -30272,7 +30273,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="80" spans="1:23" ht="45">
+    <row r="80" spans="1:23" ht="45" hidden="1">
       <c r="A80" s="4" t="s">
         <v>10</v>
       </c>
@@ -30343,7 +30344,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="81" spans="1:23" ht="45">
+    <row r="81" spans="1:23" ht="45" hidden="1">
       <c r="A81" s="4" t="s">
         <v>10</v>
       </c>
@@ -30414,7 +30415,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="82" spans="1:23" ht="30">
+    <row r="82" spans="1:23" ht="30" hidden="1">
       <c r="A82" s="4" t="s">
         <v>10</v>
       </c>
@@ -30485,7 +30486,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="83" spans="1:23" ht="30">
+    <row r="83" spans="1:23" ht="30" hidden="1">
       <c r="A83" s="4" t="s">
         <v>10</v>
       </c>
@@ -30556,7 +30557,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="84" spans="1:23" ht="30">
+    <row r="84" spans="1:23" ht="30" hidden="1">
       <c r="A84" s="4" t="s">
         <v>10</v>
       </c>
@@ -30627,7 +30628,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="85" spans="1:23" ht="30">
+    <row r="85" spans="1:23" ht="30" hidden="1">
       <c r="A85" s="4" t="s">
         <v>10</v>
       </c>
@@ -30698,7 +30699,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="86" spans="1:23" ht="45">
+    <row r="86" spans="1:23" ht="45" hidden="1">
       <c r="A86" s="4" t="s">
         <v>10</v>
       </c>
@@ -30769,7 +30770,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="87" spans="1:23" ht="30">
+    <row r="87" spans="1:23" ht="30" hidden="1">
       <c r="A87" s="4" t="s">
         <v>10</v>
       </c>
@@ -30840,7 +30841,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="88" spans="1:23" ht="30">
+    <row r="88" spans="1:23" ht="30" hidden="1">
       <c r="A88" s="4" t="s">
         <v>490</v>
       </c>
@@ -30911,7 +30912,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="89" spans="1:23" ht="30">
+    <row r="89" spans="1:23" ht="30" hidden="1">
       <c r="A89" s="4" t="s">
         <v>490</v>
       </c>
@@ -30982,7 +30983,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="90" spans="1:23" ht="30">
+    <row r="90" spans="1:23" ht="30" hidden="1">
       <c r="A90" s="4" t="s">
         <v>490</v>
       </c>
@@ -31053,7 +31054,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="91" spans="1:23" ht="30">
+    <row r="91" spans="1:23" ht="30" hidden="1">
       <c r="A91" s="4" t="s">
         <v>490</v>
       </c>
@@ -31124,7 +31125,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="92" spans="1:23">
+    <row r="92" spans="1:23" hidden="1">
       <c r="A92" s="4" t="s">
         <v>490</v>
       </c>
@@ -31195,7 +31196,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="93" spans="1:23">
+    <row r="93" spans="1:23" hidden="1">
       <c r="A93" s="4" t="s">
         <v>490</v>
       </c>
@@ -31266,7 +31267,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="94" spans="1:23" ht="45">
+    <row r="94" spans="1:23" ht="45" hidden="1">
       <c r="A94" s="4" t="s">
         <v>490</v>
       </c>
@@ -31337,7 +31338,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="95" spans="1:23" ht="30">
+    <row r="95" spans="1:23" ht="30" hidden="1">
       <c r="A95" s="4" t="s">
         <v>490</v>
       </c>
@@ -31408,7 +31409,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="96" spans="1:23" ht="30">
+    <row r="96" spans="1:23" ht="30" hidden="1">
       <c r="A96" s="4" t="s">
         <v>490</v>
       </c>
@@ -31479,7 +31480,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="97" spans="1:23" ht="45">
+    <row r="97" spans="1:23" ht="45" hidden="1">
       <c r="A97" s="4" t="s">
         <v>490</v>
       </c>
@@ -31550,7 +31551,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="98" spans="1:23" ht="30">
+    <row r="98" spans="1:23" ht="30" hidden="1">
       <c r="A98" s="4" t="s">
         <v>490</v>
       </c>
@@ -31621,7 +31622,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="99" spans="1:23" ht="30">
+    <row r="99" spans="1:23" ht="30" hidden="1">
       <c r="A99" s="4" t="s">
         <v>490</v>
       </c>
@@ -31692,7 +31693,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="100" spans="1:23" ht="30">
+    <row r="100" spans="1:23" ht="30" hidden="1">
       <c r="A100" s="4" t="s">
         <v>490</v>
       </c>
@@ -31763,7 +31764,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="101" spans="1:23" ht="30">
+    <row r="101" spans="1:23" ht="30" hidden="1">
       <c r="A101" s="4" t="s">
         <v>490</v>
       </c>
@@ -31834,7 +31835,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="102" spans="1:23" ht="30">
+    <row r="102" spans="1:23" ht="30" hidden="1">
       <c r="A102" s="4" t="s">
         <v>490</v>
       </c>
@@ -31905,7 +31906,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="103" spans="1:23" ht="30">
+    <row r="103" spans="1:23" ht="30" hidden="1">
       <c r="A103" s="4" t="s">
         <v>490</v>
       </c>
@@ -31976,7 +31977,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="104" spans="1:23" ht="30">
+    <row r="104" spans="1:23" ht="30" hidden="1">
       <c r="A104" s="4" t="s">
         <v>490</v>
       </c>
@@ -32047,7 +32048,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="105" spans="1:23" ht="30">
+    <row r="105" spans="1:23" ht="30" hidden="1">
       <c r="A105" s="4" t="s">
         <v>490</v>
       </c>
@@ -32118,7 +32119,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="106" spans="1:23" ht="30">
+    <row r="106" spans="1:23" ht="30" hidden="1">
       <c r="A106" s="4" t="s">
         <v>490</v>
       </c>
@@ -32189,7 +32190,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="107" spans="1:23" ht="30">
+    <row r="107" spans="1:23" ht="30" hidden="1">
       <c r="A107" s="4" t="s">
         <v>548</v>
       </c>
@@ -32260,7 +32261,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="108" spans="1:23" ht="30">
+    <row r="108" spans="1:23" ht="30" hidden="1">
       <c r="A108" s="4" t="s">
         <v>548</v>
       </c>
@@ -32331,7 +32332,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="109" spans="1:23" ht="30">
+    <row r="109" spans="1:23" ht="30" hidden="1">
       <c r="A109" s="4" t="s">
         <v>548</v>
       </c>
@@ -32402,7 +32403,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="110" spans="1:23" ht="30">
+    <row r="110" spans="1:23" ht="30" hidden="1">
       <c r="A110" s="4" t="s">
         <v>548</v>
       </c>
@@ -32473,7 +32474,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="111" spans="1:23" ht="30">
+    <row r="111" spans="1:23" ht="30" hidden="1">
       <c r="A111" s="4" t="s">
         <v>548</v>
       </c>
@@ -32544,7 +32545,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="112" spans="1:23">
+    <row r="112" spans="1:23" hidden="1">
       <c r="A112" s="4" t="s">
         <v>548</v>
       </c>
@@ -32615,7 +32616,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="113" spans="1:23">
+    <row r="113" spans="1:23" hidden="1">
       <c r="A113" s="4" t="s">
         <v>548</v>
       </c>
@@ -32686,7 +32687,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="114" spans="1:23">
+    <row r="114" spans="1:23" hidden="1">
       <c r="A114" s="4" t="s">
         <v>548</v>
       </c>
@@ -32757,7 +32758,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="115" spans="1:23" ht="30">
+    <row r="115" spans="1:23" ht="30" hidden="1">
       <c r="A115" s="4" t="s">
         <v>548</v>
       </c>
@@ -32828,7 +32829,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="116" spans="1:23">
+    <row r="116" spans="1:23" hidden="1">
       <c r="A116" s="4" t="s">
         <v>548</v>
       </c>
@@ -32899,7 +32900,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="117" spans="1:23" ht="30">
+    <row r="117" spans="1:23" ht="30" hidden="1">
       <c r="A117" s="4" t="s">
         <v>548</v>
       </c>
@@ -32970,7 +32971,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="118" spans="1:23">
+    <row r="118" spans="1:23" hidden="1">
       <c r="A118" s="4" t="s">
         <v>548</v>
       </c>
@@ -33041,7 +33042,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="119" spans="1:23" ht="30">
+    <row r="119" spans="1:23" ht="30" hidden="1">
       <c r="A119" s="4" t="s">
         <v>548</v>
       </c>
@@ -33112,7 +33113,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="120" spans="1:23">
+    <row r="120" spans="1:23" hidden="1">
       <c r="A120" s="4" t="s">
         <v>548</v>
       </c>
@@ -33183,7 +33184,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="121" spans="1:23" ht="30">
+    <row r="121" spans="1:23" ht="30" hidden="1">
       <c r="A121" s="4" t="s">
         <v>548</v>
       </c>
@@ -33254,7 +33255,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="122" spans="1:23">
+    <row r="122" spans="1:23" hidden="1">
       <c r="A122" s="4" t="s">
         <v>548</v>
       </c>
@@ -33325,7 +33326,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="123" spans="1:23">
+    <row r="123" spans="1:23" hidden="1">
       <c r="A123" s="4" t="s">
         <v>548</v>
       </c>
@@ -33396,7 +33397,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="124" spans="1:23">
+    <row r="124" spans="1:23" hidden="1">
       <c r="A124" s="4" t="s">
         <v>548</v>
       </c>
@@ -33467,7 +33468,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="125" spans="1:23" ht="30">
+    <row r="125" spans="1:23" ht="30" hidden="1">
       <c r="A125" s="4" t="s">
         <v>620</v>
       </c>
@@ -33538,7 +33539,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="126" spans="1:23" ht="30">
+    <row r="126" spans="1:23" ht="30" hidden="1">
       <c r="A126" s="4" t="s">
         <v>620</v>
       </c>
@@ -33609,7 +33610,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="127" spans="1:23">
+    <row r="127" spans="1:23" hidden="1">
       <c r="A127" s="4" t="s">
         <v>620</v>
       </c>
@@ -33680,7 +33681,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="128" spans="1:23" ht="30">
+    <row r="128" spans="1:23" ht="30" hidden="1">
       <c r="A128" s="4" t="s">
         <v>620</v>
       </c>
@@ -33751,7 +33752,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="129" spans="1:23">
+    <row r="129" spans="1:23" hidden="1">
       <c r="A129" s="4" t="s">
         <v>620</v>
       </c>
@@ -33822,7 +33823,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="130" spans="1:23" ht="30">
+    <row r="130" spans="1:23" ht="30" hidden="1">
       <c r="A130" s="4" t="s">
         <v>620</v>
       </c>
@@ -33893,7 +33894,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="131" spans="1:23">
+    <row r="131" spans="1:23" hidden="1">
       <c r="A131" s="4" t="s">
         <v>620</v>
       </c>
@@ -33964,7 +33965,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="132" spans="1:23">
+    <row r="132" spans="1:23" hidden="1">
       <c r="A132" s="4" t="s">
         <v>620</v>
       </c>
@@ -34035,7 +34036,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="133" spans="1:23" ht="30">
+    <row r="133" spans="1:23" ht="30" hidden="1">
       <c r="A133" s="4" t="s">
         <v>620</v>
       </c>
@@ -34106,7 +34107,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="134" spans="1:23" ht="30">
+    <row r="134" spans="1:23" ht="30" hidden="1">
       <c r="A134" s="4" t="s">
         <v>620</v>
       </c>
@@ -34177,7 +34178,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="135" spans="1:23">
+    <row r="135" spans="1:23" hidden="1">
       <c r="A135" s="4" t="s">
         <v>620</v>
       </c>
@@ -34248,7 +34249,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="136" spans="1:23" ht="30">
+    <row r="136" spans="1:23" ht="30" hidden="1">
       <c r="A136" s="4" t="s">
         <v>620</v>
       </c>
@@ -34319,7 +34320,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="137" spans="1:23">
+    <row r="137" spans="1:23" hidden="1">
       <c r="A137" s="4" t="s">
         <v>620</v>
       </c>
@@ -34390,7 +34391,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="138" spans="1:23">
+    <row r="138" spans="1:23" hidden="1">
       <c r="A138" s="4" t="s">
         <v>620</v>
       </c>
@@ -34461,7 +34462,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="139" spans="1:23">
+    <row r="139" spans="1:23" hidden="1">
       <c r="A139" s="4" t="s">
         <v>620</v>
       </c>
@@ -34532,7 +34533,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="140" spans="1:23" ht="30">
+    <row r="140" spans="1:23" ht="30" hidden="1">
       <c r="A140" s="4" t="s">
         <v>673</v>
       </c>
@@ -34603,7 +34604,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="141" spans="1:23" ht="30">
+    <row r="141" spans="1:23" ht="30" hidden="1">
       <c r="A141" s="4" t="s">
         <v>673</v>
       </c>
@@ -34674,7 +34675,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="142" spans="1:23" ht="30">
+    <row r="142" spans="1:23" ht="30" hidden="1">
       <c r="A142" s="4" t="s">
         <v>673</v>
       </c>
@@ -34745,7 +34746,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="143" spans="1:23" ht="30">
+    <row r="143" spans="1:23" ht="30" hidden="1">
       <c r="A143" s="4" t="s">
         <v>673</v>
       </c>
@@ -34816,7 +34817,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="144" spans="1:23" ht="30">
+    <row r="144" spans="1:23" ht="30" hidden="1">
       <c r="A144" s="4" t="s">
         <v>673</v>
       </c>
@@ -34887,7 +34888,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="145" spans="1:23" ht="30">
+    <row r="145" spans="1:23" ht="30" hidden="1">
       <c r="A145" s="4" t="s">
         <v>673</v>
       </c>
@@ -34958,7 +34959,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="146" spans="1:23" ht="30">
+    <row r="146" spans="1:23" ht="30" hidden="1">
       <c r="A146" s="4" t="s">
         <v>673</v>
       </c>
@@ -35029,7 +35030,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="147" spans="1:23">
+    <row r="147" spans="1:23" hidden="1">
       <c r="A147" s="4" t="s">
         <v>673</v>
       </c>
@@ -35100,7 +35101,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="148" spans="1:23" ht="30">
+    <row r="148" spans="1:23" ht="30" hidden="1">
       <c r="A148" s="4" t="s">
         <v>673</v>
       </c>
@@ -35171,7 +35172,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="149" spans="1:23" ht="30">
+    <row r="149" spans="1:23" ht="30" hidden="1">
       <c r="A149" s="4" t="s">
         <v>673</v>
       </c>
@@ -35242,7 +35243,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="150" spans="1:23" ht="30">
+    <row r="150" spans="1:23" ht="30" hidden="1">
       <c r="A150" s="4" t="s">
         <v>673</v>
       </c>
@@ -35313,7 +35314,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="151" spans="1:23" ht="30">
+    <row r="151" spans="1:23" ht="30" hidden="1">
       <c r="A151" s="4" t="s">
         <v>673</v>
       </c>
@@ -35384,7 +35385,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="152" spans="1:23" ht="30">
+    <row r="152" spans="1:23" ht="30" hidden="1">
       <c r="A152" s="4" t="s">
         <v>673</v>
       </c>
@@ -35455,7 +35456,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="153" spans="1:23" ht="30">
+    <row r="153" spans="1:23" ht="30" hidden="1">
       <c r="A153" s="4" t="s">
         <v>673</v>
       </c>
@@ -35526,7 +35527,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="154" spans="1:23">
+    <row r="154" spans="1:23" hidden="1">
       <c r="A154" s="4" t="s">
         <v>673</v>
       </c>
@@ -35597,7 +35598,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="155" spans="1:23" ht="30">
+    <row r="155" spans="1:23" ht="30" hidden="1">
       <c r="A155" s="4" t="s">
         <v>34</v>
       </c>
@@ -35668,7 +35669,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="156" spans="1:23" ht="30">
+    <row r="156" spans="1:23" ht="30" hidden="1">
       <c r="A156" s="4" t="s">
         <v>34</v>
       </c>
@@ -35739,7 +35740,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="157" spans="1:23" ht="30">
+    <row r="157" spans="1:23" ht="30" hidden="1">
       <c r="A157" s="4" t="s">
         <v>34</v>
       </c>
@@ -35810,7 +35811,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="158" spans="1:23" ht="30">
+    <row r="158" spans="1:23" ht="30" hidden="1">
       <c r="A158" s="4" t="s">
         <v>34</v>
       </c>
@@ -35881,7 +35882,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="159" spans="1:23">
+    <row r="159" spans="1:23" hidden="1">
       <c r="A159" s="4" t="s">
         <v>34</v>
       </c>
@@ -35952,7 +35953,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="160" spans="1:23" ht="30">
+    <row r="160" spans="1:23" ht="30" hidden="1">
       <c r="A160" s="4" t="s">
         <v>34</v>
       </c>
@@ -36023,7 +36024,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="161" spans="1:23" ht="30">
+    <row r="161" spans="1:23" ht="30" hidden="1">
       <c r="A161" s="4" t="s">
         <v>34</v>
       </c>
@@ -36094,7 +36095,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="162" spans="1:23" ht="30">
+    <row r="162" spans="1:23" ht="30" hidden="1">
       <c r="A162" s="4" t="s">
         <v>34</v>
       </c>
@@ -36165,7 +36166,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="163" spans="1:23" ht="30">
+    <row r="163" spans="1:23" ht="30" hidden="1">
       <c r="A163" s="4" t="s">
         <v>34</v>
       </c>
@@ -36236,7 +36237,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="164" spans="1:23" ht="30">
+    <row r="164" spans="1:23" ht="30" hidden="1">
       <c r="A164" s="4" t="s">
         <v>34</v>
       </c>
@@ -36307,7 +36308,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="165" spans="1:23" ht="30">
+    <row r="165" spans="1:23" ht="30" hidden="1">
       <c r="A165" s="4" t="s">
         <v>34</v>
       </c>
@@ -36378,7 +36379,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="166" spans="1:23" ht="30">
+    <row r="166" spans="1:23" ht="30" hidden="1">
       <c r="A166" s="4" t="s">
         <v>34</v>
       </c>
@@ -36449,7 +36450,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="167" spans="1:23" ht="30">
+    <row r="167" spans="1:23" ht="30" hidden="1">
       <c r="A167" s="4" t="s">
         <v>34</v>
       </c>
@@ -36520,7 +36521,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="168" spans="1:23" ht="30">
+    <row r="168" spans="1:23" ht="30" hidden="1">
       <c r="A168" s="4" t="s">
         <v>34</v>
       </c>
@@ -36591,7 +36592,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="169" spans="1:23" ht="30">
+    <row r="169" spans="1:23" ht="30" hidden="1">
       <c r="A169" s="4" t="s">
         <v>34</v>
       </c>
@@ -36662,7 +36663,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="170" spans="1:23" ht="30">
+    <row r="170" spans="1:23" ht="30" hidden="1">
       <c r="A170" s="4" t="s">
         <v>34</v>
       </c>
@@ -36733,7 +36734,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="171" spans="1:23" ht="30">
+    <row r="171" spans="1:23" ht="30" hidden="1">
       <c r="A171" s="4" t="s">
         <v>34</v>
       </c>
@@ -36804,7 +36805,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="172" spans="1:23" ht="30">
+    <row r="172" spans="1:23" ht="30" hidden="1">
       <c r="A172" s="4" t="s">
         <v>34</v>
       </c>
@@ -36875,7 +36876,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="173" spans="1:23">
+    <row r="173" spans="1:23" hidden="1">
       <c r="A173" s="4" t="s">
         <v>34</v>
       </c>
@@ -36946,7 +36947,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="174" spans="1:23" ht="30">
+    <row r="174" spans="1:23" ht="30" hidden="1">
       <c r="A174" s="4" t="s">
         <v>34</v>
       </c>
@@ -37017,7 +37018,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="175" spans="1:23" ht="30">
+    <row r="175" spans="1:23" ht="30" hidden="1">
       <c r="A175" s="4" t="s">
         <v>34</v>
       </c>
@@ -37088,7 +37089,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="176" spans="1:23" ht="30">
+    <row r="176" spans="1:23" ht="30" hidden="1">
       <c r="A176" s="4" t="s">
         <v>34</v>
       </c>
@@ -37159,7 +37160,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="177" spans="1:23" ht="30">
+    <row r="177" spans="1:23" ht="30" hidden="1">
       <c r="A177" s="4" t="s">
         <v>34</v>
       </c>
@@ -37230,7 +37231,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="178" spans="1:23" ht="30">
+    <row r="178" spans="1:23" ht="30" hidden="1">
       <c r="A178" s="4" t="s">
         <v>35</v>
       </c>
@@ -37301,7 +37302,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="179" spans="1:23" ht="30">
+    <row r="179" spans="1:23" ht="30" hidden="1">
       <c r="A179" s="4" t="s">
         <v>35</v>
       </c>
@@ -37372,7 +37373,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="180" spans="1:23" ht="30">
+    <row r="180" spans="1:23" ht="30" hidden="1">
       <c r="A180" s="4" t="s">
         <v>35</v>
       </c>
@@ -37443,7 +37444,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="181" spans="1:23" ht="30">
+    <row r="181" spans="1:23" ht="30" hidden="1">
       <c r="A181" s="4" t="s">
         <v>35</v>
       </c>
@@ -37514,7 +37515,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="182" spans="1:23">
+    <row r="182" spans="1:23" hidden="1">
       <c r="A182" s="4" t="s">
         <v>35</v>
       </c>
@@ -37565,7 +37566,7 @@
       <c r="V182" s="1"/>
       <c r="W182" s="1"/>
     </row>
-    <row r="183" spans="1:23">
+    <row r="183" spans="1:23" hidden="1">
       <c r="A183" s="4" t="s">
         <v>35</v>
       </c>
@@ -37614,7 +37615,7 @@
       <c r="V183" s="1"/>
       <c r="W183" s="1"/>
     </row>
-    <row r="184" spans="1:23" ht="30">
+    <row r="184" spans="1:23" ht="30" hidden="1">
       <c r="A184" s="3" t="s">
         <v>35</v>
       </c>
@@ -37685,7 +37686,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="185" spans="1:23" ht="30">
+    <row r="185" spans="1:23" ht="30" hidden="1">
       <c r="A185" s="3" t="s">
         <v>35</v>
       </c>
@@ -37756,7 +37757,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="186" spans="1:23" ht="30">
+    <row r="186" spans="1:23" ht="30" hidden="1">
       <c r="A186" s="4" t="s">
         <v>35</v>
       </c>
@@ -37827,7 +37828,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="187" spans="1:23" ht="30">
+    <row r="187" spans="1:23" ht="30" hidden="1">
       <c r="A187" s="4" t="s">
         <v>35</v>
       </c>
@@ -37898,7 +37899,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="188" spans="1:23" ht="30">
+    <row r="188" spans="1:23" ht="30" hidden="1">
       <c r="A188" s="4" t="s">
         <v>35</v>
       </c>
@@ -37969,7 +37970,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="189" spans="1:23" ht="30">
+    <row r="189" spans="1:23" ht="30" hidden="1">
       <c r="A189" s="4" t="s">
         <v>35</v>
       </c>
@@ -38040,7 +38041,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="190" spans="1:23" ht="30">
+    <row r="190" spans="1:23" ht="30" hidden="1">
       <c r="A190" s="4" t="s">
         <v>35</v>
       </c>
@@ -38111,7 +38112,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="191" spans="1:23" ht="30">
+    <row r="191" spans="1:23" ht="30" hidden="1">
       <c r="A191" s="4" t="s">
         <v>35</v>
       </c>
@@ -38182,7 +38183,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="192" spans="1:23" ht="30">
+    <row r="192" spans="1:23" ht="30" hidden="1">
       <c r="A192" s="4" t="s">
         <v>35</v>
       </c>
@@ -38253,7 +38254,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="193" spans="1:23" ht="30">
+    <row r="193" spans="1:23" ht="30" hidden="1">
       <c r="A193" s="4" t="s">
         <v>35</v>
       </c>
@@ -38324,7 +38325,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="194" spans="1:23" ht="30">
+    <row r="194" spans="1:23" ht="30" hidden="1">
       <c r="A194" s="4" t="s">
         <v>35</v>
       </c>
@@ -38395,7 +38396,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="195" spans="1:23" ht="30">
+    <row r="195" spans="1:23" ht="30" hidden="1">
       <c r="A195" s="4" t="s">
         <v>35</v>
       </c>
@@ -38466,7 +38467,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="196" spans="1:23" ht="30">
+    <row r="196" spans="1:23" ht="30" hidden="1">
       <c r="A196" s="4" t="s">
         <v>35</v>
       </c>
@@ -38537,7 +38538,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="197" spans="1:23" ht="30">
+    <row r="197" spans="1:23" ht="30" hidden="1">
       <c r="A197" s="3" t="s">
         <v>94</v>
       </c>
@@ -38604,7 +38605,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="198" spans="1:23" ht="30">
+    <row r="198" spans="1:23" ht="30" hidden="1">
       <c r="A198" s="3" t="s">
         <v>94</v>
       </c>
@@ -38673,7 +38674,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="199" spans="1:23" ht="30">
+    <row r="199" spans="1:23" ht="30" hidden="1">
       <c r="A199" s="3" t="s">
         <v>94</v>
       </c>
@@ -38742,7 +38743,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="200" spans="1:23" ht="30">
+    <row r="200" spans="1:23" ht="30" hidden="1">
       <c r="A200" s="3" t="s">
         <v>94</v>
       </c>
@@ -38811,7 +38812,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="201" spans="1:23" ht="30">
+    <row r="201" spans="1:23" ht="30" hidden="1">
       <c r="A201" s="3" t="s">
         <v>94</v>
       </c>
@@ -38880,7 +38881,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="202" spans="1:23" ht="30">
+    <row r="202" spans="1:23" ht="30" hidden="1">
       <c r="A202" s="3" t="s">
         <v>94</v>
       </c>
@@ -38949,7 +38950,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="203" spans="1:23">
+    <row r="203" spans="1:23" hidden="1">
       <c r="A203" s="3" t="s">
         <v>42</v>
       </c>
@@ -39016,7 +39017,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="204" spans="1:23">
+    <row r="204" spans="1:23" hidden="1">
       <c r="A204" s="3" t="s">
         <v>42</v>
       </c>
@@ -39085,7 +39086,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="205" spans="1:23">
+    <row r="205" spans="1:23" hidden="1">
       <c r="A205" s="3" t="s">
         <v>42</v>
       </c>
@@ -39154,7 +39155,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="206" spans="1:23" ht="30">
+    <row r="206" spans="1:23" ht="30" hidden="1">
       <c r="A206" s="3" t="s">
         <v>42</v>
       </c>
@@ -39223,7 +39224,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="207" spans="1:23">
+    <row r="207" spans="1:23" hidden="1">
       <c r="A207" s="3" t="s">
         <v>42</v>
       </c>
@@ -39292,7 +39293,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="208" spans="1:23" ht="30">
+    <row r="208" spans="1:23" ht="30" hidden="1">
       <c r="A208" s="3" t="s">
         <v>42</v>
       </c>
@@ -39361,7 +39362,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="209" spans="1:23">
+    <row r="209" spans="1:23" hidden="1">
       <c r="A209" s="3" t="s">
         <v>129</v>
       </c>
@@ -39428,7 +39429,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="210" spans="1:23">
+    <row r="210" spans="1:23" hidden="1">
       <c r="A210" s="3" t="s">
         <v>129</v>
       </c>
@@ -39497,7 +39498,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="211" spans="1:23">
+    <row r="211" spans="1:23" hidden="1">
       <c r="A211" s="3" t="s">
         <v>129</v>
       </c>
@@ -39566,7 +39567,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="212" spans="1:23">
+    <row r="212" spans="1:23" hidden="1">
       <c r="A212" s="3" t="s">
         <v>129</v>
       </c>
@@ -39635,7 +39636,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="213" spans="1:23">
+    <row r="213" spans="1:23" hidden="1">
       <c r="A213" s="3" t="s">
         <v>129</v>
       </c>
@@ -39704,7 +39705,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="214" spans="1:23" ht="30">
+    <row r="214" spans="1:23" ht="30" hidden="1">
       <c r="A214" s="3" t="s">
         <v>129</v>
       </c>
@@ -39773,7 +39774,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="215" spans="1:23" ht="30">
+    <row r="215" spans="1:23" ht="30" hidden="1">
       <c r="A215" s="3" t="s">
         <v>129</v>
       </c>
@@ -39842,7 +39843,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="216" spans="1:23">
+    <row r="216" spans="1:23" hidden="1">
       <c r="A216" s="3" t="s">
         <v>126</v>
       </c>
@@ -39909,7 +39910,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="217" spans="1:23">
+    <row r="217" spans="1:23" hidden="1">
       <c r="A217" s="3" t="s">
         <v>126</v>
       </c>
@@ -39978,7 +39979,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="218" spans="1:23">
+    <row r="218" spans="1:23" hidden="1">
       <c r="A218" s="3" t="s">
         <v>126</v>
       </c>
@@ -40047,7 +40048,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="219" spans="1:23" ht="30">
+    <row r="219" spans="1:23" ht="30" hidden="1">
       <c r="A219" s="3" t="s">
         <v>126</v>
       </c>
@@ -40116,7 +40117,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="220" spans="1:23" ht="30">
+    <row r="220" spans="1:23" ht="30" hidden="1">
       <c r="A220" s="3" t="s">
         <v>126</v>
       </c>
@@ -40185,7 +40186,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="221" spans="1:23">
+    <row r="221" spans="1:23" hidden="1">
       <c r="A221" s="3" t="s">
         <v>126</v>
       </c>
@@ -40254,7 +40255,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="222" spans="1:23" ht="30">
+    <row r="222" spans="1:23" ht="30" hidden="1">
       <c r="A222" s="3" t="s">
         <v>126</v>
       </c>
@@ -40323,7 +40324,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="223" spans="1:23" ht="30">
+    <row r="223" spans="1:23" ht="30" hidden="1">
       <c r="A223" s="3" t="s">
         <v>126</v>
       </c>
@@ -40392,7 +40393,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="224" spans="1:23" ht="30">
+    <row r="224" spans="1:23" ht="30" hidden="1">
       <c r="A224" s="3" t="s">
         <v>313</v>
       </c>
@@ -40459,7 +40460,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="225" spans="1:23" ht="30">
+    <row r="225" spans="1:23" ht="30" hidden="1">
       <c r="A225" s="3" t="s">
         <v>313</v>
       </c>
@@ -40528,7 +40529,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="226" spans="1:23" ht="30">
+    <row r="226" spans="1:23" ht="30" hidden="1">
       <c r="A226" s="3" t="s">
         <v>313</v>
       </c>
@@ -40597,7 +40598,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="227" spans="1:23" ht="30">
+    <row r="227" spans="1:23" ht="30" hidden="1">
       <c r="A227" s="3" t="s">
         <v>313</v>
       </c>
@@ -40666,7 +40667,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="228" spans="1:23" ht="30">
+    <row r="228" spans="1:23" ht="30" hidden="1">
       <c r="A228" s="3" t="s">
         <v>313</v>
       </c>
@@ -40735,7 +40736,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="229" spans="1:23" ht="45">
+    <row r="229" spans="1:23" ht="45" hidden="1">
       <c r="A229" s="3" t="s">
         <v>313</v>
       </c>
@@ -40804,7 +40805,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="230" spans="1:23" ht="30">
+    <row r="230" spans="1:23" ht="30" hidden="1">
       <c r="A230" s="3" t="s">
         <v>445</v>
       </c>
@@ -40871,7 +40872,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="231" spans="1:23" ht="30">
+    <row r="231" spans="1:23" ht="30" hidden="1">
       <c r="A231" s="3" t="s">
         <v>445</v>
       </c>
@@ -40940,7 +40941,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="232" spans="1:23" ht="30">
+    <row r="232" spans="1:23" ht="30" hidden="1">
       <c r="A232" s="3" t="s">
         <v>445</v>
       </c>
@@ -41009,7 +41010,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="233" spans="1:23" ht="30">
+    <row r="233" spans="1:23" ht="30" hidden="1">
       <c r="A233" s="3" t="s">
         <v>445</v>
       </c>
@@ -41078,7 +41079,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="234" spans="1:23" ht="30">
+    <row r="234" spans="1:23" ht="30" hidden="1">
       <c r="A234" s="3" t="s">
         <v>445</v>
       </c>
@@ -41147,7 +41148,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="235" spans="1:23" ht="30">
+    <row r="235" spans="1:23" ht="30" hidden="1">
       <c r="A235" s="3" t="s">
         <v>445</v>
       </c>
@@ -41216,7 +41217,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="236" spans="1:23" ht="30">
+    <row r="236" spans="1:23" ht="30" hidden="1">
       <c r="A236" s="3" t="s">
         <v>451</v>
       </c>
@@ -41283,7 +41284,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="237" spans="1:23">
+    <row r="237" spans="1:23" hidden="1">
       <c r="A237" s="3" t="s">
         <v>451</v>
       </c>
@@ -41352,7 +41353,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="238" spans="1:23">
+    <row r="238" spans="1:23" hidden="1">
       <c r="A238" s="3" t="s">
         <v>451</v>
       </c>
@@ -41421,7 +41422,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="239" spans="1:23" ht="30">
+    <row r="239" spans="1:23" ht="30" hidden="1">
       <c r="A239" s="3" t="s">
         <v>451</v>
       </c>
@@ -41490,7 +41491,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="240" spans="1:23">
+    <row r="240" spans="1:23" hidden="1">
       <c r="A240" s="3" t="s">
         <v>451</v>
       </c>
@@ -41559,7 +41560,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="241" spans="1:23" ht="30">
+    <row r="241" spans="1:23" ht="30" hidden="1">
       <c r="A241" s="3" t="s">
         <v>451</v>
       </c>
@@ -41628,7 +41629,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="242" spans="1:23" ht="30">
+    <row r="242" spans="1:23" ht="30" hidden="1">
       <c r="A242" s="3" t="s">
         <v>512</v>
       </c>
@@ -41695,7 +41696,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="243" spans="1:23" ht="30">
+    <row r="243" spans="1:23" ht="30" hidden="1">
       <c r="A243" s="3" t="s">
         <v>512</v>
       </c>
@@ -41764,7 +41765,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="244" spans="1:23" ht="30">
+    <row r="244" spans="1:23" ht="30" hidden="1">
       <c r="A244" s="3" t="s">
         <v>512</v>
       </c>
@@ -41833,7 +41834,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="245" spans="1:23" ht="30">
+    <row r="245" spans="1:23" ht="30" hidden="1">
       <c r="A245" s="3" t="s">
         <v>512</v>
       </c>
@@ -41902,7 +41903,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="246" spans="1:23" ht="30">
+    <row r="246" spans="1:23" ht="30" hidden="1">
       <c r="A246" s="3" t="s">
         <v>512</v>
       </c>
@@ -41971,7 +41972,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="247" spans="1:23" ht="30">
+    <row r="247" spans="1:23" ht="30" hidden="1">
       <c r="A247" s="3" t="s">
         <v>512</v>
       </c>
@@ -42040,7 +42041,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="248" spans="1:23" ht="30">
+    <row r="248" spans="1:23" ht="30" hidden="1">
       <c r="A248" s="3" t="s">
         <v>518</v>
       </c>
@@ -42107,7 +42108,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="249" spans="1:23">
+    <row r="249" spans="1:23" hidden="1">
       <c r="A249" s="3" t="s">
         <v>518</v>
       </c>
@@ -42176,7 +42177,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="250" spans="1:23">
+    <row r="250" spans="1:23" hidden="1">
       <c r="A250" s="3" t="s">
         <v>518</v>
       </c>
@@ -42245,7 +42246,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="251" spans="1:23" ht="30">
+    <row r="251" spans="1:23" ht="30" hidden="1">
       <c r="A251" s="3" t="s">
         <v>518</v>
       </c>
@@ -42314,7 +42315,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="252" spans="1:23">
+    <row r="252" spans="1:23" hidden="1">
       <c r="A252" s="3" t="s">
         <v>518</v>
       </c>
@@ -42383,7 +42384,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="253" spans="1:23" ht="30">
+    <row r="253" spans="1:23" ht="30" hidden="1">
       <c r="A253" s="3" t="s">
         <v>518</v>
       </c>
@@ -42452,7 +42453,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="254" spans="1:23" ht="30">
+    <row r="254" spans="1:23" ht="30" hidden="1">
       <c r="A254" s="3" t="s">
         <v>756</v>
       </c>
@@ -42519,7 +42520,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="255" spans="1:23">
+    <row r="255" spans="1:23" hidden="1">
       <c r="A255" s="3" t="s">
         <v>756</v>
       </c>
@@ -42588,7 +42589,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="256" spans="1:23">
+    <row r="256" spans="1:23" hidden="1">
       <c r="A256" s="3" t="s">
         <v>756</v>
       </c>
@@ -42657,7 +42658,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="257" spans="1:23">
+    <row r="257" spans="1:23" hidden="1">
       <c r="A257" s="3" t="s">
         <v>756</v>
       </c>
@@ -42726,7 +42727,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="258" spans="1:23">
+    <row r="258" spans="1:23" hidden="1">
       <c r="A258" s="3" t="s">
         <v>756</v>
       </c>
@@ -42795,7 +42796,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="259" spans="1:23" ht="30">
+    <row r="259" spans="1:23" ht="30" hidden="1">
       <c r="A259" s="3" t="s">
         <v>756</v>
       </c>
@@ -42864,7 +42865,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="260" spans="1:23" ht="30">
+    <row r="260" spans="1:23" ht="30" hidden="1">
       <c r="A260" s="3" t="s">
         <v>1514</v>
       </c>
@@ -42931,7 +42932,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="261" spans="1:23" ht="30">
+    <row r="261" spans="1:23" ht="30" hidden="1">
       <c r="A261" s="3" t="s">
         <v>1514</v>
       </c>
@@ -42998,7 +42999,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="262" spans="1:23" ht="30">
+    <row r="262" spans="1:23" ht="30" hidden="1">
       <c r="A262" s="3" t="s">
         <v>1514</v>
       </c>
@@ -43067,7 +43068,7 @@
         <v>1443</v>
       </c>
     </row>
-    <row r="263" spans="1:23" ht="30">
+    <row r="263" spans="1:23" ht="30" hidden="1">
       <c r="A263" s="3" t="s">
         <v>1514</v>
       </c>
@@ -43136,7 +43137,7 @@
         <v>1443</v>
       </c>
     </row>
-    <row r="264" spans="1:23">
+    <row r="264" spans="1:23" hidden="1">
       <c r="A264" s="3" t="s">
         <v>1514</v>
       </c>
@@ -43205,7 +43206,7 @@
         <v>1443</v>
       </c>
     </row>
-    <row r="265" spans="1:23" ht="30">
+    <row r="265" spans="1:23" ht="30" hidden="1">
       <c r="A265" s="3" t="s">
         <v>1514</v>
       </c>
@@ -43274,7 +43275,7 @@
         <v>1443</v>
       </c>
     </row>
-    <row r="266" spans="1:23">
+    <row r="266" spans="1:23" hidden="1">
       <c r="A266" s="3" t="s">
         <v>1514</v>
       </c>
@@ -43343,7 +43344,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="267" spans="1:23">
+    <row r="267" spans="1:23" hidden="1">
       <c r="A267" s="3" t="s">
         <v>1514</v>
       </c>
@@ -43412,7 +43413,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="268" spans="1:23">
+    <row r="268" spans="1:23" hidden="1">
       <c r="A268" s="3" t="s">
         <v>1514</v>
       </c>
@@ -43481,7 +43482,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="269" spans="1:23">
+    <row r="269" spans="1:23" hidden="1">
       <c r="A269" s="3" t="s">
         <v>1514</v>
       </c>
@@ -43550,7 +43551,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="270" spans="1:23">
+    <row r="270" spans="1:23" hidden="1">
       <c r="A270" s="3" t="s">
         <v>1514</v>
       </c>
@@ -43619,7 +43620,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="271" spans="1:23">
+    <row r="271" spans="1:23" hidden="1">
       <c r="A271" s="3" t="s">
         <v>1514</v>
       </c>
@@ -43688,7 +43689,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="272" spans="1:23" ht="30">
+    <row r="272" spans="1:23" ht="30" hidden="1">
       <c r="A272" s="3" t="s">
         <v>1514</v>
       </c>
@@ -43757,7 +43758,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="273" spans="1:23" ht="30">
+    <row r="273" spans="1:23" ht="30" hidden="1">
       <c r="A273" s="3" t="s">
         <v>1514</v>
       </c>
@@ -43826,7 +43827,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="274" spans="1:23">
+    <row r="274" spans="1:23" hidden="1">
       <c r="A274" s="3" t="s">
         <v>1514</v>
       </c>
@@ -43893,7 +43894,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="275" spans="1:23">
+    <row r="275" spans="1:23" hidden="1">
       <c r="A275" s="3" t="s">
         <v>1514</v>
       </c>
@@ -43960,7 +43961,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="276" spans="1:23">
+    <row r="276" spans="1:23" hidden="1">
       <c r="A276" s="3" t="s">
         <v>1514</v>
       </c>
@@ -44027,7 +44028,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="277" spans="1:23">
+    <row r="277" spans="1:23" hidden="1">
       <c r="A277" s="3" t="s">
         <v>1514</v>
       </c>
@@ -44096,7 +44097,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="278" spans="1:23">
+    <row r="278" spans="1:23" hidden="1">
       <c r="A278" s="3" t="s">
         <v>1514</v>
       </c>
@@ -44165,7 +44166,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="279" spans="1:23" ht="30">
+    <row r="279" spans="1:23" ht="30" hidden="1">
       <c r="A279" s="3" t="s">
         <v>1515</v>
       </c>
@@ -44232,7 +44233,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="280" spans="1:23" ht="30">
+    <row r="280" spans="1:23" ht="30" hidden="1">
       <c r="A280" s="3" t="s">
         <v>1515</v>
       </c>
@@ -44299,7 +44300,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="281" spans="1:23" ht="30">
+    <row r="281" spans="1:23" ht="30" hidden="1">
       <c r="A281" s="3" t="s">
         <v>1515</v>
       </c>
@@ -44370,7 +44371,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="282" spans="1:23">
+    <row r="282" spans="1:23" hidden="1">
       <c r="A282" s="3" t="s">
         <v>1515</v>
       </c>
@@ -44437,7 +44438,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="283" spans="1:23" ht="30">
+    <row r="283" spans="1:23" ht="30" hidden="1">
       <c r="A283" s="3" t="s">
         <v>1515</v>
       </c>
@@ -44506,7 +44507,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="284" spans="1:23">
+    <row r="284" spans="1:23" hidden="1">
       <c r="A284" s="3" t="s">
         <v>1515</v>
       </c>
@@ -44575,7 +44576,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="285" spans="1:23">
+    <row r="285" spans="1:23" hidden="1">
       <c r="A285" s="3" t="s">
         <v>1515</v>
       </c>
@@ -44644,7 +44645,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="286" spans="1:23" ht="45">
+    <row r="286" spans="1:23" ht="45" hidden="1">
       <c r="A286" s="3" t="s">
         <v>1515</v>
       </c>
@@ -44713,7 +44714,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="287" spans="1:23" ht="30">
+    <row r="287" spans="1:23" ht="30" hidden="1">
       <c r="A287" s="3" t="s">
         <v>1515</v>
       </c>
@@ -44782,7 +44783,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="288" spans="1:23" ht="45">
+    <row r="288" spans="1:23" ht="30" hidden="1">
       <c r="A288" s="3" t="s">
         <v>1515</v>
       </c>
@@ -44851,7 +44852,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="289" spans="1:23" ht="45">
+    <row r="289" spans="1:23" ht="45" hidden="1">
       <c r="A289" s="3" t="s">
         <v>1515</v>
       </c>
@@ -44920,7 +44921,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="290" spans="1:23" ht="30">
+    <row r="290" spans="1:23" ht="30" hidden="1">
       <c r="A290" s="3" t="s">
         <v>1515</v>
       </c>
@@ -44987,7 +44988,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="291" spans="1:23" ht="30">
+    <row r="291" spans="1:23" ht="30" hidden="1">
       <c r="A291" s="3" t="s">
         <v>1515</v>
       </c>
@@ -45054,7 +45055,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="292" spans="1:23">
+    <row r="292" spans="1:23" hidden="1">
       <c r="A292" s="3" t="s">
         <v>1515</v>
       </c>
@@ -45119,7 +45120,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="293" spans="1:23">
+    <row r="293" spans="1:23" hidden="1">
       <c r="A293" s="3" t="s">
         <v>1515</v>
       </c>
@@ -45184,7 +45185,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="294" spans="1:23">
+    <row r="294" spans="1:23" hidden="1">
       <c r="A294" s="3" t="s">
         <v>1515</v>
       </c>
@@ -45249,7 +45250,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="295" spans="1:23">
+    <row r="295" spans="1:23" hidden="1">
       <c r="A295" s="3" t="s">
         <v>1515</v>
       </c>
@@ -45318,7 +45319,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="296" spans="1:23">
+    <row r="296" spans="1:23" hidden="1">
       <c r="A296" s="3" t="s">
         <v>1515</v>
       </c>
@@ -45387,7 +45388,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="297" spans="1:23" ht="30">
+    <row r="297" spans="1:23" ht="30" hidden="1">
       <c r="A297" s="3" t="s">
         <v>1575</v>
       </c>
@@ -45454,7 +45455,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="298" spans="1:23" ht="30">
+    <row r="298" spans="1:23" ht="30" hidden="1">
       <c r="A298" s="3" t="s">
         <v>1575</v>
       </c>
@@ -45521,7 +45522,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="299" spans="1:23" ht="45">
+    <row r="299" spans="1:23" ht="45" hidden="1">
       <c r="A299" s="3" t="s">
         <v>1575</v>
       </c>
@@ -45592,7 +45593,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="300" spans="1:23" ht="30">
+    <row r="300" spans="1:23" ht="30" hidden="1">
       <c r="A300" s="3" t="s">
         <v>1575</v>
       </c>
@@ -45661,7 +45662,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="301" spans="1:23" ht="30">
+    <row r="301" spans="1:23" ht="30" hidden="1">
       <c r="A301" s="3" t="s">
         <v>1575</v>
       </c>
@@ -45730,7 +45731,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="302" spans="1:23" ht="30">
+    <row r="302" spans="1:23" ht="30" hidden="1">
       <c r="A302" s="3" t="s">
         <v>1575</v>
       </c>
@@ -45799,7 +45800,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="303" spans="1:23" ht="30">
+    <row r="303" spans="1:23" ht="30" hidden="1">
       <c r="A303" s="3" t="s">
         <v>1575</v>
       </c>
@@ -45868,7 +45869,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="304" spans="1:23" ht="30">
+    <row r="304" spans="1:23" ht="30" hidden="1">
       <c r="A304" s="3" t="s">
         <v>1575</v>
       </c>
@@ -45937,7 +45938,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="305" spans="1:23" ht="30">
+    <row r="305" spans="1:23" ht="30" hidden="1">
       <c r="A305" s="3" t="s">
         <v>1575</v>
       </c>
@@ -46004,7 +46005,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="306" spans="1:23" ht="30">
+    <row r="306" spans="1:23" ht="30" hidden="1">
       <c r="A306" s="3" t="s">
         <v>1575</v>
       </c>
@@ -46071,7 +46072,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="307" spans="1:23" ht="30">
+    <row r="307" spans="1:23" ht="30" hidden="1">
       <c r="A307" s="3" t="s">
         <v>1575</v>
       </c>
@@ -46136,7 +46137,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="308" spans="1:23" ht="30">
+    <row r="308" spans="1:23" ht="30" hidden="1">
       <c r="A308" s="3" t="s">
         <v>1575</v>
       </c>
@@ -46201,7 +46202,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="309" spans="1:23" ht="30">
+    <row r="309" spans="1:23" ht="30" hidden="1">
       <c r="A309" s="3" t="s">
         <v>1575</v>
       </c>
@@ -46266,7 +46267,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="310" spans="1:23" ht="30">
+    <row r="310" spans="1:23" ht="30" hidden="1">
       <c r="A310" s="3" t="s">
         <v>1575</v>
       </c>
@@ -46335,7 +46336,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="311" spans="1:23" ht="30">
+    <row r="311" spans="1:23" ht="30" hidden="1">
       <c r="A311" s="3" t="s">
         <v>1575</v>
       </c>
@@ -46404,7 +46405,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="312" spans="1:23" ht="30">
+    <row r="312" spans="1:23" ht="30" hidden="1">
       <c r="A312" s="3" t="s">
         <v>1632</v>
       </c>
@@ -46471,7 +46472,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="313" spans="1:23" ht="30">
+    <row r="313" spans="1:23" ht="30" hidden="1">
       <c r="A313" s="3" t="s">
         <v>1632</v>
       </c>
@@ -46538,7 +46539,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="314" spans="1:23" ht="45">
+    <row r="314" spans="1:23" ht="45" hidden="1">
       <c r="A314" s="3" t="s">
         <v>1632</v>
       </c>
@@ -46607,7 +46608,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="315" spans="1:23">
+    <row r="315" spans="1:23" hidden="1">
       <c r="A315" s="3" t="s">
         <v>1632</v>
       </c>
@@ -46674,7 +46675,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="316" spans="1:23">
+    <row r="316" spans="1:23" hidden="1">
       <c r="A316" s="3" t="s">
         <v>1632</v>
       </c>
@@ -46741,7 +46742,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="317" spans="1:23" ht="30">
+    <row r="317" spans="1:23" ht="30" hidden="1">
       <c r="A317" s="3" t="s">
         <v>1632</v>
       </c>
@@ -46808,7 +46809,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="318" spans="1:23">
+    <row r="318" spans="1:23" hidden="1">
       <c r="A318" s="3" t="s">
         <v>1632</v>
       </c>
@@ -46875,7 +46876,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="319" spans="1:23" ht="45">
+    <row r="319" spans="1:23" ht="45" hidden="1">
       <c r="A319" s="3" t="s">
         <v>1632</v>
       </c>
@@ -46944,7 +46945,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="320" spans="1:23" ht="30">
+    <row r="320" spans="1:23" ht="30" hidden="1">
       <c r="A320" s="3" t="s">
         <v>1632</v>
       </c>
@@ -47009,7 +47010,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="321" spans="1:23" ht="30">
+    <row r="321" spans="1:23" ht="30" hidden="1">
       <c r="A321" s="3" t="s">
         <v>1632</v>
       </c>
@@ -47078,7 +47079,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="322" spans="1:23" ht="30">
+    <row r="322" spans="1:23" ht="30" hidden="1">
       <c r="A322" s="3" t="s">
         <v>1632</v>
       </c>
@@ -47145,7 +47146,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="323" spans="1:23" ht="30">
+    <row r="323" spans="1:23" ht="30" hidden="1">
       <c r="A323" s="3" t="s">
         <v>1686</v>
       </c>
@@ -47212,7 +47213,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="324" spans="1:23" ht="30">
+    <row r="324" spans="1:23" ht="30" hidden="1">
       <c r="A324" s="3" t="s">
         <v>1686</v>
       </c>
@@ -47279,7 +47280,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="325" spans="1:23" ht="30">
+    <row r="325" spans="1:23" ht="30" hidden="1">
       <c r="A325" s="3" t="s">
         <v>1686</v>
       </c>
@@ -47348,7 +47349,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="326" spans="1:23" ht="30">
+    <row r="326" spans="1:23" ht="30" hidden="1">
       <c r="A326" s="3" t="s">
         <v>1686</v>
       </c>
@@ -47415,7 +47416,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="327" spans="1:23" ht="30">
+    <row r="327" spans="1:23" ht="30" hidden="1">
       <c r="A327" s="3" t="s">
         <v>1686</v>
       </c>
@@ -47484,7 +47485,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="328" spans="1:23" ht="30">
+    <row r="328" spans="1:23" ht="30" hidden="1">
       <c r="A328" s="3" t="s">
         <v>1686</v>
       </c>
@@ -47553,7 +47554,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="329" spans="1:23" ht="30">
+    <row r="329" spans="1:23" ht="30" hidden="1">
       <c r="A329" s="3" t="s">
         <v>1686</v>
       </c>
@@ -47620,7 +47621,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="330" spans="1:23" ht="30">
+    <row r="330" spans="1:23" ht="30" hidden="1">
       <c r="A330" s="3" t="s">
         <v>1686</v>
       </c>
@@ -47687,7 +47688,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="331" spans="1:23" ht="30">
+    <row r="331" spans="1:23" ht="30" hidden="1">
       <c r="A331" s="3" t="s">
         <v>1686</v>
       </c>
@@ -47752,7 +47753,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="332" spans="1:23" ht="30">
+    <row r="332" spans="1:23" ht="30" hidden="1">
       <c r="A332" s="3" t="s">
         <v>1686</v>
       </c>
@@ -47819,7 +47820,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="333" spans="1:23" ht="45">
+    <row r="333" spans="1:23" ht="45" hidden="1">
       <c r="A333" s="3" t="s">
         <v>1686</v>
       </c>
@@ -47888,7 +47889,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="334" spans="1:23" ht="30">
+    <row r="334" spans="1:23" ht="30" hidden="1">
       <c r="A334" s="3" t="s">
         <v>1686</v>
       </c>
@@ -47957,7 +47958,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="335" spans="1:23" ht="30">
+    <row r="335" spans="1:23" ht="30" hidden="1">
       <c r="A335" s="3" t="s">
         <v>1701</v>
       </c>
@@ -48024,7 +48025,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="336" spans="1:23" ht="30">
+    <row r="336" spans="1:23" ht="30" hidden="1">
       <c r="A336" s="3" t="s">
         <v>1701</v>
       </c>
@@ -48093,7 +48094,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="337" spans="1:23">
+    <row r="337" spans="1:23" hidden="1">
       <c r="A337" s="3" t="s">
         <v>1701</v>
       </c>
@@ -48162,7 +48163,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="338" spans="1:23" ht="30">
+    <row r="338" spans="1:23" ht="30" hidden="1">
       <c r="A338" s="3" t="s">
         <v>1701</v>
       </c>
@@ -48231,7 +48232,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="339" spans="1:23">
+    <row r="339" spans="1:23" hidden="1">
       <c r="A339" s="3" t="s">
         <v>1701</v>
       </c>
@@ -48300,7 +48301,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="340" spans="1:23" ht="30">
+    <row r="340" spans="1:23" ht="30" hidden="1">
       <c r="A340" s="3" t="s">
         <v>1701</v>
       </c>
@@ -48369,7 +48370,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="341" spans="1:23" ht="30">
+    <row r="341" spans="1:23" ht="30" hidden="1">
       <c r="A341" s="3" t="s">
         <v>1701</v>
       </c>
@@ -48436,7 +48437,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="342" spans="1:23">
+    <row r="342" spans="1:23" hidden="1">
       <c r="A342" s="3" t="s">
         <v>1701</v>
       </c>
@@ -48501,7 +48502,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="343" spans="1:23" ht="30">
+    <row r="343" spans="1:23" ht="30" hidden="1">
       <c r="A343" s="3" t="s">
         <v>1701</v>
       </c>
@@ -48570,7 +48571,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="344" spans="1:23">
+    <row r="344" spans="1:23" hidden="1">
       <c r="A344" s="3" t="s">
         <v>1701</v>
       </c>
@@ -48639,7 +48640,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="345" spans="1:23" ht="30">
+    <row r="345" spans="1:23" ht="30" hidden="1">
       <c r="A345" s="3" t="s">
         <v>1803</v>
       </c>
@@ -48706,7 +48707,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="346" spans="1:23" ht="30">
+    <row r="346" spans="1:23" ht="30" hidden="1">
       <c r="A346" s="3" t="s">
         <v>1803</v>
       </c>
@@ -48773,7 +48774,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="347" spans="1:23" ht="30">
+    <row r="347" spans="1:23" ht="30" hidden="1">
       <c r="A347" s="3" t="s">
         <v>1803</v>
       </c>
@@ -48840,7 +48841,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="348" spans="1:23" ht="30">
+    <row r="348" spans="1:23" ht="30" hidden="1">
       <c r="A348" s="3" t="s">
         <v>1803</v>
       </c>
@@ -48909,7 +48910,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="349" spans="1:23" ht="45">
+    <row r="349" spans="1:23" ht="45" hidden="1">
       <c r="A349" s="3" t="s">
         <v>1803</v>
       </c>
@@ -48978,7 +48979,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="350" spans="1:23" ht="30">
+    <row r="350" spans="1:23" ht="30" hidden="1">
       <c r="A350" s="3" t="s">
         <v>1803</v>
       </c>
@@ -49045,7 +49046,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="351" spans="1:23" ht="30">
+    <row r="351" spans="1:23" ht="30" hidden="1">
       <c r="A351" s="3" t="s">
         <v>1803</v>
       </c>
@@ -49112,7 +49113,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="352" spans="1:23" ht="30">
+    <row r="352" spans="1:23" ht="30" hidden="1">
       <c r="A352" s="3" t="s">
         <v>1803</v>
       </c>
@@ -49181,7 +49182,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="353" spans="1:23" ht="30">
+    <row r="353" spans="1:23" ht="30" hidden="1">
       <c r="A353" s="3" t="s">
         <v>1803</v>
       </c>
@@ -49248,7 +49249,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="354" spans="1:23" ht="30">
+    <row r="354" spans="1:23" ht="30" hidden="1">
       <c r="A354" s="3" t="s">
         <v>1803</v>
       </c>
@@ -49315,7 +49316,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="355" spans="1:23" ht="30">
+    <row r="355" spans="1:23" ht="30" hidden="1">
       <c r="A355" s="3" t="s">
         <v>1803</v>
       </c>
@@ -49380,7 +49381,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="356" spans="1:23" ht="30">
+    <row r="356" spans="1:23" ht="30" hidden="1">
       <c r="A356" s="3" t="s">
         <v>1803</v>
       </c>
@@ -49447,7 +49448,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="357" spans="1:23" ht="45">
+    <row r="357" spans="1:23" ht="45" hidden="1">
       <c r="A357" s="3" t="s">
         <v>1803</v>
       </c>
@@ -49516,7 +49517,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="358" spans="1:23" ht="30">
+    <row r="358" spans="1:23" ht="30" hidden="1">
       <c r="A358" s="3" t="s">
         <v>1803</v>
       </c>
@@ -49585,7 +49586,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="359" spans="1:23">
+    <row r="359" spans="1:23" hidden="1">
       <c r="A359" s="3" t="s">
         <v>1911</v>
       </c>
@@ -49654,7 +49655,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="360" spans="1:23">
+    <row r="360" spans="1:23" hidden="1">
       <c r="A360" s="3" t="s">
         <v>1911</v>
       </c>
@@ -49723,7 +49724,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="361" spans="1:23">
+    <row r="361" spans="1:23" hidden="1">
       <c r="A361" s="3" t="s">
         <v>1911</v>
       </c>
@@ -49792,7 +49793,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="362" spans="1:23" ht="30">
+    <row r="362" spans="1:23" ht="30" hidden="1">
       <c r="A362" s="3" t="s">
         <v>1911</v>
       </c>
@@ -49861,7 +49862,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="363" spans="1:23" ht="30">
+    <row r="363" spans="1:23" ht="30" hidden="1">
       <c r="A363" s="3" t="s">
         <v>1911</v>
       </c>
@@ -49930,7 +49931,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="364" spans="1:23" ht="30">
+    <row r="364" spans="1:23" ht="30" hidden="1">
       <c r="A364" s="3" t="s">
         <v>1911</v>
       </c>
@@ -50001,7 +50002,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="365" spans="1:23" ht="30">
+    <row r="365" spans="1:23" ht="30" hidden="1">
       <c r="A365" s="3" t="s">
         <v>1911</v>
       </c>
@@ -50070,7 +50071,7 @@
         <v>1956</v>
       </c>
     </row>
-    <row r="366" spans="1:23">
+    <row r="366" spans="1:23" hidden="1">
       <c r="A366" s="3" t="s">
         <v>1911</v>
       </c>
@@ -50141,7 +50142,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="367" spans="1:23" ht="30">
+    <row r="367" spans="1:23" ht="30" hidden="1">
       <c r="A367" s="3" t="s">
         <v>1911</v>
       </c>
@@ -50212,7 +50213,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="368" spans="1:23" ht="45">
+    <row r="368" spans="1:23" ht="45" hidden="1">
       <c r="A368" s="3" t="s">
         <v>1911</v>
       </c>
@@ -50283,7 +50284,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="369" spans="1:23" ht="30">
+    <row r="369" spans="1:23" ht="30" hidden="1">
       <c r="A369" s="3" t="s">
         <v>1911</v>
       </c>
@@ -50354,7 +50355,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="370" spans="1:23">
+    <row r="370" spans="1:23" hidden="1">
       <c r="A370" s="3" t="s">
         <v>1911</v>
       </c>
@@ -50423,7 +50424,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="371" spans="1:23" ht="30">
+    <row r="371" spans="1:23" ht="30" hidden="1">
       <c r="A371" s="3" t="s">
         <v>1911</v>
       </c>
@@ -50494,7 +50495,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="372" spans="1:23" ht="30">
+    <row r="372" spans="1:23" ht="30" hidden="1">
       <c r="A372" s="3" t="s">
         <v>1911</v>
       </c>
@@ -50563,7 +50564,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="373" spans="1:23" ht="30">
+    <row r="373" spans="1:23" ht="30" hidden="1">
       <c r="A373" s="3" t="s">
         <v>1911</v>
       </c>
@@ -50634,7 +50635,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="374" spans="1:23" ht="30">
+    <row r="374" spans="1:23" ht="30" hidden="1">
       <c r="A374" s="3" t="s">
         <v>1911</v>
       </c>
@@ -50705,7 +50706,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="375" spans="1:23" ht="30">
+    <row r="375" spans="1:23" ht="30" hidden="1">
       <c r="A375" s="3" t="s">
         <v>1919</v>
       </c>
@@ -50774,7 +50775,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="376" spans="1:23" ht="30">
+    <row r="376" spans="1:23" ht="30" hidden="1">
       <c r="A376" s="3" t="s">
         <v>1919</v>
       </c>
@@ -50843,7 +50844,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="377" spans="1:23">
+    <row r="377" spans="1:23" hidden="1">
       <c r="A377" s="3" t="s">
         <v>1919</v>
       </c>
@@ -50912,7 +50913,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="378" spans="1:23" ht="45">
+    <row r="378" spans="1:23" ht="45" hidden="1">
       <c r="A378" s="3" t="s">
         <v>1919</v>
       </c>
@@ -50981,7 +50982,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="379" spans="1:23" ht="30">
+    <row r="379" spans="1:23" ht="30" hidden="1">
       <c r="A379" s="3" t="s">
         <v>1919</v>
       </c>
@@ -51052,7 +51053,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="380" spans="1:23" ht="30">
+    <row r="380" spans="1:23" ht="30" hidden="1">
       <c r="A380" s="4" t="s">
         <v>2014</v>
       </c>
@@ -51123,7 +51124,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="381" spans="1:23" ht="30">
+    <row r="381" spans="1:23" ht="30" hidden="1">
       <c r="A381" s="4" t="s">
         <v>2014</v>
       </c>
@@ -51194,7 +51195,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="382" spans="1:23" ht="30">
+    <row r="382" spans="1:23" ht="30" hidden="1">
       <c r="A382" s="4" t="s">
         <v>2014</v>
       </c>
@@ -51265,7 +51266,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="383" spans="1:23" ht="45">
+    <row r="383" spans="1:23" ht="45" hidden="1">
       <c r="A383" s="4" t="s">
         <v>2014</v>
       </c>
@@ -51336,7 +51337,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="384" spans="1:23" ht="30">
+    <row r="384" spans="1:23" ht="30" hidden="1">
       <c r="A384" s="4" t="s">
         <v>2014</v>
       </c>
@@ -51407,7 +51408,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="385" spans="1:23" ht="30">
+    <row r="385" spans="1:23" ht="30" hidden="1">
       <c r="A385" s="4" t="s">
         <v>2014</v>
       </c>
@@ -51478,7 +51479,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="386" spans="1:23" ht="30">
+    <row r="386" spans="1:23" ht="30" hidden="1">
       <c r="A386" s="4" t="s">
         <v>2014</v>
       </c>
@@ -51549,7 +51550,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="387" spans="1:23" ht="30">
+    <row r="387" spans="1:23" ht="30" hidden="1">
       <c r="A387" s="4" t="s">
         <v>2014</v>
       </c>
@@ -51620,7 +51621,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="388" spans="1:23" ht="30">
+    <row r="388" spans="1:23" ht="30" hidden="1">
       <c r="A388" s="4" t="s">
         <v>2014</v>
       </c>
@@ -51691,7 +51692,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="389" spans="1:23" ht="30">
+    <row r="389" spans="1:23" ht="30" hidden="1">
       <c r="A389" s="4" t="s">
         <v>2014</v>
       </c>
@@ -51762,7 +51763,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="390" spans="1:23" ht="30">
+    <row r="390" spans="1:23" ht="30" hidden="1">
       <c r="A390" s="4" t="s">
         <v>2058</v>
       </c>
@@ -51833,7 +51834,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="391" spans="1:23" ht="30">
+    <row r="391" spans="1:23" ht="30" hidden="1">
       <c r="A391" s="4" t="s">
         <v>2058</v>
       </c>
@@ -51904,7 +51905,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="392" spans="1:23" ht="30">
+    <row r="392" spans="1:23" ht="30" hidden="1">
       <c r="A392" s="4" t="s">
         <v>2058</v>
       </c>
@@ -51975,7 +51976,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="393" spans="1:23" ht="30">
+    <row r="393" spans="1:23" ht="30" hidden="1">
       <c r="A393" s="4" t="s">
         <v>2058</v>
       </c>
@@ -52046,7 +52047,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="394" spans="1:23" ht="30">
+    <row r="394" spans="1:23" ht="30" hidden="1">
       <c r="A394" s="4" t="s">
         <v>2058</v>
       </c>
@@ -52117,7 +52118,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="395" spans="1:23" ht="45">
+    <row r="395" spans="1:23" ht="45" hidden="1">
       <c r="A395" s="4" t="s">
         <v>2058</v>
       </c>
@@ -52188,7 +52189,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="396" spans="1:23" ht="30">
+    <row r="396" spans="1:23" ht="30" hidden="1">
       <c r="A396" s="4" t="s">
         <v>2058</v>
       </c>
@@ -52259,7 +52260,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="397" spans="1:23" ht="30">
+    <row r="397" spans="1:23" ht="30" hidden="1">
       <c r="A397" s="4" t="s">
         <v>2058</v>
       </c>
@@ -52330,7 +52331,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="398" spans="1:23" ht="30">
+    <row r="398" spans="1:23" ht="30" hidden="1">
       <c r="A398" s="4" t="s">
         <v>2058</v>
       </c>
@@ -52401,7 +52402,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="399" spans="1:23" ht="30">
+    <row r="399" spans="1:23" ht="30" hidden="1">
       <c r="A399" s="4" t="s">
         <v>2058</v>
       </c>
@@ -52472,7 +52473,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="400" spans="1:23" ht="30">
+    <row r="400" spans="1:23" ht="30" hidden="1">
       <c r="A400" s="4" t="s">
         <v>2058</v>
       </c>
@@ -52543,7 +52544,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="401" spans="1:23" ht="30">
+    <row r="401" spans="1:23" ht="30" hidden="1">
       <c r="A401" s="4" t="s">
         <v>2058</v>
       </c>
@@ -52614,7 +52615,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="402" spans="1:23">
+    <row r="402" spans="1:23" hidden="1">
       <c r="A402" s="4" t="s">
         <v>2106</v>
       </c>
@@ -52685,7 +52686,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="403" spans="1:23" ht="30">
+    <row r="403" spans="1:23" ht="30" hidden="1">
       <c r="A403" s="4" t="s">
         <v>2106</v>
       </c>
@@ -52756,7 +52757,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="404" spans="1:23" ht="30">
+    <row r="404" spans="1:23" ht="30" hidden="1">
       <c r="A404" s="4" t="s">
         <v>2106</v>
       </c>
@@ -52827,7 +52828,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="405" spans="1:23" ht="45">
+    <row r="405" spans="1:23" ht="45" hidden="1">
       <c r="A405" s="4" t="s">
         <v>2106</v>
       </c>
@@ -52895,7 +52896,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="406" spans="1:23" ht="30">
+    <row r="406" spans="1:23" ht="30" hidden="1">
       <c r="A406" s="4" t="s">
         <v>2106</v>
       </c>
@@ -52963,7 +52964,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="407" spans="1:23" ht="45">
+    <row r="407" spans="1:23" ht="45" hidden="1">
       <c r="A407" s="4" t="s">
         <v>2106</v>
       </c>
@@ -53034,7 +53035,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="408" spans="1:23" ht="30">
+    <row r="408" spans="1:23" ht="30" hidden="1">
       <c r="A408" s="4" t="s">
         <v>2106</v>
       </c>
@@ -53105,7 +53106,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="409" spans="1:23" ht="30">
+    <row r="409" spans="1:23" ht="30" hidden="1">
       <c r="A409" s="4" t="s">
         <v>2106</v>
       </c>
@@ -53176,7 +53177,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="410" spans="1:23" ht="30">
+    <row r="410" spans="1:23" ht="30" hidden="1">
       <c r="A410" s="4" t="s">
         <v>2106</v>
       </c>
@@ -53247,7 +53248,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="411" spans="1:23" ht="45">
+    <row r="411" spans="1:23" ht="45" hidden="1">
       <c r="A411" s="4" t="s">
         <v>2106</v>
       </c>
@@ -53318,7 +53319,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="412" spans="1:23" ht="30">
+    <row r="412" spans="1:23" ht="30" hidden="1">
       <c r="A412" s="4" t="s">
         <v>2106</v>
       </c>
@@ -53389,7 +53390,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="413" spans="1:23" ht="45">
+    <row r="413" spans="1:23" ht="45" hidden="1">
       <c r="A413" s="4" t="s">
         <v>2106</v>
       </c>
@@ -53460,7 +53461,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="414" spans="1:23" ht="30">
+    <row r="414" spans="1:23" ht="30" hidden="1">
       <c r="A414" s="4" t="s">
         <v>2106</v>
       </c>
@@ -53531,7 +53532,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="415" spans="1:23" ht="30">
+    <row r="415" spans="1:23" ht="30" hidden="1">
       <c r="A415" s="4" t="s">
         <v>2106</v>
       </c>
@@ -53599,7 +53600,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="416" spans="1:23" ht="30">
+    <row r="416" spans="1:23" ht="30" hidden="1">
       <c r="A416" s="4" t="s">
         <v>2106</v>
       </c>
@@ -53667,7 +53668,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="417" spans="1:23" ht="30">
+    <row r="417" spans="1:23" ht="30" hidden="1">
       <c r="A417" s="4" t="s">
         <v>2106</v>
       </c>
@@ -53735,7 +53736,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="418" spans="1:23" ht="30">
+    <row r="418" spans="1:23" ht="30" hidden="1">
       <c r="A418" s="4" t="s">
         <v>2106</v>
       </c>
@@ -53806,7 +53807,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="419" spans="1:23" ht="30">
+    <row r="419" spans="1:23" ht="30" hidden="1">
       <c r="A419" s="4" t="s">
         <v>2106</v>
       </c>
@@ -53877,7 +53878,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="420" spans="1:23" ht="30">
+    <row r="420" spans="1:23" ht="30" hidden="1">
       <c r="A420" s="4" t="s">
         <v>2106</v>
       </c>
@@ -53948,7 +53949,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="421" spans="1:23" ht="30">
+    <row r="421" spans="1:23" ht="30" hidden="1">
       <c r="A421" s="4" t="s">
         <v>2106</v>
       </c>
@@ -54019,7 +54020,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="422" spans="1:23" ht="30">
+    <row r="422" spans="1:23" ht="30" hidden="1">
       <c r="A422" s="4" t="s">
         <v>2106</v>
       </c>
@@ -54090,7 +54091,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="423" spans="1:23" ht="30">
+    <row r="423" spans="1:23" ht="30" hidden="1">
       <c r="A423" s="4" t="s">
         <v>2106</v>
       </c>
@@ -54161,7 +54162,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="424" spans="1:23" ht="30">
+    <row r="424" spans="1:23" ht="30" hidden="1">
       <c r="A424" s="4" t="s">
         <v>2106</v>
       </c>
@@ -54232,7 +54233,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="425" spans="1:23" ht="45">
+    <row r="425" spans="1:23" ht="45" hidden="1">
       <c r="A425" s="3" t="s">
         <v>2349</v>
       </c>
@@ -54303,7 +54304,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="426" spans="1:23" ht="30">
+    <row r="426" spans="1:23" ht="30" hidden="1">
       <c r="A426" s="3" t="s">
         <v>2349</v>
       </c>
@@ -54374,7 +54375,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="427" spans="1:23" ht="45">
+    <row r="427" spans="1:23" ht="45" hidden="1">
       <c r="A427" s="3" t="s">
         <v>2349</v>
       </c>
@@ -54445,7 +54446,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="428" spans="1:23" ht="30">
+    <row r="428" spans="1:23" ht="30" hidden="1">
       <c r="A428" s="3" t="s">
         <v>2349</v>
       </c>
@@ -54516,7 +54517,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="429" spans="1:23" ht="45">
+    <row r="429" spans="1:23" ht="45" hidden="1">
       <c r="A429" s="3" t="s">
         <v>2349</v>
       </c>
@@ -54587,7 +54588,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="430" spans="1:23" ht="45">
+    <row r="430" spans="1:23" ht="45" hidden="1">
       <c r="A430" s="3" t="s">
         <v>2349</v>
       </c>
@@ -54658,7 +54659,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="431" spans="1:23" ht="45">
+    <row r="431" spans="1:23" ht="45" hidden="1">
       <c r="A431" s="3" t="s">
         <v>2349</v>
       </c>
@@ -54729,7 +54730,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="432" spans="1:23" ht="30">
+    <row r="432" spans="1:23" ht="30" hidden="1">
       <c r="A432" s="3" t="s">
         <v>2349</v>
       </c>
@@ -54800,7 +54801,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="433" spans="1:23" ht="30">
+    <row r="433" spans="1:23" ht="30" hidden="1">
       <c r="A433" s="3" t="s">
         <v>2349</v>
       </c>
@@ -54871,7 +54872,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="434" spans="1:23" ht="30">
+    <row r="434" spans="1:23" ht="30" hidden="1">
       <c r="A434" s="3" t="s">
         <v>2349</v>
       </c>
@@ -54942,7 +54943,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="435" spans="1:23" ht="30">
+    <row r="435" spans="1:23" ht="30" hidden="1">
       <c r="A435" s="3" t="s">
         <v>2349</v>
       </c>
@@ -55013,7 +55014,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="436" spans="1:23" ht="30">
+    <row r="436" spans="1:23" ht="30" hidden="1">
       <c r="A436" s="3" t="s">
         <v>2349</v>
       </c>
@@ -55084,7 +55085,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="437" spans="1:23" ht="30">
+    <row r="437" spans="1:23" ht="30" hidden="1">
       <c r="A437" s="3" t="s">
         <v>2349</v>
       </c>
@@ -55155,7 +55156,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="438" spans="1:23" ht="30">
+    <row r="438" spans="1:23" ht="30" hidden="1">
       <c r="A438" s="3" t="s">
         <v>2349</v>
       </c>
@@ -55226,7 +55227,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="439" spans="1:23">
+    <row r="439" spans="1:23" hidden="1">
       <c r="A439" s="4" t="s">
         <v>2426</v>
       </c>
@@ -55297,7 +55298,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="440" spans="1:23" ht="30">
+    <row r="440" spans="1:23" ht="30" hidden="1">
       <c r="A440" s="4" t="s">
         <v>2426</v>
       </c>
@@ -55368,7 +55369,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="441" spans="1:23" ht="30">
+    <row r="441" spans="1:23" ht="30" hidden="1">
       <c r="A441" s="4" t="s">
         <v>2426</v>
       </c>
@@ -55439,7 +55440,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="442" spans="1:23" ht="45">
+    <row r="442" spans="1:23" ht="45" hidden="1">
       <c r="A442" s="4" t="s">
         <v>2426</v>
       </c>
@@ -55510,7 +55511,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="443" spans="1:23" ht="30">
+    <row r="443" spans="1:23" ht="30" hidden="1">
       <c r="A443" s="4" t="s">
         <v>2426</v>
       </c>
@@ -55581,7 +55582,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="444" spans="1:23" ht="45">
+    <row r="444" spans="1:23" ht="45" hidden="1">
       <c r="A444" s="4" t="s">
         <v>2426</v>
       </c>
@@ -55652,7 +55653,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="445" spans="1:23" ht="30">
+    <row r="445" spans="1:23" ht="30" hidden="1">
       <c r="A445" s="4" t="s">
         <v>2426</v>
       </c>
@@ -55723,7 +55724,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="446" spans="1:23" ht="30">
+    <row r="446" spans="1:23" ht="30" hidden="1">
       <c r="A446" s="4" t="s">
         <v>2426</v>
       </c>
@@ -55794,7 +55795,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="447" spans="1:23" ht="30">
+    <row r="447" spans="1:23" ht="30" hidden="1">
       <c r="A447" s="4" t="s">
         <v>2426</v>
       </c>
@@ -55865,7 +55866,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="448" spans="1:23" ht="30">
+    <row r="448" spans="1:23" ht="30" hidden="1">
       <c r="A448" s="4" t="s">
         <v>2426</v>
       </c>
@@ -55936,7 +55937,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="449" spans="1:23" ht="30">
+    <row r="449" spans="1:23" ht="30" hidden="1">
       <c r="A449" s="4" t="s">
         <v>2426</v>
       </c>
@@ -56007,7 +56008,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="450" spans="1:23" ht="30">
+    <row r="450" spans="1:23" ht="30" hidden="1">
       <c r="A450" s="4" t="s">
         <v>2426</v>
       </c>
@@ -56078,7 +56079,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="451" spans="1:23" ht="30">
+    <row r="451" spans="1:23" ht="30" hidden="1">
       <c r="A451" s="3" t="s">
         <v>3691</v>
       </c>
@@ -56145,7 +56146,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="452" spans="1:23" ht="30">
+    <row r="452" spans="1:23" ht="30" hidden="1">
       <c r="A452" s="3" t="s">
         <v>3691</v>
       </c>
@@ -56212,7 +56213,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="453" spans="1:23" ht="30">
+    <row r="453" spans="1:23" ht="30" hidden="1">
       <c r="A453" s="3" t="s">
         <v>3691</v>
       </c>
@@ -56279,7 +56280,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="454" spans="1:23" ht="30">
+    <row r="454" spans="1:23" ht="30" hidden="1">
       <c r="A454" s="3" t="s">
         <v>3691</v>
       </c>
@@ -56346,7 +56347,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="455" spans="1:23" ht="30">
+    <row r="455" spans="1:23" ht="30" hidden="1">
       <c r="A455" s="3" t="s">
         <v>3691</v>
       </c>
@@ -56415,7 +56416,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="456" spans="1:23" ht="45">
+    <row r="456" spans="1:23" ht="45" hidden="1">
       <c r="A456" s="3" t="s">
         <v>3691</v>
       </c>
@@ -56484,7 +56485,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="457" spans="1:23" ht="30">
+    <row r="457" spans="1:23" ht="30" hidden="1">
       <c r="A457" s="3" t="s">
         <v>3684</v>
       </c>
@@ -56551,7 +56552,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="458" spans="1:23" ht="30">
+    <row r="458" spans="1:23" ht="30" hidden="1">
       <c r="A458" s="3" t="s">
         <v>3684</v>
       </c>
@@ -56620,7 +56621,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="459" spans="1:23">
+    <row r="459" spans="1:23" hidden="1">
       <c r="A459" s="3" t="s">
         <v>3684</v>
       </c>
@@ -56689,7 +56690,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="460" spans="1:23" ht="45">
+    <row r="460" spans="1:23" ht="45" hidden="1">
       <c r="A460" s="3" t="s">
         <v>3684</v>
       </c>
@@ -56758,7 +56759,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="461" spans="1:23" ht="30">
+    <row r="461" spans="1:23" ht="30" hidden="1">
       <c r="A461" s="3" t="s">
         <v>3684</v>
       </c>
@@ -56825,7 +56826,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="462" spans="1:23" ht="30">
+    <row r="462" spans="1:23" ht="30" hidden="1">
       <c r="A462" s="3" t="s">
         <v>3684</v>
       </c>
@@ -56895,7 +56896,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W462" xr:uid="{7E21F442-9136-4C15-8BA3-92E07332B93A}"/>
+  <autoFilter ref="A1:W462" xr:uid="{7E21F442-9136-4C15-8BA3-92E07332B93A}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="User"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <hyperlinks>
     <hyperlink ref="Q9" r:id="rId1" display="mailto:admin@memgine.com" xr:uid="{93170BB8-77D4-4002-829B-D89928109808}"/>
     <hyperlink ref="Q11" r:id="rId2" display="https://memgine.com/" xr:uid="{F8EB4105-6CCB-4B06-B657-948DB365F556}"/>

</xml_diff>

<commit_message>
Offer rule engine changes
</commit_message>
<xml_diff>
--- a/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
+++ b/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MynikaTech\memgine\docs\domain\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37E0F9B4-2252-41F4-AF4D-A47E50054D73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13023519-5769-475F-869A-4F4517D0FB98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="3" xr2:uid="{AA28BC4D-8219-43B9-8C16-6977709D904A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="6" activeTab="13" xr2:uid="{AA28BC4D-8219-43B9-8C16-6977709D904A}"/>
   </bookViews>
   <sheets>
     <sheet name="Entity Catalogue" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16878" uniqueCount="4397">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17338" uniqueCount="4432">
   <si>
     <t>Domain</t>
   </si>
@@ -13235,6 +13235,111 @@
   </si>
   <si>
     <t>REL075</t>
+  </si>
+  <si>
+    <t>OFFRULE</t>
+  </si>
+  <si>
+    <t>Promotion</t>
+  </si>
+  <si>
+    <t>Offer Usage Rule</t>
+  </si>
+  <si>
+    <t>offer_usage_rule</t>
+  </si>
+  <si>
+    <t>Defines the usage, frequency and time-window rules that control when and how often a customer may redeem an offer.</t>
+  </si>
+  <si>
+    <t>offer_usage_rule_id</t>
+  </si>
+  <si>
+    <t>Offer Usage Rule Name</t>
+  </si>
+  <si>
+    <t>Allows offers to support recurring usage limits and time-based redemption windows such as daily offers, monthly offers and offers available only during specified hours.</t>
+  </si>
+  <si>
+    <t>Offer Usage Rule ID</t>
+  </si>
+  <si>
+    <t>Uniquely identifies an offer usage rule.</t>
+  </si>
+  <si>
+    <t>System-generated identifier for the offer usage rule.</t>
+  </si>
+  <si>
+    <t>Primary identifier for the usage rule controlling offer redemption eligibility.</t>
+  </si>
+  <si>
+    <t>Identifies the offer to which the usage rule applies.</t>
+  </si>
+  <si>
+    <t>References the offer governed by this usage rule.</t>
+  </si>
+  <si>
+    <t>Associates the usage rule with the applicable offer.</t>
+  </si>
+  <si>
+    <t>Name used to identify the purpose of the usage rule.</t>
+  </si>
+  <si>
+    <t>Weekend Offer Rule</t>
+  </si>
+  <si>
+    <t>Defines the recurring frequency at which the offer may be redeemed.</t>
+  </si>
+  <si>
+    <t>Defines whether the offer usage is Daily, Weekly, Monthly, Yearly or One Time.</t>
+  </si>
+  <si>
+    <t>Maximum number of times the offer may be redeemed during each applicable frequency period.</t>
+  </si>
+  <si>
+    <t>Controls limits such as one offer per day or two redemptions per month.</t>
+  </si>
+  <si>
+    <t>Time of day from which the offer becomes redeemable.</t>
+  </si>
+  <si>
+    <t>Supports offers that are available only during specified hours.</t>
+  </si>
+  <si>
+    <t>Time of day after which the offer is no longer redeemable.</t>
+  </si>
+  <si>
+    <t>Offer Usage Rule Status</t>
+  </si>
+  <si>
+    <t>offer_usage_rule_status_id</t>
+  </si>
+  <si>
+    <t>REL079</t>
+  </si>
+  <si>
+    <t>Offer Usage Rules</t>
+  </si>
+  <si>
+    <t>Each Offer may have one or more usage rules that define its redemption frequency, limits and time windows.</t>
+  </si>
+  <si>
+    <t>REL080</t>
+  </si>
+  <si>
+    <t>Each Offer Usage Rule has one lifecycle status.</t>
+  </si>
+  <si>
+    <t>REL081</t>
+  </si>
+  <si>
+    <t>Identifies the user who created the Offer Usage Rule.</t>
+  </si>
+  <si>
+    <t>REL082</t>
+  </si>
+  <si>
+    <t>Identifies the user who last updated the Offer Usage Rule.</t>
   </si>
 </sst>
 </file>
@@ -13466,7 +13571,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3841114F-D1EC-49B1-850B-590431E39412}" name="Table2" displayName="Table2" ref="A1:Q46" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3841114F-D1EC-49B1-850B-590431E39412}" name="Table2" displayName="Table2" ref="A1:Q47" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{FEF6275C-74E6-4563-BFF3-6461E4A3D8DA}" name="Entity Code" dataDxfId="16"/>
     <tableColumn id="2" xr3:uid="{67FE23FD-539D-4023-BA73-D2A0B84718BF}" name="Domain" dataDxfId="15"/>
@@ -13787,7 +13892,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4659496D-1A4F-4BC3-BD65-377E70E6B8BE}">
-  <dimension ref="A1:Q46"/>
+  <dimension ref="A1:Q47"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="31.85546875" style="4" customWidth="1"/>
@@ -16227,6 +16332,59 @@
         <v>4314</v>
       </c>
     </row>
+    <row r="47" spans="1:17" ht="75">
+      <c r="A47" s="4" t="s">
+        <v>4397</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>417</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>4398</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>4399</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>4400</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>4401</v>
+      </c>
+      <c r="G47" s="4" t="s">
+        <v>1517</v>
+      </c>
+      <c r="H47" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="I47" s="4" t="s">
+        <v>2106</v>
+      </c>
+      <c r="J47" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K47" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="L47" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="M47" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="N47" s="4" t="s">
+        <v>4402</v>
+      </c>
+      <c r="O47" s="4" t="s">
+        <v>4403</v>
+      </c>
+      <c r="P47" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q47" s="4" t="s">
+        <v>4404</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -19788,7 +19946,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C85B9BC7-C8C8-4E3E-A0EF-02B9554CEAE5}">
-  <dimension ref="A1:K79"/>
+  <dimension ref="A1:K83"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.5703125" style="4" bestFit="1" customWidth="1"/>
@@ -22568,6 +22726,146 @@
       </c>
       <c r="K79" s="4" t="s">
         <v>4395</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11">
+      <c r="A80" s="4" t="s">
+        <v>4423</v>
+      </c>
+      <c r="B80" s="4" t="s">
+        <v>2106</v>
+      </c>
+      <c r="C80" s="4" t="s">
+        <v>4399</v>
+      </c>
+      <c r="D80" s="4" t="s">
+        <v>4424</v>
+      </c>
+      <c r="E80" s="4" t="s">
+        <v>2110</v>
+      </c>
+      <c r="F80" s="4" t="s">
+        <v>2110</v>
+      </c>
+      <c r="G80" s="4" t="s">
+        <v>1298</v>
+      </c>
+      <c r="H80" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I80" s="4" t="s">
+        <v>1334</v>
+      </c>
+      <c r="J80" s="4" t="s">
+        <v>1311</v>
+      </c>
+      <c r="K80" s="4" t="s">
+        <v>4425</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11">
+      <c r="A81" s="4" t="s">
+        <v>4426</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>4399</v>
+      </c>
+      <c r="D81" s="4" t="s">
+        <v>4421</v>
+      </c>
+      <c r="E81" s="4" t="s">
+        <v>1013</v>
+      </c>
+      <c r="F81" s="4" t="s">
+        <v>4422</v>
+      </c>
+      <c r="G81" s="4" t="s">
+        <v>1298</v>
+      </c>
+      <c r="H81" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I81" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="J81" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K81" s="4" t="s">
+        <v>4427</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11">
+      <c r="A82" s="4" t="s">
+        <v>4428</v>
+      </c>
+      <c r="B82" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C82" s="4" t="s">
+        <v>4399</v>
+      </c>
+      <c r="D82" s="4" t="s">
+        <v>4390</v>
+      </c>
+      <c r="E82" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="F82" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="G82" s="4" t="s">
+        <v>1298</v>
+      </c>
+      <c r="H82" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I82" s="4" t="s">
+        <v>4392</v>
+      </c>
+      <c r="J82" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K82" s="4" t="s">
+        <v>4429</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11">
+      <c r="A83" s="4" t="s">
+        <v>4430</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>4399</v>
+      </c>
+      <c r="D83" s="4" t="s">
+        <v>4394</v>
+      </c>
+      <c r="E83" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="F83" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="G83" s="4" t="s">
+        <v>1298</v>
+      </c>
+      <c r="H83" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I83" s="4" t="s">
+        <v>4392</v>
+      </c>
+      <c r="J83" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K83" s="4" t="s">
+        <v>4431</v>
       </c>
     </row>
   </sheetData>
@@ -26625,7 +26923,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E21F442-9136-4C15-8BA3-92E07332B93A}">
-  <dimension ref="A1:W543"/>
+  <dimension ref="A1:W562"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.140625" style="4" customWidth="1"/>
@@ -62695,7 +62993,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="525" spans="1:23">
+    <row r="525" spans="1:23" ht="30">
       <c r="A525" s="4" t="s">
         <v>4309</v>
       </c>
@@ -62766,7 +63064,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="526" spans="1:23">
+    <row r="526" spans="1:23" ht="30">
       <c r="A526" s="4" t="s">
         <v>4309</v>
       </c>
@@ -62837,7 +63135,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="527" spans="1:23">
+    <row r="527" spans="1:23" ht="30">
       <c r="A527" s="4" t="s">
         <v>4309</v>
       </c>
@@ -62908,7 +63206,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="528" spans="1:23">
+    <row r="528" spans="1:23" ht="45">
       <c r="A528" s="4" t="s">
         <v>4309</v>
       </c>
@@ -62979,7 +63277,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="529" spans="1:23">
+    <row r="529" spans="1:23" ht="45">
       <c r="A529" s="4" t="s">
         <v>4309</v>
       </c>
@@ -63050,7 +63348,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="530" spans="1:23">
+    <row r="530" spans="1:23" ht="60">
       <c r="A530" s="4" t="s">
         <v>4309</v>
       </c>
@@ -63121,7 +63419,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="531" spans="1:23">
+    <row r="531" spans="1:23" ht="30">
       <c r="A531" s="4" t="s">
         <v>4309</v>
       </c>
@@ -63192,7 +63490,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="532" spans="1:23">
+    <row r="532" spans="1:23" ht="30">
       <c r="A532" s="4" t="s">
         <v>4309</v>
       </c>
@@ -63263,7 +63561,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="533" spans="1:23">
+    <row r="533" spans="1:23" ht="30">
       <c r="A533" s="4" t="s">
         <v>4309</v>
       </c>
@@ -63334,7 +63632,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="534" spans="1:23">
+    <row r="534" spans="1:23" ht="45">
       <c r="A534" s="4" t="s">
         <v>4309</v>
       </c>
@@ -63405,7 +63703,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="535" spans="1:23">
+    <row r="535" spans="1:23" ht="60">
       <c r="A535" s="4" t="s">
         <v>4309</v>
       </c>
@@ -63473,7 +63771,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="536" spans="1:23">
+    <row r="536" spans="1:23" ht="60">
       <c r="A536" s="4" t="s">
         <v>4309</v>
       </c>
@@ -63541,7 +63839,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="537" spans="1:23">
+    <row r="537" spans="1:23" ht="30">
       <c r="A537" s="4" t="s">
         <v>4309</v>
       </c>
@@ -63612,7 +63910,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="538" spans="1:23">
+    <row r="538" spans="1:23" ht="30">
       <c r="A538" s="4" t="s">
         <v>4309</v>
       </c>
@@ -63683,7 +63981,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="539" spans="1:23">
+    <row r="539" spans="1:23" ht="30">
       <c r="A539" s="4" t="s">
         <v>4309</v>
       </c>
@@ -63754,7 +64052,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="540" spans="1:23">
+    <row r="540" spans="1:23" ht="30">
       <c r="A540" s="4" t="s">
         <v>4309</v>
       </c>
@@ -63825,7 +64123,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="541" spans="1:23">
+    <row r="541" spans="1:23" ht="30">
       <c r="A541" s="4" t="s">
         <v>4309</v>
       </c>
@@ -63896,7 +64194,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="542" spans="1:23">
+    <row r="542" spans="1:23" ht="30">
       <c r="A542" s="4" t="s">
         <v>4309</v>
       </c>
@@ -63967,7 +64265,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="543" spans="1:23">
+    <row r="543" spans="1:23" ht="30">
       <c r="A543" s="4" t="s">
         <v>4309</v>
       </c>
@@ -64035,6 +64333,1349 @@
         <v>6</v>
       </c>
       <c r="W543" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="544" spans="1:23">
+      <c r="A544" s="4" t="s">
+        <v>4399</v>
+      </c>
+      <c r="B544" s="4">
+        <v>1</v>
+      </c>
+      <c r="C544" s="4" t="s">
+        <v>4405</v>
+      </c>
+      <c r="D544" s="4" t="s">
+        <v>4402</v>
+      </c>
+      <c r="E544" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F544" s="4">
+        <v>36</v>
+      </c>
+      <c r="G544" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H544" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I544" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="J544" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K544" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L544" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="M544" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="N544" s="4" t="s">
+        <v>4406</v>
+      </c>
+      <c r="O544" s="4" t="s">
+        <v>4407</v>
+      </c>
+      <c r="P544" s="4" t="s">
+        <v>4408</v>
+      </c>
+      <c r="Q544" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="R544" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="S544" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="T544" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="U544" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="V544" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W544" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="545" spans="1:23">
+      <c r="A545" s="4" t="s">
+        <v>4399</v>
+      </c>
+      <c r="B545" s="4">
+        <v>2</v>
+      </c>
+      <c r="C545" s="4" t="s">
+        <v>2106</v>
+      </c>
+      <c r="D545" s="4" t="s">
+        <v>2110</v>
+      </c>
+      <c r="E545" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F545" s="4">
+        <v>36</v>
+      </c>
+      <c r="G545" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H545" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I545" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J545" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K545" s="4" t="s">
+        <v>2106</v>
+      </c>
+      <c r="L545" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M545" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N545" s="4" t="s">
+        <v>4409</v>
+      </c>
+      <c r="O545" s="4" t="s">
+        <v>4410</v>
+      </c>
+      <c r="P545" s="4" t="s">
+        <v>4411</v>
+      </c>
+      <c r="Q545" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="R545" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S545" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T545" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U545" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V545" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="W545" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="546" spans="1:23">
+      <c r="A546" s="4" t="s">
+        <v>4399</v>
+      </c>
+      <c r="B546" s="4">
+        <v>3</v>
+      </c>
+      <c r="C546" s="4" t="s">
+        <v>4322</v>
+      </c>
+      <c r="D546" s="4" t="s">
+        <v>4323</v>
+      </c>
+      <c r="E546" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="F546" s="4">
+        <v>100</v>
+      </c>
+      <c r="G546" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H546" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I546" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J546" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K546" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L546" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M546" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N546" s="4" t="s">
+        <v>4324</v>
+      </c>
+      <c r="O546" s="4" t="s">
+        <v>4412</v>
+      </c>
+      <c r="P546" s="4" t="s">
+        <v>4326</v>
+      </c>
+      <c r="Q546" s="4" t="s">
+        <v>4413</v>
+      </c>
+      <c r="R546" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S546" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T546" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U546" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V546" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="W546" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="547" spans="1:23">
+      <c r="A547" s="4" t="s">
+        <v>4399</v>
+      </c>
+      <c r="B547" s="4">
+        <v>4</v>
+      </c>
+      <c r="C547" s="4" t="s">
+        <v>4328</v>
+      </c>
+      <c r="D547" s="4" t="s">
+        <v>4329</v>
+      </c>
+      <c r="E547" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="F547" s="4">
+        <v>30</v>
+      </c>
+      <c r="G547" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H547" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I547" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J547" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K547" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L547" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M547" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N547" s="4" t="s">
+        <v>4414</v>
+      </c>
+      <c r="O547" s="4" t="s">
+        <v>4415</v>
+      </c>
+      <c r="P547" s="4" t="s">
+        <v>4332</v>
+      </c>
+      <c r="Q547" s="4" t="s">
+        <v>4333</v>
+      </c>
+      <c r="R547" s="4" t="s">
+        <v>4333</v>
+      </c>
+      <c r="S547" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T547" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U547" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V547" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="W547" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="548" spans="1:23">
+      <c r="A548" s="4" t="s">
+        <v>4399</v>
+      </c>
+      <c r="B548" s="4">
+        <v>5</v>
+      </c>
+      <c r="C548" s="4" t="s">
+        <v>4334</v>
+      </c>
+      <c r="D548" s="4" t="s">
+        <v>4335</v>
+      </c>
+      <c r="E548" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="F548" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="G548" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H548" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I548" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J548" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K548" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L548" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M548" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N548" s="4" t="s">
+        <v>4336</v>
+      </c>
+      <c r="O548" s="4" t="s">
+        <v>4337</v>
+      </c>
+      <c r="P548" s="4" t="s">
+        <v>4338</v>
+      </c>
+      <c r="Q548" s="4">
+        <v>1</v>
+      </c>
+      <c r="R548" s="4">
+        <v>1</v>
+      </c>
+      <c r="S548" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T548" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U548" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V548" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="W548" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="549" spans="1:23">
+      <c r="A549" s="4" t="s">
+        <v>4399</v>
+      </c>
+      <c r="B549" s="4">
+        <v>6</v>
+      </c>
+      <c r="C549" s="4" t="s">
+        <v>4339</v>
+      </c>
+      <c r="D549" s="4" t="s">
+        <v>4340</v>
+      </c>
+      <c r="E549" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="F549" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="G549" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H549" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I549" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J549" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K549" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L549" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M549" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N549" s="4" t="s">
+        <v>4341</v>
+      </c>
+      <c r="O549" s="4" t="s">
+        <v>4416</v>
+      </c>
+      <c r="P549" s="4" t="s">
+        <v>4417</v>
+      </c>
+      <c r="Q549" s="4">
+        <v>1</v>
+      </c>
+      <c r="R549" s="4">
+        <v>1</v>
+      </c>
+      <c r="S549" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T549" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U549" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V549" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="W549" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="550" spans="1:23">
+      <c r="A550" s="4" t="s">
+        <v>4399</v>
+      </c>
+      <c r="B550" s="4">
+        <v>7</v>
+      </c>
+      <c r="C550" s="4" t="s">
+        <v>4344</v>
+      </c>
+      <c r="D550" s="4" t="s">
+        <v>4345</v>
+      </c>
+      <c r="E550" s="4" t="s">
+        <v>4346</v>
+      </c>
+      <c r="F550" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="G550" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H550" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I550" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J550" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K550" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L550" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M550" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N550" s="4" t="s">
+        <v>4347</v>
+      </c>
+      <c r="O550" s="4" t="s">
+        <v>4418</v>
+      </c>
+      <c r="P550" s="4" t="s">
+        <v>4419</v>
+      </c>
+      <c r="Q550" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="R550" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S550" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T550" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U550" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V550" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="W550" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="551" spans="1:23">
+      <c r="A551" s="4" t="s">
+        <v>4399</v>
+      </c>
+      <c r="B551" s="4">
+        <v>8</v>
+      </c>
+      <c r="C551" s="4" t="s">
+        <v>4350</v>
+      </c>
+      <c r="D551" s="4" t="s">
+        <v>4351</v>
+      </c>
+      <c r="E551" s="4" t="s">
+        <v>4346</v>
+      </c>
+      <c r="F551" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="G551" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H551" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I551" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J551" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K551" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L551" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M551" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N551" s="4" t="s">
+        <v>4352</v>
+      </c>
+      <c r="O551" s="4" t="s">
+        <v>4420</v>
+      </c>
+      <c r="P551" s="4" t="s">
+        <v>4419</v>
+      </c>
+      <c r="Q551" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="R551" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S551" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T551" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U551" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V551" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="W551" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="552" spans="1:23">
+      <c r="A552" s="4" t="s">
+        <v>4399</v>
+      </c>
+      <c r="B552" s="4">
+        <v>9</v>
+      </c>
+      <c r="C552" s="4" t="s">
+        <v>4354</v>
+      </c>
+      <c r="D552" s="4" t="s">
+        <v>4355</v>
+      </c>
+      <c r="E552" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="F552" s="4">
+        <v>100</v>
+      </c>
+      <c r="G552" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H552" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I552" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J552" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K552" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L552" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M552" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N552" s="4" t="s">
+        <v>4356</v>
+      </c>
+      <c r="O552" s="4" t="s">
+        <v>4357</v>
+      </c>
+      <c r="P552" s="4" t="s">
+        <v>4358</v>
+      </c>
+      <c r="Q552" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="R552" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S552" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T552" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U552" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V552" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="W552" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="553" spans="1:23">
+      <c r="A553" s="4" t="s">
+        <v>4399</v>
+      </c>
+      <c r="B553" s="4">
+        <v>10</v>
+      </c>
+      <c r="C553" s="4" t="s">
+        <v>4360</v>
+      </c>
+      <c r="D553" s="4" t="s">
+        <v>4361</v>
+      </c>
+      <c r="E553" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="F553" s="4">
+        <v>100</v>
+      </c>
+      <c r="G553" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H553" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I553" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J553" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K553" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L553" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M553" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N553" s="4" t="s">
+        <v>4362</v>
+      </c>
+      <c r="O553" s="4" t="s">
+        <v>4363</v>
+      </c>
+      <c r="P553" s="4" t="s">
+        <v>4364</v>
+      </c>
+      <c r="Q553" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="R553" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S553" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T553" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U553" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V553" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="W553" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="554" spans="1:23">
+      <c r="A554" s="4" t="s">
+        <v>4399</v>
+      </c>
+      <c r="B554" s="4">
+        <v>11</v>
+      </c>
+      <c r="C554" s="4" t="s">
+        <v>466</v>
+      </c>
+      <c r="D554" s="4" t="s">
+        <v>467</v>
+      </c>
+      <c r="E554" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="F554" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G554" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H554" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I554" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J554" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="K554" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="L554" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M554" s="4" t="s">
+        <v>4365</v>
+      </c>
+      <c r="N554" s="4" t="s">
+        <v>4366</v>
+      </c>
+      <c r="O554" s="4" t="s">
+        <v>4367</v>
+      </c>
+      <c r="P554" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="Q554" s="4" t="s">
+        <v>295</v>
+      </c>
+      <c r="R554" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="S554" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T554" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U554" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V554" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="555" spans="1:23">
+      <c r="A555" s="4" t="s">
+        <v>4399</v>
+      </c>
+      <c r="B555" s="4">
+        <v>12</v>
+      </c>
+      <c r="C555" s="4" t="s">
+        <v>471</v>
+      </c>
+      <c r="D555" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="E555" s="4" t="s">
+        <v>291</v>
+      </c>
+      <c r="F555" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G555" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H555" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I555" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J555" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="K555" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="L555" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M555" s="4" t="s">
+        <v>4368</v>
+      </c>
+      <c r="N555" s="4" t="s">
+        <v>4369</v>
+      </c>
+      <c r="O555" s="4" t="s">
+        <v>4370</v>
+      </c>
+      <c r="P555" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="Q555" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="R555" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="S555" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T555" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U555" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V555" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="556" spans="1:23">
+      <c r="A556" s="4" t="s">
+        <v>4399</v>
+      </c>
+      <c r="B556" s="4">
+        <v>13</v>
+      </c>
+      <c r="C556" s="4" t="s">
+        <v>4421</v>
+      </c>
+      <c r="D556" s="4" t="s">
+        <v>4422</v>
+      </c>
+      <c r="E556" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F556" s="4">
+        <v>36</v>
+      </c>
+      <c r="G556" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H556" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I556" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J556" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K556" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="L556" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M556" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N556" s="4" t="s">
+        <v>4373</v>
+      </c>
+      <c r="O556" s="4" t="s">
+        <v>4374</v>
+      </c>
+      <c r="P556" s="4" t="s">
+        <v>4375</v>
+      </c>
+      <c r="Q556" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="R556" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="S556" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T556" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U556" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V556" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="W556" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="557" spans="1:23">
+      <c r="A557" s="4" t="s">
+        <v>4399</v>
+      </c>
+      <c r="B557" s="4">
+        <v>14</v>
+      </c>
+      <c r="C557" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="D557" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="E557" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="F557" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="G557" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H557" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I557" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J557" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K557" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L557" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M557" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="N557" s="4" t="s">
+        <v>4376</v>
+      </c>
+      <c r="O557" s="4" t="s">
+        <v>4377</v>
+      </c>
+      <c r="P557" s="4" t="s">
+        <v>478</v>
+      </c>
+      <c r="Q557" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="R557" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="S557" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="T557" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="U557" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V557" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W557" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="558" spans="1:23">
+      <c r="A558" s="4" t="s">
+        <v>4399</v>
+      </c>
+      <c r="B558" s="4">
+        <v>15</v>
+      </c>
+      <c r="C558" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="D558" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="E558" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F558" s="4">
+        <v>36</v>
+      </c>
+      <c r="G558" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H558" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I558" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J558" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K558" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="L558" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M558" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N558" s="4" t="s">
+        <v>4378</v>
+      </c>
+      <c r="O558" s="4" t="s">
+        <v>4379</v>
+      </c>
+      <c r="P558" s="4" t="s">
+        <v>478</v>
+      </c>
+      <c r="Q558" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="R558" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S558" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T558" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U558" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="V558" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W558" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="559" spans="1:23">
+      <c r="A559" s="4" t="s">
+        <v>4399</v>
+      </c>
+      <c r="B559" s="4">
+        <v>16</v>
+      </c>
+      <c r="C559" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="D559" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="E559" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="F559" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="G559" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H559" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I559" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J559" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K559" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L559" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M559" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="N559" s="4" t="s">
+        <v>4380</v>
+      </c>
+      <c r="O559" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="P559" s="4" t="s">
+        <v>478</v>
+      </c>
+      <c r="Q559" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="R559" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="S559" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="T559" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="U559" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V559" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W559" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="560" spans="1:23">
+      <c r="A560" s="4" t="s">
+        <v>4399</v>
+      </c>
+      <c r="B560" s="4">
+        <v>17</v>
+      </c>
+      <c r="C560" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="D560" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="E560" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F560" s="4">
+        <v>36</v>
+      </c>
+      <c r="G560" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H560" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I560" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J560" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K560" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="L560" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M560" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N560" s="4" t="s">
+        <v>4381</v>
+      </c>
+      <c r="O560" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="P560" s="4" t="s">
+        <v>478</v>
+      </c>
+      <c r="Q560" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="R560" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S560" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T560" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U560" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="V560" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W560" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="561" spans="1:23">
+      <c r="A561" s="4" t="s">
+        <v>4399</v>
+      </c>
+      <c r="B561" s="4">
+        <v>18</v>
+      </c>
+      <c r="C561" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="D561" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="E561" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="F561" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="G561" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H561" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I561" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J561" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K561" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L561" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M561" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N561" s="4" t="s">
+        <v>4382</v>
+      </c>
+      <c r="O561" s="4" t="s">
+        <v>484</v>
+      </c>
+      <c r="P561" s="4" t="s">
+        <v>485</v>
+      </c>
+      <c r="Q561" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="R561" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="S561" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="T561" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U561" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="V561" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W561" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="562" spans="1:23">
+      <c r="A562" s="4" t="s">
+        <v>4399</v>
+      </c>
+      <c r="B562" s="4">
+        <v>19</v>
+      </c>
+      <c r="C562" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="D562" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="E562" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="F562" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="G562" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H562" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I562" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J562" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K562" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L562" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M562" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="N562" s="4" t="s">
+        <v>486</v>
+      </c>
+      <c r="O562" s="4" t="s">
+        <v>487</v>
+      </c>
+      <c r="P562" s="4" t="s">
+        <v>4383</v>
+      </c>
+      <c r="Q562" s="4">
+        <v>1</v>
+      </c>
+      <c r="R562" s="4">
+        <v>1</v>
+      </c>
+      <c r="S562" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="T562" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="U562" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V562" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W562" s="4" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Initial QR  engien set up -Stage 1
</commit_message>
<xml_diff>
--- a/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
+++ b/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MynikaTech\memgine\docs\domain\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13023519-5769-475F-869A-4F4517D0FB98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E648539-C542-4F56-B93B-FFAA79B83836}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="6" activeTab="13" xr2:uid="{AA28BC4D-8219-43B9-8C16-6977709D904A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="11" xr2:uid="{AA28BC4D-8219-43B9-8C16-6977709D904A}"/>
   </bookViews>
   <sheets>
     <sheet name="Entity Catalogue" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17338" uniqueCount="4432">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18252" uniqueCount="4635">
   <si>
     <t>Domain</t>
   </si>
@@ -13340,6 +13340,615 @@
   </si>
   <si>
     <t>Identifies the user who last updated the Offer Usage Rule.</t>
+  </si>
+  <si>
+    <t>QRCODE</t>
+  </si>
+  <si>
+    <t>QR Management</t>
+  </si>
+  <si>
+    <t>QR Code</t>
+  </si>
+  <si>
+    <t>qr_codes</t>
+  </si>
+  <si>
+    <t>Represents a reusable QR code configured by an Organization to initiate a supported Memgine journey such as viewing available memberships, opening a specific membership, or initiating a redemption flow.</t>
+  </si>
+  <si>
+    <t>qr_code_id</t>
+  </si>
+  <si>
+    <t>QR Code Name</t>
+  </si>
+  <si>
+    <t>A generic QR definition that can support multiple QR Code Types and target different business journeys or entities.</t>
+  </si>
+  <si>
+    <t>QRSCNHIST</t>
+  </si>
+  <si>
+    <t>QR Scan History</t>
+  </si>
+  <si>
+    <t>qr_scan_history</t>
+  </si>
+  <si>
+    <t>Records each attempt to scan a QR code, including successful, failed and anonymous scans, to support operational auditing and membership acquisition analysis.</t>
+  </si>
+  <si>
+    <t>qr_scan_history_id</t>
+  </si>
+  <si>
+    <t>QR Scan Time</t>
+  </si>
+  <si>
+    <t>Scan history is retained for analytics and audit purposes and must not be physically deleted.</t>
+  </si>
+  <si>
+    <t>QRCODETYPE</t>
+  </si>
+  <si>
+    <t>QR Code Type</t>
+  </si>
+  <si>
+    <t>qr_code_types</t>
+  </si>
+  <si>
+    <t>Represents the supported business purpose of a QR code, such as displaying all available memberships, opening a specific membership, or initiating an offer or benefit redemption.</t>
+  </si>
+  <si>
+    <t>qr_code_type_id</t>
+  </si>
+  <si>
+    <t>QR Code Type Name</t>
+  </si>
+  <si>
+    <t>Platform-managed reference data defining the supported QR-driven customer journeys.</t>
+  </si>
+  <si>
+    <t>QRSCANRESULT</t>
+  </si>
+  <si>
+    <t>QR Scan Result</t>
+  </si>
+  <si>
+    <t>qr_scan_results</t>
+  </si>
+  <si>
+    <t>Represents the outcome of a QR code scan, such as successful resolution, invalid QR, expired QR or inactive QR.</t>
+  </si>
+  <si>
+    <t>qr_scan_result_id</t>
+  </si>
+  <si>
+    <t>QR Scan Result Name</t>
+  </si>
+  <si>
+    <t>Platform-managed reference data used to classify QR scan outcomes for operational and analytical purposes.</t>
+  </si>
+  <si>
+    <t>QR Code Identifier</t>
+  </si>
+  <si>
+    <t>Uniquely identifies a QR code definition.</t>
+  </si>
+  <si>
+    <t>System-generated identifier for the QR code.</t>
+  </si>
+  <si>
+    <t>Represents the persistent identity of a reusable QR code.</t>
+  </si>
+  <si>
+    <t>Identifies the organization that owns the QR code.</t>
+  </si>
+  <si>
+    <t>References the organization that created and manages the QR code.</t>
+  </si>
+  <si>
+    <t>Establishes tenant ownership of the QR code.</t>
+  </si>
+  <si>
+    <t>qr_code_name</t>
+  </si>
+  <si>
+    <t>Provides a business-friendly name for the QR code.</t>
+  </si>
+  <si>
+    <t>Name used by organization administrators to identify the QR code and its placement or campaign.</t>
+  </si>
+  <si>
+    <t>Represents the human-readable administrative name of the QR code.</t>
+  </si>
+  <si>
+    <t>Store Membership Poster</t>
+  </si>
+  <si>
+    <t>Defines the customer journey initiated by the QR code.</t>
+  </si>
+  <si>
+    <t>References the type of QR-driven journey such as all memberships, a specific membership, offer redemption or benefit redemption.</t>
+  </si>
+  <si>
+    <t>Determines how Memgine interprets the QR code.</t>
+  </si>
+  <si>
+    <t>QR Code Token</t>
+  </si>
+  <si>
+    <t>qr_code_token</t>
+  </si>
+  <si>
+    <t>Stores the opaque value encoded into the QR destination.</t>
+  </si>
+  <si>
+    <t>Unique system-generated token used to resolve the QR code without exposing business data directly in the QR payload.</t>
+  </si>
+  <si>
+    <t>Represents the secure public identifier carried by the QR code.</t>
+  </si>
+  <si>
+    <t>Opaque Token</t>
+  </si>
+  <si>
+    <t>Target Entity Type</t>
+  </si>
+  <si>
+    <t>target_entity_type</t>
+  </si>
+  <si>
+    <t>Identifies the type of business entity targeted by the QR code when applicable.</t>
+  </si>
+  <si>
+    <t>Specifies the target entity represented by target_entity_id, such as Membership Product, Offer or Benefit.</t>
+  </si>
+  <si>
+    <t>Supports generic QR targeting without coupling the QR entity to a single business domain.</t>
+  </si>
+  <si>
+    <t>Target Entity ID</t>
+  </si>
+  <si>
+    <t>target_entity_id</t>
+  </si>
+  <si>
+    <t>Identifies the specific entity targeted by the QR code when applicable.</t>
+  </si>
+  <si>
+    <t>References the business entity to be opened or acted upon according to the QR Code Type.</t>
+  </si>
+  <si>
+    <t>Provides the generic target identifier for a QR-driven journey.</t>
+  </si>
+  <si>
+    <t>Placement Name</t>
+  </si>
+  <si>
+    <t>placement_name</t>
+  </si>
+  <si>
+    <t>Identifies where or how the QR code is promoted.</t>
+  </si>
+  <si>
+    <t>Business-defined placement or campaign label used to distinguish physical or promotional placements for analysis.</t>
+  </si>
+  <si>
+    <t>Supports analysis of membership acquisition by QR placement or promotion source.</t>
+  </si>
+  <si>
+    <t>Store Entrance Poster</t>
+  </si>
+  <si>
+    <t>Identifies the store associated with the QR placement when applicable.</t>
+  </si>
+  <si>
+    <t>References the store where the QR code is displayed when the placement is store-specific.</t>
+  </si>
+  <si>
+    <t>Supports store-level QR scan and acquisition analysis.</t>
+  </si>
+  <si>
+    <t>Indicates the operational status of the QR code.</t>
+  </si>
+  <si>
+    <t>References the lifecycle status of the QR code.</t>
+  </si>
+  <si>
+    <t>Determines whether the QR code is currently usable.</t>
+  </si>
+  <si>
+    <t>Records when the QR code was created.</t>
+  </si>
+  <si>
+    <t>Timestamp when the QR code definition was first created.</t>
+  </si>
+  <si>
+    <t>Records who created the QR code.</t>
+  </si>
+  <si>
+    <t>References the user who created the QR code definition.</t>
+  </si>
+  <si>
+    <t>Records the most recent update to the QR code.</t>
+  </si>
+  <si>
+    <t>Records who last updated the QR code.</t>
+  </si>
+  <si>
+    <t>Indicates whether the QR code has been soft deleted.</t>
+  </si>
+  <si>
+    <t>Logical deletion flag used to preserve the QR code definition and its history.</t>
+  </si>
+  <si>
+    <t>Supports controlled retirement without physical removal.</t>
+  </si>
+  <si>
+    <t>Represents the current business version of the QR code.</t>
+  </si>
+  <si>
+    <t>QR Scan History Identifier</t>
+  </si>
+  <si>
+    <t>Uniquely identifies a QR scan history record.</t>
+  </si>
+  <si>
+    <t>System-generated identifier for each recorded QR scan event.</t>
+  </si>
+  <si>
+    <t>Represents the unique identity of a scan event.</t>
+  </si>
+  <si>
+    <t>Identifies the QR code that was scanned.</t>
+  </si>
+  <si>
+    <t>References the persistent QR code definition associated with the scan.</t>
+  </si>
+  <si>
+    <t>Links each scan event to its QR code for operational and acquisition analysis.</t>
+  </si>
+  <si>
+    <t>Identifies the customer associated with the scan when known.</t>
+  </si>
+  <si>
+    <t>References the global user when the scanner or application can associate the scan with a customer.</t>
+  </si>
+  <si>
+    <t>Supports customer-level acquisition funnel analysis while allowing anonymous scans.</t>
+  </si>
+  <si>
+    <t>qr_scan_datetime</t>
+  </si>
+  <si>
+    <t>Records when the QR scan occurred.</t>
+  </si>
+  <si>
+    <t>Timestamp of the QR scan event.</t>
+  </si>
+  <si>
+    <t>Represents the exact time at which the QR code was scanned.</t>
+  </si>
+  <si>
+    <t>Records the outcome of the QR scan.</t>
+  </si>
+  <si>
+    <t>References the result classification for the scan attempt.</t>
+  </si>
+  <si>
+    <t>Supports operational monitoring and analysis of successful and unsuccessful scans.</t>
+  </si>
+  <si>
+    <t>Identifies the store where the scan occurred when applicable.</t>
+  </si>
+  <si>
+    <t>References the store associated with the scan location when known.</t>
+  </si>
+  <si>
+    <t>Supports store-level scan and acquisition analysis.</t>
+  </si>
+  <si>
+    <t>Identifies the staff member involved in the scan when applicable.</t>
+  </si>
+  <si>
+    <t>References the staff member operating a counter scanner or assisting the customer.</t>
+  </si>
+  <si>
+    <t>Supports operational and redemption analysis.</t>
+  </si>
+  <si>
+    <t>Scan Source</t>
+  </si>
+  <si>
+    <t>scan_source</t>
+  </si>
+  <si>
+    <t>Identifies the channel from which the scan was initiated.</t>
+  </si>
+  <si>
+    <t>Records whether the scan originated from a customer device, counter scanner, web or another supported channel.</t>
+  </si>
+  <si>
+    <t>Supports channel-level QR performance analysis.</t>
+  </si>
+  <si>
+    <t>Customer Device</t>
+  </si>
+  <si>
+    <t>Captures the target entity type resolved at scan time.</t>
+  </si>
+  <si>
+    <t>Records the entity type associated with the QR target when applicable.</t>
+  </si>
+  <si>
+    <t>Preserves scan-time targeting context for historical analysis even if QR configuration later changes.</t>
+  </si>
+  <si>
+    <t>Captures the target entity identifier resolved at scan time.</t>
+  </si>
+  <si>
+    <t>Records the target identifier associated with the QR scan when applicable.</t>
+  </si>
+  <si>
+    <t>Preserves the business target associated with the historical scan event.</t>
+  </si>
+  <si>
+    <t>Failure Reason</t>
+  </si>
+  <si>
+    <t>failure_reason</t>
+  </si>
+  <si>
+    <t>Stores additional information when a QR scan cannot be successfully resolved.</t>
+  </si>
+  <si>
+    <t>Provides a human-readable or system-generated explanation for an unsuccessful scan.</t>
+  </si>
+  <si>
+    <t>Supports operational troubleshooting and analysis of failed scans.</t>
+  </si>
+  <si>
+    <t>Expired QR Code</t>
+  </si>
+  <si>
+    <t>Records when the scan history record was created.</t>
+  </si>
+  <si>
+    <t>Timestamp when the scan event was persisted.</t>
+  </si>
+  <si>
+    <t>Supports auditability of scan history.</t>
+  </si>
+  <si>
+    <t>Records the user responsible for creating the scan history record when applicable.</t>
+  </si>
+  <si>
+    <t>References the authenticated user or system actor that persisted the scan event.</t>
+  </si>
+  <si>
+    <t>Supports auditability while allowing system-generated or anonymous scan records.</t>
+  </si>
+  <si>
+    <t>Supports version tracking for scan history records.</t>
+  </si>
+  <si>
+    <t>Version number for the persisted scan event record.</t>
+  </si>
+  <si>
+    <t>Supports controlled updates if scan history metadata is corrected.</t>
+  </si>
+  <si>
+    <t>REL083</t>
+  </si>
+  <si>
+    <t>Each QR Code has one QR Code Type defining the customer journey it initiates.</t>
+  </si>
+  <si>
+    <t>REL084</t>
+  </si>
+  <si>
+    <t>Organization QR Codes</t>
+  </si>
+  <si>
+    <t>Each Organization may configure multiple QR codes.</t>
+  </si>
+  <si>
+    <t>REL085</t>
+  </si>
+  <si>
+    <t>QR Code Status</t>
+  </si>
+  <si>
+    <t>Each QR Code has one lifecycle status.</t>
+  </si>
+  <si>
+    <t>REL086</t>
+  </si>
+  <si>
+    <t>QR Code Store Placement</t>
+  </si>
+  <si>
+    <t>A QR Code may optionally be associated with a Store when the QR is displayed at a specific store.</t>
+  </si>
+  <si>
+    <t>REL087</t>
+  </si>
+  <si>
+    <t>QR Code Created By</t>
+  </si>
+  <si>
+    <t>Identifies the user who created the QR Code.</t>
+  </si>
+  <si>
+    <t>REL088</t>
+  </si>
+  <si>
+    <t>QR Code Updated By</t>
+  </si>
+  <si>
+    <t>Identifies the user who last updated the QR Code.</t>
+  </si>
+  <si>
+    <t>REL089</t>
+  </si>
+  <si>
+    <t>QR Code Scans</t>
+  </si>
+  <si>
+    <t>Each QR Code may have many scan history records.</t>
+  </si>
+  <si>
+    <t>REL090</t>
+  </si>
+  <si>
+    <t>Customer QR Scans</t>
+  </si>
+  <si>
+    <t>A User may be associated with multiple QR scan history records when the customer is known.</t>
+  </si>
+  <si>
+    <t>REL091</t>
+  </si>
+  <si>
+    <t>Each QR Scan History record has one scan result classification.</t>
+  </si>
+  <si>
+    <t>REL092</t>
+  </si>
+  <si>
+    <t>Store QR Scans</t>
+  </si>
+  <si>
+    <t>A QR Scan History record may optionally identify the Store where the scan occurred.</t>
+  </si>
+  <si>
+    <t>REL093</t>
+  </si>
+  <si>
+    <t>Staff QR Scans</t>
+  </si>
+  <si>
+    <t>A QR Scan History record may optionally identify the Staff member involved in the scan.</t>
+  </si>
+  <si>
+    <t>REL094</t>
+  </si>
+  <si>
+    <t>Scan History Created By</t>
+  </si>
+  <si>
+    <t>Identifies the authenticated user or system actor that created the scan history record.</t>
+  </si>
+  <si>
+    <t>QR_BUSINESS_MEMBERSHIPS</t>
+  </si>
+  <si>
+    <t>Business Memberships</t>
+  </si>
+  <si>
+    <t>Opens the memberships available for the QR code's organization.</t>
+  </si>
+  <si>
+    <t>Customer scans a generic business QR and is taken to the organization's available memberships.</t>
+  </si>
+  <si>
+    <t>QR_MEMBERSHIP</t>
+  </si>
+  <si>
+    <t>Specific Membership</t>
+  </si>
+  <si>
+    <t>Opens a specific membership product for the customer to review and purchase.</t>
+  </si>
+  <si>
+    <t>Customer scans a QR promoting a specific membership.</t>
+  </si>
+  <si>
+    <t>QR_OFFER_REDEMPTION</t>
+  </si>
+  <si>
+    <t>Offer Redemption</t>
+  </si>
+  <si>
+    <t>Represents a QR-driven offer redemption journey.</t>
+  </si>
+  <si>
+    <t>Used when a customer presents a QR for an offer redemption.</t>
+  </si>
+  <si>
+    <t>QR_BENEFIT_REDEMPTION</t>
+  </si>
+  <si>
+    <t>Benefit Redemption</t>
+  </si>
+  <si>
+    <t>Represents a QR-driven benefit redemption journey.</t>
+  </si>
+  <si>
+    <t>Used when a customer presents a QR for a benefit redemption.</t>
+  </si>
+  <si>
+    <t>QR was successfully resolved and the requested journey can proceed.</t>
+  </si>
+  <si>
+    <t>Successful QR resolution.</t>
+  </si>
+  <si>
+    <t>INVALID</t>
+  </si>
+  <si>
+    <t>Invalid QR</t>
+  </si>
+  <si>
+    <t>The QR could not be recognized or its token is invalid.</t>
+  </si>
+  <si>
+    <t>Invalid or malformed QR.</t>
+  </si>
+  <si>
+    <t>Expired QR</t>
+  </si>
+  <si>
+    <t>The QR or its associated journey is no longer valid.</t>
+  </si>
+  <si>
+    <t>QR has expired or its associated target is no longer valid.</t>
+  </si>
+  <si>
+    <t>Inactive QR</t>
+  </si>
+  <si>
+    <t>The QR code has been disabled or is not currently active.</t>
+  </si>
+  <si>
+    <t>QR code is not operational.</t>
+  </si>
+  <si>
+    <t>TARGET_NOT_FOUND</t>
+  </si>
+  <si>
+    <t>Target Not Found</t>
+  </si>
+  <si>
+    <t>The QR resolved but its configured target could not be found.</t>
+  </si>
+  <si>
+    <t>Target membership, offer, benefit or other entity could not be resolved.</t>
+  </si>
+  <si>
+    <t>ACCESS_DENIED</t>
+  </si>
+  <si>
+    <t>Access Denied</t>
+  </si>
+  <si>
+    <t>The QR resolved but the requested journey cannot be accessed by the current user or context.</t>
+  </si>
+  <si>
+    <t>QR target exists but access or eligibility prevents proceeding.</t>
+  </si>
+  <si>
+    <t>QR_CODE</t>
   </si>
 </sst>
 </file>
@@ -13571,7 +14180,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3841114F-D1EC-49B1-850B-590431E39412}" name="Table2" displayName="Table2" ref="A1:Q47" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3841114F-D1EC-49B1-850B-590431E39412}" name="Table2" displayName="Table2" ref="A1:Q51" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{FEF6275C-74E6-4563-BFF3-6461E4A3D8DA}" name="Entity Code" dataDxfId="16"/>
     <tableColumn id="2" xr3:uid="{67FE23FD-539D-4023-BA73-D2A0B84718BF}" name="Domain" dataDxfId="15"/>
@@ -13892,7 +14501,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4659496D-1A4F-4BC3-BD65-377E70E6B8BE}">
-  <dimension ref="A1:Q47"/>
+  <dimension ref="A1:Q51"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="31.85546875" style="4" customWidth="1"/>
@@ -16385,6 +16994,218 @@
         <v>4404</v>
       </c>
     </row>
+    <row r="48" spans="1:17" ht="75">
+      <c r="A48" s="4" t="s">
+        <v>4432</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>417</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>4433</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="E48" s="4" t="s">
+        <v>4435</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>4436</v>
+      </c>
+      <c r="G48" s="4" t="s">
+        <v>1517</v>
+      </c>
+      <c r="H48" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="I48" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="J48" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K48" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="L48" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="M48" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="N48" s="4" t="s">
+        <v>4437</v>
+      </c>
+      <c r="O48" s="4" t="s">
+        <v>4438</v>
+      </c>
+      <c r="P48" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q48" s="4" t="s">
+        <v>4439</v>
+      </c>
+    </row>
+    <row r="49" spans="1:17" ht="60">
+      <c r="A49" s="4" t="s">
+        <v>4440</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>417</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>4433</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>4441</v>
+      </c>
+      <c r="E49" s="4" t="s">
+        <v>4442</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>4443</v>
+      </c>
+      <c r="G49" s="4" t="s">
+        <v>623</v>
+      </c>
+      <c r="H49" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="I49" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="J49" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K49" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="L49" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="M49" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="N49" s="4" t="s">
+        <v>4444</v>
+      </c>
+      <c r="O49" s="4" t="s">
+        <v>4445</v>
+      </c>
+      <c r="P49" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q49" s="4" t="s">
+        <v>4446</v>
+      </c>
+    </row>
+    <row r="50" spans="1:17" ht="60">
+      <c r="A50" s="4" t="s">
+        <v>4447</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>4433</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>4448</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>4449</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>4450</v>
+      </c>
+      <c r="G50" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="H50" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="I50" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="J50" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K50" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="L50" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M50" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N50" s="4" t="s">
+        <v>4451</v>
+      </c>
+      <c r="O50" s="4" t="s">
+        <v>4452</v>
+      </c>
+      <c r="P50" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q50" s="4" t="s">
+        <v>4453</v>
+      </c>
+    </row>
+    <row r="51" spans="1:17" ht="45">
+      <c r="A51" s="4" t="s">
+        <v>4454</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>4433</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>4455</v>
+      </c>
+      <c r="E51" s="4" t="s">
+        <v>4456</v>
+      </c>
+      <c r="F51" s="4" t="s">
+        <v>4457</v>
+      </c>
+      <c r="G51" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="H51" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="I51" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="J51" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K51" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="L51" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M51" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N51" s="4" t="s">
+        <v>4458</v>
+      </c>
+      <c r="O51" s="4" t="s">
+        <v>4459</v>
+      </c>
+      <c r="P51" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q51" s="4" t="s">
+        <v>4460</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -17895,7 +18716,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B7B29B1-81FD-48F8-9727-C5470F35164D}">
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="3" style="4" bestFit="1" customWidth="1"/>
@@ -18253,6 +19074,20 @@
       </c>
       <c r="D25" s="3" t="s">
         <v>2253</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" s="5">
+        <v>25</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>4634</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>2234</v>
       </c>
     </row>
   </sheetData>
@@ -19946,7 +20781,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C85B9BC7-C8C8-4E3E-A0EF-02B9554CEAE5}">
-  <dimension ref="A1:K83"/>
+  <dimension ref="A1:K95"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.5703125" style="4" bestFit="1" customWidth="1"/>
@@ -22728,7 +23563,7 @@
         <v>4395</v>
       </c>
     </row>
-    <row r="80" spans="1:11">
+    <row r="80" spans="1:11" ht="30">
       <c r="A80" s="4" t="s">
         <v>4423</v>
       </c>
@@ -22866,6 +23701,426 @@
       </c>
       <c r="K83" s="4" t="s">
         <v>4431</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11">
+      <c r="A84" s="4" t="s">
+        <v>4564</v>
+      </c>
+      <c r="B84" s="4" t="s">
+        <v>4448</v>
+      </c>
+      <c r="C84" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="D84" s="4" t="s">
+        <v>4448</v>
+      </c>
+      <c r="E84" s="4" t="s">
+        <v>4451</v>
+      </c>
+      <c r="F84" s="4" t="s">
+        <v>4451</v>
+      </c>
+      <c r="G84" s="4" t="s">
+        <v>1298</v>
+      </c>
+      <c r="H84" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I84" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="J84" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K84" s="4" t="s">
+        <v>4565</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11">
+      <c r="A85" s="4" t="s">
+        <v>4566</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>4567</v>
+      </c>
+      <c r="E85" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F85" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="G85" s="4" t="s">
+        <v>1298</v>
+      </c>
+      <c r="H85" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I85" s="4" t="s">
+        <v>1517</v>
+      </c>
+      <c r="J85" s="4" t="s">
+        <v>1311</v>
+      </c>
+      <c r="K85" s="4" t="s">
+        <v>4568</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11">
+      <c r="A86" s="4" t="s">
+        <v>4569</v>
+      </c>
+      <c r="B86" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C86" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="D86" s="4" t="s">
+        <v>4570</v>
+      </c>
+      <c r="E86" s="4" t="s">
+        <v>1013</v>
+      </c>
+      <c r="F86" s="4" t="s">
+        <v>1013</v>
+      </c>
+      <c r="G86" s="4" t="s">
+        <v>1298</v>
+      </c>
+      <c r="H86" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I86" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="J86" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K86" s="4" t="s">
+        <v>4571</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11">
+      <c r="A87" s="4" t="s">
+        <v>4572</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C87" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="D87" s="4" t="s">
+        <v>4573</v>
+      </c>
+      <c r="E87" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="F87" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="G87" s="4" t="s">
+        <v>1298</v>
+      </c>
+      <c r="H87" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I87" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="J87" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K87" s="4" t="s">
+        <v>4574</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11">
+      <c r="A88" s="4" t="s">
+        <v>4575</v>
+      </c>
+      <c r="B88" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C88" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="D88" s="4" t="s">
+        <v>4576</v>
+      </c>
+      <c r="E88" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="F88" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="G88" s="4" t="s">
+        <v>1298</v>
+      </c>
+      <c r="H88" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I88" s="4" t="s">
+        <v>4392</v>
+      </c>
+      <c r="J88" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K88" s="4" t="s">
+        <v>4577</v>
+      </c>
+    </row>
+    <row r="89" spans="1:11">
+      <c r="A89" s="4" t="s">
+        <v>4578</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C89" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="D89" s="4" t="s">
+        <v>4579</v>
+      </c>
+      <c r="E89" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="F89" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="G89" s="4" t="s">
+        <v>1298</v>
+      </c>
+      <c r="H89" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I89" s="4" t="s">
+        <v>4392</v>
+      </c>
+      <c r="J89" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K89" s="4" t="s">
+        <v>4580</v>
+      </c>
+    </row>
+    <row r="90" spans="1:11">
+      <c r="A90" s="4" t="s">
+        <v>4581</v>
+      </c>
+      <c r="B90" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="C90" s="4" t="s">
+        <v>4441</v>
+      </c>
+      <c r="D90" s="4" t="s">
+        <v>4582</v>
+      </c>
+      <c r="E90" s="4" t="s">
+        <v>4437</v>
+      </c>
+      <c r="F90" s="4" t="s">
+        <v>4437</v>
+      </c>
+      <c r="G90" s="4" t="s">
+        <v>1298</v>
+      </c>
+      <c r="H90" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I90" s="4" t="s">
+        <v>623</v>
+      </c>
+      <c r="J90" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K90" s="4" t="s">
+        <v>4583</v>
+      </c>
+    </row>
+    <row r="91" spans="1:11">
+      <c r="A91" s="4" t="s">
+        <v>4584</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C91" s="4" t="s">
+        <v>4441</v>
+      </c>
+      <c r="D91" s="4" t="s">
+        <v>4585</v>
+      </c>
+      <c r="E91" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="F91" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G91" s="4" t="s">
+        <v>1298</v>
+      </c>
+      <c r="H91" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I91" s="4" t="s">
+        <v>1307</v>
+      </c>
+      <c r="J91" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K91" s="4" t="s">
+        <v>4586</v>
+      </c>
+    </row>
+    <row r="92" spans="1:11">
+      <c r="A92" s="4" t="s">
+        <v>4587</v>
+      </c>
+      <c r="B92" s="4" t="s">
+        <v>4455</v>
+      </c>
+      <c r="C92" s="4" t="s">
+        <v>4441</v>
+      </c>
+      <c r="D92" s="4" t="s">
+        <v>4455</v>
+      </c>
+      <c r="E92" s="4" t="s">
+        <v>4458</v>
+      </c>
+      <c r="F92" s="4" t="s">
+        <v>4458</v>
+      </c>
+      <c r="G92" s="4" t="s">
+        <v>1298</v>
+      </c>
+      <c r="H92" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I92" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="J92" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K92" s="4" t="s">
+        <v>4588</v>
+      </c>
+    </row>
+    <row r="93" spans="1:11">
+      <c r="A93" s="4" t="s">
+        <v>4589</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C93" s="4" t="s">
+        <v>4441</v>
+      </c>
+      <c r="D93" s="4" t="s">
+        <v>4590</v>
+      </c>
+      <c r="E93" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="F93" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="G93" s="4" t="s">
+        <v>1298</v>
+      </c>
+      <c r="H93" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I93" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="J93" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K93" s="4" t="s">
+        <v>4591</v>
+      </c>
+    </row>
+    <row r="94" spans="1:11">
+      <c r="A94" s="4" t="s">
+        <v>4592</v>
+      </c>
+      <c r="B94" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C94" s="4" t="s">
+        <v>4441</v>
+      </c>
+      <c r="D94" s="4" t="s">
+        <v>4593</v>
+      </c>
+      <c r="E94" s="4" t="s">
+        <v>698</v>
+      </c>
+      <c r="F94" s="4" t="s">
+        <v>698</v>
+      </c>
+      <c r="G94" s="4" t="s">
+        <v>1298</v>
+      </c>
+      <c r="H94" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I94" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="J94" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K94" s="4" t="s">
+        <v>4594</v>
+      </c>
+    </row>
+    <row r="95" spans="1:11">
+      <c r="A95" s="4" t="s">
+        <v>4595</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>4441</v>
+      </c>
+      <c r="D95" s="4" t="s">
+        <v>4596</v>
+      </c>
+      <c r="E95" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="F95" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="G95" s="4" t="s">
+        <v>1298</v>
+      </c>
+      <c r="H95" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I95" s="4" t="s">
+        <v>4392</v>
+      </c>
+      <c r="J95" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K95" s="4" t="s">
+        <v>4597</v>
       </c>
     </row>
   </sheetData>
@@ -26923,7 +28178,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E21F442-9136-4C15-8BA3-92E07332B93A}">
-  <dimension ref="A1:W562"/>
+  <dimension ref="A1:W592"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.140625" style="4" customWidth="1"/>
@@ -64336,7 +65591,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="544" spans="1:23">
+    <row r="544" spans="1:23" ht="30">
       <c r="A544" s="4" t="s">
         <v>4399</v>
       </c>
@@ -64407,7 +65662,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="545" spans="1:23">
+    <row r="545" spans="1:23" ht="30">
       <c r="A545" s="4" t="s">
         <v>4399</v>
       </c>
@@ -64478,7 +65733,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="546" spans="1:23">
+    <row r="546" spans="1:23" ht="30">
       <c r="A546" s="4" t="s">
         <v>4399</v>
       </c>
@@ -64549,7 +65804,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="547" spans="1:23">
+    <row r="547" spans="1:23" ht="45">
       <c r="A547" s="4" t="s">
         <v>4399</v>
       </c>
@@ -64620,7 +65875,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="548" spans="1:23">
+    <row r="548" spans="1:23" ht="45">
       <c r="A548" s="4" t="s">
         <v>4399</v>
       </c>
@@ -64691,7 +65946,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="549" spans="1:23">
+    <row r="549" spans="1:23" ht="60">
       <c r="A549" s="4" t="s">
         <v>4399</v>
       </c>
@@ -64762,7 +66017,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="550" spans="1:23">
+    <row r="550" spans="1:23" ht="30">
       <c r="A550" s="4" t="s">
         <v>4399</v>
       </c>
@@ -64833,7 +66088,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="551" spans="1:23">
+    <row r="551" spans="1:23" ht="30">
       <c r="A551" s="4" t="s">
         <v>4399</v>
       </c>
@@ -64904,7 +66159,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="552" spans="1:23">
+    <row r="552" spans="1:23" ht="30">
       <c r="A552" s="4" t="s">
         <v>4399</v>
       </c>
@@ -64975,7 +66230,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="553" spans="1:23">
+    <row r="553" spans="1:23" ht="45">
       <c r="A553" s="4" t="s">
         <v>4399</v>
       </c>
@@ -65046,7 +66301,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="554" spans="1:23">
+    <row r="554" spans="1:23" ht="60">
       <c r="A554" s="4" t="s">
         <v>4399</v>
       </c>
@@ -65114,7 +66369,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="555" spans="1:23">
+    <row r="555" spans="1:23" ht="60">
       <c r="A555" s="4" t="s">
         <v>4399</v>
       </c>
@@ -65182,7 +66437,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="556" spans="1:23">
+    <row r="556" spans="1:23" ht="30">
       <c r="A556" s="4" t="s">
         <v>4399</v>
       </c>
@@ -65253,7 +66508,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="557" spans="1:23">
+    <row r="557" spans="1:23" ht="30">
       <c r="A557" s="4" t="s">
         <v>4399</v>
       </c>
@@ -65324,7 +66579,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="558" spans="1:23">
+    <row r="558" spans="1:23" ht="30">
       <c r="A558" s="4" t="s">
         <v>4399</v>
       </c>
@@ -65395,7 +66650,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="559" spans="1:23">
+    <row r="559" spans="1:23" ht="30">
       <c r="A559" s="4" t="s">
         <v>4399</v>
       </c>
@@ -65466,7 +66721,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="560" spans="1:23">
+    <row r="560" spans="1:23" ht="30">
       <c r="A560" s="4" t="s">
         <v>4399</v>
       </c>
@@ -65537,7 +66792,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="561" spans="1:23">
+    <row r="561" spans="1:23" ht="30">
       <c r="A561" s="4" t="s">
         <v>4399</v>
       </c>
@@ -65608,7 +66863,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="562" spans="1:23">
+    <row r="562" spans="1:23" ht="30">
       <c r="A562" s="4" t="s">
         <v>4399</v>
       </c>
@@ -65676,6 +66931,2136 @@
         <v>6</v>
       </c>
       <c r="W562" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="563" spans="1:23">
+      <c r="A563" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="B563" s="4">
+        <v>1</v>
+      </c>
+      <c r="C563" s="4" t="s">
+        <v>4461</v>
+      </c>
+      <c r="D563" s="4" t="s">
+        <v>4437</v>
+      </c>
+      <c r="E563" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F563" s="4">
+        <v>36</v>
+      </c>
+      <c r="G563" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H563" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I563" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="J563" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K563" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L563" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="M563" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="N563" s="4" t="s">
+        <v>4462</v>
+      </c>
+      <c r="O563" s="4" t="s">
+        <v>4463</v>
+      </c>
+      <c r="P563" s="4" t="s">
+        <v>4464</v>
+      </c>
+      <c r="Q563" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="R563" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="S563" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="T563" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="U563" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="V563" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W563" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="564" spans="1:23">
+      <c r="A564" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="B564" s="4">
+        <v>2</v>
+      </c>
+      <c r="C564" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D564" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E564" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F564" s="4">
+        <v>36</v>
+      </c>
+      <c r="G564" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H564" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I564" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J564" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K564" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="L564" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M564" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N564" s="4" t="s">
+        <v>4465</v>
+      </c>
+      <c r="O564" s="4" t="s">
+        <v>4466</v>
+      </c>
+      <c r="P564" s="4" t="s">
+        <v>4467</v>
+      </c>
+      <c r="Q564" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="R564" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S564" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T564" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U564" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="V564" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W564" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="565" spans="1:23">
+      <c r="A565" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="B565" s="4">
+        <v>3</v>
+      </c>
+      <c r="C565" s="4" t="s">
+        <v>4438</v>
+      </c>
+      <c r="D565" s="4" t="s">
+        <v>4468</v>
+      </c>
+      <c r="E565" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="F565" s="4">
+        <v>100</v>
+      </c>
+      <c r="G565" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H565" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I565" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J565" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K565" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L565" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M565" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N565" s="4" t="s">
+        <v>4469</v>
+      </c>
+      <c r="O565" s="4" t="s">
+        <v>4470</v>
+      </c>
+      <c r="P565" s="4" t="s">
+        <v>4471</v>
+      </c>
+      <c r="Q565" s="4" t="s">
+        <v>4472</v>
+      </c>
+      <c r="R565" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S565" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T565" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U565" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V565" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="W565" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="566" spans="1:23">
+      <c r="A566" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="B566" s="4">
+        <v>4</v>
+      </c>
+      <c r="C566" s="4" t="s">
+        <v>4448</v>
+      </c>
+      <c r="D566" s="4" t="s">
+        <v>4451</v>
+      </c>
+      <c r="E566" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F566" s="4">
+        <v>36</v>
+      </c>
+      <c r="G566" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H566" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I566" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J566" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K566" s="4" t="s">
+        <v>4448</v>
+      </c>
+      <c r="L566" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M566" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N566" s="4" t="s">
+        <v>4473</v>
+      </c>
+      <c r="O566" s="4" t="s">
+        <v>4474</v>
+      </c>
+      <c r="P566" s="4" t="s">
+        <v>4475</v>
+      </c>
+      <c r="Q566" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="R566" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S566" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T566" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U566" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V566" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="W566" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="567" spans="1:23">
+      <c r="A567" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="B567" s="4">
+        <v>5</v>
+      </c>
+      <c r="C567" s="4" t="s">
+        <v>4476</v>
+      </c>
+      <c r="D567" s="4" t="s">
+        <v>4477</v>
+      </c>
+      <c r="E567" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="F567" s="4">
+        <v>200</v>
+      </c>
+      <c r="G567" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H567" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I567" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J567" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K567" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L567" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="M567" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="N567" s="4" t="s">
+        <v>4478</v>
+      </c>
+      <c r="O567" s="4" t="s">
+        <v>4479</v>
+      </c>
+      <c r="P567" s="4" t="s">
+        <v>4480</v>
+      </c>
+      <c r="Q567" s="4" t="s">
+        <v>4481</v>
+      </c>
+      <c r="R567" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="S567" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T567" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U567" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V567" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W567" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="568" spans="1:23">
+      <c r="A568" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="B568" s="4">
+        <v>6</v>
+      </c>
+      <c r="C568" s="4" t="s">
+        <v>4482</v>
+      </c>
+      <c r="D568" s="4" t="s">
+        <v>4483</v>
+      </c>
+      <c r="E568" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="F568" s="4">
+        <v>50</v>
+      </c>
+      <c r="G568" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H568" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I568" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J568" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K568" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L568" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M568" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N568" s="4" t="s">
+        <v>4484</v>
+      </c>
+      <c r="O568" s="4" t="s">
+        <v>4485</v>
+      </c>
+      <c r="P568" s="4" t="s">
+        <v>4486</v>
+      </c>
+      <c r="Q568" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="R568" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S568" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T568" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U568" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V568" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="W568" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="569" spans="1:23">
+      <c r="A569" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="B569" s="4">
+        <v>7</v>
+      </c>
+      <c r="C569" s="4" t="s">
+        <v>4487</v>
+      </c>
+      <c r="D569" s="4" t="s">
+        <v>4488</v>
+      </c>
+      <c r="E569" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F569" s="4">
+        <v>36</v>
+      </c>
+      <c r="G569" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H569" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I569" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J569" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K569" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L569" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M569" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N569" s="4" t="s">
+        <v>4489</v>
+      </c>
+      <c r="O569" s="4" t="s">
+        <v>4490</v>
+      </c>
+      <c r="P569" s="4" t="s">
+        <v>4491</v>
+      </c>
+      <c r="Q569" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="R569" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S569" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T569" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U569" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V569" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="W569" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="570" spans="1:23">
+      <c r="A570" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="B570" s="4">
+        <v>8</v>
+      </c>
+      <c r="C570" s="4" t="s">
+        <v>4492</v>
+      </c>
+      <c r="D570" s="4" t="s">
+        <v>4493</v>
+      </c>
+      <c r="E570" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="F570" s="4">
+        <v>150</v>
+      </c>
+      <c r="G570" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H570" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I570" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J570" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K570" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L570" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M570" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N570" s="4" t="s">
+        <v>4494</v>
+      </c>
+      <c r="O570" s="4" t="s">
+        <v>4495</v>
+      </c>
+      <c r="P570" s="4" t="s">
+        <v>4496</v>
+      </c>
+      <c r="Q570" s="4" t="s">
+        <v>4497</v>
+      </c>
+      <c r="R570" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S570" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T570" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U570" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V570" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="W570" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="571" spans="1:23">
+      <c r="A571" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="B571" s="4">
+        <v>9</v>
+      </c>
+      <c r="C571" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D571" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="E571" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F571" s="4">
+        <v>36</v>
+      </c>
+      <c r="G571" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H571" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I571" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J571" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K571" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="L571" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M571" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N571" s="4" t="s">
+        <v>4498</v>
+      </c>
+      <c r="O571" s="4" t="s">
+        <v>4499</v>
+      </c>
+      <c r="P571" s="4" t="s">
+        <v>4500</v>
+      </c>
+      <c r="Q571" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="R571" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S571" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T571" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U571" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V571" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="W571" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="572" spans="1:23">
+      <c r="A572" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="B572" s="4">
+        <v>10</v>
+      </c>
+      <c r="C572" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="D572" s="4" t="s">
+        <v>1013</v>
+      </c>
+      <c r="E572" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F572" s="4">
+        <v>36</v>
+      </c>
+      <c r="G572" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H572" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I572" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J572" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K572" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="L572" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M572" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N572" s="4" t="s">
+        <v>4501</v>
+      </c>
+      <c r="O572" s="4" t="s">
+        <v>4502</v>
+      </c>
+      <c r="P572" s="4" t="s">
+        <v>4503</v>
+      </c>
+      <c r="Q572" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="R572" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="S572" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T572" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U572" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V572" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="W572" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="573" spans="1:23">
+      <c r="A573" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="B573" s="4">
+        <v>11</v>
+      </c>
+      <c r="C573" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="D573" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="E573" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="F573" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="G573" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H573" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I573" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J573" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K573" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L573" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M573" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="N573" s="4" t="s">
+        <v>4504</v>
+      </c>
+      <c r="O573" s="4" t="s">
+        <v>4505</v>
+      </c>
+      <c r="P573" s="4" t="s">
+        <v>478</v>
+      </c>
+      <c r="Q573" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="R573" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="S573" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="T573" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="U573" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V573" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W573" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="574" spans="1:23">
+      <c r="A574" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="B574" s="4">
+        <v>12</v>
+      </c>
+      <c r="C574" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="D574" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="E574" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F574" s="4">
+        <v>36</v>
+      </c>
+      <c r="G574" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H574" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I574" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J574" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K574" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="L574" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M574" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N574" s="4" t="s">
+        <v>4506</v>
+      </c>
+      <c r="O574" s="4" t="s">
+        <v>4507</v>
+      </c>
+      <c r="P574" s="4" t="s">
+        <v>478</v>
+      </c>
+      <c r="Q574" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="R574" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S574" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T574" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U574" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="V574" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W574" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="575" spans="1:23">
+      <c r="A575" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="B575" s="4">
+        <v>13</v>
+      </c>
+      <c r="C575" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="D575" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="E575" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="F575" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="G575" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H575" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I575" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J575" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K575" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L575" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M575" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="N575" s="4" t="s">
+        <v>4508</v>
+      </c>
+      <c r="O575" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="P575" s="4" t="s">
+        <v>478</v>
+      </c>
+      <c r="Q575" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="R575" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="S575" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="T575" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="U575" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V575" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W575" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="576" spans="1:23">
+      <c r="A576" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="B576" s="4">
+        <v>14</v>
+      </c>
+      <c r="C576" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="D576" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="E576" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F576" s="4">
+        <v>36</v>
+      </c>
+      <c r="G576" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H576" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I576" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J576" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K576" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="L576" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M576" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N576" s="4" t="s">
+        <v>4509</v>
+      </c>
+      <c r="O576" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="P576" s="4" t="s">
+        <v>478</v>
+      </c>
+      <c r="Q576" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="R576" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S576" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T576" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U576" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="V576" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W576" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="577" spans="1:23">
+      <c r="A577" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="B577" s="4">
+        <v>15</v>
+      </c>
+      <c r="C577" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="D577" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="E577" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="F577" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="G577" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H577" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I577" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J577" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K577" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L577" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M577" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N577" s="4" t="s">
+        <v>4510</v>
+      </c>
+      <c r="O577" s="4" t="s">
+        <v>4511</v>
+      </c>
+      <c r="P577" s="4" t="s">
+        <v>4512</v>
+      </c>
+      <c r="Q577" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="R577" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="S577" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="T577" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U577" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="V577" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W577" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="578" spans="1:23">
+      <c r="A578" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="B578" s="4">
+        <v>16</v>
+      </c>
+      <c r="C578" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="D578" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="E578" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="F578" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="G578" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H578" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I578" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J578" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K578" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L578" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M578" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="N578" s="4" t="s">
+        <v>486</v>
+      </c>
+      <c r="O578" s="4" t="s">
+        <v>487</v>
+      </c>
+      <c r="P578" s="4" t="s">
+        <v>4513</v>
+      </c>
+      <c r="Q578" s="4">
+        <v>1</v>
+      </c>
+      <c r="R578" s="4">
+        <v>1</v>
+      </c>
+      <c r="S578" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="T578" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="U578" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V578" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W578" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="579" spans="1:23">
+      <c r="A579" s="4" t="s">
+        <v>4441</v>
+      </c>
+      <c r="B579" s="4">
+        <v>1</v>
+      </c>
+      <c r="C579" s="4" t="s">
+        <v>4514</v>
+      </c>
+      <c r="D579" s="4" t="s">
+        <v>4444</v>
+      </c>
+      <c r="E579" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F579" s="4">
+        <v>36</v>
+      </c>
+      <c r="G579" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H579" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I579" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="J579" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K579" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L579" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="M579" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="N579" s="4" t="s">
+        <v>4515</v>
+      </c>
+      <c r="O579" s="4" t="s">
+        <v>4516</v>
+      </c>
+      <c r="P579" s="4" t="s">
+        <v>4517</v>
+      </c>
+      <c r="Q579" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="R579" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="S579" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="T579" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="U579" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="V579" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W579" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="580" spans="1:23">
+      <c r="A580" s="4" t="s">
+        <v>4441</v>
+      </c>
+      <c r="B580" s="4">
+        <v>2</v>
+      </c>
+      <c r="C580" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="D580" s="4" t="s">
+        <v>4437</v>
+      </c>
+      <c r="E580" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F580" s="4">
+        <v>36</v>
+      </c>
+      <c r="G580" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H580" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I580" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J580" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K580" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="L580" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M580" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N580" s="4" t="s">
+        <v>4518</v>
+      </c>
+      <c r="O580" s="4" t="s">
+        <v>4519</v>
+      </c>
+      <c r="P580" s="4" t="s">
+        <v>4520</v>
+      </c>
+      <c r="Q580" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="R580" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S580" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T580" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U580" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="V580" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W580" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="581" spans="1:23">
+      <c r="A581" s="4" t="s">
+        <v>4441</v>
+      </c>
+      <c r="B581" s="4">
+        <v>3</v>
+      </c>
+      <c r="C581" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D581" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="E581" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F581" s="4">
+        <v>36</v>
+      </c>
+      <c r="G581" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H581" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I581" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J581" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K581" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="L581" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M581" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N581" s="4" t="s">
+        <v>4521</v>
+      </c>
+      <c r="O581" s="4" t="s">
+        <v>4522</v>
+      </c>
+      <c r="P581" s="4" t="s">
+        <v>4523</v>
+      </c>
+      <c r="Q581" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="R581" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S581" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T581" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U581" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="V581" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W581" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="582" spans="1:23">
+      <c r="A582" s="4" t="s">
+        <v>4441</v>
+      </c>
+      <c r="B582" s="4">
+        <v>4</v>
+      </c>
+      <c r="C582" s="4" t="s">
+        <v>4445</v>
+      </c>
+      <c r="D582" s="4" t="s">
+        <v>4524</v>
+      </c>
+      <c r="E582" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="F582" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="G582" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H582" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I582" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J582" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K582" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L582" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M582" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="N582" s="4" t="s">
+        <v>4525</v>
+      </c>
+      <c r="O582" s="4" t="s">
+        <v>4526</v>
+      </c>
+      <c r="P582" s="4" t="s">
+        <v>4527</v>
+      </c>
+      <c r="Q582" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="R582" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="S582" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T582" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U582" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V582" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W582" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="583" spans="1:23">
+      <c r="A583" s="4" t="s">
+        <v>4441</v>
+      </c>
+      <c r="B583" s="4">
+        <v>5</v>
+      </c>
+      <c r="C583" s="4" t="s">
+        <v>4455</v>
+      </c>
+      <c r="D583" s="4" t="s">
+        <v>4458</v>
+      </c>
+      <c r="E583" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F583" s="4">
+        <v>36</v>
+      </c>
+      <c r="G583" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H583" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I583" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J583" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K583" s="4" t="s">
+        <v>4455</v>
+      </c>
+      <c r="L583" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M583" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N583" s="4" t="s">
+        <v>4528</v>
+      </c>
+      <c r="O583" s="4" t="s">
+        <v>4529</v>
+      </c>
+      <c r="P583" s="4" t="s">
+        <v>4530</v>
+      </c>
+      <c r="Q583" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="R583" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S583" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T583" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U583" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V583" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W583" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="584" spans="1:23">
+      <c r="A584" s="4" t="s">
+        <v>4441</v>
+      </c>
+      <c r="B584" s="4">
+        <v>6</v>
+      </c>
+      <c r="C584" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D584" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="E584" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F584" s="4">
+        <v>36</v>
+      </c>
+      <c r="G584" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H584" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I584" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J584" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K584" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="L584" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M584" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N584" s="4" t="s">
+        <v>4531</v>
+      </c>
+      <c r="O584" s="4" t="s">
+        <v>4532</v>
+      </c>
+      <c r="P584" s="4" t="s">
+        <v>4533</v>
+      </c>
+      <c r="Q584" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="R584" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S584" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T584" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U584" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="V584" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W584" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="585" spans="1:23">
+      <c r="A585" s="4" t="s">
+        <v>4441</v>
+      </c>
+      <c r="B585" s="4">
+        <v>7</v>
+      </c>
+      <c r="C585" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D585" s="4" t="s">
+        <v>698</v>
+      </c>
+      <c r="E585" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F585" s="4">
+        <v>36</v>
+      </c>
+      <c r="G585" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H585" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I585" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J585" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K585" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="L585" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M585" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N585" s="4" t="s">
+        <v>4534</v>
+      </c>
+      <c r="O585" s="4" t="s">
+        <v>4535</v>
+      </c>
+      <c r="P585" s="4" t="s">
+        <v>4536</v>
+      </c>
+      <c r="Q585" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="R585" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S585" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T585" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U585" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="V585" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W585" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="586" spans="1:23">
+      <c r="A586" s="4" t="s">
+        <v>4441</v>
+      </c>
+      <c r="B586" s="4">
+        <v>8</v>
+      </c>
+      <c r="C586" s="4" t="s">
+        <v>4537</v>
+      </c>
+      <c r="D586" s="4" t="s">
+        <v>4538</v>
+      </c>
+      <c r="E586" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="F586" s="4">
+        <v>50</v>
+      </c>
+      <c r="G586" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H586" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I586" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J586" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K586" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L586" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M586" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N586" s="4" t="s">
+        <v>4539</v>
+      </c>
+      <c r="O586" s="4" t="s">
+        <v>4540</v>
+      </c>
+      <c r="P586" s="4" t="s">
+        <v>4541</v>
+      </c>
+      <c r="Q586" s="4" t="s">
+        <v>4542</v>
+      </c>
+      <c r="R586" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S586" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T586" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U586" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V586" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="W586" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="587" spans="1:23">
+      <c r="A587" s="4" t="s">
+        <v>4441</v>
+      </c>
+      <c r="B587" s="4">
+        <v>9</v>
+      </c>
+      <c r="C587" s="4" t="s">
+        <v>4482</v>
+      </c>
+      <c r="D587" s="4" t="s">
+        <v>4483</v>
+      </c>
+      <c r="E587" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="F587" s="4">
+        <v>50</v>
+      </c>
+      <c r="G587" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H587" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I587" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J587" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K587" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L587" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M587" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N587" s="4" t="s">
+        <v>4543</v>
+      </c>
+      <c r="O587" s="4" t="s">
+        <v>4544</v>
+      </c>
+      <c r="P587" s="4" t="s">
+        <v>4545</v>
+      </c>
+      <c r="Q587" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="R587" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S587" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T587" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U587" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V587" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W587" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="588" spans="1:23">
+      <c r="A588" s="4" t="s">
+        <v>4441</v>
+      </c>
+      <c r="B588" s="4">
+        <v>10</v>
+      </c>
+      <c r="C588" s="4" t="s">
+        <v>4487</v>
+      </c>
+      <c r="D588" s="4" t="s">
+        <v>4488</v>
+      </c>
+      <c r="E588" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F588" s="4">
+        <v>36</v>
+      </c>
+      <c r="G588" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H588" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I588" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J588" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K588" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L588" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M588" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N588" s="4" t="s">
+        <v>4546</v>
+      </c>
+      <c r="O588" s="4" t="s">
+        <v>4547</v>
+      </c>
+      <c r="P588" s="4" t="s">
+        <v>4548</v>
+      </c>
+      <c r="Q588" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="R588" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S588" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T588" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U588" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V588" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W588" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="589" spans="1:23">
+      <c r="A589" s="4" t="s">
+        <v>4441</v>
+      </c>
+      <c r="B589" s="4">
+        <v>11</v>
+      </c>
+      <c r="C589" s="4" t="s">
+        <v>4549</v>
+      </c>
+      <c r="D589" s="4" t="s">
+        <v>4550</v>
+      </c>
+      <c r="E589" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="F589" s="4">
+        <v>500</v>
+      </c>
+      <c r="G589" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H589" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I589" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J589" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K589" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L589" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M589" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N589" s="4" t="s">
+        <v>4551</v>
+      </c>
+      <c r="O589" s="4" t="s">
+        <v>4552</v>
+      </c>
+      <c r="P589" s="4" t="s">
+        <v>4553</v>
+      </c>
+      <c r="Q589" s="4" t="s">
+        <v>4554</v>
+      </c>
+      <c r="R589" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S589" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T589" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="U589" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="V589" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="W589" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="590" spans="1:23">
+      <c r="A590" s="4" t="s">
+        <v>4441</v>
+      </c>
+      <c r="B590" s="4">
+        <v>12</v>
+      </c>
+      <c r="C590" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="D590" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="E590" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="F590" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="G590" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H590" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I590" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J590" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K590" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L590" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M590" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="N590" s="4" t="s">
+        <v>4555</v>
+      </c>
+      <c r="O590" s="4" t="s">
+        <v>4556</v>
+      </c>
+      <c r="P590" s="4" t="s">
+        <v>4557</v>
+      </c>
+      <c r="Q590" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="R590" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="S590" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="T590" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="U590" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V590" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W590" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="591" spans="1:23">
+      <c r="A591" s="4" t="s">
+        <v>4441</v>
+      </c>
+      <c r="B591" s="4">
+        <v>13</v>
+      </c>
+      <c r="C591" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="D591" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="E591" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F591" s="4">
+        <v>36</v>
+      </c>
+      <c r="G591" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H591" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I591" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J591" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K591" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="L591" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M591" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N591" s="4" t="s">
+        <v>4558</v>
+      </c>
+      <c r="O591" s="4" t="s">
+        <v>4559</v>
+      </c>
+      <c r="P591" s="4" t="s">
+        <v>4560</v>
+      </c>
+      <c r="Q591" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="R591" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S591" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T591" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U591" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="V591" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W591" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="592" spans="1:23">
+      <c r="A592" s="4" t="s">
+        <v>4441</v>
+      </c>
+      <c r="B592" s="4">
+        <v>14</v>
+      </c>
+      <c r="C592" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="D592" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="E592" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="F592" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="G592" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H592" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I592" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J592" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K592" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L592" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M592" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="N592" s="4" t="s">
+        <v>4561</v>
+      </c>
+      <c r="O592" s="4" t="s">
+        <v>4562</v>
+      </c>
+      <c r="P592" s="4" t="s">
+        <v>4563</v>
+      </c>
+      <c r="Q592" s="4">
+        <v>1</v>
+      </c>
+      <c r="R592" s="4">
+        <v>1</v>
+      </c>
+      <c r="S592" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="T592" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="U592" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V592" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W592" s="4" t="s">
         <v>6</v>
       </c>
     </row>
@@ -65921,7 +69306,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96FF8F3C-B975-44A1-AEC1-A0B924B73AFA}">
-  <dimension ref="A1:I96"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="28.28515625" style="4" customWidth="1"/>
@@ -68590,6 +71975,296 @@
       </c>
       <c r="I96" s="4" t="s">
         <v>3928</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9">
+      <c r="A97" s="4" t="s">
+        <v>4448</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="C97" s="4" t="s">
+        <v>4598</v>
+      </c>
+      <c r="D97" s="4" t="s">
+        <v>4599</v>
+      </c>
+      <c r="E97" s="4" t="s">
+        <v>4600</v>
+      </c>
+      <c r="F97" s="4">
+        <v>1</v>
+      </c>
+      <c r="G97" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H97" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I97" s="4" t="s">
+        <v>4601</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9">
+      <c r="A98" s="4" t="s">
+        <v>4448</v>
+      </c>
+      <c r="B98" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="C98" s="4" t="s">
+        <v>4602</v>
+      </c>
+      <c r="D98" s="4" t="s">
+        <v>4603</v>
+      </c>
+      <c r="E98" s="4" t="s">
+        <v>4604</v>
+      </c>
+      <c r="F98" s="4">
+        <v>2</v>
+      </c>
+      <c r="G98" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H98" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I98" s="4" t="s">
+        <v>4605</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9">
+      <c r="A99" s="4" t="s">
+        <v>4448</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="C99" s="4" t="s">
+        <v>4606</v>
+      </c>
+      <c r="D99" s="4" t="s">
+        <v>4607</v>
+      </c>
+      <c r="E99" s="4" t="s">
+        <v>4608</v>
+      </c>
+      <c r="F99" s="4">
+        <v>3</v>
+      </c>
+      <c r="G99" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H99" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I99" s="4" t="s">
+        <v>4609</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9">
+      <c r="A100" s="4" t="s">
+        <v>4448</v>
+      </c>
+      <c r="B100" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="C100" s="4" t="s">
+        <v>4610</v>
+      </c>
+      <c r="D100" s="4" t="s">
+        <v>4611</v>
+      </c>
+      <c r="E100" s="4" t="s">
+        <v>4612</v>
+      </c>
+      <c r="F100" s="4">
+        <v>4</v>
+      </c>
+      <c r="G100" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H100" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I100" s="4" t="s">
+        <v>4613</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9">
+      <c r="A101" s="4" t="s">
+        <v>4455</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="C101" s="4" t="s">
+        <v>872</v>
+      </c>
+      <c r="D101" s="4" t="s">
+        <v>717</v>
+      </c>
+      <c r="E101" s="4" t="s">
+        <v>4614</v>
+      </c>
+      <c r="F101" s="4">
+        <v>1</v>
+      </c>
+      <c r="G101" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H101" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I101" s="4" t="s">
+        <v>4615</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9">
+      <c r="A102" s="4" t="s">
+        <v>4455</v>
+      </c>
+      <c r="B102" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="C102" s="4" t="s">
+        <v>4616</v>
+      </c>
+      <c r="D102" s="4" t="s">
+        <v>4617</v>
+      </c>
+      <c r="E102" s="4" t="s">
+        <v>4618</v>
+      </c>
+      <c r="F102" s="4">
+        <v>2</v>
+      </c>
+      <c r="G102" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H102" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I102" s="4" t="s">
+        <v>4619</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9">
+      <c r="A103" s="4" t="s">
+        <v>4455</v>
+      </c>
+      <c r="B103" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="C103" s="4" t="s">
+        <v>866</v>
+      </c>
+      <c r="D103" s="4" t="s">
+        <v>4620</v>
+      </c>
+      <c r="E103" s="4" t="s">
+        <v>4621</v>
+      </c>
+      <c r="F103" s="4">
+        <v>3</v>
+      </c>
+      <c r="G103" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H103" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I103" s="4" t="s">
+        <v>4622</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9">
+      <c r="A104" s="4" t="s">
+        <v>4455</v>
+      </c>
+      <c r="B104" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="C104" s="4" t="s">
+        <v>877</v>
+      </c>
+      <c r="D104" s="4" t="s">
+        <v>4623</v>
+      </c>
+      <c r="E104" s="4" t="s">
+        <v>4624</v>
+      </c>
+      <c r="F104" s="4">
+        <v>4</v>
+      </c>
+      <c r="G104" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H104" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I104" s="4" t="s">
+        <v>4625</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9">
+      <c r="A105" s="4" t="s">
+        <v>4455</v>
+      </c>
+      <c r="B105" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="C105" s="4" t="s">
+        <v>4626</v>
+      </c>
+      <c r="D105" s="4" t="s">
+        <v>4627</v>
+      </c>
+      <c r="E105" s="4" t="s">
+        <v>4628</v>
+      </c>
+      <c r="F105" s="4">
+        <v>5</v>
+      </c>
+      <c r="G105" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H105" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I105" s="4" t="s">
+        <v>4629</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9">
+      <c r="A106" s="4" t="s">
+        <v>4455</v>
+      </c>
+      <c r="B106" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="C106" s="4" t="s">
+        <v>4630</v>
+      </c>
+      <c r="D106" s="4" t="s">
+        <v>4631</v>
+      </c>
+      <c r="E106" s="4" t="s">
+        <v>4632</v>
+      </c>
+      <c r="F106" s="4">
+        <v>6</v>
+      </c>
+      <c r="G106" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H106" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I106" s="4" t="s">
+        <v>4633</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
QR implementation Stage 4
</commit_message>
<xml_diff>
--- a/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
+++ b/docs/domain/Memgine_Physical_Data_Model_catalogue.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MynikaTech\memgine\docs\domain\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E648539-C542-4F56-B93B-FFAA79B83836}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{354F09F5-5A12-44DB-88BA-14394BAE67E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="3" activeTab="11" xr2:uid="{AA28BC4D-8219-43B9-8C16-6977709D904A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="6" activeTab="13" xr2:uid="{AA28BC4D-8219-43B9-8C16-6977709D904A}"/>
   </bookViews>
   <sheets>
     <sheet name="Entity Catalogue" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18252" uniqueCount="4635">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18546" uniqueCount="4690">
   <si>
     <t>Domain</t>
   </si>
@@ -13949,6 +13949,171 @@
   </si>
   <si>
     <t>QR_CODE</t>
+  </si>
+  <si>
+    <t>QRACQATTR</t>
+  </si>
+  <si>
+    <t>QR Acquisition</t>
+  </si>
+  <si>
+    <t>QR Membership Acquisition Attribution</t>
+  </si>
+  <si>
+    <t>qr_membership_acquisition_attributions</t>
+  </si>
+  <si>
+    <t>Links a successful business-membership QR scan to the membership subscription created from that acquisition journey.</t>
+  </si>
+  <si>
+    <t>qr_membership_acquisition_attribution_id</t>
+  </si>
+  <si>
+    <t>Attributed At</t>
+  </si>
+  <si>
+    <t>Relationship entity connecting a qualifying QR scan to the resulting membership subscription without modifying QR Scan History.</t>
+  </si>
+  <si>
+    <t>QR Membership Acquisition Attribution Identifier</t>
+  </si>
+  <si>
+    <t>Uniquely identifies the acquisition attribution record.</t>
+  </si>
+  <si>
+    <t>System-generated identifier for the attribution record.</t>
+  </si>
+  <si>
+    <t>Represents the relationship between a QR scan and the resulting membership subscription.</t>
+  </si>
+  <si>
+    <t>Identifies the QR scan that generated the acquisition journey.</t>
+  </si>
+  <si>
+    <t>References the source QR Scan History record.</t>
+  </si>
+  <si>
+    <t>Links the membership acquisition attribution to the immutable QR scan event.</t>
+  </si>
+  <si>
+    <t>Identifies the membership subscription created from the QR acquisition journey.</t>
+  </si>
+  <si>
+    <t>References the resulting membership subscription.</t>
+  </si>
+  <si>
+    <t>Links the QR scan to the membership purchased from that journey.</t>
+  </si>
+  <si>
+    <t>Identifies the organization associated with the acquisition.</t>
+  </si>
+  <si>
+    <t>References the organization owning the QR and membership.</t>
+  </si>
+  <si>
+    <t>Preserves tenant context for attribution reporting.</t>
+  </si>
+  <si>
+    <t>Identifies the membership product acquired.</t>
+  </si>
+  <si>
+    <t>References the membership product associated with the subscription plan.</t>
+  </si>
+  <si>
+    <t>Supports membership-product-level acquisition analytics.</t>
+  </si>
+  <si>
+    <t>customer_id</t>
+  </si>
+  <si>
+    <t>Identifies the customer associated with the attributed acquisition when known.</t>
+  </si>
+  <si>
+    <t>References the customer associated with the organization user.</t>
+  </si>
+  <si>
+    <t>Supports customer-level QR acquisition analytics.</t>
+  </si>
+  <si>
+    <t>attributed_at</t>
+  </si>
+  <si>
+    <t>Records when the QR scan was attributed to the subscription.</t>
+  </si>
+  <si>
+    <t>Timestamp when attribution was created.</t>
+  </si>
+  <si>
+    <t>Records the point at which the scan-to-subscription relationship was established.</t>
+  </si>
+  <si>
+    <t>Timestamp when the attribution record was created.</t>
+  </si>
+  <si>
+    <t>Identifies the user or system that created the attribution.</t>
+  </si>
+  <si>
+    <t>References the creating user when available.</t>
+  </si>
+  <si>
+    <t>Organization has QR Membership Acquisition Attributions</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>Each acquisition attribution belongs to one organization.</t>
+  </si>
+  <si>
+    <t>Scan History has Acquisition Attribution</t>
+  </si>
+  <si>
+    <t>1:0..1</t>
+  </si>
+  <si>
+    <t>A QR scan may result in zero or one membership acquisition attribution.</t>
+  </si>
+  <si>
+    <t>Subscription has QR Acquisition Attribution</t>
+  </si>
+  <si>
+    <t>A membership subscription may have zero or one QR acquisition attribution.</t>
+  </si>
+  <si>
+    <t>Membership Product has QR Acquisition Attributions</t>
+  </si>
+  <si>
+    <t>Identifies the membership product acquired through the QR journey.</t>
+  </si>
+  <si>
+    <t>QR Code has Scan History</t>
+  </si>
+  <si>
+    <t>Each QR scan history record references the QR Code that was scanned.</t>
+  </si>
+  <si>
+    <t>QR Code has QR Code Type</t>
+  </si>
+  <si>
+    <t>Identifies the journey type configured for the QR Code.</t>
+  </si>
+  <si>
+    <t>REL095</t>
+  </si>
+  <si>
+    <t>REL096</t>
+  </si>
+  <si>
+    <t>REL097</t>
+  </si>
+  <si>
+    <t>REL098</t>
+  </si>
+  <si>
+    <t>REL099</t>
+  </si>
+  <si>
+    <t>REL100</t>
   </si>
 </sst>
 </file>
@@ -14180,7 +14345,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3841114F-D1EC-49B1-850B-590431E39412}" name="Table2" displayName="Table2" ref="A1:Q51" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{3841114F-D1EC-49B1-850B-590431E39412}" name="Table2" displayName="Table2" ref="A1:Q52" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{FEF6275C-74E6-4563-BFF3-6461E4A3D8DA}" name="Entity Code" dataDxfId="16"/>
     <tableColumn id="2" xr3:uid="{67FE23FD-539D-4023-BA73-D2A0B84718BF}" name="Domain" dataDxfId="15"/>
@@ -14501,7 +14666,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4659496D-1A4F-4BC3-BD65-377E70E6B8BE}">
-  <dimension ref="A1:Q51"/>
+  <dimension ref="A1:Q52"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="31.85546875" style="4" customWidth="1"/>
@@ -17206,6 +17371,59 @@
         <v>4460</v>
       </c>
     </row>
+    <row r="52" spans="1:17" ht="60">
+      <c r="A52" s="4" t="s">
+        <v>4635</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>733</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>4636</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>4637</v>
+      </c>
+      <c r="E52" s="4" t="s">
+        <v>4638</v>
+      </c>
+      <c r="F52" s="4" t="s">
+        <v>4639</v>
+      </c>
+      <c r="G52" s="4" t="s">
+        <v>623</v>
+      </c>
+      <c r="H52" s="4" t="s">
+        <v>733</v>
+      </c>
+      <c r="I52" s="4" t="s">
+        <v>4441</v>
+      </c>
+      <c r="J52" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K52" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="L52" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="M52" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="N52" s="4" t="s">
+        <v>4640</v>
+      </c>
+      <c r="O52" s="4" t="s">
+        <v>4641</v>
+      </c>
+      <c r="P52" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q52" s="4" t="s">
+        <v>4642</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -20781,7 +20999,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C85B9BC7-C8C8-4E3E-A0EF-02B9554CEAE5}">
-  <dimension ref="A1:K95"/>
+  <dimension ref="A1:K101"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14.5703125" style="4" bestFit="1" customWidth="1"/>
@@ -23703,7 +23921,7 @@
         <v>4431</v>
       </c>
     </row>
-    <row r="84" spans="1:11">
+    <row r="84" spans="1:11" ht="30">
       <c r="A84" s="4" t="s">
         <v>4564</v>
       </c>
@@ -23808,7 +24026,7 @@
         <v>4571</v>
       </c>
     </row>
-    <row r="87" spans="1:11">
+    <row r="87" spans="1:11" ht="30">
       <c r="A87" s="4" t="s">
         <v>4572</v>
       </c>
@@ -23948,7 +24166,7 @@
         <v>4583</v>
       </c>
     </row>
-    <row r="91" spans="1:11">
+    <row r="91" spans="1:11" ht="30">
       <c r="A91" s="4" t="s">
         <v>4584</v>
       </c>
@@ -24018,7 +24236,7 @@
         <v>4588</v>
       </c>
     </row>
-    <row r="93" spans="1:11">
+    <row r="93" spans="1:11" ht="30">
       <c r="A93" s="4" t="s">
         <v>4589</v>
       </c>
@@ -24053,7 +24271,7 @@
         <v>4591</v>
       </c>
     </row>
-    <row r="94" spans="1:11">
+    <row r="94" spans="1:11" ht="30">
       <c r="A94" s="4" t="s">
         <v>4592</v>
       </c>
@@ -24088,7 +24306,7 @@
         <v>4594</v>
       </c>
     </row>
-    <row r="95" spans="1:11">
+    <row r="95" spans="1:11" ht="30">
       <c r="A95" s="4" t="s">
         <v>4595</v>
       </c>
@@ -24121,6 +24339,216 @@
       </c>
       <c r="K95" s="4" t="s">
         <v>4597</v>
+      </c>
+    </row>
+    <row r="96" spans="1:11" ht="45">
+      <c r="A96" s="4" t="s">
+        <v>4684</v>
+      </c>
+      <c r="B96" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C96" s="4" t="s">
+        <v>4637</v>
+      </c>
+      <c r="D96" s="4" t="s">
+        <v>4670</v>
+      </c>
+      <c r="E96" s="4" t="s">
+        <v>4671</v>
+      </c>
+      <c r="F96" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="G96" s="4" t="s">
+        <v>1298</v>
+      </c>
+      <c r="H96" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I96" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="J96" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K96" s="4" t="s">
+        <v>4672</v>
+      </c>
+    </row>
+    <row r="97" spans="1:11" ht="30">
+      <c r="A97" s="4" t="s">
+        <v>4685</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>4441</v>
+      </c>
+      <c r="C97" s="4" t="s">
+        <v>4637</v>
+      </c>
+      <c r="D97" s="4" t="s">
+        <v>4673</v>
+      </c>
+      <c r="E97" s="4" t="s">
+        <v>4671</v>
+      </c>
+      <c r="F97" s="4" t="s">
+        <v>4444</v>
+      </c>
+      <c r="G97" s="4" t="s">
+        <v>4674</v>
+      </c>
+      <c r="H97" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I97" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="J97" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K97" s="4" t="s">
+        <v>4675</v>
+      </c>
+    </row>
+    <row r="98" spans="1:11" ht="30">
+      <c r="A98" s="4" t="s">
+        <v>4686</v>
+      </c>
+      <c r="B98" s="4" t="s">
+        <v>620</v>
+      </c>
+      <c r="C98" s="4" t="s">
+        <v>4637</v>
+      </c>
+      <c r="D98" s="4" t="s">
+        <v>4676</v>
+      </c>
+      <c r="E98" s="4" t="s">
+        <v>4671</v>
+      </c>
+      <c r="F98" s="4" t="s">
+        <v>624</v>
+      </c>
+      <c r="G98" s="4" t="s">
+        <v>4674</v>
+      </c>
+      <c r="H98" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I98" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="J98" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K98" s="4" t="s">
+        <v>4677</v>
+      </c>
+    </row>
+    <row r="99" spans="1:11" ht="30">
+      <c r="A99" s="4" t="s">
+        <v>4687</v>
+      </c>
+      <c r="B99" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C99" s="4" t="s">
+        <v>4637</v>
+      </c>
+      <c r="D99" s="4" t="s">
+        <v>4678</v>
+      </c>
+      <c r="E99" s="4" t="s">
+        <v>4671</v>
+      </c>
+      <c r="F99" s="4" t="s">
+        <v>420</v>
+      </c>
+      <c r="G99" s="4" t="s">
+        <v>1298</v>
+      </c>
+      <c r="H99" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I99" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="J99" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K99" s="4" t="s">
+        <v>4679</v>
+      </c>
+    </row>
+    <row r="100" spans="1:11" ht="30">
+      <c r="A100" s="4" t="s">
+        <v>4688</v>
+      </c>
+      <c r="B100" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="C100" s="4" t="s">
+        <v>4441</v>
+      </c>
+      <c r="D100" s="4" t="s">
+        <v>4680</v>
+      </c>
+      <c r="E100" s="4" t="s">
+        <v>4671</v>
+      </c>
+      <c r="F100" s="4" t="s">
+        <v>4437</v>
+      </c>
+      <c r="G100" s="4" t="s">
+        <v>1298</v>
+      </c>
+      <c r="H100" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I100" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="J100" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K100" s="4" t="s">
+        <v>4681</v>
+      </c>
+    </row>
+    <row r="101" spans="1:11">
+      <c r="A101" s="4" t="s">
+        <v>4689</v>
+      </c>
+      <c r="B101" s="4" t="s">
+        <v>4448</v>
+      </c>
+      <c r="C101" s="4" t="s">
+        <v>4434</v>
+      </c>
+      <c r="D101" s="4" t="s">
+        <v>4682</v>
+      </c>
+      <c r="E101" s="4" t="s">
+        <v>4671</v>
+      </c>
+      <c r="F101" s="4" t="s">
+        <v>4451</v>
+      </c>
+      <c r="G101" s="4" t="s">
+        <v>1298</v>
+      </c>
+      <c r="H101" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I101" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="J101" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K101" s="4" t="s">
+        <v>4683</v>
       </c>
     </row>
   </sheetData>
@@ -28178,7 +28606,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E21F442-9136-4C15-8BA3-92E07332B93A}">
-  <dimension ref="A1:W592"/>
+  <dimension ref="A1:W602"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="22.140625" style="4" customWidth="1"/>
@@ -66934,7 +67362,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="563" spans="1:23">
+    <row r="563" spans="1:23" ht="30">
       <c r="A563" s="4" t="s">
         <v>4434</v>
       </c>
@@ -67005,7 +67433,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="564" spans="1:23">
+    <row r="564" spans="1:23" ht="30">
       <c r="A564" s="4" t="s">
         <v>4434</v>
       </c>
@@ -67076,7 +67504,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="565" spans="1:23">
+    <row r="565" spans="1:23" ht="45">
       <c r="A565" s="4" t="s">
         <v>4434</v>
       </c>
@@ -67147,7 +67575,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="566" spans="1:23">
+    <row r="566" spans="1:23" ht="60">
       <c r="A566" s="4" t="s">
         <v>4434</v>
       </c>
@@ -67218,7 +67646,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="567" spans="1:23">
+    <row r="567" spans="1:23" ht="45">
       <c r="A567" s="4" t="s">
         <v>4434</v>
       </c>
@@ -67289,7 +67717,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="568" spans="1:23">
+    <row r="568" spans="1:23" ht="45">
       <c r="A568" s="4" t="s">
         <v>4434</v>
       </c>
@@ -67360,7 +67788,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="569" spans="1:23">
+    <row r="569" spans="1:23" ht="45">
       <c r="A569" s="4" t="s">
         <v>4434</v>
       </c>
@@ -67431,7 +67859,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="570" spans="1:23">
+    <row r="570" spans="1:23" ht="45">
       <c r="A570" s="4" t="s">
         <v>4434</v>
       </c>
@@ -67502,7 +67930,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="571" spans="1:23">
+    <row r="571" spans="1:23" ht="45">
       <c r="A571" s="4" t="s">
         <v>4434</v>
       </c>
@@ -67573,7 +68001,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="572" spans="1:23">
+    <row r="572" spans="1:23" ht="30">
       <c r="A572" s="4" t="s">
         <v>4434</v>
       </c>
@@ -67644,7 +68072,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="573" spans="1:23">
+    <row r="573" spans="1:23" ht="30">
       <c r="A573" s="4" t="s">
         <v>4434</v>
       </c>
@@ -67715,7 +68143,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="574" spans="1:23">
+    <row r="574" spans="1:23" ht="30">
       <c r="A574" s="4" t="s">
         <v>4434</v>
       </c>
@@ -67786,7 +68214,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="575" spans="1:23">
+    <row r="575" spans="1:23" ht="30">
       <c r="A575" s="4" t="s">
         <v>4434</v>
       </c>
@@ -67857,7 +68285,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="576" spans="1:23">
+    <row r="576" spans="1:23" ht="30">
       <c r="A576" s="4" t="s">
         <v>4434</v>
       </c>
@@ -67928,7 +68356,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="577" spans="1:23">
+    <row r="577" spans="1:23" ht="30">
       <c r="A577" s="4" t="s">
         <v>4434</v>
       </c>
@@ -67999,7 +68427,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="578" spans="1:23">
+    <row r="578" spans="1:23" ht="30">
       <c r="A578" s="4" t="s">
         <v>4434</v>
       </c>
@@ -68070,7 +68498,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="579" spans="1:23">
+    <row r="579" spans="1:23" ht="30">
       <c r="A579" s="4" t="s">
         <v>4441</v>
       </c>
@@ -68141,7 +68569,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="580" spans="1:23">
+    <row r="580" spans="1:23" ht="30">
       <c r="A580" s="4" t="s">
         <v>4441</v>
       </c>
@@ -68212,7 +68640,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="581" spans="1:23">
+    <row r="581" spans="1:23" ht="45">
       <c r="A581" s="4" t="s">
         <v>4441</v>
       </c>
@@ -68283,7 +68711,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="582" spans="1:23">
+    <row r="582" spans="1:23" ht="30">
       <c r="A582" s="4" t="s">
         <v>4441</v>
       </c>
@@ -68354,7 +68782,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="583" spans="1:23">
+    <row r="583" spans="1:23" ht="30">
       <c r="A583" s="4" t="s">
         <v>4441</v>
       </c>
@@ -68425,7 +68853,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="584" spans="1:23">
+    <row r="584" spans="1:23" ht="30">
       <c r="A584" s="4" t="s">
         <v>4441</v>
       </c>
@@ -68496,7 +68924,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="585" spans="1:23">
+    <row r="585" spans="1:23" ht="45">
       <c r="A585" s="4" t="s">
         <v>4441</v>
       </c>
@@ -68567,7 +68995,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="586" spans="1:23">
+    <row r="586" spans="1:23" ht="45">
       <c r="A586" s="4" t="s">
         <v>4441</v>
       </c>
@@ -68638,7 +69066,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="587" spans="1:23">
+    <row r="587" spans="1:23" ht="30">
       <c r="A587" s="4" t="s">
         <v>4441</v>
       </c>
@@ -68709,7 +69137,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="588" spans="1:23">
+    <row r="588" spans="1:23" ht="30">
       <c r="A588" s="4" t="s">
         <v>4441</v>
       </c>
@@ -68780,7 +69208,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="589" spans="1:23">
+    <row r="589" spans="1:23" ht="45">
       <c r="A589" s="4" t="s">
         <v>4441</v>
       </c>
@@ -68851,7 +69279,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="590" spans="1:23">
+    <row r="590" spans="1:23" ht="30">
       <c r="A590" s="4" t="s">
         <v>4441</v>
       </c>
@@ -68922,7 +69350,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="591" spans="1:23">
+    <row r="591" spans="1:23" ht="45">
       <c r="A591" s="4" t="s">
         <v>4441</v>
       </c>
@@ -68993,7 +69421,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="592" spans="1:23">
+    <row r="592" spans="1:23" ht="30">
       <c r="A592" s="4" t="s">
         <v>4441</v>
       </c>
@@ -69061,6 +69489,716 @@
         <v>6</v>
       </c>
       <c r="W592" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="593" spans="1:23">
+      <c r="A593" s="4" t="s">
+        <v>4637</v>
+      </c>
+      <c r="B593" s="4">
+        <v>1</v>
+      </c>
+      <c r="C593" s="4" t="s">
+        <v>4643</v>
+      </c>
+      <c r="D593" s="4" t="s">
+        <v>4640</v>
+      </c>
+      <c r="E593" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F593" s="4">
+        <v>36</v>
+      </c>
+      <c r="G593" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H593" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I593" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="J593" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K593" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L593" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="M593" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="N593" s="4" t="s">
+        <v>4644</v>
+      </c>
+      <c r="O593" s="4" t="s">
+        <v>4645</v>
+      </c>
+      <c r="P593" s="4" t="s">
+        <v>4646</v>
+      </c>
+      <c r="Q593" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="R593" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="S593" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="T593" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="U593" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="V593" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W593" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="594" spans="1:23">
+      <c r="A594" s="4" t="s">
+        <v>4637</v>
+      </c>
+      <c r="B594" s="4">
+        <v>2</v>
+      </c>
+      <c r="C594" s="4" t="s">
+        <v>4441</v>
+      </c>
+      <c r="D594" s="4" t="s">
+        <v>4444</v>
+      </c>
+      <c r="E594" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F594" s="4">
+        <v>36</v>
+      </c>
+      <c r="G594" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H594" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I594" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J594" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K594" s="4" t="s">
+        <v>4441</v>
+      </c>
+      <c r="L594" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M594" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N594" s="4" t="s">
+        <v>4647</v>
+      </c>
+      <c r="O594" s="4" t="s">
+        <v>4648</v>
+      </c>
+      <c r="P594" s="4" t="s">
+        <v>4649</v>
+      </c>
+      <c r="Q594" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="R594" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S594" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T594" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U594" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V594" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W594" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="595" spans="1:23">
+      <c r="A595" s="4" t="s">
+        <v>4637</v>
+      </c>
+      <c r="B595" s="4">
+        <v>3</v>
+      </c>
+      <c r="C595" s="4" t="s">
+        <v>620</v>
+      </c>
+      <c r="D595" s="4" t="s">
+        <v>624</v>
+      </c>
+      <c r="E595" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F595" s="4">
+        <v>36</v>
+      </c>
+      <c r="G595" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H595" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I595" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J595" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K595" s="4" t="s">
+        <v>620</v>
+      </c>
+      <c r="L595" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M595" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N595" s="4" t="s">
+        <v>4650</v>
+      </c>
+      <c r="O595" s="4" t="s">
+        <v>4651</v>
+      </c>
+      <c r="P595" s="4" t="s">
+        <v>4652</v>
+      </c>
+      <c r="Q595" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="R595" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S595" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T595" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U595" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V595" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W595" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="596" spans="1:23">
+      <c r="A596" s="4" t="s">
+        <v>4637</v>
+      </c>
+      <c r="B596" s="4">
+        <v>4</v>
+      </c>
+      <c r="C596" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D596" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E596" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F596" s="4">
+        <v>36</v>
+      </c>
+      <c r="G596" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H596" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I596" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J596" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K596" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="L596" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M596" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N596" s="4" t="s">
+        <v>4653</v>
+      </c>
+      <c r="O596" s="4" t="s">
+        <v>4654</v>
+      </c>
+      <c r="P596" s="4" t="s">
+        <v>4655</v>
+      </c>
+      <c r="Q596" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="R596" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S596" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T596" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U596" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V596" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W596" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="597" spans="1:23">
+      <c r="A597" s="4" t="s">
+        <v>4637</v>
+      </c>
+      <c r="B597" s="4">
+        <v>5</v>
+      </c>
+      <c r="C597" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D597" s="4" t="s">
+        <v>420</v>
+      </c>
+      <c r="E597" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F597" s="4">
+        <v>36</v>
+      </c>
+      <c r="G597" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H597" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I597" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J597" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K597" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="L597" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M597" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N597" s="4" t="s">
+        <v>4656</v>
+      </c>
+      <c r="O597" s="4" t="s">
+        <v>4657</v>
+      </c>
+      <c r="P597" s="4" t="s">
+        <v>4658</v>
+      </c>
+      <c r="Q597" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="R597" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S597" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T597" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U597" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V597" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W597" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="598" spans="1:23">
+      <c r="A598" s="4" t="s">
+        <v>4637</v>
+      </c>
+      <c r="B598" s="4">
+        <v>6</v>
+      </c>
+      <c r="C598" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D598" s="4" t="s">
+        <v>4659</v>
+      </c>
+      <c r="E598" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F598" s="4">
+        <v>36</v>
+      </c>
+      <c r="G598" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H598" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I598" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J598" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K598" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="L598" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M598" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N598" s="4" t="s">
+        <v>4660</v>
+      </c>
+      <c r="O598" s="4" t="s">
+        <v>4661</v>
+      </c>
+      <c r="P598" s="4" t="s">
+        <v>4662</v>
+      </c>
+      <c r="Q598" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="R598" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S598" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T598" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U598" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="V598" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="W598" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="599" spans="1:23">
+      <c r="A599" s="4" t="s">
+        <v>4637</v>
+      </c>
+      <c r="B599" s="4">
+        <v>7</v>
+      </c>
+      <c r="C599" s="4" t="s">
+        <v>4641</v>
+      </c>
+      <c r="D599" s="4" t="s">
+        <v>4663</v>
+      </c>
+      <c r="E599" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="F599" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="G599" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H599" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I599" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J599" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K599" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L599" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M599" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N599" s="4" t="s">
+        <v>4664</v>
+      </c>
+      <c r="O599" s="4" t="s">
+        <v>4665</v>
+      </c>
+      <c r="P599" s="4" t="s">
+        <v>4666</v>
+      </c>
+      <c r="Q599" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="R599" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="S599" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T599" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U599" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V599" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W599" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="600" spans="1:23">
+      <c r="A600" s="4" t="s">
+        <v>4637</v>
+      </c>
+      <c r="B600" s="4">
+        <v>8</v>
+      </c>
+      <c r="C600" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="D600" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="E600" s="4" t="s">
+        <v>296</v>
+      </c>
+      <c r="F600" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="G600" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H600" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I600" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J600" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K600" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L600" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M600" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="N600" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="O600" s="4" t="s">
+        <v>4667</v>
+      </c>
+      <c r="P600" s="4" t="s">
+        <v>297</v>
+      </c>
+      <c r="Q600" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="R600" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="S600" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="T600" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="U600" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V600" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W600" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="601" spans="1:23">
+      <c r="A601" s="4" t="s">
+        <v>4637</v>
+      </c>
+      <c r="B601" s="4">
+        <v>9</v>
+      </c>
+      <c r="C601" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="D601" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="E601" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="F601" s="4">
+        <v>36</v>
+      </c>
+      <c r="G601" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H601" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I601" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J601" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="K601" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="L601" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M601" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="N601" s="4" t="s">
+        <v>4668</v>
+      </c>
+      <c r="O601" s="4" t="s">
+        <v>4669</v>
+      </c>
+      <c r="P601" s="4" t="s">
+        <v>297</v>
+      </c>
+      <c r="Q601" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="R601" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="S601" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="T601" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="U601" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="V601" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W601" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="602" spans="1:23">
+      <c r="A602" s="4" t="s">
+        <v>4637</v>
+      </c>
+      <c r="B602" s="4">
+        <v>10</v>
+      </c>
+      <c r="C602" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="D602" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="E602" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="F602" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="G602" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H602" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I602" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J602" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="K602" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="L602" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M602" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="N602" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="O602" s="4" t="s">
+        <v>617</v>
+      </c>
+      <c r="P602" s="4" t="s">
+        <v>618</v>
+      </c>
+      <c r="Q602" s="4">
+        <v>1</v>
+      </c>
+      <c r="R602" s="4">
+        <v>1</v>
+      </c>
+      <c r="S602" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="T602" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="U602" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="V602" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="W602" s="4" t="s">
         <v>6</v>
       </c>
     </row>
@@ -71977,7 +73115,7 @@
         <v>3928</v>
       </c>
     </row>
-    <row r="97" spans="1:9">
+    <row r="97" spans="1:9" ht="90">
       <c r="A97" s="4" t="s">
         <v>4448</v>
       </c>
@@ -72006,7 +73144,7 @@
         <v>4601</v>
       </c>
     </row>
-    <row r="98" spans="1:9">
+    <row r="98" spans="1:9" ht="60">
       <c r="A98" s="4" t="s">
         <v>4448</v>
       </c>
@@ -72035,7 +73173,7 @@
         <v>4605</v>
       </c>
     </row>
-    <row r="99" spans="1:9">
+    <row r="99" spans="1:9" ht="75">
       <c r="A99" s="4" t="s">
         <v>4448</v>
       </c>
@@ -72064,7 +73202,7 @@
         <v>4609</v>
       </c>
     </row>
-    <row r="100" spans="1:9">
+    <row r="100" spans="1:9" ht="75">
       <c r="A100" s="4" t="s">
         <v>4448</v>
       </c>
@@ -72093,7 +73231,7 @@
         <v>4613</v>
       </c>
     </row>
-    <row r="101" spans="1:9">
+    <row r="101" spans="1:9" ht="30">
       <c r="A101" s="4" t="s">
         <v>4455</v>
       </c>
@@ -72122,7 +73260,7 @@
         <v>4615</v>
       </c>
     </row>
-    <row r="102" spans="1:9">
+    <row r="102" spans="1:9" ht="30">
       <c r="A102" s="4" t="s">
         <v>4455</v>
       </c>
@@ -72151,7 +73289,7 @@
         <v>4619</v>
       </c>
     </row>
-    <row r="103" spans="1:9">
+    <row r="103" spans="1:9" ht="60">
       <c r="A103" s="4" t="s">
         <v>4455</v>
       </c>
@@ -72180,7 +73318,7 @@
         <v>4622</v>
       </c>
     </row>
-    <row r="104" spans="1:9">
+    <row r="104" spans="1:9" ht="30">
       <c r="A104" s="4" t="s">
         <v>4455</v>
       </c>
@@ -72209,7 +73347,7 @@
         <v>4625</v>
       </c>
     </row>
-    <row r="105" spans="1:9">
+    <row r="105" spans="1:9" ht="75">
       <c r="A105" s="4" t="s">
         <v>4455</v>
       </c>
@@ -72238,7 +73376,7 @@
         <v>4629</v>
       </c>
     </row>
-    <row r="106" spans="1:9">
+    <row r="106" spans="1:9" ht="75">
       <c r="A106" s="4" t="s">
         <v>4455</v>
       </c>

</xml_diff>